<commit_message>
Lauf 2026-08-05 02:27 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firmen entdeckt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$102</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$81</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L100"/>
+  <dimension ref="A1:L102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1506,27 +1506,23 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Digital Marketing &amp; Category Management</t>
+          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Benrath, Düsseldorf</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F21" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
+      <c r="G21" s="2" t="inlineStr"/>
       <c r="H21" s="2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1545,7 +1541,7 @@
       <c r="K21" s="2" t="inlineStr"/>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816415884?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1560,23 +1556,27 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich Marketing für die Marke BE-KIND DACH</t>
+          <t>Praktikum Digital Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Unterhaching, München (Kreis)</t>
+          <t>Benrath, Düsseldorf</t>
         </is>
       </c>
       <c r="F22" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="G22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1595,7 +1595,7 @@
       <c r="K22" s="2" t="inlineStr"/>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5752932983?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5816415884?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1610,17 +1610,17 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>P&amp;G</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum im Bereich Marketing für die Marke BE-KIND DACH</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Unterhaching, München (Kreis)</t>
         </is>
       </c>
       <c r="F23" s="2" t="n">
@@ -1645,7 +1645,7 @@
       <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5752932983?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1660,17 +1660,17 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>P&amp;G</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Category Management Non Food Vertrieb (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F24" s="2" t="n">
@@ -1695,7 +1695,7 @@
       <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5795118484?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1715,7 +1715,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Praktikum CNX Category Management Home &amp; Living (m/w/d)</t>
+          <t>Praktikum Category Management Non Food Vertrieb (m/w/d)</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1745,7 +1745,7 @@
       <c r="K25" s="2" t="inlineStr"/>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5765078175?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5795118484?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1765,7 +1765,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing Tchibo (m/w/d)</t>
+          <t>Praktikum CNX Category Management Home &amp; Living (m/w/d)</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1795,7 +1795,7 @@
       <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5744245447?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5765078175?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1815,7 +1815,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing Eduscho (m/w/d)</t>
+          <t>Praktikum Trade Marketing Tchibo (m/w/d)</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1845,7 +1845,7 @@
       <c r="K27" s="2" t="inlineStr"/>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5773205889?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5744245447?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1856,25 +1856,25 @@
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>Tchibo GmbH</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Trade Marketing Eduscho (m/w/d)</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G28" s="2" t="inlineStr"/>
       <c r="H28" s="2" t="inlineStr">
@@ -1895,7 +1895,7 @@
       <c r="K28" s="2" t="inlineStr"/>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5773205889?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1910,21 +1910,21 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>markenbaumarkt24</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
+          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Feuersbach, Siegen</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G29" s="2" t="inlineStr"/>
       <c r="H29" s="2" t="inlineStr">
@@ -1945,7 +1945,7 @@
       <c r="K29" s="2" t="inlineStr"/>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1956,24 +1956,26 @@
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>markenbaumarkt24</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr"/>
+          <t>Feuersbach, Siegen</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="G30" s="2" t="inlineStr"/>
       <c r="H30" s="2" t="inlineStr">
         <is>
@@ -1993,7 +1995,7 @@
       <c r="K30" s="2" t="inlineStr"/>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
+          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2004,26 +2006,24 @@
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="n">
-        <v>6</v>
-      </c>
+          <t>Hamburg, Deutschland</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr"/>
       <c r="G31" s="2" t="inlineStr"/>
       <c r="H31" s="2" t="inlineStr">
         <is>
@@ -2043,7 +2043,7 @@
       <c r="K31" s="2" t="inlineStr"/>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
         </is>
       </c>
     </row>
@@ -3604,19 +3604,15 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E63" s="2" t="inlineStr">
-        <is>
-          <t>Schwabing-Freimann, München</t>
-        </is>
-      </c>
+          <t>Marketing Intern - Trade Marketing</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr"/>
       <c r="F63" s="2" t="inlineStr"/>
       <c r="G63" s="2" t="inlineStr"/>
       <c r="H63" s="2" t="inlineStr">
@@ -3637,7 +3633,7 @@
       <c r="K63" s="2" t="inlineStr"/>
       <c r="L63" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
         </is>
       </c>
     </row>
@@ -3652,24 +3648,20 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="inlineStr">
-        <is>
-          <t>DEU-Bayern-Unterhaching</t>
-        </is>
-      </c>
+          <t>Operational Trade Marketing Intern</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr"/>
       <c r="F64" s="2" t="inlineStr"/>
       <c r="G64" s="2" t="inlineStr"/>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
@@ -3685,7 +3677,7 @@
       <c r="K64" s="2" t="inlineStr"/>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
+          <t>https://careers.coty.com/job/Toronto-Operational-Trade-Marketing-Intern-ON-M5H4H2/1397938633/</t>
         </is>
       </c>
     </row>
@@ -3700,17 +3692,17 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>Schwabing-Freimann, München</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr"/>
@@ -3733,7 +3725,7 @@
       <c r="K65" s="2" t="inlineStr"/>
       <c r="L65" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3748,24 +3740,24 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
+          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>DEU-Bayern-Unterhaching</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr"/>
       <c r="G66" s="2" t="inlineStr"/>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
@@ -3781,7 +3773,7 @@
       <c r="K66" s="2" t="inlineStr"/>
       <c r="L66" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
         </is>
       </c>
     </row>
@@ -3796,17 +3788,17 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr"/>
@@ -3829,7 +3821,7 @@
       <c r="K67" s="2" t="inlineStr"/>
       <c r="L67" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
+          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3849,7 +3841,7 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -3877,7 +3869,7 @@
       <c r="K68" s="2" t="inlineStr"/>
       <c r="L68" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
+          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
         </is>
       </c>
     </row>
@@ -3892,17 +3884,17 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr"/>
@@ -3925,7 +3917,7 @@
       <c r="K69" s="2" t="inlineStr"/>
       <c r="L69" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
         </is>
       </c>
     </row>
@@ -3936,21 +3928,21 @@
         </is>
       </c>
       <c r="B70" s="2" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>AUTO1 Global Services SE &amp; Co. KG</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (d/m/w)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr"/>
@@ -3973,7 +3965,7 @@
       <c r="K70" s="2" t="inlineStr"/>
       <c r="L70" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5789927805?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
         </is>
       </c>
     </row>
@@ -3984,21 +3976,21 @@
         </is>
       </c>
       <c r="B71" s="2" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Amolina</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr"/>
@@ -4021,7 +4013,7 @@
       <c r="K71" s="2" t="inlineStr"/>
       <c r="L71" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727292709?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4036,17 +4028,17 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>CTG Consulting</t>
+          <t>AUTO1 Global Services SE &amp; Co. KG</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Sales/Business Development // Hamburg oder Berlin</t>
+          <t>Praktikum Business Development (d/m/w)</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr"/>
@@ -4069,7 +4061,7 @@
       <c r="K72" s="2" t="inlineStr"/>
       <c r="L72" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5694221323?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5789927805?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4084,17 +4076,17 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Dronesperhour</t>
+          <t>Amolina</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development eines Startups (m/w/d)</t>
+          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>Mitte, Berlin</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr"/>
@@ -4117,7 +4109,7 @@
       <c r="K73" s="2" t="inlineStr"/>
       <c r="L73" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5669955732?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5727292709?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4132,17 +4124,17 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>GrantLift GmbH</t>
+          <t>CTG Consulting</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
+          <t>Praktikum Sales/Business Development // Hamburg oder Berlin</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr"/>
@@ -4165,7 +4157,7 @@
       <c r="K74" s="2" t="inlineStr"/>
       <c r="L74" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5803032426?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5694221323?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4180,17 +4172,17 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>GrantLift GmbH</t>
+          <t>Dronesperhour</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
+          <t>Praktikum im Business Development eines Startups (m/w/d)</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Mitte, Berlin</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr"/>
@@ -4213,7 +4205,7 @@
       <c r="K75" s="2" t="inlineStr"/>
       <c r="L75" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804575149?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5669955732?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4228,17 +4220,17 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Otto Group one.O GmbH</t>
+          <t>GrantLift GmbH</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Knowledge Management - Corporate Strategy (w/m/d)</t>
+          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr"/>
@@ -4261,7 +4253,7 @@
       <c r="K76" s="2" t="inlineStr"/>
       <c r="L76" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5809516963?se=mrUvpGeQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=7970F7260CB99374DD6661F2025E46043B457CE4</t>
+          <t>https://www.adzuna.de/details/5803032426?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4276,17 +4268,17 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Pflegia</t>
+          <t>GrantLift GmbH</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr"/>
@@ -4309,7 +4301,7 @@
       <c r="K77" s="2" t="inlineStr"/>
       <c r="L77" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5821302522?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804575149?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4324,17 +4316,17 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Pflegia</t>
+          <t>Otto Group one.O GmbH</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Praktikum im Knowledge Management - Corporate Strategy (w/m/d)</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr"/>
@@ -4357,7 +4349,7 @@
       <c r="K78" s="2" t="inlineStr"/>
       <c r="L78" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802953545?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5809516963?se=mrUvpGeQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=7970F7260CB99374DD6661F2025E46043B457CE4</t>
         </is>
       </c>
     </row>
@@ -4377,7 +4369,7 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (Projektmanagement &amp; Prozessoptimierung) (m/w/d)</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
@@ -4405,7 +4397,7 @@
       <c r="K79" s="2" t="inlineStr"/>
       <c r="L79" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802984051?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5821302522?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4425,12 +4417,12 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (Business Analyst/Automation Engineer/Applied AI Engineer) (m/w/d)</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr"/>
@@ -4453,7 +4445,7 @@
       <c r="K80" s="2" t="inlineStr"/>
       <c r="L80" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802977130?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802953545?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4468,17 +4460,17 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>REWE Group</t>
+          <t>Pflegia</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Praktikum im Business Development (Projektmanagement &amp; Prozessoptimierung) (m/w/d)</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Wedding, Berlin</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr"/>
@@ -4501,7 +4493,7 @@
       <c r="K81" s="2" t="inlineStr"/>
       <c r="L81" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5712965755?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802984051?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4516,17 +4508,17 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>SHAVENT - ARA Sustainable Products</t>
+          <t>Pflegia</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Business Development in nachhaltigem Start-Up (w/m/d) Remote in DE</t>
+          <t>Praktikum im Business Development (Business Analyst/Automation Engineer/Applied AI Engineer) (m/w/d)</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Sendling, München</t>
+          <t>Wedding, Berlin</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr"/>
@@ -4549,7 +4541,7 @@
       <c r="K82" s="2" t="inlineStr"/>
       <c r="L82" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802951937?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802977130?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4564,17 +4556,17 @@
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>SINN Power</t>
+          <t>REWE Group</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im AI Business Development (m/w/d)</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Kasten, München (Kreis)</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr"/>
@@ -4597,7 +4589,7 @@
       <c r="K83" s="2" t="inlineStr"/>
       <c r="L83" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727348338?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5712965755?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4612,17 +4604,17 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>SHAVENT - ARA Sustainable Products</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Strategy &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Business Development in nachhaltigem Start-Up (w/m/d) Remote in DE</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Sendling, München</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr"/>
@@ -4645,7 +4637,7 @@
       <c r="K84" s="2" t="inlineStr"/>
       <c r="L84" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5799516357?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802951937?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4660,17 +4652,17 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>Vitolus</t>
+          <t>SINN Power</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
+          <t>Praktikum im AI Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Kasten, München (Kreis)</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr"/>
@@ -4693,7 +4685,7 @@
       <c r="K85" s="2" t="inlineStr"/>
       <c r="L85" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5785872138?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5727348338?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4708,17 +4700,17 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Vivanta Gmbh</t>
+          <t>Tchibo GmbH</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Praktikum Strategy &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr"/>
@@ -4741,7 +4733,7 @@
       <c r="K86" s="2" t="inlineStr"/>
       <c r="L86" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802952325?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5799516357?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4756,17 +4748,17 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>Vivanta Gmbh</t>
+          <t>Vitolus</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr"/>
@@ -4789,7 +4781,7 @@
       <c r="K87" s="2" t="inlineStr"/>
       <c r="L87" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804549349?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5785872138?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4804,17 +4796,17 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Werkia</t>
+          <t>Vivanta Gmbh</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d) - Datenanalyse &amp; Automatisierung</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr"/>
@@ -4837,7 +4829,7 @@
       <c r="K88" s="2" t="inlineStr"/>
       <c r="L88" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802974922?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802952325?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4852,12 +4844,12 @@
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>Werkia</t>
+          <t>Vivanta Gmbh</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d) - Berlin</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
@@ -4885,7 +4877,7 @@
       <c r="K89" s="2" t="inlineStr"/>
       <c r="L89" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802950225?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804549349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4900,17 +4892,17 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>innpuls</t>
+          <t>Werkia</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/d) - Datenanalyse &amp; Automatisierung</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Wedding, Berlin</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr"/>
@@ -4933,7 +4925,7 @@
       <c r="K90" s="2" t="inlineStr"/>
       <c r="L90" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5735591887?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802974922?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4948,17 +4940,17 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>paero</t>
+          <t>Werkia</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im Business Development (m/w/d) - Berlin</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>Ludwigsvorstadt-Isarvorstadt, München</t>
+          <t>Wedding, Berlin</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr"/>
@@ -4981,7 +4973,7 @@
       <c r="K91" s="2" t="inlineStr"/>
       <c r="L91" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813846665?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802950225?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4992,21 +4984,21 @@
         </is>
       </c>
       <c r="B92" s="2" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>innpuls</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr"/>
@@ -5029,7 +5021,7 @@
       <c r="K92" s="2" t="inlineStr"/>
       <c r="L92" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5735591887?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5040,21 +5032,21 @@
         </is>
       </c>
       <c r="B93" s="2" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>paero</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>Altstadt-Nord, Köln</t>
+          <t>Ludwigsvorstadt-Isarvorstadt, München</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr"/>
@@ -5077,7 +5069,7 @@
       <c r="K93" s="2" t="inlineStr"/>
       <c r="L93" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5813846665?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5088,21 +5080,21 @@
         </is>
       </c>
       <c r="B94" s="2" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Devoteam G Cloud Germany</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr"/>
@@ -5125,7 +5117,7 @@
       <c r="K94" s="2" t="inlineStr"/>
       <c r="L94" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811135653?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5136,21 +5128,21 @@
         </is>
       </c>
       <c r="B95" s="2" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt-Nord, Köln</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr"/>
@@ -5173,7 +5165,7 @@
       <c r="K95" s="2" t="inlineStr"/>
       <c r="L95" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5188,12 +5180,12 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>Devoteam G Cloud Germany</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -5221,7 +5213,7 @@
       <c r="K96" s="2" t="inlineStr"/>
       <c r="L96" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5811135653?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5246,7 +5238,7 @@
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr"/>
@@ -5269,7 +5261,7 @@
       <c r="K97" s="2" t="inlineStr"/>
       <c r="L97" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5294,7 +5286,7 @@
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr"/>
@@ -5317,7 +5309,7 @@
       <c r="K98" s="2" t="inlineStr"/>
       <c r="L98" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5332,17 +5324,17 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>sailwithus</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr"/>
@@ -5365,7 +5357,7 @@
       <c r="K99" s="2" t="inlineStr"/>
       <c r="L99" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5380,12 +5372,12 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>sailwithus</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
@@ -5413,12 +5405,108 @@
       <c r="K100" s="2" t="inlineStr"/>
       <c r="L100" s="2" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>sailwithus</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr"/>
+      <c r="G101" s="2" t="inlineStr"/>
+      <c r="H101" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I101" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J101" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K101" s="2" t="inlineStr"/>
+      <c r="L101" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>sailwithus</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr"/>
+      <c r="G102" s="2" t="inlineStr"/>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I102" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J102" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K102" s="2" t="inlineStr"/>
+      <c r="L102" s="2" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5804544237?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L100"/>
+  <autoFilter ref="A1:L102"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5485,7 +5573,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2" t="n">
         <v>107</v>
@@ -5510,7 +5598,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C3" t="n">
         <v>91</v>
@@ -5535,7 +5623,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C4" t="n">
         <v>89</v>
@@ -5560,7 +5648,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C5" t="n">
         <v>84</v>
@@ -5585,7 +5673,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C6" t="n">
         <v>84</v>
@@ -5610,7 +5698,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C7" t="n">
         <v>84</v>
@@ -5635,7 +5723,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C8" t="n">
         <v>84</v>
@@ -5668,7 +5756,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C9" t="n">
         <v>84</v>
@@ -5693,7 +5781,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
@@ -5718,7 +5806,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C11" t="n">
         <v>80</v>
@@ -5743,7 +5831,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C12" t="n">
         <v>79</v>
@@ -5768,7 +5856,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C13" t="n">
         <v>79</v>
@@ -5793,7 +5881,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C14" t="n">
         <v>78</v>
@@ -5818,7 +5906,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C15" t="n">
         <v>78</v>
@@ -5851,7 +5939,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C16" t="n">
         <v>73</v>
@@ -5880,18 +5968,18 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>P&amp;G</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C17" t="n">
         <v>73</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
@@ -5905,18 +5993,18 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>markenbaumarkt24</t>
+          <t>P&amp;G</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C18" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
@@ -5930,18 +6018,18 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>markenbaumarkt24</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C19" t="n">
         <v>72</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
@@ -5955,18 +6043,18 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>3</v>
       </c>
       <c r="C20" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
@@ -5980,18 +6068,18 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C21" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
@@ -6005,22 +6093,30 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C22" t="n">
         <v>68</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
+          <t>Intern Category Growth</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>successfactors</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -6030,30 +6126,22 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C23" t="n">
         <v>68</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Intern Category Growth</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>successfactors</t>
-        </is>
-      </c>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -6067,7 +6155,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C24" t="n">
         <v>68</v>
@@ -6092,7 +6180,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C25" t="n">
         <v>68</v>
@@ -6117,7 +6205,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C26" t="n">
         <v>62</v>
@@ -6142,7 +6230,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C27" t="n">
         <v>62</v>
@@ -6167,7 +6255,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C28" t="n">
         <v>57</v>
@@ -6200,7 +6288,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C29" t="n">
         <v>56</v>
@@ -6225,7 +6313,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C30" t="n">
         <v>55</v>
@@ -6250,7 +6338,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C31" t="n">
         <v>54</v>
@@ -6275,7 +6363,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C32" t="n">
         <v>54</v>
@@ -6300,7 +6388,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C33" t="n">
         <v>54</v>
@@ -6325,7 +6413,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C34" t="n">
         <v>54</v>
@@ -6350,7 +6438,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C35" t="n">
         <v>53</v>
@@ -6375,7 +6463,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C36" t="n">
         <v>53</v>
@@ -6400,7 +6488,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C37" t="n">
         <v>53</v>
@@ -6425,7 +6513,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C38" t="n">
         <v>52</v>
@@ -6450,7 +6538,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C39" t="n">
         <v>51</v>
@@ -6475,7 +6563,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C40" t="n">
         <v>51</v>
@@ -6500,7 +6588,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C41" t="n">
         <v>51</v>
@@ -6525,7 +6613,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C42" t="n">
         <v>51</v>
@@ -6550,7 +6638,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C43" t="n">
         <v>51</v>
@@ -6575,7 +6663,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C44" t="n">
         <v>49</v>
@@ -6600,7 +6688,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C45" t="n">
         <v>49</v>
@@ -6625,7 +6713,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C46" t="n">
         <v>49</v>
@@ -6650,7 +6738,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C47" t="n">
         <v>49</v>
@@ -6675,7 +6763,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C48" t="n">
         <v>49</v>
@@ -6725,7 +6813,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C50" t="n">
         <v>48</v>
@@ -7075,7 +7163,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C64" t="n">
         <v>46</v>

</xml_diff>

<commit_message>
Lauf 2026-08-05 08:43 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firmen entdeckt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$102</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$103</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$82</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L102"/>
+  <dimension ref="A1:L103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1502,26 +1502,24 @@
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>Miles &amp; More GmbH</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
+          <t>Internship Marketing Strategy &amp; Delivery</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="n">
-        <v>6</v>
-      </c>
+          <t>Flughafen, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr"/>
       <c r="G21" s="2" t="inlineStr"/>
       <c r="H21" s="2" t="inlineStr">
         <is>
@@ -1541,7 +1539,7 @@
       <c r="K21" s="2" t="inlineStr"/>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5828674997?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1556,27 +1554,23 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Digital Marketing &amp; Category Management</t>
+          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Benrath, Düsseldorf</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F22" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
+      <c r="G22" s="2" t="inlineStr"/>
       <c r="H22" s="2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1595,7 +1589,7 @@
       <c r="K22" s="2" t="inlineStr"/>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816415884?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1610,23 +1604,27 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich Marketing für die Marke BE-KIND DACH</t>
+          <t>Praktikum Digital Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Unterhaching, München (Kreis)</t>
+          <t>Benrath, Düsseldorf</t>
         </is>
       </c>
       <c r="F23" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="G23" s="2" t="inlineStr"/>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1645,7 +1643,7 @@
       <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5752932983?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5816415884?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1660,17 +1658,17 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>P&amp;G</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum im Bereich Marketing für die Marke BE-KIND DACH</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Unterhaching, München (Kreis)</t>
         </is>
       </c>
       <c r="F24" s="2" t="n">
@@ -1695,7 +1693,7 @@
       <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5752932983?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1710,17 +1708,17 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>P&amp;G</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Category Management Non Food Vertrieb (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F25" s="2" t="n">
@@ -1745,7 +1743,7 @@
       <c r="K25" s="2" t="inlineStr"/>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5795118484?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1765,7 +1763,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Praktikum CNX Category Management Home &amp; Living (m/w/d)</t>
+          <t>Praktikum Category Management Non Food Vertrieb (m/w/d)</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1795,7 +1793,7 @@
       <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5765078175?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5795118484?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1815,7 +1813,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing Tchibo (m/w/d)</t>
+          <t>Praktikum CNX Category Management Home &amp; Living (m/w/d)</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1845,7 +1843,7 @@
       <c r="K27" s="2" t="inlineStr"/>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5744245447?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5765078175?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1865,7 +1863,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing Eduscho (m/w/d)</t>
+          <t>Praktikum Trade Marketing Tchibo (m/w/d)</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1895,7 +1893,7 @@
       <c r="K28" s="2" t="inlineStr"/>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5773205889?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5744245447?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1906,25 +1904,25 @@
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>Tchibo GmbH</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Trade Marketing Eduscho (m/w/d)</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G29" s="2" t="inlineStr"/>
       <c r="H29" s="2" t="inlineStr">
@@ -1945,7 +1943,7 @@
       <c r="K29" s="2" t="inlineStr"/>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5773205889?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1960,21 +1958,21 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>markenbaumarkt24</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
+          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Feuersbach, Siegen</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G30" s="2" t="inlineStr"/>
       <c r="H30" s="2" t="inlineStr">
@@ -1995,7 +1993,7 @@
       <c r="K30" s="2" t="inlineStr"/>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2006,24 +2004,26 @@
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>markenbaumarkt24</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr"/>
+          <t>Feuersbach, Siegen</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="G31" s="2" t="inlineStr"/>
       <c r="H31" s="2" t="inlineStr">
         <is>
@@ -2043,7 +2043,7 @@
       <c r="K31" s="2" t="inlineStr"/>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
+          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2054,26 +2054,24 @@
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="n">
-        <v>6</v>
-      </c>
+          <t>Hamburg, Deutschland</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr"/>
       <c r="G32" s="2" t="inlineStr"/>
       <c r="H32" s="2" t="inlineStr">
         <is>
@@ -2093,7 +2091,7 @@
       <c r="K32" s="2" t="inlineStr"/>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
         </is>
       </c>
     </row>
@@ -2113,7 +2111,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
+          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -2124,11 +2122,7 @@
       <c r="F33" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="G33" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G33" s="2" t="inlineStr"/>
       <c r="H33" s="2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2147,7 +2141,7 @@
       <c r="K33" s="2" t="inlineStr"/>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2162,17 +2156,17 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Bosch Thermotechnik GmbH</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im internationalen Brand Management</t>
+          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Wernau (Neckar), Esslingen (Kreis)</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F34" s="2" t="n">
@@ -2180,7 +2174,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -2201,7 +2195,7 @@
       <c r="K34" s="2" t="inlineStr"/>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5799981240?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2216,17 +2210,17 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Bosch Thermotechnik GmbH</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Intern Category Growth</t>
+          <t>Praktikum im internationalen Brand Management</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Darmstadt, Hessen</t>
+          <t>Wernau (Neckar), Esslingen (Kreis)</t>
         </is>
       </c>
       <c r="F35" s="2" t="n">
@@ -2234,7 +2228,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>2025-08-15</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -2255,7 +2249,7 @@
       <c r="K35" s="2" t="inlineStr"/>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5754086625?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5799981240?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2270,17 +2264,17 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>L’ORÉAL</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>PRAKTIKUM (M/W/D) Product Marketing - Start ab August/September/Oktober für 6 Monate</t>
+          <t>Intern Category Growth</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Nordrhein-Westfalen, Deutschland</t>
+          <t>Darmstadt, Hessen</t>
         </is>
       </c>
       <c r="F36" s="2" t="n">
@@ -2288,7 +2282,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2025-08-15</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -2309,7 +2303,7 @@
       <c r="K36" s="2" t="inlineStr"/>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5754061318?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5754086625?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2324,17 +2318,17 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>L’ORÉAL</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>PRAKTIKUM (M/W/D) Product Marketing - Start ab August/September/Oktober für 6 Monate</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Nordrhein-Westfalen, Deutschland</t>
         </is>
       </c>
       <c r="F37" s="2" t="n">
@@ -2363,7 +2357,7 @@
       <c r="K37" s="2" t="inlineStr"/>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5754061318?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2378,17 +2372,17 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>coty</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Darmstadt, Hessen</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F38" s="2" t="n">
@@ -2396,7 +2390,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>2025-08-15</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2417,7 +2411,7 @@
       <c r="K38" s="2" t="inlineStr"/>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2428,27 +2422,29 @@
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>coty</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>Marketing Intern - Trade Marketing</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F39" s="2" t="inlineStr"/>
+          <t>Darmstadt, Hessen</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>6</v>
+      </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2025-08-15</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2469,7 +2465,7 @@
       <c r="K39" s="2" t="inlineStr"/>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5822943276?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=580C236799B96DFD395A1EC1CBBF7474C7F58435</t>
+          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2480,25 +2476,29 @@
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr"/>
-      <c r="G40" s="2" t="inlineStr"/>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2517,7 +2517,7 @@
       <c r="K40" s="2" t="inlineStr"/>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5822943276?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=580C236799B96DFD395A1EC1CBBF7474C7F58435</t>
         </is>
       </c>
     </row>
@@ -2542,7 +2542,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Altstadt, Düsseldorf</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr"/>
@@ -2565,7 +2565,7 @@
       <c r="K41" s="2" t="inlineStr"/>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2580,17 +2580,17 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Calypso Ventures GmbH</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Altstadt, Düsseldorf</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr"/>
@@ -2613,7 +2613,7 @@
       <c r="K42" s="2" t="inlineStr"/>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2624,28 +2624,28 @@
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Calypso Ventures GmbH</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
+          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr"/>
       <c r="G43" s="2" t="inlineStr"/>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
@@ -2661,7 +2661,7 @@
       <c r="K43" s="2" t="inlineStr"/>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
+          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2672,28 +2672,28 @@
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr"/>
       <c r="G44" s="2" t="inlineStr"/>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
@@ -2709,7 +2709,7 @@
       <c r="K44" s="2" t="inlineStr"/>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
         </is>
       </c>
     </row>
@@ -2734,7 +2734,7 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr"/>
@@ -2757,7 +2757,7 @@
       <c r="K45" s="2" t="inlineStr"/>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2768,21 +2768,21 @@
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Sayano Deutschland GmbH</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr"/>
@@ -2805,7 +2805,7 @@
       <c r="K46" s="2" t="inlineStr"/>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816572451?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2816,21 +2816,21 @@
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Abrio</t>
+          <t>Sayano Deutschland GmbH</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
+          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Mitte, Stuttgart</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr"/>
@@ -2853,7 +2853,7 @@
       <c r="K47" s="2" t="inlineStr"/>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5816572451?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2868,17 +2868,17 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>Abrio</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Internship International Marketing Schwarzkopf Coloration - Legacy Brands</t>
+          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Benrath, Düsseldorf</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr"/>
@@ -2901,7 +2901,7 @@
       <c r="K48" s="2" t="inlineStr"/>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5819890143?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2916,22 +2916,20 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Lidl Stiftung</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food in Neckarsulm</t>
+          <t>Internship International Marketing Schwarzkopf Coloration - Legacy Brands</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F49" s="2" t="n">
-        <v>6</v>
-      </c>
+          <t>Benrath, Düsseldorf</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr"/>
       <c r="G49" s="2" t="inlineStr"/>
       <c r="H49" s="2" t="inlineStr">
         <is>
@@ -2951,7 +2949,7 @@
       <c r="K49" s="2" t="inlineStr"/>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813494719?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5819890143?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2966,12 +2964,12 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Lidl Stiftung &amp; Co. KG</t>
+          <t>Lidl Stiftung</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food in Neckarsulm</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -2979,7 +2977,9 @@
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="F50" s="2" t="inlineStr"/>
+      <c r="F50" s="2" t="n">
+        <v>6</v>
+      </c>
       <c r="G50" s="2" t="inlineStr"/>
       <c r="H50" s="2" t="inlineStr">
         <is>
@@ -2999,7 +2999,7 @@
       <c r="K50" s="2" t="inlineStr"/>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
+          <t>https://www.adzuna.de/details/5813494719?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3014,12 +3014,12 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Marc O'Polo</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -3028,11 +3028,7 @@
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr"/>
-      <c r="G51" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
+      <c r="G51" s="2" t="inlineStr"/>
       <c r="H51" s="2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3051,7 +3047,7 @@
       <c r="K51" s="2" t="inlineStr"/>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
         </is>
       </c>
     </row>
@@ -3066,21 +3062,25 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>Marc O'Polo</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Marketing (m/w/d)</t>
+          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr"/>
-      <c r="G52" s="2" t="inlineStr"/>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3099,7 +3099,7 @@
       <c r="K52" s="2" t="inlineStr"/>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899691?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3114,7 +3114,7 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -3124,14 +3124,14 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr"/>
       <c r="G53" s="2" t="inlineStr"/>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
@@ -3147,7 +3147,7 @@
       <c r="K53" s="2" t="inlineStr"/>
       <c r="L53" s="2" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
+          <t>https://www.adzuna.de/details/5802899691?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3158,34 +3158,28 @@
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>LIGANOVA I Karriere</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Buying (all genders) – August/September 2026</t>
+          <t>Praktikum Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
-        </is>
-      </c>
-      <c r="F54" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="G54" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+          <t>Frankfurt am Main, DE, 60329</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr"/>
+      <c r="G54" s="2" t="inlineStr"/>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
@@ -3201,7 +3195,7 @@
       <c r="K54" s="2" t="inlineStr"/>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805407495?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
         </is>
       </c>
     </row>
@@ -3216,24 +3210,30 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>LIGANOVA I Karriere</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Marketing &amp; Merchandising Assistant Trainee</t>
+          <t>Praktikum Buying (all genders) – August/September 2026</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>MILAN</t>
-        </is>
-      </c>
-      <c r="F55" s="2" t="inlineStr"/>
-      <c r="G55" s="2" t="inlineStr"/>
+          <t>Mitte, Stuttgart</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
@@ -3249,7 +3249,7 @@
       <c r="K55" s="2" t="inlineStr"/>
       <c r="L55" s="2" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
+          <t>https://www.adzuna.de/details/5805407495?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3269,7 +3269,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Marketing and Merchandising Assistant Trainee</t>
+          <t>Marketing &amp; Merchandising Assistant Trainee</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -3297,7 +3297,7 @@
       <c r="K56" s="2" t="inlineStr"/>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing-and-Merchandising-Assistant-Trainee_JR128690</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
         </is>
       </c>
     </row>
@@ -3308,28 +3308,28 @@
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Digitalagenten</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
+          <t>Marketing and Merchandising Assistant Trainee</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Charlottenburg, Berlin</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr"/>
       <c r="G57" s="2" t="inlineStr"/>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr">
@@ -3345,7 +3345,7 @@
       <c r="K57" s="2" t="inlineStr"/>
       <c r="L57" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804948828?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing-and-Merchandising-Assistant-Trainee_JR128690</t>
         </is>
       </c>
     </row>
@@ -3360,17 +3360,17 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>LIMITD by Wunderproducts GmbH</t>
+          <t>Digitalagenten</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Kreuzberg, Berlin</t>
+          <t>Charlottenburg, Berlin</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr"/>
@@ -3393,7 +3393,7 @@
       <c r="K58" s="2" t="inlineStr"/>
       <c r="L58" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804948828?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3408,25 +3408,21 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers GmbH WPG</t>
+          <t>LIMITD by Wunderproducts GmbH</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Kreuzberg, Berlin</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr"/>
-      <c r="G59" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
+      <c r="G59" s="2" t="inlineStr"/>
       <c r="H59" s="2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3445,7 +3441,7 @@
       <c r="K59" s="2" t="inlineStr"/>
       <c r="L59" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3460,21 +3456,25 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>THE VERSE Ventures</t>
+          <t>PricewaterhouseCoopers GmbH WPG</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr"/>
-      <c r="G60" s="2" t="inlineStr"/>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3493,7 +3493,7 @@
       <c r="K60" s="2" t="inlineStr"/>
       <c r="L60" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3508,17 +3508,17 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>WirWinzer</t>
+          <t>THE VERSE Ventures</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Business Development Weinhandel (all genders)</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr"/>
@@ -3541,7 +3541,7 @@
       <c r="K61" s="2" t="inlineStr"/>
       <c r="L61" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3552,21 +3552,21 @@
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Brand Trust</t>
+          <t>WirWinzer</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
+          <t>Praktikum Business Development Weinhandel (all genders)</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Gleißbühl, Nürnberg</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr"/>
@@ -3589,7 +3589,7 @@
       <c r="K62" s="2" t="inlineStr"/>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5669847401?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3604,15 +3604,19 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Brand Trust</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
-        </is>
-      </c>
-      <c r="E63" s="2" t="inlineStr"/>
+          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>Gleißbühl, Nürnberg</t>
+        </is>
+      </c>
       <c r="F63" s="2" t="inlineStr"/>
       <c r="G63" s="2" t="inlineStr"/>
       <c r="H63" s="2" t="inlineStr">
@@ -3633,7 +3637,7 @@
       <c r="K63" s="2" t="inlineStr"/>
       <c r="L63" s="2" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
+          <t>https://www.adzuna.de/details/5669847401?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3653,7 +3657,7 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Operational Trade Marketing Intern</t>
+          <t>Marketing Intern - Trade Marketing</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr"/>
@@ -3677,7 +3681,7 @@
       <c r="K64" s="2" t="inlineStr"/>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Toronto-Operational-Trade-Marketing-Intern-ON-M5H4H2/1397938633/</t>
+          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
         </is>
       </c>
     </row>
@@ -3692,19 +3696,15 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="inlineStr">
-        <is>
-          <t>Schwabing-Freimann, München</t>
-        </is>
-      </c>
+          <t>Operational Trade Marketing Intern</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr"/>
       <c r="F65" s="2" t="inlineStr"/>
       <c r="G65" s="2" t="inlineStr"/>
       <c r="H65" s="2" t="inlineStr">
@@ -3725,7 +3725,7 @@
       <c r="K65" s="2" t="inlineStr"/>
       <c r="L65" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://careers.coty.com/job/Toronto-Operational-Trade-Marketing-Intern-ON-M5H4H2/1397938633/</t>
         </is>
       </c>
     </row>
@@ -3740,24 +3740,24 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>DEU-Bayern-Unterhaching</t>
+          <t>Schwabing-Freimann, München</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr"/>
       <c r="G66" s="2" t="inlineStr"/>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
@@ -3773,7 +3773,7 @@
       <c r="K66" s="2" t="inlineStr"/>
       <c r="L66" s="2" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
+          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3788,24 +3788,24 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>DEU-Bayern-Unterhaching</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr"/>
       <c r="G67" s="2" t="inlineStr"/>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
@@ -3821,7 +3821,7 @@
       <c r="K67" s="2" t="inlineStr"/>
       <c r="L67" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
         </is>
       </c>
     </row>
@@ -3836,17 +3836,17 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr"/>
@@ -3869,7 +3869,7 @@
       <c r="K68" s="2" t="inlineStr"/>
       <c r="L68" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
+          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3889,7 +3889,7 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
@@ -3917,7 +3917,7 @@
       <c r="K69" s="2" t="inlineStr"/>
       <c r="L69" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
+          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
         </is>
       </c>
     </row>
@@ -3937,7 +3937,7 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -3965,7 +3965,7 @@
       <c r="K70" s="2" t="inlineStr"/>
       <c r="L70" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
+          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
         </is>
       </c>
     </row>
@@ -3980,17 +3980,17 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr"/>
@@ -4013,7 +4013,7 @@
       <c r="K71" s="2" t="inlineStr"/>
       <c r="L71" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
         </is>
       </c>
     </row>
@@ -4024,21 +4024,21 @@
         </is>
       </c>
       <c r="B72" s="2" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>AUTO1 Global Services SE &amp; Co. KG</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (d/m/w)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr"/>
@@ -4061,7 +4061,7 @@
       <c r="K72" s="2" t="inlineStr"/>
       <c r="L72" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5789927805?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4076,17 +4076,17 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Amolina</t>
+          <t>AUTO1 Global Services SE &amp; Co. KG</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
+          <t>Praktikum Business Development (d/m/w)</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr"/>
@@ -4109,7 +4109,7 @@
       <c r="K73" s="2" t="inlineStr"/>
       <c r="L73" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727292709?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5789927805?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4124,17 +4124,17 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>CTG Consulting</t>
+          <t>Amolina</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Sales/Business Development // Hamburg oder Berlin</t>
+          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr"/>
@@ -4157,7 +4157,7 @@
       <c r="K74" s="2" t="inlineStr"/>
       <c r="L74" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5694221323?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5727292709?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4172,17 +4172,17 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Dronesperhour</t>
+          <t>CTG Consulting</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development eines Startups (m/w/d)</t>
+          <t>Praktikum Sales/Business Development // Hamburg oder Berlin</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Mitte, Berlin</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr"/>
@@ -4205,7 +4205,7 @@
       <c r="K75" s="2" t="inlineStr"/>
       <c r="L75" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5669955732?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5694221323?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4220,17 +4220,17 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>GrantLift GmbH</t>
+          <t>Dronesperhour</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
+          <t>Praktikum im Business Development eines Startups (m/w/d)</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Mitte, Berlin</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr"/>
@@ -4253,7 +4253,7 @@
       <c r="K76" s="2" t="inlineStr"/>
       <c r="L76" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5803032426?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5669955732?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4278,7 +4278,7 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr"/>
@@ -4301,7 +4301,7 @@
       <c r="K77" s="2" t="inlineStr"/>
       <c r="L77" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804575149?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5803032426?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4316,17 +4316,17 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Otto Group one.O GmbH</t>
+          <t>GrantLift GmbH</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Knowledge Management - Corporate Strategy (w/m/d)</t>
+          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr"/>
@@ -4349,7 +4349,7 @@
       <c r="K78" s="2" t="inlineStr"/>
       <c r="L78" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5809516963?se=mrUvpGeQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=7970F7260CB99374DD6661F2025E46043B457CE4</t>
+          <t>https://www.adzuna.de/details/5804575149?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4364,17 +4364,17 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>Pflegia</t>
+          <t>Otto Group one.O GmbH</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Praktikum im Knowledge Management - Corporate Strategy (w/m/d)</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr"/>
@@ -4397,7 +4397,7 @@
       <c r="K79" s="2" t="inlineStr"/>
       <c r="L79" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5821302522?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5809516963?se=mrUvpGeQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=7970F7260CB99374DD6661F2025E46043B457CE4</t>
         </is>
       </c>
     </row>
@@ -4422,7 +4422,7 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Wedding, Berlin</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr"/>
@@ -4445,7 +4445,7 @@
       <c r="K80" s="2" t="inlineStr"/>
       <c r="L80" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802953545?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5821302522?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4465,12 +4465,12 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (Projektmanagement &amp; Prozessoptimierung) (m/w/d)</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr"/>
@@ -4493,7 +4493,7 @@
       <c r="K81" s="2" t="inlineStr"/>
       <c r="L81" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802984051?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802953545?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4513,7 +4513,7 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (Business Analyst/Automation Engineer/Applied AI Engineer) (m/w/d)</t>
+          <t>Praktikum im Business Development (Projektmanagement &amp; Prozessoptimierung) (m/w/d)</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
@@ -4541,7 +4541,7 @@
       <c r="K82" s="2" t="inlineStr"/>
       <c r="L82" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802977130?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802984051?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4556,17 +4556,17 @@
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>REWE Group</t>
+          <t>Pflegia</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Praktikum im Business Development (Business Analyst/Automation Engineer/Applied AI Engineer) (m/w/d)</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Wedding, Berlin</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr"/>
@@ -4589,7 +4589,7 @@
       <c r="K83" s="2" t="inlineStr"/>
       <c r="L83" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5712965755?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802977130?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4604,17 +4604,17 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>SHAVENT - ARA Sustainable Products</t>
+          <t>REWE Group</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Business Development in nachhaltigem Start-Up (w/m/d) Remote in DE</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Sendling, München</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr"/>
@@ -4637,7 +4637,7 @@
       <c r="K84" s="2" t="inlineStr"/>
       <c r="L84" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802951937?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5712965755?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4652,17 +4652,17 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>SINN Power</t>
+          <t>SHAVENT - ARA Sustainable Products</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im AI Business Development (m/w/d)</t>
+          <t>Praktikum Business Development in nachhaltigem Start-Up (w/m/d) Remote in DE</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Kasten, München (Kreis)</t>
+          <t>Sendling, München</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr"/>
@@ -4685,7 +4685,7 @@
       <c r="K85" s="2" t="inlineStr"/>
       <c r="L85" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727348338?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802951937?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4700,17 +4700,17 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>SINN Power</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Strategy &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im AI Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Kasten, München (Kreis)</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr"/>
@@ -4733,7 +4733,7 @@
       <c r="K86" s="2" t="inlineStr"/>
       <c r="L86" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5799516357?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5727348338?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4748,17 +4748,17 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>Vitolus</t>
+          <t>Tchibo GmbH</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
+          <t>Praktikum Strategy &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr"/>
@@ -4781,7 +4781,7 @@
       <c r="K87" s="2" t="inlineStr"/>
       <c r="L87" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5785872138?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5799516357?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4796,17 +4796,17 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Vivanta Gmbh</t>
+          <t>Vitolus</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr"/>
@@ -4829,7 +4829,7 @@
       <c r="K88" s="2" t="inlineStr"/>
       <c r="L88" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802952325?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5785872138?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4854,7 +4854,7 @@
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr"/>
@@ -4877,7 +4877,7 @@
       <c r="K89" s="2" t="inlineStr"/>
       <c r="L89" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804549349?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802952325?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4892,12 +4892,12 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Werkia</t>
+          <t>Vivanta Gmbh</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d) - Datenanalyse &amp; Automatisierung</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -4925,7 +4925,7 @@
       <c r="K90" s="2" t="inlineStr"/>
       <c r="L90" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802974922?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804549349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4945,7 +4945,7 @@
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d) - Berlin</t>
+          <t>Praktikum Business Development (m/w/d) - Datenanalyse &amp; Automatisierung</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
@@ -4973,7 +4973,7 @@
       <c r="K91" s="2" t="inlineStr"/>
       <c r="L91" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802950225?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802974922?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4988,17 +4988,17 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>innpuls</t>
+          <t>Werkia</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Praktikum im Business Development (m/w/d) - Berlin</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Wedding, Berlin</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr"/>
@@ -5021,7 +5021,7 @@
       <c r="K92" s="2" t="inlineStr"/>
       <c r="L92" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5735591887?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802950225?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5036,17 +5036,17 @@
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>paero</t>
+          <t>innpuls</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>Ludwigsvorstadt-Isarvorstadt, München</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr"/>
@@ -5069,7 +5069,7 @@
       <c r="K93" s="2" t="inlineStr"/>
       <c r="L93" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813846665?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5735591887?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5080,21 +5080,21 @@
         </is>
       </c>
       <c r="B94" s="2" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>paero</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Ludwigsvorstadt-Isarvorstadt, München</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr"/>
@@ -5117,7 +5117,7 @@
       <c r="K94" s="2" t="inlineStr"/>
       <c r="L94" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5813846665?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5142,7 +5142,7 @@
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>Altstadt-Nord, Köln</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr"/>
@@ -5165,7 +5165,7 @@
       <c r="K95" s="2" t="inlineStr"/>
       <c r="L95" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5176,21 +5176,21 @@
         </is>
       </c>
       <c r="B96" s="2" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>Devoteam G Cloud Germany</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt-Nord, Köln</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr"/>
@@ -5213,7 +5213,7 @@
       <c r="K96" s="2" t="inlineStr"/>
       <c r="L96" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811135653?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5228,12 +5228,12 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>Devoteam G Cloud Germany</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
@@ -5261,7 +5261,7 @@
       <c r="K97" s="2" t="inlineStr"/>
       <c r="L97" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5811135653?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5281,7 +5281,7 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
@@ -5309,7 +5309,7 @@
       <c r="K98" s="2" t="inlineStr"/>
       <c r="L98" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5329,12 +5329,12 @@
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr"/>
@@ -5357,7 +5357,7 @@
       <c r="K99" s="2" t="inlineStr"/>
       <c r="L99" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5377,7 +5377,7 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
@@ -5405,7 +5405,7 @@
       <c r="K100" s="2" t="inlineStr"/>
       <c r="L100" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5420,17 +5420,17 @@
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>sailwithus</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr"/>
@@ -5453,7 +5453,7 @@
       <c r="K101" s="2" t="inlineStr"/>
       <c r="L101" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5478,7 +5478,7 @@
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr"/>
@@ -5501,12 +5501,60 @@
       <c r="K102" s="2" t="inlineStr"/>
       <c r="L102" s="2" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>sailwithus</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr"/>
+      <c r="G103" s="2" t="inlineStr"/>
+      <c r="H103" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I103" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J103" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K103" s="2" t="inlineStr"/>
+      <c r="L103" s="2" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5804544237?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L102"/>
+  <autoFilter ref="A1:L103"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5517,7 +5565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G81"/>
+  <dimension ref="A1:G82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -5573,7 +5621,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C2" t="n">
         <v>107</v>
@@ -5598,7 +5646,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C3" t="n">
         <v>91</v>
@@ -5623,7 +5671,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C4" t="n">
         <v>89</v>
@@ -5644,11 +5692,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C5" t="n">
         <v>84</v>
@@ -5669,11 +5717,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C6" t="n">
         <v>84</v>
@@ -5694,22 +5742,30 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Nestle</t>
+          <t>Picnic</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C7" t="n">
         <v>84</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
+          <t>Category Management Praktikum (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>smartrecruiters</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -5719,30 +5775,22 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Picnic</t>
+          <t>Nestle</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C8" t="n">
         <v>84</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Category Management Praktikum (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>smartrecruiters</t>
-        </is>
-      </c>
+          <t>Praktikum Brand Management (m/w/d(</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -5756,7 +5804,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C9" t="n">
         <v>84</v>
@@ -5781,7 +5829,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
@@ -5806,7 +5854,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C11" t="n">
         <v>80</v>
@@ -5831,7 +5879,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C12" t="n">
         <v>79</v>
@@ -5856,7 +5904,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C13" t="n">
         <v>79</v>
@@ -5881,7 +5929,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C14" t="n">
         <v>78</v>
@@ -5906,7 +5954,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C15" t="n">
         <v>78</v>
@@ -5935,30 +5983,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>Miles &amp; More GmbH</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="C16" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Praktikum Category Management Non Food Vertrieb (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>successfactors</t>
-        </is>
-      </c>
+          <t>Internship Marketing Strategy &amp; Delivery</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -5968,22 +6008,30 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>Tchibo GmbH</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="C17" t="n">
         <v>73</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
+          <t>Praktikum Category Management Non Food Vertrieb (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>successfactors</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -5993,18 +6041,18 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>P&amp;G</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="C18" t="n">
         <v>73</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
@@ -6018,18 +6066,18 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>markenbaumarkt24</t>
+          <t>P&amp;G</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C19" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
@@ -6043,18 +6091,18 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>markenbaumarkt24</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C20" t="n">
         <v>72</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
@@ -6068,18 +6116,18 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>4</v>
       </c>
       <c r="C21" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
@@ -6093,30 +6141,22 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C22" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Intern Category Growth</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>successfactors</t>
-        </is>
-      </c>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -6126,22 +6166,30 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C23" t="n">
         <v>68</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
+          <t>Intern Category Growth</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>successfactors</t>
+        </is>
+      </c>
       <c r="G23" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -6151,18 +6199,18 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Bosch Thermotechnik GmbH</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C24" t="n">
         <v>68</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Praktikum im internationalen Brand Management</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr"/>
@@ -6176,18 +6224,18 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>L’ORÉAL</t>
+          <t>Bosch Thermotechnik GmbH</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C25" t="n">
         <v>68</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>PRAKTIKUM (M/W/D) Product Marketing - Start ab August/September/Oktober für 6 Monate</t>
+          <t>Praktikum im internationalen Brand Management</t>
         </is>
       </c>
       <c r="E25" t="inlineStr"/>
@@ -6201,18 +6249,18 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>L’ORÉAL</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C26" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>PRAKTIKUM (M/W/D) Product Marketing - Start ab August/September/Oktober für 6 Monate</t>
         </is>
       </c>
       <c r="E26" t="inlineStr"/>
@@ -6226,18 +6274,18 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Calypso Ventures GmbH</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C27" t="n">
         <v>62</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr"/>
@@ -6251,30 +6299,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Calypso Ventures GmbH</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C28" t="n">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>workday</t>
-        </is>
-      </c>
+          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -6284,22 +6324,30 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C29" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
+          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>workday</t>
+        </is>
+      </c>
       <c r="G29" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -6309,18 +6357,18 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Sayano Deutschland GmbH</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C30" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E30" t="inlineStr"/>
@@ -6334,18 +6382,18 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Lidl Stiftung &amp; Co. KG</t>
+          <t>Sayano Deutschland GmbH</t>
         </is>
       </c>
       <c r="B31" t="n">
         <v>4</v>
       </c>
       <c r="C31" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
@@ -6359,18 +6407,18 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Marc O'Polo</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C32" t="n">
         <v>54</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E32" t="inlineStr"/>
@@ -6384,18 +6432,18 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Abrio</t>
+          <t>Marc O'Polo</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C33" t="n">
         <v>54</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
+          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
         </is>
       </c>
       <c r="E33" t="inlineStr"/>
@@ -6409,18 +6457,18 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Lidl Stiftung</t>
+          <t>Abrio</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C34" t="n">
         <v>54</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food in Neckarsulm</t>
+          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
@@ -6434,18 +6482,18 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>Lidl Stiftung</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="C35" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food in Neckarsulm</t>
         </is>
       </c>
       <c r="E35" t="inlineStr"/>
@@ -6459,18 +6507,18 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>sailwithus</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="C36" t="n">
         <v>53</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr"/>
@@ -6484,18 +6532,18 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Devoteam G Cloud Germany</t>
+          <t>sailwithus</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C37" t="n">
         <v>53</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
         </is>
       </c>
       <c r="E37" t="inlineStr"/>
@@ -6509,18 +6557,18 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>LIGANOVA I Karriere</t>
+          <t>Devoteam G Cloud Germany</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C38" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Praktikum Buying (all genders) – August/September 2026</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr"/>
@@ -6534,18 +6582,18 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>LIMITD by Wunderproducts GmbH</t>
+          <t>LIGANOVA I Karriere</t>
         </is>
       </c>
       <c r="B39" t="n">
         <v>4</v>
       </c>
       <c r="C39" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Praktikum Buying (all genders) – August/September 2026</t>
         </is>
       </c>
       <c r="E39" t="inlineStr"/>
@@ -6559,11 +6607,11 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>THE VERSE Ventures</t>
+          <t>LIMITD by Wunderproducts GmbH</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C40" t="n">
         <v>51</v>
@@ -6584,18 +6632,18 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>WirWinzer</t>
+          <t>THE VERSE Ventures</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C41" t="n">
         <v>51</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Praktikum Business Development Weinhandel (all genders)</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr"/>
@@ -6609,18 +6657,18 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers GmbH WPG</t>
+          <t>WirWinzer</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C42" t="n">
         <v>51</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
+          <t>Praktikum Business Development Weinhandel (all genders)</t>
         </is>
       </c>
       <c r="E42" t="inlineStr"/>
@@ -6634,18 +6682,18 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Digitalagenten</t>
+          <t>PricewaterhouseCoopers GmbH WPG</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C43" t="n">
         <v>51</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr"/>
@@ -6659,18 +6707,18 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Digitalagenten</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C44" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
+          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr"/>
@@ -6684,18 +6732,18 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Brand Trust</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="C45" t="n">
         <v>49</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
+          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr"/>
@@ -6709,18 +6757,18 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>Brand Trust</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C46" t="n">
         <v>49</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
         </is>
       </c>
       <c r="E46" t="inlineStr"/>
@@ -6734,18 +6782,18 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C47" t="n">
         <v>49</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
@@ -6759,18 +6807,18 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C48" t="n">
         <v>49</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
@@ -6784,18 +6832,18 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Pflegia</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C49" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr"/>
@@ -6809,18 +6857,18 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>REWE Group</t>
+          <t>Pflegia</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C50" t="n">
         <v>48</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
@@ -6834,18 +6882,18 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Werkia</t>
+          <t>REWE Group</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C51" t="n">
         <v>48</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d) - Datenanalyse &amp; Automatisierung</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr"/>
@@ -6859,7 +6907,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>paero</t>
+          <t>Werkia</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -6870,7 +6918,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/d) - Datenanalyse &amp; Automatisierung</t>
         </is>
       </c>
       <c r="E52" t="inlineStr"/>
@@ -6884,7 +6932,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Vivanta Gmbh</t>
+          <t>paero</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -6895,7 +6943,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
@@ -6909,7 +6957,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Vitolus</t>
+          <t>Vivanta Gmbh</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -6920,7 +6968,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr"/>
@@ -6934,7 +6982,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>GrantLift GmbH</t>
+          <t>Vitolus</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -6945,7 +6993,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
+          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr"/>
@@ -6959,7 +7007,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Otto Group one.O GmbH</t>
+          <t>GrantLift GmbH</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -6970,7 +7018,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Praktikum im Knowledge Management - Corporate Strategy (w/m/d)</t>
+          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr"/>
@@ -6984,18 +7032,18 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>AUTO1 Global Services SE &amp; Co. KG</t>
+          <t>Otto Group one.O GmbH</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C57" t="n">
         <v>48</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (d/m/w)</t>
+          <t>Praktikum im Knowledge Management - Corporate Strategy (w/m/d)</t>
         </is>
       </c>
       <c r="E57" t="inlineStr"/>
@@ -7009,7 +7057,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>SHAVENT - ARA Sustainable Products</t>
+          <t>AUTO1 Global Services SE &amp; Co. KG</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -7020,7 +7068,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Praktikum Business Development in nachhaltigem Start-Up (w/m/d) Remote in DE</t>
+          <t>Praktikum Business Development (d/m/w)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
@@ -7034,7 +7082,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CTG Consulting</t>
+          <t>SHAVENT - ARA Sustainable Products</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -7045,7 +7093,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Praktikum Sales/Business Development // Hamburg oder Berlin</t>
+          <t>Praktikum Business Development in nachhaltigem Start-Up (w/m/d) Remote in DE</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
@@ -7059,7 +7107,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Dronesperhour</t>
+          <t>CTG Consulting</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -7070,7 +7118,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development eines Startups (m/w/d)</t>
+          <t>Praktikum Sales/Business Development // Hamburg oder Berlin</t>
         </is>
       </c>
       <c r="E60" t="inlineStr"/>
@@ -7084,7 +7132,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>SINN Power</t>
+          <t>Dronesperhour</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -7095,7 +7143,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Praktikum im AI Business Development (m/w/d)</t>
+          <t>Praktikum im Business Development eines Startups (m/w/d)</t>
         </is>
       </c>
       <c r="E61" t="inlineStr"/>
@@ -7109,7 +7157,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>innpuls</t>
+          <t>SINN Power</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -7120,7 +7168,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Praktikum im AI Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
@@ -7134,7 +7182,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Amolina</t>
+          <t>innpuls</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -7145,7 +7193,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
@@ -7159,18 +7207,18 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>Amolina</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C64" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
@@ -7184,18 +7232,18 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>STARTPLATZ Gruppe</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C65" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Sales (m/w/d) – STARTPLATZ</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
@@ -7209,7 +7257,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>spring.gate business consulting UG</t>
+          <t>STARTPLATZ Gruppe</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -7220,7 +7268,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development &amp; B2B Akquise (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Sales (m/w/d) – STARTPLATZ</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
@@ -7234,7 +7282,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>specter automation</t>
+          <t>spring.gate business consulting UG</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -7245,7 +7293,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Praktikum (M/W/D) im Business Development</t>
+          <t>Praktikum im Business Development &amp; B2B Akquise (m/w/d)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
@@ -7259,18 +7307,18 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Closd Kunststoffprodukte GmbH</t>
+          <t>specter automation</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C68" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Praktikum beim E-Commerce Startup Closd als Founders Associate (m/w/d)</t>
+          <t>Praktikum (M/W/D) im Business Development</t>
         </is>
       </c>
       <c r="E68" t="inlineStr"/>
@@ -7284,18 +7332,18 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Bosch Rexroth AG</t>
+          <t>Closd Kunststoffprodukte GmbH</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C69" t="n">
         <v>38</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Praktikum Business Development – Software Defined Business</t>
+          <t>Praktikum beim E-Commerce Startup Closd als Founders Associate (m/w/d)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
@@ -7309,7 +7357,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Weenect</t>
+          <t>Bosch Rexroth AG</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -7320,7 +7368,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d) – Markt DACH – Standort Brüssel</t>
+          <t>Praktikum Business Development – Software Defined Business</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
@@ -7334,18 +7382,18 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Lidl Dienstleistung GmbH &amp; Co. KG</t>
+          <t>Weenect</t>
         </is>
       </c>
       <c r="B71" t="n">
         <v>1</v>
       </c>
       <c r="C71" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Praktikum Business Development (m/w/d) – Markt DACH – Standort Brüssel</t>
         </is>
       </c>
       <c r="E71" t="inlineStr"/>
@@ -7359,18 +7407,18 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Drägerwerk AG &amp; Co. KGaA</t>
+          <t>Lidl Dienstleistung GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C72" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Praktikum New Business Development</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E72" t="inlineStr"/>
@@ -7384,18 +7432,18 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Arteus Energy</t>
+          <t>Drägerwerk AG &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C73" t="n">
         <v>28</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Praktikum Business Development und Marketing Photovoltaik</t>
+          <t>Praktikum New Business Development</t>
         </is>
       </c>
       <c r="E73" t="inlineStr"/>
@@ -7409,7 +7457,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>aramido</t>
+          <t>Arteus Energy</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -7420,7 +7468,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/x)</t>
+          <t>Praktikum Business Development und Marketing Photovoltaik</t>
         </is>
       </c>
       <c r="E74" t="inlineStr"/>
@@ -7434,7 +7482,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>pacemaker.ai by thyssenkrupp</t>
+          <t>aramido</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -7445,7 +7493,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/x)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr"/>
@@ -7459,7 +7507,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Wonder Natural GmbH</t>
+          <t>pacemaker.ai by thyssenkrupp</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -7470,7 +7518,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr"/>
@@ -7484,7 +7532,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Molly Suh GmbH</t>
+          <t>Wonder Natural GmbH</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -7495,7 +7543,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; B2B Sales (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr"/>
@@ -7509,7 +7557,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>homewise</t>
+          <t>Molly Suh GmbH</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -7520,7 +7568,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development &amp; Strategie (m/w/d)</t>
+          <t>Praktikum Business Development &amp; B2B Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E78" t="inlineStr"/>
@@ -7534,7 +7582,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>ClipMyHorse.TV</t>
+          <t>homewise</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -7545,7 +7593,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Praktikum HR &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im Business Development &amp; Strategie (m/w/d)</t>
         </is>
       </c>
       <c r="E79" t="inlineStr"/>
@@ -7559,7 +7607,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>AUMOVIO</t>
+          <t>ClipMyHorse.TV</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -7570,7 +7618,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Praktikum - Administration/Assistenz &amp; Business Development</t>
+          <t>Praktikum HR &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E80" t="inlineStr"/>
@@ -7584,7 +7632,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>TRUMPF Group</t>
+          <t>AUMOVIO</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -7595,7 +7643,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich Business Development für Smart Factory Solutions (WS26/27)</t>
+          <t>Praktikum - Administration/Assistenz &amp; Business Development</t>
         </is>
       </c>
       <c r="E81" t="inlineStr"/>
@@ -7606,8 +7654,33 @@
         </is>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>TRUMPF Group</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>1</v>
+      </c>
+      <c r="C82" t="n">
+        <v>28</v>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Praktikum im Bereich Business Development für Smart Factory Solutions (WS26/27)</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G81"/>
+  <autoFilter ref="A1:G82"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Lauf 2026-08-06 08:43 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firmen entdeckt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$103</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$105</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$82</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L103"/>
+  <dimension ref="A1:L105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -572,31 +572,27 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>Peek &amp; Cloppenburg* Düsseldorf</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management &amp; Shopper Marketing</t>
+          <t>Praktikum Strategic Brand Management (m/w/d)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Benrath, Düsseldorf</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+      <c r="G3" s="2" t="inlineStr"/>
       <c r="H3" s="2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -604,7 +600,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -615,7 +611,7 @@
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816411046?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5829419056?se=DOVmNHGR8RGawatf7LFQeQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59B7BE074DA3DBF8AEEEF0748268FCDE2EB4436F</t>
         </is>
       </c>
     </row>
@@ -626,27 +622,31 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>VEYNOU GmbH</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d) 3-6 Monate</t>
+          <t>Praktikum Brand Management &amp; Shopper Marketing</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Benrath, Düsseldorf</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="G4" s="2" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -665,7 +665,7 @@
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5646645887?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5816411046?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -676,21 +676,21 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Carwow</t>
+          <t>VEYNOU GmbH</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Media (m/w/d) - OEM Partnerships @ Carwow</t>
+          <t>Praktikum Business Development (m/w/d) 3-6 Monate</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
@@ -715,7 +715,7 @@
       <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5822522402?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5646645887?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -730,17 +730,17 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>FC Viktoria 1889 Berlin Frauen-Fußball GmbH</t>
+          <t>Carwow</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>PRAKTIKUM // Business Development</t>
+          <t>Praktikum Business Development &amp; Media (m/w/d) - OEM Partnerships @ Carwow</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Mitte, Berlin</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
@@ -765,7 +765,7 @@
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802962068?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5822522402?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -780,27 +780,23 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>FC Viktoria 1889 Berlin Frauen-Fußball GmbH</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Internship Digital Brand Marketing</t>
+          <t>PRAKTIKUM // Business Development</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Benrath, Düsseldorf</t>
+          <t>Mitte, Berlin</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
       <c r="H7" s="2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -819,7 +815,7 @@
       <c r="K7" s="2" t="inlineStr"/>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816488136?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802962068?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -839,7 +835,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Internship Digital Brand Marketing Schwarzkopf</t>
+          <t>Internship Digital Brand Marketing</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -852,7 +848,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -873,7 +869,7 @@
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816486591?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5816488136?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -888,23 +884,27 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Internship Digital Brand Marketing Schwarzkopf</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Benrath, Düsseldorf</t>
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="G9" s="2" t="inlineStr"/>
+        <v>6</v>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -923,7 +923,7 @@
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5816486591?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -938,7 +938,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Nestle</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -948,17 +948,13 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F10" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-01</t>
-        </is>
-      </c>
+      <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -977,7 +973,7 @@
       <c r="K10" s="2" t="inlineStr"/>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -992,23 +988,27 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Picnic</t>
+          <t>Nestle</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Category Management Praktikum (m/w/d)</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F11" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="G11" s="2" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1027,7 +1027,7 @@
       <c r="K11" s="2" t="inlineStr"/>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1042,17 +1042,17 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Picnic</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Category Management Praktikum (m/w/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Hamburg-Altstadt, Hamburg</t>
         </is>
       </c>
       <c r="F12" s="2" t="n">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1077,7 +1077,7 @@
       <c r="K12" s="2" t="inlineStr"/>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759088383?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5829732882?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1088,29 +1088,27 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
+          <t>Picnic</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management National</t>
+          <t>Category Management Praktikum (m/w/d)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Au-Haidhausen, München</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr"/>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
+          <t>Hamburg, Deutschland</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G13" s="2" t="inlineStr"/>
       <c r="H13" s="2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1129,7 +1127,7 @@
       <c r="K13" s="2" t="inlineStr"/>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805399065?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1140,26 +1138,30 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>EAT HAPPY GROUP</t>
+          <t>Picnic</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Brand Marketing (m/w/d) Marketing · Köln</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr"/>
+          <t>Category Management Praktikum (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
       <c r="F14" s="2" t="n">
         <v>6</v>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1175,7 +1177,7 @@
       <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>https://eathappygroup.teamtailor.com/jobs/7902845-praktikum-brand-marketing-m-w-d</t>
+          <t>https://www.adzuna.de/details/5759088383?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1186,27 +1188,29 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Yogi Tea</t>
+          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Marketing - Brand &amp; Product / mindestens 5 Monate</t>
+          <t>Praktikum Brand Management National</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="G15" s="2" t="inlineStr"/>
+          <t>Au-Haidhausen, München</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1225,7 +1229,7 @@
       <c r="K15" s="2" t="inlineStr"/>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5744980745?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805399065?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1236,34 +1240,26 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Ferrero</t>
+          <t>EAT HAPPY GROUP</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
+          <t>Praktikum Brand Marketing (m/w/d) Marketing · Köln</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
+      <c r="G16" s="2" t="inlineStr"/>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1279,7 +1275,7 @@
       <c r="K16" s="2" t="inlineStr"/>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://eathappygroup.teamtailor.com/jobs/7902845-praktikum-brand-marketing-m-w-d</t>
         </is>
       </c>
     </row>
@@ -1290,31 +1286,27 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Ferrero</t>
+          <t>Yogi Tea</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikum im Marketing - Brand &amp; Product / mindestens 5 Monate</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F17" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="G17" s="2" t="inlineStr"/>
       <c r="H17" s="2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1333,7 +1325,7 @@
       <c r="K17" s="2" t="inlineStr"/>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5799961458?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5744980745?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1353,7 +1345,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1366,7 +1358,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1387,7 +1379,7 @@
       <c r="K18" s="2" t="inlineStr"/>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1402,23 +1394,27 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich Marketing für die Marke BE-KIND DACH</t>
+          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F19" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="G19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1437,7 +1433,7 @@
       <c r="K19" s="2" t="inlineStr"/>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5753617280?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5799961458?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1452,17 +1448,17 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F20" s="2" t="n">
@@ -1470,7 +1466,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1491,7 +1487,7 @@
       <c r="K20" s="2" t="inlineStr"/>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899675?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1502,24 +1498,26 @@
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Miles &amp; More GmbH</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Internship Marketing Strategy &amp; Delivery</t>
+          <t>Praktikum im Bereich Marketing für die Marke BE-KIND DACH</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Flughafen, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr"/>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>6</v>
+      </c>
       <c r="G21" s="2" t="inlineStr"/>
       <c r="H21" s="2" t="inlineStr">
         <is>
@@ -1539,7 +1537,7 @@
       <c r="K21" s="2" t="inlineStr"/>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5828674997?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5753617280?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1550,27 +1548,31 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
+          <t>Praktikum Brand Management (m/w/d)</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F22" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="G22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1589,7 +1591,7 @@
       <c r="K22" s="2" t="inlineStr"/>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802899675?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1600,31 +1602,25 @@
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>Miles &amp; More GmbH</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Digital Marketing &amp; Category Management</t>
+          <t>Internship Marketing Strategy &amp; Delivery</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Benrath, Düsseldorf</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
+          <t>Flughafen, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr"/>
+      <c r="G23" s="2" t="inlineStr"/>
       <c r="H23" s="2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1643,7 +1639,7 @@
       <c r="K23" s="2" t="inlineStr"/>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816415884?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5828674997?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1658,17 +1654,17 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich Marketing für die Marke BE-KIND DACH</t>
+          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Unterhaching, München (Kreis)</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F24" s="2" t="n">
@@ -1693,7 +1689,7 @@
       <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5752932983?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1708,23 +1704,27 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>P&amp;G</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum Digital Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Benrath, Düsseldorf</t>
         </is>
       </c>
       <c r="F25" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="G25" s="2" t="inlineStr"/>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1743,7 +1743,7 @@
       <c r="K25" s="2" t="inlineStr"/>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5816415884?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1758,17 +1758,17 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Category Management Non Food Vertrieb (m/w/d)</t>
+          <t>Praktikum im Bereich Marketing für die Marke BE-KIND DACH</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Unterhaching, München (Kreis)</t>
         </is>
       </c>
       <c r="F26" s="2" t="n">
@@ -1793,7 +1793,7 @@
       <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5795118484?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5752932983?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1808,17 +1808,17 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>P&amp;G</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Praktikum CNX Category Management Home &amp; Living (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F27" s="2" t="n">
@@ -1843,7 +1843,7 @@
       <c r="K27" s="2" t="inlineStr"/>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5765078175?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1863,7 +1863,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing Tchibo (m/w/d)</t>
+          <t>Praktikum Category Management Non Food Vertrieb (m/w/d)</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1893,7 +1893,7 @@
       <c r="K28" s="2" t="inlineStr"/>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5744245447?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5795118484?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1913,7 +1913,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing Eduscho (m/w/d)</t>
+          <t>Praktikum CNX Category Management Home &amp; Living (m/w/d)</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -1943,7 +1943,7 @@
       <c r="K29" s="2" t="inlineStr"/>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5773205889?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5765078175?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1954,25 +1954,25 @@
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>Tchibo GmbH</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Trade Marketing Tchibo (m/w/d)</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G30" s="2" t="inlineStr"/>
       <c r="H30" s="2" t="inlineStr">
@@ -1993,7 +1993,7 @@
       <c r="K30" s="2" t="inlineStr"/>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5744245447?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2004,25 +2004,25 @@
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>markenbaumarkt24</t>
+          <t>Tchibo GmbH</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
+          <t>Praktikum Trade Marketing Eduscho (m/w/d)</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Feuersbach, Siegen</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G31" s="2" t="inlineStr"/>
       <c r="H31" s="2" t="inlineStr">
@@ -2043,7 +2043,7 @@
       <c r="K31" s="2" t="inlineStr"/>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5773205889?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2054,24 +2054,26 @@
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr"/>
+          <t>Düsseltal, Düsseldorf</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="n">
+        <v>5</v>
+      </c>
       <c r="G32" s="2" t="inlineStr"/>
       <c r="H32" s="2" t="inlineStr">
         <is>
@@ -2091,7 +2093,7 @@
       <c r="K32" s="2" t="inlineStr"/>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
+          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2102,25 +2104,25 @@
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>markenbaumarkt24</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
+          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Feuersbach, Siegen</t>
         </is>
       </c>
       <c r="F33" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G33" s="2" t="inlineStr"/>
       <c r="H33" s="2" t="inlineStr">
@@ -2141,7 +2143,7 @@
       <c r="K33" s="2" t="inlineStr"/>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2152,31 +2154,25 @@
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="G34" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>Hamburg, Deutschland</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr"/>
+      <c r="G34" s="2" t="inlineStr"/>
       <c r="H34" s="2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2195,7 +2191,7 @@
       <c r="K34" s="2" t="inlineStr"/>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
         </is>
       </c>
     </row>
@@ -2210,27 +2206,23 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Bosch Thermotechnik GmbH</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im internationalen Brand Management</t>
+          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Wernau (Neckar), Esslingen (Kreis)</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F35" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="G35" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+      <c r="G35" s="2" t="inlineStr"/>
       <c r="H35" s="2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2249,7 +2241,7 @@
       <c r="K35" s="2" t="inlineStr"/>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5799981240?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2264,17 +2256,17 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Intern Category Growth</t>
+          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Darmstadt, Hessen</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F36" s="2" t="n">
@@ -2282,7 +2274,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>2025-08-15</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -2303,7 +2295,7 @@
       <c r="K36" s="2" t="inlineStr"/>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5754086625?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2318,17 +2310,17 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>L’ORÉAL</t>
+          <t>Bosch Thermotechnik GmbH</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>PRAKTIKUM (M/W/D) Product Marketing - Start ab August/September/Oktober für 6 Monate</t>
+          <t>Praktikum im internationalen Brand Management</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Nordrhein-Westfalen, Deutschland</t>
+          <t>Wernau (Neckar), Esslingen (Kreis)</t>
         </is>
       </c>
       <c r="F37" s="2" t="n">
@@ -2336,7 +2328,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2357,7 +2349,7 @@
       <c r="K37" s="2" t="inlineStr"/>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5754061318?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5799981240?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2372,17 +2364,17 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>Intern Category Growth</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Darmstadt, Hessen</t>
         </is>
       </c>
       <c r="F38" s="2" t="n">
@@ -2390,7 +2382,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2025-08-15</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2411,7 +2403,7 @@
       <c r="K38" s="2" t="inlineStr"/>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5754086625?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2426,17 +2418,17 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>coty</t>
+          <t>L’ORÉAL</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
+          <t>PRAKTIKUM (M/W/D) Product Marketing - Start ab August/September/Oktober für 6 Monate</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Darmstadt, Hessen</t>
+          <t>Nordrhein-Westfalen, Deutschland</t>
         </is>
       </c>
       <c r="F39" s="2" t="n">
@@ -2444,7 +2436,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>2025-08-15</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2465,7 +2457,7 @@
       <c r="K39" s="2" t="inlineStr"/>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5754061318?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2476,7 +2468,7 @@
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
@@ -2490,10 +2482,12 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr"/>
+          <t>Braunsfeld, Köln</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>6</v>
+      </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
           <t>2026-10-01</t>
@@ -2517,7 +2511,7 @@
       <c r="K40" s="2" t="inlineStr"/>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5822943276?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=580C236799B96DFD395A1EC1CBBF7474C7F58435</t>
+          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2528,25 +2522,31 @@
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>coty</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Marketing Intern - Trade Marketing</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr"/>
-      <c r="G41" s="2" t="inlineStr"/>
+          <t>Darmstadt, Hessen</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>2025-08-15</t>
+        </is>
+      </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2565,7 +2565,7 @@
       <c r="K41" s="2" t="inlineStr"/>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2576,25 +2576,29 @@
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Altstadt, Düsseldorf</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr"/>
-      <c r="G42" s="2" t="inlineStr"/>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2613,7 +2617,7 @@
       <c r="K42" s="2" t="inlineStr"/>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5822943276?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=580C236799B96DFD395A1EC1CBBF7474C7F58435</t>
         </is>
       </c>
     </row>
@@ -2628,17 +2632,17 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Calypso Ventures GmbH</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr"/>
@@ -2661,7 +2665,7 @@
       <c r="K43" s="2" t="inlineStr"/>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2672,28 +2676,28 @@
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Altstadt, Düsseldorf</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr"/>
       <c r="G44" s="2" t="inlineStr"/>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
@@ -2709,7 +2713,7 @@
       <c r="K44" s="2" t="inlineStr"/>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
+          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2720,21 +2724,21 @@
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>Calypso Ventures GmbH</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr"/>
@@ -2757,7 +2761,7 @@
       <c r="K45" s="2" t="inlineStr"/>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2768,28 +2772,28 @@
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr"/>
       <c r="G46" s="2" t="inlineStr"/>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
@@ -2805,7 +2809,7 @@
       <c r="K46" s="2" t="inlineStr"/>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
         </is>
       </c>
     </row>
@@ -2816,21 +2820,21 @@
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Sayano Deutschland GmbH</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr"/>
@@ -2853,7 +2857,7 @@
       <c r="K47" s="2" t="inlineStr"/>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816572451?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2864,21 +2868,21 @@
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Abrio</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr"/>
@@ -2901,7 +2905,7 @@
       <c r="K48" s="2" t="inlineStr"/>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2912,21 +2916,21 @@
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>Sayano Deutschland GmbH</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Internship International Marketing Schwarzkopf Coloration - Legacy Brands</t>
+          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Benrath, Düsseldorf</t>
+          <t>Mitte, Stuttgart</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr"/>
@@ -2949,7 +2953,7 @@
       <c r="K49" s="2" t="inlineStr"/>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5819890143?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5816572451?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2964,22 +2968,20 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Lidl Stiftung</t>
+          <t>Abrio</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food in Neckarsulm</t>
+          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F50" s="2" t="n">
-        <v>6</v>
-      </c>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr"/>
       <c r="G50" s="2" t="inlineStr"/>
       <c r="H50" s="2" t="inlineStr">
         <is>
@@ -2999,7 +3001,7 @@
       <c r="K50" s="2" t="inlineStr"/>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813494719?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3014,17 +3016,17 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Lidl Stiftung &amp; Co. KG</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Internship International Marketing Schwarzkopf Coloration - Legacy Brands</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Benrath, Düsseldorf</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr"/>
@@ -3047,7 +3049,7 @@
       <c r="K51" s="2" t="inlineStr"/>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
+          <t>https://www.adzuna.de/details/5819890143?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3062,12 +3064,12 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Marc O'Polo</t>
+          <t>Lidl Stiftung</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food in Neckarsulm</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -3075,12 +3077,10 @@
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr"/>
-      <c r="G52" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
+      <c r="F52" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G52" s="2" t="inlineStr"/>
       <c r="H52" s="2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3099,7 +3099,7 @@
       <c r="K52" s="2" t="inlineStr"/>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5813494719?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3114,17 +3114,17 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Marketing (m/w/d)</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr"/>
@@ -3147,7 +3147,7 @@
       <c r="K53" s="2" t="inlineStr"/>
       <c r="L53" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899691?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
         </is>
       </c>
     </row>
@@ -3162,24 +3162,28 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Marc O'Polo</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Marketing (m/w/d)</t>
+          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr"/>
-      <c r="G54" s="2" t="inlineStr"/>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
@@ -3195,7 +3199,7 @@
       <c r="K54" s="2" t="inlineStr"/>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
+          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3206,31 +3210,25 @@
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>LIGANOVA I Karriere</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Buying (all genders) – August/September 2026</t>
+          <t>Praktikum Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
-        </is>
-      </c>
-      <c r="F55" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="G55" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr"/>
+      <c r="G55" s="2" t="inlineStr"/>
       <c r="H55" s="2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3249,7 +3247,7 @@
       <c r="K55" s="2" t="inlineStr"/>
       <c r="L55" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805407495?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802899691?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3260,28 +3258,28 @@
         </is>
       </c>
       <c r="B56" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Marketing &amp; Merchandising Assistant Trainee</t>
+          <t>Praktikum Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr"/>
       <c r="G56" s="2" t="inlineStr"/>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
@@ -3297,7 +3295,7 @@
       <c r="K56" s="2" t="inlineStr"/>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
         </is>
       </c>
     </row>
@@ -3312,24 +3310,30 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>LIGANOVA I Karriere</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Marketing and Merchandising Assistant Trainee</t>
+          <t>Praktikum Buying (all genders) – August/September 2026</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>MILAN</t>
-        </is>
-      </c>
-      <c r="F57" s="2" t="inlineStr"/>
-      <c r="G57" s="2" t="inlineStr"/>
+          <t>Mitte, Stuttgart</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr">
@@ -3345,7 +3349,7 @@
       <c r="K57" s="2" t="inlineStr"/>
       <c r="L57" s="2" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing-and-Merchandising-Assistant-Trainee_JR128690</t>
+          <t>https://www.adzuna.de/details/5805407495?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3356,28 +3360,28 @@
         </is>
       </c>
       <c r="B58" s="2" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Digitalagenten</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
+          <t>Marketing &amp; Merchandising Assistant Trainee</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Charlottenburg, Berlin</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr"/>
       <c r="G58" s="2" t="inlineStr"/>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
@@ -3393,7 +3397,7 @@
       <c r="K58" s="2" t="inlineStr"/>
       <c r="L58" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804948828?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
         </is>
       </c>
     </row>
@@ -3404,28 +3408,28 @@
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>LIMITD by Wunderproducts GmbH</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Marketing and Merchandising Assistant Trainee</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Kreuzberg, Berlin</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr"/>
       <c r="G59" s="2" t="inlineStr"/>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr">
@@ -3441,7 +3445,7 @@
       <c r="K59" s="2" t="inlineStr"/>
       <c r="L59" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing-and-Merchandising-Assistant-Trainee_JR128690</t>
         </is>
       </c>
     </row>
@@ -3456,25 +3460,21 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers GmbH WPG</t>
+          <t>Digitalagenten</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
+          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Charlottenburg, Berlin</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr"/>
-      <c r="G60" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
+      <c r="G60" s="2" t="inlineStr"/>
       <c r="H60" s="2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3493,7 +3493,7 @@
       <c r="K60" s="2" t="inlineStr"/>
       <c r="L60" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804948828?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3508,7 +3508,7 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>THE VERSE Ventures</t>
+          <t>LIMITD by Wunderproducts GmbH</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
@@ -3518,7 +3518,7 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Kreuzberg, Berlin</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr"/>
@@ -3541,7 +3541,7 @@
       <c r="K61" s="2" t="inlineStr"/>
       <c r="L61" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3556,21 +3556,25 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>WirWinzer</t>
+          <t>PricewaterhouseCoopers GmbH WPG</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Business Development Weinhandel (all genders)</t>
+          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr"/>
-      <c r="G62" s="2" t="inlineStr"/>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3589,7 +3593,7 @@
       <c r="K62" s="2" t="inlineStr"/>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3600,21 +3604,21 @@
         </is>
       </c>
       <c r="B63" s="2" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Brand Trust</t>
+          <t>THE VERSE Ventures</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Gleißbühl, Nürnberg</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr"/>
@@ -3637,7 +3641,7 @@
       <c r="K63" s="2" t="inlineStr"/>
       <c r="L63" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5669847401?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3648,19 +3652,23 @@
         </is>
       </c>
       <c r="B64" s="2" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>WirWinzer</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="inlineStr"/>
+          <t>Praktikum Business Development Weinhandel (all genders)</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>Altstadt-Lehel, München</t>
+        </is>
+      </c>
       <c r="F64" s="2" t="inlineStr"/>
       <c r="G64" s="2" t="inlineStr"/>
       <c r="H64" s="2" t="inlineStr">
@@ -3681,7 +3689,7 @@
       <c r="K64" s="2" t="inlineStr"/>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
+          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3696,15 +3704,19 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Brand Trust</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Operational Trade Marketing Intern</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="inlineStr"/>
+          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>Gleißbühl, Nürnberg</t>
+        </is>
+      </c>
       <c r="F65" s="2" t="inlineStr"/>
       <c r="G65" s="2" t="inlineStr"/>
       <c r="H65" s="2" t="inlineStr">
@@ -3725,7 +3737,7 @@
       <c r="K65" s="2" t="inlineStr"/>
       <c r="L65" s="2" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Toronto-Operational-Trade-Marketing-Intern-ON-M5H4H2/1397938633/</t>
+          <t>https://www.adzuna.de/details/5669847401?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3740,19 +3752,15 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E66" s="2" t="inlineStr">
-        <is>
-          <t>Schwabing-Freimann, München</t>
-        </is>
-      </c>
+          <t>Marketing Intern - Trade Marketing</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr"/>
       <c r="F66" s="2" t="inlineStr"/>
       <c r="G66" s="2" t="inlineStr"/>
       <c r="H66" s="2" t="inlineStr">
@@ -3773,7 +3781,7 @@
       <c r="K66" s="2" t="inlineStr"/>
       <c r="L66" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
         </is>
       </c>
     </row>
@@ -3788,24 +3796,20 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="inlineStr">
-        <is>
-          <t>DEU-Bayern-Unterhaching</t>
-        </is>
-      </c>
+          <t>Operational Trade Marketing Intern</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr"/>
       <c r="F67" s="2" t="inlineStr"/>
       <c r="G67" s="2" t="inlineStr"/>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
@@ -3821,7 +3825,7 @@
       <c r="K67" s="2" t="inlineStr"/>
       <c r="L67" s="2" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
+          <t>https://careers.coty.com/job/Toronto-Operational-Trade-Marketing-Intern-ON-M5H4H2/1397938633/</t>
         </is>
       </c>
     </row>
@@ -3836,17 +3840,17 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>Schwabing-Freimann, München</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr"/>
@@ -3869,7 +3873,7 @@
       <c r="K68" s="2" t="inlineStr"/>
       <c r="L68" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3884,24 +3888,24 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
+          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>DEU-Bayern-Unterhaching</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr"/>
       <c r="G69" s="2" t="inlineStr"/>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr">
@@ -3917,7 +3921,7 @@
       <c r="K69" s="2" t="inlineStr"/>
       <c r="L69" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
         </is>
       </c>
     </row>
@@ -3932,17 +3936,17 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr"/>
@@ -3965,7 +3969,7 @@
       <c r="K70" s="2" t="inlineStr"/>
       <c r="L70" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
+          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3985,7 +3989,7 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
@@ -4013,7 +4017,7 @@
       <c r="K71" s="2" t="inlineStr"/>
       <c r="L71" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
+          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
         </is>
       </c>
     </row>
@@ -4028,17 +4032,17 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr"/>
@@ -4061,7 +4065,7 @@
       <c r="K72" s="2" t="inlineStr"/>
       <c r="L72" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
         </is>
       </c>
     </row>
@@ -4072,21 +4076,21 @@
         </is>
       </c>
       <c r="B73" s="2" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>AUTO1 Global Services SE &amp; Co. KG</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (d/m/w)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr"/>
@@ -4109,7 +4113,7 @@
       <c r="K73" s="2" t="inlineStr"/>
       <c r="L73" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5789927805?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
         </is>
       </c>
     </row>
@@ -4120,21 +4124,21 @@
         </is>
       </c>
       <c r="B74" s="2" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Amolina</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr"/>
@@ -4157,7 +4161,7 @@
       <c r="K74" s="2" t="inlineStr"/>
       <c r="L74" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727292709?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4172,17 +4176,17 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>CTG Consulting</t>
+          <t>AUTO1 Global Services SE &amp; Co. KG</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Sales/Business Development // Hamburg oder Berlin</t>
+          <t>Praktikum Business Development (d/m/w)</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr"/>
@@ -4205,7 +4209,7 @@
       <c r="K75" s="2" t="inlineStr"/>
       <c r="L75" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5694221323?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5789927805?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4220,17 +4224,17 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Dronesperhour</t>
+          <t>Amolina</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development eines Startups (m/w/d)</t>
+          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Mitte, Berlin</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr"/>
@@ -4253,7 +4257,7 @@
       <c r="K76" s="2" t="inlineStr"/>
       <c r="L76" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5669955732?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5727292709?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4268,17 +4272,17 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>GrantLift GmbH</t>
+          <t>CTG Consulting</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
+          <t>Praktikum Sales/Business Development // Hamburg oder Berlin</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr"/>
@@ -4301,7 +4305,7 @@
       <c r="K77" s="2" t="inlineStr"/>
       <c r="L77" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5803032426?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5694221323?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4316,17 +4320,17 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>GrantLift GmbH</t>
+          <t>Dronesperhour</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
+          <t>Praktikum im Business Development eines Startups (m/w/d)</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Mitte, Berlin</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr"/>
@@ -4349,7 +4353,7 @@
       <c r="K78" s="2" t="inlineStr"/>
       <c r="L78" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804575149?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5669955732?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4364,17 +4368,17 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>Otto Group one.O GmbH</t>
+          <t>GrantLift GmbH</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Knowledge Management - Corporate Strategy (w/m/d)</t>
+          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr"/>
@@ -4397,7 +4401,7 @@
       <c r="K79" s="2" t="inlineStr"/>
       <c r="L79" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5809516963?se=mrUvpGeQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=7970F7260CB99374DD6661F2025E46043B457CE4</t>
+          <t>https://www.adzuna.de/details/5803032426?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4412,17 +4416,17 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Pflegia</t>
+          <t>GrantLift GmbH</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr"/>
@@ -4445,7 +4449,7 @@
       <c r="K80" s="2" t="inlineStr"/>
       <c r="L80" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5821302522?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804575149?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4460,17 +4464,17 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>Pflegia</t>
+          <t>Otto Group one.O GmbH</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Praktikum im Knowledge Management - Corporate Strategy (w/m/d)</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr"/>
@@ -4493,7 +4497,7 @@
       <c r="K81" s="2" t="inlineStr"/>
       <c r="L81" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802953545?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5809516963?se=mrUvpGeQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=7970F7260CB99374DD6661F2025E46043B457CE4</t>
         </is>
       </c>
     </row>
@@ -4513,7 +4517,7 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (Projektmanagement &amp; Prozessoptimierung) (m/w/d)</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
@@ -4541,7 +4545,7 @@
       <c r="K82" s="2" t="inlineStr"/>
       <c r="L82" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802984051?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5821302522?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4561,12 +4565,12 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (Business Analyst/Automation Engineer/Applied AI Engineer) (m/w/d)</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr"/>
@@ -4589,7 +4593,7 @@
       <c r="K83" s="2" t="inlineStr"/>
       <c r="L83" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802977130?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802953545?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4604,17 +4608,17 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>REWE Group</t>
+          <t>Pflegia</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Praktikum im Business Development (Projektmanagement &amp; Prozessoptimierung) (m/w/d)</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Wedding, Berlin</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr"/>
@@ -4637,7 +4641,7 @@
       <c r="K84" s="2" t="inlineStr"/>
       <c r="L84" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5712965755?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802984051?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4652,17 +4656,17 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>SHAVENT - ARA Sustainable Products</t>
+          <t>Pflegia</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Business Development in nachhaltigem Start-Up (w/m/d) Remote in DE</t>
+          <t>Praktikum im Business Development (Business Analyst/Automation Engineer/Applied AI Engineer) (m/w/d)</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Sendling, München</t>
+          <t>Wedding, Berlin</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr"/>
@@ -4685,7 +4689,7 @@
       <c r="K85" s="2" t="inlineStr"/>
       <c r="L85" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802951937?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802977130?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4700,17 +4704,17 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>SINN Power</t>
+          <t>REWE Group</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im AI Business Development (m/w/d)</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Kasten, München (Kreis)</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr"/>
@@ -4733,7 +4737,7 @@
       <c r="K86" s="2" t="inlineStr"/>
       <c r="L86" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727348338?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5712965755?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4748,17 +4752,17 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>SHAVENT - ARA Sustainable Products</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Strategy &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Business Development in nachhaltigem Start-Up (w/m/d) Remote in DE</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Sendling, München</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr"/>
@@ -4781,7 +4785,7 @@
       <c r="K87" s="2" t="inlineStr"/>
       <c r="L87" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5799516357?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802951937?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4796,17 +4800,17 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Vitolus</t>
+          <t>SINN Power</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
+          <t>Praktikum im AI Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Kasten, München (Kreis)</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr"/>
@@ -4829,7 +4833,7 @@
       <c r="K88" s="2" t="inlineStr"/>
       <c r="L88" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5785872138?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5727348338?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4844,17 +4848,17 @@
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>Vivanta Gmbh</t>
+          <t>Tchibo GmbH</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Praktikum Strategy &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr"/>
@@ -4877,7 +4881,7 @@
       <c r="K89" s="2" t="inlineStr"/>
       <c r="L89" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802952325?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5799516357?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4892,17 +4896,17 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Vivanta Gmbh</t>
+          <t>Vitolus</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr"/>
@@ -4925,7 +4929,7 @@
       <c r="K90" s="2" t="inlineStr"/>
       <c r="L90" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804549349?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5785872138?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4940,17 +4944,17 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>Werkia</t>
+          <t>Vivanta Gmbh</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d) - Datenanalyse &amp; Automatisierung</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr"/>
@@ -4973,7 +4977,7 @@
       <c r="K91" s="2" t="inlineStr"/>
       <c r="L91" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802974922?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802952325?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4988,12 +4992,12 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Werkia</t>
+          <t>Vivanta Gmbh</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d) - Berlin</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -5021,7 +5025,7 @@
       <c r="K92" s="2" t="inlineStr"/>
       <c r="L92" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802950225?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804549349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5036,17 +5040,17 @@
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>innpuls</t>
+          <t>Werkia</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/d) - Datenanalyse &amp; Automatisierung</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Wedding, Berlin</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr"/>
@@ -5069,7 +5073,7 @@
       <c r="K93" s="2" t="inlineStr"/>
       <c r="L93" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5735591887?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802974922?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5084,17 +5088,17 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>paero</t>
+          <t>Werkia</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im Business Development (m/w/d) - Berlin</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>Ludwigsvorstadt-Isarvorstadt, München</t>
+          <t>Wedding, Berlin</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr"/>
@@ -5117,7 +5121,7 @@
       <c r="K94" s="2" t="inlineStr"/>
       <c r="L94" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813846665?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802950225?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5128,21 +5132,21 @@
         </is>
       </c>
       <c r="B95" s="2" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>innpuls</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr"/>
@@ -5165,7 +5169,7 @@
       <c r="K95" s="2" t="inlineStr"/>
       <c r="L95" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5735591887?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5176,21 +5180,21 @@
         </is>
       </c>
       <c r="B96" s="2" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>paero</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>Altstadt-Nord, Köln</t>
+          <t>Ludwigsvorstadt-Isarvorstadt, München</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr"/>
@@ -5213,7 +5217,7 @@
       <c r="K96" s="2" t="inlineStr"/>
       <c r="L96" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5813846665?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5224,21 +5228,21 @@
         </is>
       </c>
       <c r="B97" s="2" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>Devoteam G Cloud Germany</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr"/>
@@ -5261,7 +5265,7 @@
       <c r="K97" s="2" t="inlineStr"/>
       <c r="L97" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811135653?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5272,21 +5276,21 @@
         </is>
       </c>
       <c r="B98" s="2" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt-Nord, Köln</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr"/>
@@ -5309,7 +5313,7 @@
       <c r="K98" s="2" t="inlineStr"/>
       <c r="L98" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5324,12 +5328,12 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>Devoteam G Cloud Germany</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
@@ -5357,7 +5361,7 @@
       <c r="K99" s="2" t="inlineStr"/>
       <c r="L99" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5811135653?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5382,7 +5386,7 @@
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr"/>
@@ -5405,7 +5409,7 @@
       <c r="K100" s="2" t="inlineStr"/>
       <c r="L100" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5430,7 +5434,7 @@
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr"/>
@@ -5453,7 +5457,7 @@
       <c r="K101" s="2" t="inlineStr"/>
       <c r="L101" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5468,17 +5472,17 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>sailwithus</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr"/>
@@ -5501,7 +5505,7 @@
       <c r="K102" s="2" t="inlineStr"/>
       <c r="L102" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5516,12 +5520,12 @@
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>sailwithus</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
@@ -5549,12 +5553,108 @@
       <c r="K103" s="2" t="inlineStr"/>
       <c r="L103" s="2" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>sailwithus</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr"/>
+      <c r="G104" s="2" t="inlineStr"/>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I104" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J104" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K104" s="2" t="inlineStr"/>
+      <c r="L104" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>sailwithus</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr"/>
+      <c r="G105" s="2" t="inlineStr"/>
+      <c r="H105" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I105" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J105" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K105" s="2" t="inlineStr"/>
+      <c r="L105" s="2" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5804544237?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L103"/>
+  <autoFilter ref="A1:L105"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5621,7 +5721,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C2" t="n">
         <v>107</v>
@@ -5646,7 +5746,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C3" t="n">
         <v>91</v>
@@ -5671,7 +5771,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C4" t="n">
         <v>89</v>
@@ -5696,7 +5796,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C5" t="n">
         <v>84</v>
@@ -5721,7 +5821,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C6" t="n">
         <v>84</v>
@@ -5746,7 +5846,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C7" t="n">
         <v>84</v>
@@ -5779,7 +5879,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C8" t="n">
         <v>84</v>
@@ -5800,18 +5900,18 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>FC Viktoria 1889 Berlin Frauen-Fußball GmbH</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C9" t="n">
         <v>84</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>PRAKTIKUM // Business Development</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
@@ -5825,18 +5925,18 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Carwow</t>
+          <t>FC Viktoria 1889 Berlin Frauen-Fußball GmbH</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Media (m/w/d) - OEM Partnerships @ Carwow</t>
+          <t>PRAKTIKUM // Business Development</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
@@ -5850,18 +5950,18 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
+          <t>Carwow</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C11" t="n">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management National</t>
+          <t>Praktikum Business Development &amp; Media (m/w/d) - OEM Partnerships @ Carwow</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
@@ -5875,18 +5975,18 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Yogi Tea</t>
+          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C12" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Praktikum im Marketing - Brand &amp; Product / mindestens 5 Monate</t>
+          <t>Praktikum Brand Management National</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
@@ -5904,7 +6004,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C13" t="n">
         <v>79</v>
@@ -5925,18 +6025,18 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Yogi Tea</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="C14" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich Marketing für die Marke BE-KIND DACH</t>
+          <t>Praktikum im Marketing - Brand &amp; Product / mindestens 5 Monate</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
@@ -5950,30 +6050,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Ferrero</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C15" t="n">
         <v>78</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>successfactors</t>
-        </is>
-      </c>
+          <t>Praktikum im Bereich Marketing für die Marke BE-KIND DACH</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -5983,22 +6075,30 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Miles &amp; More GmbH</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C16" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Internship Marketing Strategy &amp; Delivery</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>successfactors</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -6008,30 +6108,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>Miles &amp; More GmbH</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="C17" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Praktikum Category Management Non Food Vertrieb (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>successfactors</t>
-        </is>
-      </c>
+          <t>Internship Marketing Strategy &amp; Delivery</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -6041,22 +6133,30 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>Tchibo GmbH</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="C18" t="n">
         <v>73</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
+          <t>Praktikum Category Management Non Food Vertrieb (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>successfactors</t>
+        </is>
+      </c>
       <c r="G18" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -6066,18 +6166,18 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>P&amp;G</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="C19" t="n">
         <v>73</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
@@ -6091,18 +6191,18 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>markenbaumarkt24</t>
+          <t>P&amp;G</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C20" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
@@ -6116,18 +6216,18 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>markenbaumarkt24</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C21" t="n">
         <v>72</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
@@ -6141,18 +6241,18 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>5</v>
       </c>
       <c r="C22" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr"/>
@@ -6170,7 +6270,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C23" t="n">
         <v>68</v>
@@ -6203,7 +6303,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C24" t="n">
         <v>68</v>
@@ -6228,7 +6328,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C25" t="n">
         <v>68</v>
@@ -6278,7 +6378,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C27" t="n">
         <v>62</v>
@@ -6303,7 +6403,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C28" t="n">
         <v>62</v>
@@ -6328,7 +6428,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C29" t="n">
         <v>57</v>
@@ -6361,7 +6461,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C30" t="n">
         <v>56</v>
@@ -6386,7 +6486,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C31" t="n">
         <v>55</v>
@@ -6411,7 +6511,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C32" t="n">
         <v>54</v>
@@ -6436,7 +6536,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C33" t="n">
         <v>54</v>
@@ -6461,7 +6561,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C34" t="n">
         <v>54</v>
@@ -6486,7 +6586,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C35" t="n">
         <v>54</v>
@@ -6511,7 +6611,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C36" t="n">
         <v>53</v>
@@ -6536,7 +6636,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C37" t="n">
         <v>53</v>
@@ -6561,7 +6661,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C38" t="n">
         <v>53</v>
@@ -6586,7 +6686,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C39" t="n">
         <v>52</v>
@@ -6611,7 +6711,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C40" t="n">
         <v>51</v>
@@ -6636,7 +6736,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C41" t="n">
         <v>51</v>
@@ -6661,7 +6761,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C42" t="n">
         <v>51</v>
@@ -6686,7 +6786,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C43" t="n">
         <v>51</v>
@@ -6711,7 +6811,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C44" t="n">
         <v>51</v>
@@ -6736,7 +6836,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C45" t="n">
         <v>49</v>
@@ -6761,7 +6861,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C46" t="n">
         <v>49</v>
@@ -6786,7 +6886,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C47" t="n">
         <v>49</v>
@@ -6811,7 +6911,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C48" t="n">
         <v>49</v>
@@ -6836,7 +6936,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C49" t="n">
         <v>49</v>
@@ -6857,7 +6957,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Pflegia</t>
+          <t>REWE Group</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -6868,7 +6968,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
@@ -6882,18 +6982,18 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>REWE Group</t>
+          <t>Pflegia</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C51" t="n">
         <v>48</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr"/>
@@ -7236,7 +7336,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C65" t="n">
         <v>46</v>

</xml_diff>

<commit_message>
Lauf 2026-08-08 06:58 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firmen entdeckt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$105</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$106</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$83</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L105"/>
+  <dimension ref="A1:L106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -562,50 +562,46 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="n">
         <v>107</v>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Peek &amp; Cloppenburg* Düsseldorf</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Praktikum Strategic Brand Management (m/w/d)</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="F3" t="n">
         <v>4</v>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
         <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr"/>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
         <is>
           <t>https://www.adzuna.de/land/ad/5829419056?se=DOVmNHGR8RGawatf7LFQeQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59B7BE074DA3DBF8AEEEF0748268FCDE2EB4436F</t>
         </is>
@@ -996,50 +992,46 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="n">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="n">
         <v>84</v>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>Hamburg-Altstadt, Hamburg</t>
         </is>
       </c>
-      <c r="F12" s="2" t="n">
+      <c r="F12" t="n">
         <v>6</v>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
         <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
         <is>
           <t>https://www.adzuna.de/details/5829732882?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
@@ -1526,21 +1518,27 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Miles &amp; More GmbH</t>
+          <t>Marc O'Polo</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Internship Marketing Strategy &amp; Delivery</t>
+          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Flughafen, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>6</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
       <c r="H23" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1559,33 +1557,31 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5828674997?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>Miles &amp; More GmbH</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
+          <t>Internship Marketing Strategy &amp; Delivery</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F24" t="n">
-        <v>6</v>
-      </c>
+          <t>Flughafen, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
@@ -1605,38 +1601,32 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5828674997?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Praktikum Digital Marketing &amp; Category Management</t>
+          <t>Praktikum Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Benrath, Düsseldorf</t>
-        </is>
-      </c>
-      <c r="F25" t="n">
-        <v>6</v>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1655,7 +1645,7 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816415884?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802899691?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1666,17 +1656,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich Marketing für die Marke BE-KIND DACH</t>
+          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Unterhaching, München (Kreis)</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F26" t="n">
@@ -1701,7 +1691,7 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5752932983?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1712,23 +1702,27 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>P&amp;G</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum Digital Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Benrath, Düsseldorf</t>
         </is>
       </c>
       <c r="F27" t="n">
         <v>6</v>
       </c>
-      <c r="G27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
       <c r="H27" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1747,7 +1741,7 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5816415884?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1758,17 +1752,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Praktikum Category Management Non Food Vertrieb (m/w/d)</t>
+          <t>Praktikum im Bereich Marketing für die Marke BE-KIND DACH</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Unterhaching, München (Kreis)</t>
         </is>
       </c>
       <c r="F28" t="n">
@@ -1793,7 +1787,7 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5795118484?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5752932983?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1804,17 +1798,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>P&amp;G</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Praktikum CNX Category Management Home &amp; Living (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F29" t="n">
@@ -1839,7 +1833,7 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5765078175?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1855,7 +1849,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing Tchibo (m/w/d)</t>
+          <t>Praktikum Category Management Non Food Vertrieb (m/w/d)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1885,7 +1879,7 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5744245447?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5795118484?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1901,7 +1895,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing Eduscho (m/w/d)</t>
+          <t>Praktikum CNX Category Management Home &amp; Living (m/w/d)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1931,32 +1925,32 @@
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5773205889?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5765078175?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr"/>
       <c r="B32" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>Tchibo GmbH</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Trade Marketing Tchibo (m/w/d)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
@@ -1977,32 +1971,32 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5744245447?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr"/>
       <c r="B33" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>markenbaumarkt24</t>
+          <t>Tchibo GmbH</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
+          <t>Praktikum Trade Marketing Eduscho (m/w/d)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Feuersbach, Siegen</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
@@ -2023,31 +2017,33 @@
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5773205889?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr"/>
       <c r="B34" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr"/>
+          <t>Düsseltal, Düsseldorf</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>5</v>
+      </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
@@ -2067,32 +2063,32 @@
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
+          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr"/>
       <c r="B35" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>markenbaumarkt24</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
+          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Feuersbach, Siegen</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
@@ -2113,88 +2109,82 @@
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr"/>
-      <c r="B36" t="n">
-        <v>68</v>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Barilla</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Köln, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F36" t="n">
-        <v>6</v>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>PARSA Haar- und Modeartikel GmbH</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr"/>
+      <c r="G36" s="2" t="inlineStr"/>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr"/>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Bosch Thermotechnik GmbH</t>
+          <t>Lidl Stiftung</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Praktikum im internationalen Brand Management</t>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food in Neckarsulm</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Wernau (Neckar), Esslingen (Kreis)</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F37" t="n">
         <v>6</v>
       </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2213,38 +2203,32 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5799981240?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5813494719?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Intern Category Growth</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Darmstadt, Hessen</t>
-        </is>
-      </c>
-      <c r="F38" t="n">
-        <v>6</v>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>2025-08-15</t>
-        </is>
-      </c>
+          <t>Hamburg, Deutschland</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2263,7 +2247,7 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5754086625?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
         </is>
       </c>
     </row>
@@ -2274,27 +2258,23 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>L’ORÉAL</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>PRAKTIKUM (M/W/D) Product Marketing - Start ab August/September/Oktober für 6 Monate</t>
+          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Nordrhein-Westfalen, Deutschland</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F39" t="n">
         <v>6</v>
       </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2313,7 +2293,7 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5754061318?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2324,17 +2304,17 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F40" t="n">
@@ -2363,7 +2343,7 @@
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2374,17 +2354,17 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>coty</t>
+          <t>Bosch Thermotechnik GmbH</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
+          <t>Praktikum im internationalen Brand Management</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Darmstadt, Hessen</t>
+          <t>Wernau (Neckar), Esslingen (Kreis)</t>
         </is>
       </c>
       <c r="F41" t="n">
@@ -2392,7 +2372,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>2025-08-15</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2413,36 +2393,34 @@
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5799981240?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr"/>
       <c r="B42" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>Intern Category Growth</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>Darmstadt, Hessen</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>6</v>
+      </c>
+      <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2461,32 +2439,38 @@
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5822943276?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=580C236799B96DFD395A1EC1CBBF7474C7F58435</t>
+          <t>https://www.adzuna.de/details/5754086625?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr"/>
       <c r="B43" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>L’ORÉAL</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>PRAKTIKUM (M/W/D) Product Marketing - Start ab August/September/Oktober für 6 Monate</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
+          <t>Nordrhein-Westfalen, Deutschland</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>6</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H43" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2505,32 +2489,38 @@
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5754061318?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr"/>
       <c r="B44" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Altstadt, Düsseldorf</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
+          <t>Braunsfeld, Köln</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>6</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H44" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2549,32 +2539,38 @@
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr"/>
       <c r="B45" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Calypso Ventures GmbH</t>
+          <t>coty</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
+          <t>Marketing Intern - Trade Marketing</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
+          <t>Darmstadt, Hessen</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>6</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>2025-08-15</t>
+        </is>
+      </c>
       <c r="H45" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2593,35 +2589,37 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr"/>
       <c r="B46" t="n">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>MILAN</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr"/>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>6</v>
+      </c>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2637,31 +2635,33 @@
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
+          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr"/>
       <c r="B47" t="n">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr"/>
+          <t>Altstadt, Düsseldorf</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>6</v>
+      </c>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
@@ -2681,32 +2681,36 @@
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr"/>
       <c r="B48" t="n">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H48" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2725,36 +2729,32 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5822943276?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=580C236799B96DFD395A1EC1CBBF7474C7F58435</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr"/>
       <c r="B49" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Sayano Deutschland GmbH</t>
+          <t>Calypso Ventures GmbH</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
+          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2773,35 +2773,35 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816572451?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr"/>
       <c r="B50" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Abrio</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
+          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -2817,28 +2817,28 @@
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr"/>
       <c r="B51" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Internship International Marketing Schwarzkopf Coloration - Legacy Brands</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Benrath, Düsseldorf</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
@@ -2861,33 +2861,31 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5819890143?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr"/>
       <c r="B52" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Lidl Stiftung</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food in Neckarsulm</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F52" t="n">
-        <v>6</v>
-      </c>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr">
         <is>
@@ -2907,32 +2905,36 @@
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813494719?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr"/>
       <c r="B53" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Lidl Stiftung &amp; Co. KG</t>
+          <t>Sayano Deutschland GmbH</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Mitte, Stuttgart</t>
         </is>
       </c>
       <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr"/>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H53" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2951,7 +2953,7 @@
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
+          <t>https://www.adzuna.de/details/5816572451?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2962,25 +2964,21 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Marc O'Polo</t>
+          <t>Abrio</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
+          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
+      <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2999,7 +2997,7 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3010,17 +3008,17 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Praktikum Marketing (m/w/d)</t>
+          <t>Internship International Marketing Schwarzkopf Coloration - Legacy Brands</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Benrath, Düsseldorf</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
@@ -3043,7 +3041,7 @@
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899691?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5819890143?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3054,24 +3052,24 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Praktikum Marketing (m/w/d)</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -3087,41 +3085,35 @@
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
+          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr"/>
       <c r="B57" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>LIGANOVA I Karriere</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Praktikum Buying (all genders) – August/September 2026</t>
+          <t>Praktikum Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
-        </is>
-      </c>
-      <c r="F57" t="n">
-        <v>6</v>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+          <t>Frankfurt am Main, DE, 60329</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -3137,7 +3129,7 @@
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805407495?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
         </is>
       </c>
     </row>
@@ -3148,24 +3140,30 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>LIGANOVA I Karriere</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Marketing &amp; Merchandising Assistant Trainee</t>
+          <t>Praktikum Buying (all genders) – August/September 2026</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>MILAN</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr"/>
+          <t>Mitte, Stuttgart</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>6</v>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -3181,7 +3179,7 @@
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
+          <t>https://www.adzuna.de/details/5805407495?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3195,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Marketing and Merchandising Assistant Trainee</t>
+          <t>Marketing &amp; Merchandising Assistant Trainee</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -3225,35 +3223,35 @@
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing-and-Merchandising-Assistant-Trainee_JR128690</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr"/>
       <c r="B60" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Digitalagenten</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
+          <t>Marketing and Merchandising Assistant Trainee</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Charlottenburg, Berlin</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -3269,7 +3267,7 @@
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804948828?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing-and-Merchandising-Assistant-Trainee_JR128690</t>
         </is>
       </c>
     </row>
@@ -3280,17 +3278,17 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>LIMITD by Wunderproducts GmbH</t>
+          <t>Digitalagenten</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Kreuzberg, Berlin</t>
+          <t>Charlottenburg, Berlin</t>
         </is>
       </c>
       <c r="F61" t="inlineStr"/>
@@ -3313,7 +3311,7 @@
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804948828?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3324,25 +3322,21 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers GmbH WPG</t>
+          <t>LIMITD by Wunderproducts GmbH</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Kreuzberg, Berlin</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
+      <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3361,7 +3355,7 @@
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3372,21 +3366,25 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>THE VERSE Ventures</t>
+          <t>PricewaterhouseCoopers GmbH WPG</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
       <c r="H63" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3405,7 +3403,7 @@
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3416,17 +3414,17 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>WirWinzer</t>
+          <t>THE VERSE Ventures</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Praktikum Business Development Weinhandel (all genders)</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F64" t="inlineStr"/>
@@ -3449,28 +3447,28 @@
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr"/>
       <c r="B65" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Brand Trust</t>
+          <t>WirWinzer</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
+          <t>Praktikum Business Development Weinhandel (all genders)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Gleißbühl, Nürnberg</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F65" t="inlineStr"/>
@@ -3493,7 +3491,7 @@
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5669847401?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3504,15 +3502,19 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Brand Trust</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr"/>
+          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Gleißbühl, Nürnberg</t>
+        </is>
+      </c>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
@@ -3533,7 +3535,7 @@
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
+          <t>https://www.adzuna.de/details/5669847401?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3549,7 +3551,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Operational Trade Marketing Intern</t>
+          <t>Marketing Intern - Trade Marketing</t>
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
@@ -3573,7 +3575,7 @@
       <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Toronto-Operational-Trade-Marketing-Intern-ON-M5H4H2/1397938633/</t>
+          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
         </is>
       </c>
     </row>
@@ -3584,19 +3586,15 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>Schwabing-Freimann, München</t>
-        </is>
-      </c>
+          <t>Operational Trade Marketing Intern</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr">
@@ -3617,7 +3615,7 @@
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://careers.coty.com/job/Toronto-Operational-Trade-Marketing-Intern-ON-M5H4H2/1397938633/</t>
         </is>
       </c>
     </row>
@@ -3628,24 +3626,24 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>DEU-Bayern-Unterhaching</t>
+          <t>Schwabing-Freimann, München</t>
         </is>
       </c>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -3661,7 +3659,7 @@
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
+          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3672,24 +3670,24 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>DEU-Bayern-Unterhaching</t>
         </is>
       </c>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -3705,7 +3703,7 @@
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
         </is>
       </c>
     </row>
@@ -3716,17 +3714,17 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
@@ -3749,7 +3747,7 @@
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
+          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3765,7 +3763,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -3793,7 +3791,7 @@
       <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
+          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
         </is>
       </c>
     </row>
@@ -3809,7 +3807,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3837,7 +3835,7 @@
       <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
+          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
         </is>
       </c>
     </row>
@@ -3848,17 +3846,17 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F74" t="inlineStr"/>
@@ -3881,28 +3879,28 @@
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr"/>
       <c r="B75" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>AUTO1 Global Services SE &amp; Co. KG</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (d/m/w)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
         </is>
       </c>
       <c r="F75" t="inlineStr"/>
@@ -3925,7 +3923,7 @@
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5789927805?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3936,17 +3934,17 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Amolina</t>
+          <t>AUTO1 Global Services SE &amp; Co. KG</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
+          <t>Praktikum Business Development (d/m/w)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F76" t="inlineStr"/>
@@ -3969,7 +3967,7 @@
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727292709?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5789927805?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3980,17 +3978,17 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>CTG Consulting</t>
+          <t>Amolina</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Praktikum Sales/Business Development // Hamburg oder Berlin</t>
+          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F77" t="inlineStr"/>
@@ -4013,7 +4011,7 @@
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5694221323?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5727292709?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4024,17 +4022,17 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Dronesperhour</t>
+          <t>CTG Consulting</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development eines Startups (m/w/d)</t>
+          <t>Praktikum Sales/Business Development // Hamburg oder Berlin</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Mitte, Berlin</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F78" t="inlineStr"/>
@@ -4057,7 +4055,7 @@
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5669955732?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5694221323?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4068,17 +4066,17 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>GrantLift GmbH</t>
+          <t>Dronesperhour</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
+          <t>Praktikum im Business Development eines Startups (m/w/d)</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Mitte, Berlin</t>
         </is>
       </c>
       <c r="F79" t="inlineStr"/>
@@ -4101,7 +4099,7 @@
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5803032426?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5669955732?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4122,7 +4120,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F80" t="inlineStr"/>
@@ -4145,7 +4143,7 @@
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804575149?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5803032426?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4156,17 +4154,17 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Otto Group one.O GmbH</t>
+          <t>GrantLift GmbH</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Praktikum im Knowledge Management - Corporate Strategy (w/m/d)</t>
+          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F81" t="inlineStr"/>
@@ -4189,7 +4187,7 @@
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5809516963?se=mrUvpGeQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=7970F7260CB99374DD6661F2025E46043B457CE4</t>
+          <t>https://www.adzuna.de/details/5804575149?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4200,17 +4198,17 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Pflegia</t>
+          <t>Otto Group one.O GmbH</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Praktikum im Knowledge Management - Corporate Strategy (w/m/d)</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F82" t="inlineStr"/>
@@ -4233,7 +4231,7 @@
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5821302522?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5809516963?se=mrUvpGeQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=7970F7260CB99374DD6661F2025E46043B457CE4</t>
         </is>
       </c>
     </row>
@@ -4254,7 +4252,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Wedding, Berlin</t>
         </is>
       </c>
       <c r="F83" t="inlineStr"/>
@@ -4277,7 +4275,7 @@
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802953545?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5821302522?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4293,12 +4291,12 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (Projektmanagement &amp; Prozessoptimierung) (m/w/d)</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
@@ -4321,7 +4319,7 @@
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802984051?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802953545?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4337,7 +4335,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (Business Analyst/Automation Engineer/Applied AI Engineer) (m/w/d)</t>
+          <t>Praktikum im Business Development (Projektmanagement &amp; Prozessoptimierung) (m/w/d)</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4365,7 +4363,7 @@
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802977130?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802984051?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4376,17 +4374,17 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>REWE Group</t>
+          <t>Pflegia</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Praktikum im Business Development (Business Analyst/Automation Engineer/Applied AI Engineer) (m/w/d)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Wedding, Berlin</t>
         </is>
       </c>
       <c r="F86" t="inlineStr"/>
@@ -4409,7 +4407,7 @@
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5712965755?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802977130?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4420,17 +4418,17 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>SHAVENT - ARA Sustainable Products</t>
+          <t>REWE Group</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Praktikum Business Development in nachhaltigem Start-Up (w/m/d) Remote in DE</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Sendling, München</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F87" t="inlineStr"/>
@@ -4453,7 +4451,7 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802951937?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5712965755?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4464,17 +4462,17 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>SINN Power</t>
+          <t>SHAVENT - ARA Sustainable Products</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Praktikum im AI Business Development (m/w/d)</t>
+          <t>Praktikum Business Development in nachhaltigem Start-Up (w/m/d) Remote in DE</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Kasten, München (Kreis)</t>
+          <t>Sendling, München</t>
         </is>
       </c>
       <c r="F88" t="inlineStr"/>
@@ -4497,7 +4495,7 @@
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727348338?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802951937?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4508,17 +4506,17 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>SINN Power</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Praktikum Strategy &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im AI Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Kasten, München (Kreis)</t>
         </is>
       </c>
       <c r="F89" t="inlineStr"/>
@@ -4541,7 +4539,7 @@
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5799516357?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5727348338?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4552,17 +4550,17 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Vitolus</t>
+          <t>Tchibo GmbH</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
+          <t>Praktikum Strategy &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
@@ -4585,7 +4583,7 @@
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5785872138?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5799516357?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4596,17 +4594,17 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Vivanta Gmbh</t>
+          <t>Vitolus</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F91" t="inlineStr"/>
@@ -4629,7 +4627,7 @@
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802952325?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5785872138?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4650,7 +4648,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F92" t="inlineStr"/>
@@ -4673,7 +4671,7 @@
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804549349?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802952325?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4684,12 +4682,12 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Werkia</t>
+          <t>Vivanta Gmbh</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d) - Datenanalyse &amp; Automatisierung</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -4717,7 +4715,7 @@
       <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802974922?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804549349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4733,7 +4731,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d) - Berlin</t>
+          <t>Praktikum Business Development (m/w/d) - Datenanalyse &amp; Automatisierung</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -4761,7 +4759,7 @@
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802950225?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802974922?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4772,17 +4770,17 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>innpuls</t>
+          <t>Werkia</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Praktikum im Business Development (m/w/d) - Berlin</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Wedding, Berlin</t>
         </is>
       </c>
       <c r="F95" t="inlineStr"/>
@@ -4805,7 +4803,7 @@
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5735591887?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802950225?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4816,17 +4814,17 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>paero</t>
+          <t>innpuls</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Ludwigsvorstadt-Isarvorstadt, München</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F96" t="inlineStr"/>
@@ -4849,28 +4847,28 @@
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813846665?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5735591887?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr"/>
       <c r="B97" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>paero</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Ludwigsvorstadt-Isarvorstadt, München</t>
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -4893,7 +4891,7 @@
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5813846665?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4914,7 +4912,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Altstadt-Nord, Köln</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F98" t="inlineStr"/>
@@ -4937,28 +4935,28 @@
       <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr"/>
       <c r="B99" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Devoteam G Cloud Germany</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt-Nord, Köln</t>
         </is>
       </c>
       <c r="F99" t="inlineStr"/>
@@ -4981,7 +4979,7 @@
       <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811135653?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4992,12 +4990,12 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>Devoteam G Cloud Germany</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -5025,7 +5023,7 @@
       <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5811135653?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5041,7 +5039,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -5069,7 +5067,7 @@
       <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5085,12 +5083,12 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F102" t="inlineStr"/>
@@ -5113,7 +5111,7 @@
       <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5129,7 +5127,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -5157,7 +5155,7 @@
       <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5168,17 +5166,17 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>sailwithus</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F104" t="inlineStr"/>
@@ -5201,7 +5199,7 @@
       <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5222,7 +5220,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F105" t="inlineStr"/>
@@ -5245,12 +5243,56 @@
       <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr"/>
+      <c r="B106" t="n">
+        <v>45</v>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>sailwithus</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr"/>
+      <c r="G106" t="inlineStr"/>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr"/>
+      <c r="L106" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5804544237?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L105"/>
+  <autoFilter ref="A1:L106"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5261,7 +5303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G82"/>
+  <dimension ref="A1:G83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -5317,7 +5359,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C2" t="n">
         <v>107</v>
@@ -5367,7 +5409,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C4" t="n">
         <v>89</v>
@@ -5392,7 +5434,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C5" t="n">
         <v>84</v>
@@ -5417,7 +5459,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C6" t="n">
         <v>84</v>
@@ -5442,7 +5484,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C7" t="n">
         <v>84</v>
@@ -5475,7 +5517,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C8" t="n">
         <v>84</v>
@@ -5500,7 +5542,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C9" t="n">
         <v>84</v>
@@ -5525,7 +5567,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
@@ -5550,7 +5592,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C11" t="n">
         <v>84</v>
@@ -5575,7 +5617,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C12" t="n">
         <v>80</v>
@@ -5600,7 +5642,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C13" t="n">
         <v>79</v>
@@ -5646,22 +5688,30 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C15" t="n">
         <v>78</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich Marketing für die Marke BE-KIND DACH</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>successfactors</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -5671,30 +5721,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Ferrero</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C16" t="n">
         <v>78</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>successfactors</t>
-        </is>
-      </c>
+          <t>Praktikum im Bereich Marketing für die Marke BE-KIND DACH</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -5704,18 +5746,18 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Miles &amp; More GmbH</t>
+          <t>Marc O'Polo</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C17" t="n">
         <v>74</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Internship Marketing Strategy &amp; Delivery</t>
+          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
@@ -5729,30 +5771,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>Miles &amp; More GmbH</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="C18" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Praktikum Category Management Non Food Vertrieb (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>successfactors</t>
-        </is>
-      </c>
+          <t>Internship Marketing Strategy &amp; Delivery</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -5762,22 +5796,30 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>Tchibo GmbH</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="C19" t="n">
         <v>73</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
+          <t>Praktikum Category Management Non Food Vertrieb (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>successfactors</t>
+        </is>
+      </c>
       <c r="G19" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -5787,18 +5829,18 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>P&amp;G</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C20" t="n">
         <v>73</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
@@ -5812,18 +5854,18 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>markenbaumarkt24</t>
+          <t>P&amp;G</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C21" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
@@ -5837,18 +5879,18 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>markenbaumarkt24</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C22" t="n">
         <v>72</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
         </is>
       </c>
       <c r="E22" t="inlineStr"/>
@@ -5862,30 +5904,22 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C23" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Intern Category Growth</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>successfactors</t>
-        </is>
-      </c>
+          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -5895,43 +5929,43 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>PARSA Haar- und Modeartikel GmbH</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="C24" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-08</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Bosch Thermotechnik GmbH</t>
+          <t>Lidl Stiftung</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>6</v>
       </c>
       <c r="C25" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Praktikum im internationalen Brand Management</t>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food in Neckarsulm</t>
         </is>
       </c>
       <c r="E25" t="inlineStr"/>
@@ -5945,22 +5979,30 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>L’ORÉAL</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="C26" t="n">
         <v>68</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>PRAKTIKUM (M/W/D) Product Marketing - Start ab August/September/Oktober für 6 Monate</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
+          <t>Intern Category Growth</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>successfactors</t>
+        </is>
+      </c>
       <c r="G26" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -5970,18 +6012,18 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C27" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr"/>
@@ -5995,18 +6037,18 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Calypso Ventures GmbH</t>
+          <t>Bosch Thermotechnik GmbH</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C28" t="n">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
+          <t>Praktikum im internationalen Brand Management</t>
         </is>
       </c>
       <c r="E28" t="inlineStr"/>
@@ -6020,30 +6062,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>L’ORÉAL</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="C29" t="n">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>workday</t>
-        </is>
-      </c>
+          <t>PRAKTIKUM (M/W/D) Product Marketing - Start ab August/September/Oktober für 6 Monate</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -6053,18 +6087,18 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C30" t="n">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr"/>
@@ -6078,18 +6112,18 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Sayano Deutschland GmbH</t>
+          <t>Calypso Ventures GmbH</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C31" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
+          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
@@ -6103,22 +6137,30 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Lidl Stiftung &amp; Co. KG</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="C32" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
+          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>workday</t>
+        </is>
+      </c>
       <c r="G32" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -6128,18 +6170,18 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Marc O'Polo</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C33" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E33" t="inlineStr"/>
@@ -6153,18 +6195,18 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Abrio</t>
+          <t>Sayano Deutschland GmbH</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C34" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
+          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
@@ -6178,18 +6220,18 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Lidl Stiftung</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C35" t="n">
         <v>54</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food in Neckarsulm</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E35" t="inlineStr"/>
@@ -6203,18 +6245,18 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>Abrio</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="C36" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr"/>
@@ -6228,18 +6270,18 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>sailwithus</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="C37" t="n">
         <v>53</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr"/>
@@ -6253,18 +6295,18 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Devoteam G Cloud Germany</t>
+          <t>sailwithus</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C38" t="n">
         <v>53</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
         </is>
       </c>
       <c r="E38" t="inlineStr"/>
@@ -6278,18 +6320,18 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>LIGANOVA I Karriere</t>
+          <t>Devoteam G Cloud Germany</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C39" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Praktikum Buying (all genders) – August/September 2026</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr"/>
@@ -6303,18 +6345,18 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>LIMITD by Wunderproducts GmbH</t>
+          <t>LIGANOVA I Karriere</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C40" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Praktikum Buying (all genders) – August/September 2026</t>
         </is>
       </c>
       <c r="E40" t="inlineStr"/>
@@ -6328,11 +6370,11 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>THE VERSE Ventures</t>
+          <t>LIMITD by Wunderproducts GmbH</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C41" t="n">
         <v>51</v>
@@ -6353,18 +6395,18 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>WirWinzer</t>
+          <t>THE VERSE Ventures</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C42" t="n">
         <v>51</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Praktikum Business Development Weinhandel (all genders)</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E42" t="inlineStr"/>
@@ -6378,18 +6420,18 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers GmbH WPG</t>
+          <t>WirWinzer</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C43" t="n">
         <v>51</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
+          <t>Praktikum Business Development Weinhandel (all genders)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr"/>
@@ -6403,18 +6445,18 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Digitalagenten</t>
+          <t>PricewaterhouseCoopers GmbH WPG</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C44" t="n">
         <v>51</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr"/>
@@ -6428,18 +6470,18 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Digitalagenten</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C45" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
+          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr"/>
@@ -6453,18 +6495,18 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Brand Trust</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="C46" t="n">
         <v>49</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
+          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
         </is>
       </c>
       <c r="E46" t="inlineStr"/>
@@ -6478,18 +6520,18 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>Brand Trust</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C47" t="n">
         <v>49</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
@@ -6503,18 +6545,18 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C48" t="n">
         <v>49</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
@@ -6528,18 +6570,18 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C49" t="n">
         <v>49</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr"/>
@@ -6553,18 +6595,18 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>REWE Group</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C50" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
@@ -6578,18 +6620,18 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Pflegia</t>
+          <t>REWE Group</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C51" t="n">
         <v>48</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr"/>
@@ -6603,18 +6645,18 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Werkia</t>
+          <t>Pflegia</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C52" t="n">
         <v>48</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d) - Datenanalyse &amp; Automatisierung</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr"/>
@@ -6628,7 +6670,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>paero</t>
+          <t>Werkia</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -6639,7 +6681,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/d) - Datenanalyse &amp; Automatisierung</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
@@ -6653,7 +6695,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Vivanta Gmbh</t>
+          <t>paero</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -6664,7 +6706,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr"/>
@@ -6678,7 +6720,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Vitolus</t>
+          <t>Vivanta Gmbh</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -6689,7 +6731,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr"/>
@@ -6703,7 +6745,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>GrantLift GmbH</t>
+          <t>Vitolus</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -6714,7 +6756,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
+          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr"/>
@@ -6728,7 +6770,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Otto Group one.O GmbH</t>
+          <t>GrantLift GmbH</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -6739,7 +6781,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Praktikum im Knowledge Management - Corporate Strategy (w/m/d)</t>
+          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E57" t="inlineStr"/>
@@ -6753,18 +6795,18 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>AUTO1 Global Services SE &amp; Co. KG</t>
+          <t>Otto Group one.O GmbH</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C58" t="n">
         <v>48</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (d/m/w)</t>
+          <t>Praktikum im Knowledge Management - Corporate Strategy (w/m/d)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
@@ -6778,7 +6820,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>SHAVENT - ARA Sustainable Products</t>
+          <t>AUTO1 Global Services SE &amp; Co. KG</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -6789,7 +6831,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Praktikum Business Development in nachhaltigem Start-Up (w/m/d) Remote in DE</t>
+          <t>Praktikum Business Development (d/m/w)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
@@ -6803,7 +6845,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CTG Consulting</t>
+          <t>SHAVENT - ARA Sustainable Products</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -6814,7 +6856,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Praktikum Sales/Business Development // Hamburg oder Berlin</t>
+          <t>Praktikum Business Development in nachhaltigem Start-Up (w/m/d) Remote in DE</t>
         </is>
       </c>
       <c r="E60" t="inlineStr"/>
@@ -6828,7 +6870,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Dronesperhour</t>
+          <t>CTG Consulting</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -6839,7 +6881,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development eines Startups (m/w/d)</t>
+          <t>Praktikum Sales/Business Development // Hamburg oder Berlin</t>
         </is>
       </c>
       <c r="E61" t="inlineStr"/>
@@ -6853,7 +6895,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>SINN Power</t>
+          <t>Dronesperhour</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -6864,7 +6906,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Praktikum im AI Business Development (m/w/d)</t>
+          <t>Praktikum im Business Development eines Startups (m/w/d)</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
@@ -6878,7 +6920,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>innpuls</t>
+          <t>SINN Power</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -6889,7 +6931,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Praktikum im AI Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
@@ -6903,7 +6945,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Amolina</t>
+          <t>innpuls</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -6914,7 +6956,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
@@ -6928,18 +6970,18 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>Amolina</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="C65" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
@@ -6953,18 +6995,18 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>STARTPLATZ Gruppe</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C66" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Sales (m/w/d) – STARTPLATZ</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
@@ -6978,7 +7020,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>spring.gate business consulting UG</t>
+          <t>STARTPLATZ Gruppe</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -6989,7 +7031,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development &amp; B2B Akquise (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Sales (m/w/d) – STARTPLATZ</t>
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
@@ -7003,7 +7045,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>specter automation</t>
+          <t>spring.gate business consulting UG</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -7014,7 +7056,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Praktikum (M/W/D) im Business Development</t>
+          <t>Praktikum im Business Development &amp; B2B Akquise (m/w/d)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr"/>
@@ -7028,18 +7070,18 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Closd Kunststoffprodukte GmbH</t>
+          <t>specter automation</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C69" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Praktikum beim E-Commerce Startup Closd als Founders Associate (m/w/d)</t>
+          <t>Praktikum (M/W/D) im Business Development</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
@@ -7053,18 +7095,18 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Bosch Rexroth AG</t>
+          <t>Closd Kunststoffprodukte GmbH</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C70" t="n">
         <v>38</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Praktikum Business Development – Software Defined Business</t>
+          <t>Praktikum beim E-Commerce Startup Closd als Founders Associate (m/w/d)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
@@ -7078,7 +7120,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Weenect</t>
+          <t>Bosch Rexroth AG</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -7089,7 +7131,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d) – Markt DACH – Standort Brüssel</t>
+          <t>Praktikum Business Development – Software Defined Business</t>
         </is>
       </c>
       <c r="E71" t="inlineStr"/>
@@ -7103,18 +7145,18 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Lidl Dienstleistung GmbH &amp; Co. KG</t>
+          <t>Weenect</t>
         </is>
       </c>
       <c r="B72" t="n">
         <v>1</v>
       </c>
       <c r="C72" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Praktikum Business Development (m/w/d) – Markt DACH – Standort Brüssel</t>
         </is>
       </c>
       <c r="E72" t="inlineStr"/>
@@ -7128,18 +7170,18 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Drägerwerk AG &amp; Co. KGaA</t>
+          <t>Lidl Dienstleistung GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C73" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Praktikum New Business Development</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E73" t="inlineStr"/>
@@ -7153,18 +7195,18 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Arteus Energy</t>
+          <t>Drägerwerk AG &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C74" t="n">
         <v>28</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Praktikum Business Development und Marketing Photovoltaik</t>
+          <t>Praktikum New Business Development</t>
         </is>
       </c>
       <c r="E74" t="inlineStr"/>
@@ -7178,7 +7220,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>aramido</t>
+          <t>Arteus Energy</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -7189,7 +7231,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/x)</t>
+          <t>Praktikum Business Development und Marketing Photovoltaik</t>
         </is>
       </c>
       <c r="E75" t="inlineStr"/>
@@ -7203,7 +7245,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>pacemaker.ai by thyssenkrupp</t>
+          <t>aramido</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -7214,7 +7256,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/x)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr"/>
@@ -7228,7 +7270,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Wonder Natural GmbH</t>
+          <t>pacemaker.ai by thyssenkrupp</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -7239,7 +7281,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr"/>
@@ -7253,7 +7295,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Molly Suh GmbH</t>
+          <t>Wonder Natural GmbH</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -7264,7 +7306,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; B2B Sales (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
         </is>
       </c>
       <c r="E78" t="inlineStr"/>
@@ -7278,7 +7320,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>homewise</t>
+          <t>Molly Suh GmbH</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -7289,7 +7331,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development &amp; Strategie (m/w/d)</t>
+          <t>Praktikum Business Development &amp; B2B Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E79" t="inlineStr"/>
@@ -7303,7 +7345,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>ClipMyHorse.TV</t>
+          <t>homewise</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -7314,7 +7356,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Praktikum HR &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im Business Development &amp; Strategie (m/w/d)</t>
         </is>
       </c>
       <c r="E80" t="inlineStr"/>
@@ -7328,7 +7370,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>AUMOVIO</t>
+          <t>ClipMyHorse.TV</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -7339,7 +7381,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Praktikum - Administration/Assistenz &amp; Business Development</t>
+          <t>Praktikum HR &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E81" t="inlineStr"/>
@@ -7353,7 +7395,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>TRUMPF Group</t>
+          <t>AUMOVIO</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -7364,7 +7406,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich Business Development für Smart Factory Solutions (WS26/27)</t>
+          <t>Praktikum - Administration/Assistenz &amp; Business Development</t>
         </is>
       </c>
       <c r="E82" t="inlineStr"/>
@@ -7375,8 +7417,33 @@
         </is>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>TRUMPF Group</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>1</v>
+      </c>
+      <c r="C83" t="n">
+        <v>28</v>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Praktikum im Bereich Business Development für Smart Factory Solutions (WS26/27)</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr"/>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G82"/>
+  <autoFilter ref="A1:G83"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Lauf 2026-08-09 07:04 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -2566,11 +2566,7 @@
       <c r="F45" t="n">
         <v>6</v>
       </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>2025-08-15</t>
-        </is>
-      </c>
+      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2688,29 +2684,25 @@
     <row r="48">
       <c r="A48" t="inlineStr"/>
       <c r="B48" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>Abrio</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2729,32 +2721,36 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5822943276?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=580C236799B96DFD395A1EC1CBBF7474C7F58435</t>
+          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr"/>
       <c r="B49" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Calypso Ventures GmbH</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H49" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2773,35 +2769,35 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5822943276?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=580C236799B96DFD395A1EC1CBBF7474C7F58435</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr"/>
       <c r="B50" t="n">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Calypso Ventures GmbH</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
+          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -2817,35 +2813,35 @@
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
+          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr"/>
       <c r="B51" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -2861,7 +2857,7 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
         </is>
       </c>
     </row>
@@ -2882,7 +2878,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F52" t="inlineStr"/>
@@ -2905,36 +2901,32 @@
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr"/>
       <c r="B53" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Sayano Deutschland GmbH</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2953,32 +2945,36 @@
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816572451?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr"/>
       <c r="B54" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Abrio</t>
+          <t>Sayano Deutschland GmbH</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
+          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Mitte, Stuttgart</t>
         </is>
       </c>
       <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H54" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2997,7 +2993,7 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5816572451?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5359,7 +5355,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C2" t="n">
         <v>107</v>
@@ -5409,7 +5405,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C4" t="n">
         <v>89</v>
@@ -5434,7 +5430,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C5" t="n">
         <v>84</v>
@@ -5459,7 +5455,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C6" t="n">
         <v>84</v>
@@ -5484,7 +5480,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C7" t="n">
         <v>84</v>
@@ -5517,7 +5513,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C8" t="n">
         <v>84</v>
@@ -5542,7 +5538,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C9" t="n">
         <v>84</v>
@@ -5567,7 +5563,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
@@ -5592,7 +5588,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C11" t="n">
         <v>84</v>
@@ -5617,7 +5613,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C12" t="n">
         <v>80</v>
@@ -5642,7 +5638,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C13" t="n">
         <v>79</v>
@@ -5692,7 +5688,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C15" t="n">
         <v>78</v>
@@ -5725,7 +5721,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C16" t="n">
         <v>78</v>
@@ -5750,7 +5746,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C17" t="n">
         <v>74</v>
@@ -5775,7 +5771,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C18" t="n">
         <v>74</v>
@@ -5800,7 +5796,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C19" t="n">
         <v>73</v>
@@ -5858,7 +5854,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C21" t="n">
         <v>73</v>
@@ -5883,7 +5879,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C22" t="n">
         <v>72</v>
@@ -5908,7 +5904,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C23" t="n">
         <v>72</v>
@@ -5958,7 +5954,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C25" t="n">
         <v>69</v>
@@ -5983,7 +5979,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C26" t="n">
         <v>68</v>
@@ -6016,7 +6012,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C27" t="n">
         <v>68</v>
@@ -6041,7 +6037,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C28" t="n">
         <v>68</v>
@@ -6066,7 +6062,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C29" t="n">
         <v>68</v>
@@ -6091,7 +6087,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C30" t="n">
         <v>66</v>
@@ -6112,18 +6108,18 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Calypso Ventures GmbH</t>
+          <t>Abrio</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C31" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
+          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
@@ -6137,30 +6133,22 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Calypso Ventures GmbH</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="C32" t="n">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>workday</t>
-        </is>
-      </c>
+          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -6170,22 +6158,30 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C33" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
+          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>workday</t>
+        </is>
+      </c>
       <c r="G33" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -6195,18 +6191,18 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Sayano Deutschland GmbH</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="C34" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
@@ -6220,18 +6216,18 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Lidl Stiftung &amp; Co. KG</t>
+          <t>Sayano Deutschland GmbH</t>
         </is>
       </c>
       <c r="B35" t="n">
         <v>8</v>
       </c>
       <c r="C35" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr"/>
@@ -6245,18 +6241,18 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Abrio</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C36" t="n">
         <v>54</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E36" t="inlineStr"/>
@@ -6274,7 +6270,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C37" t="n">
         <v>53</v>
@@ -6299,7 +6295,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C38" t="n">
         <v>53</v>
@@ -6324,7 +6320,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C39" t="n">
         <v>53</v>
@@ -6374,7 +6370,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C41" t="n">
         <v>51</v>
@@ -6399,7 +6395,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C42" t="n">
         <v>51</v>
@@ -6424,7 +6420,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C43" t="n">
         <v>51</v>
@@ -6449,7 +6445,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C44" t="n">
         <v>51</v>
@@ -6474,7 +6470,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C45" t="n">
         <v>51</v>
@@ -6499,7 +6495,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C46" t="n">
         <v>49</v>
@@ -6524,7 +6520,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C47" t="n">
         <v>49</v>
@@ -6549,7 +6545,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C48" t="n">
         <v>49</v>
@@ -6574,7 +6570,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C49" t="n">
         <v>49</v>
@@ -6599,7 +6595,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C50" t="n">
         <v>49</v>
@@ -6624,7 +6620,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C51" t="n">
         <v>48</v>
@@ -6999,7 +6995,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C66" t="n">
         <v>46</v>

</xml_diff>

<commit_message>
Lauf 2026-08-10 07:39 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -34,7 +34,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -44,11 +44,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F3864"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D8F3DC"/>
       </patternFill>
     </fill>
   </fills>
@@ -64,12 +59,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2114,48 +2108,44 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="n">
+      <c r="A36" t="inlineStr"/>
+      <c r="B36" t="n">
         <v>70</v>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>PARSA Haar- und Modeartikel GmbH</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr"/>
-      <c r="G36" s="2" t="inlineStr"/>
-      <c r="H36" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I36" s="2" t="inlineStr">
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
         <is>
           <t>2026-08-08</t>
         </is>
       </c>
-      <c r="J36" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K36" s="2" t="inlineStr"/>
-      <c r="L36" s="2" t="inlineStr">
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr">
         <is>
           <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
         </is>
@@ -5312,37 +5302,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Unternehmen</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Treffer</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Bester Score</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Beispielrolle</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Wird überwacht</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>System</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Zuerst gesehen</t>
         </is>
@@ -5355,7 +5345,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C2" t="n">
         <v>107</v>
@@ -5405,7 +5395,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C4" t="n">
         <v>89</v>
@@ -5430,7 +5420,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C5" t="n">
         <v>84</v>
@@ -5455,7 +5445,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C6" t="n">
         <v>84</v>
@@ -5480,7 +5470,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C7" t="n">
         <v>84</v>
@@ -5509,18 +5499,18 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Nestle</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C8" t="n">
         <v>84</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
@@ -5534,18 +5524,18 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Nestle</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C9" t="n">
         <v>84</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
@@ -5563,7 +5553,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
@@ -5588,7 +5578,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C11" t="n">
         <v>84</v>
@@ -5613,7 +5603,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C12" t="n">
         <v>80</v>
@@ -5638,7 +5628,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C13" t="n">
         <v>79</v>
@@ -5688,7 +5678,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C15" t="n">
         <v>78</v>
@@ -5721,7 +5711,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C16" t="n">
         <v>78</v>
@@ -5746,7 +5736,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C17" t="n">
         <v>74</v>
@@ -5771,7 +5761,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C18" t="n">
         <v>74</v>
@@ -5796,7 +5786,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C19" t="n">
         <v>73</v>
@@ -5854,7 +5844,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C21" t="n">
         <v>73</v>
@@ -5879,7 +5869,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C22" t="n">
         <v>72</v>
@@ -5904,7 +5894,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C23" t="n">
         <v>72</v>
@@ -5954,7 +5944,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C25" t="n">
         <v>69</v>
@@ -5979,7 +5969,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C26" t="n">
         <v>68</v>
@@ -6012,7 +6002,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C27" t="n">
         <v>68</v>
@@ -6037,7 +6027,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C28" t="n">
         <v>68</v>
@@ -6062,7 +6052,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C29" t="n">
         <v>68</v>
@@ -6087,7 +6077,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C30" t="n">
         <v>66</v>
@@ -6112,7 +6102,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C31" t="n">
         <v>65</v>
@@ -6137,7 +6127,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C32" t="n">
         <v>62</v>
@@ -6162,7 +6152,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C33" t="n">
         <v>57</v>
@@ -6195,7 +6185,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C34" t="n">
         <v>56</v>
@@ -6220,7 +6210,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C35" t="n">
         <v>55</v>
@@ -6245,7 +6235,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C36" t="n">
         <v>54</v>
@@ -6270,7 +6260,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C37" t="n">
         <v>53</v>
@@ -6295,7 +6285,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C38" t="n">
         <v>53</v>
@@ -6320,7 +6310,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C39" t="n">
         <v>53</v>
@@ -6370,7 +6360,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C41" t="n">
         <v>51</v>
@@ -6395,7 +6385,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C42" t="n">
         <v>51</v>
@@ -6420,7 +6410,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C43" t="n">
         <v>51</v>
@@ -6445,7 +6435,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C44" t="n">
         <v>51</v>
@@ -6470,7 +6460,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C45" t="n">
         <v>51</v>
@@ -6495,7 +6485,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C46" t="n">
         <v>49</v>
@@ -6520,7 +6510,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C47" t="n">
         <v>49</v>
@@ -6545,7 +6535,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C48" t="n">
         <v>49</v>
@@ -6570,7 +6560,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C49" t="n">
         <v>49</v>
@@ -6595,7 +6585,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C50" t="n">
         <v>49</v>
@@ -6620,7 +6610,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C51" t="n">
         <v>48</v>
@@ -6995,7 +6985,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C66" t="n">
         <v>46</v>

</xml_diff>

<commit_message>
Lauf 2026-08-11 07:13 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firmen entdeckt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$106</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$107</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$83</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -34,7 +34,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -44,6 +44,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D8F3DC"/>
       </patternFill>
     </fill>
   </fills>
@@ -59,11 +64,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -430,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L106"/>
+  <dimension ref="A1:L107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2722,28 +2728,30 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>Praktikum Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr"/>
+          <t>Frankfurt am Main, DE, 60329</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>5</v>
+      </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -2759,32 +2767,36 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5822943276?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=580C236799B96DFD395A1EC1CBBF7474C7F58435</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr"/>
       <c r="B50" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Calypso Ventures GmbH</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H50" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2803,35 +2815,35 @@
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5822943276?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=580C236799B96DFD395A1EC1CBBF7474C7F58435</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr"/>
       <c r="B51" t="n">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Calypso Ventures GmbH</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
+          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -2847,35 +2859,35 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
+          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr"/>
       <c r="B52" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -2891,7 +2903,7 @@
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
         </is>
       </c>
     </row>
@@ -2912,7 +2924,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F53" t="inlineStr"/>
@@ -2935,36 +2947,32 @@
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr"/>
       <c r="B54" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Sayano Deutschland GmbH</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2983,32 +2991,36 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816572451?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr"/>
       <c r="B55" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>Sayano Deutschland GmbH</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Internship International Marketing Schwarzkopf Coloration - Legacy Brands</t>
+          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Benrath, Düsseldorf</t>
+          <t>Mitte, Stuttgart</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H55" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3027,7 +3039,7 @@
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5819890143?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5816572451?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3038,17 +3050,17 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Lidl Stiftung &amp; Co. KG</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Internship International Marketing Schwarzkopf Coloration - Legacy Brands</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Benrath, Düsseldorf</t>
         </is>
       </c>
       <c r="F56" t="inlineStr"/>
@@ -3071,7 +3083,7 @@
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
+          <t>https://www.adzuna.de/details/5819890143?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3082,24 +3094,24 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Praktikum Marketing (m/w/d)</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -3115,7 +3127,7 @@
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
+          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
         </is>
       </c>
     </row>
@@ -3606,46 +3618,50 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr"/>
-      <c r="B69" t="n">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="n">
         <v>49</v>
       </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>Honest Catch</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>Schwabing-Freimann, München</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr"/>
-      <c r="G69" t="inlineStr"/>
-      <c r="H69" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J69" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K69" t="inlineStr"/>
-      <c r="L69" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Henkel</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>Benrath, Düsseldorf</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr"/>
+      <c r="G69" s="2" t="inlineStr"/>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K69" s="2" t="inlineStr"/>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3656,24 +3672,24 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>DEU-Bayern-Unterhaching</t>
+          <t>Schwabing-Freimann, München</t>
         </is>
       </c>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -3689,7 +3705,7 @@
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
+          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3700,24 +3716,24 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>DEU-Bayern-Unterhaching</t>
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -3733,7 +3749,7 @@
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
         </is>
       </c>
     </row>
@@ -3744,17 +3760,17 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F72" t="inlineStr"/>
@@ -3777,7 +3793,7 @@
       <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
+          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3793,7 +3809,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3821,7 +3837,7 @@
       <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
+          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
         </is>
       </c>
     </row>
@@ -3837,7 +3853,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3865,7 +3881,7 @@
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
+          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
         </is>
       </c>
     </row>
@@ -3876,17 +3892,17 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F75" t="inlineStr"/>
@@ -3909,28 +3925,28 @@
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr"/>
       <c r="B76" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>AUTO1 Global Services SE &amp; Co. KG</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (d/m/w)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
         </is>
       </c>
       <c r="F76" t="inlineStr"/>
@@ -3953,7 +3969,7 @@
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5789927805?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3964,17 +3980,17 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Amolina</t>
+          <t>AUTO1 Global Services SE &amp; Co. KG</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
+          <t>Praktikum Business Development (d/m/w)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F77" t="inlineStr"/>
@@ -3997,7 +4013,7 @@
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727292709?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5789927805?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4008,17 +4024,17 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>CTG Consulting</t>
+          <t>Amolina</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Praktikum Sales/Business Development // Hamburg oder Berlin</t>
+          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F78" t="inlineStr"/>
@@ -4041,7 +4057,7 @@
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5694221323?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5727292709?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4052,17 +4068,17 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Dronesperhour</t>
+          <t>CTG Consulting</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development eines Startups (m/w/d)</t>
+          <t>Praktikum Sales/Business Development // Hamburg oder Berlin</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Mitte, Berlin</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F79" t="inlineStr"/>
@@ -4085,7 +4101,7 @@
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5669955732?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5694221323?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4096,17 +4112,17 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>GrantLift GmbH</t>
+          <t>Dronesperhour</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
+          <t>Praktikum im Business Development eines Startups (m/w/d)</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Mitte, Berlin</t>
         </is>
       </c>
       <c r="F80" t="inlineStr"/>
@@ -4129,7 +4145,7 @@
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5803032426?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5669955732?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4150,7 +4166,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F81" t="inlineStr"/>
@@ -4173,7 +4189,7 @@
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804575149?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5803032426?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4184,17 +4200,17 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Otto Group one.O GmbH</t>
+          <t>GrantLift GmbH</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Praktikum im Knowledge Management - Corporate Strategy (w/m/d)</t>
+          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F82" t="inlineStr"/>
@@ -4217,7 +4233,7 @@
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5809516963?se=mrUvpGeQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=7970F7260CB99374DD6661F2025E46043B457CE4</t>
+          <t>https://www.adzuna.de/details/5804575149?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4228,17 +4244,17 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Pflegia</t>
+          <t>Otto Group one.O GmbH</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Praktikum im Knowledge Management - Corporate Strategy (w/m/d)</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F83" t="inlineStr"/>
@@ -4261,7 +4277,7 @@
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5821302522?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5809516963?se=mrUvpGeQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=7970F7260CB99374DD6661F2025E46043B457CE4</t>
         </is>
       </c>
     </row>
@@ -4282,7 +4298,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Wedding, Berlin</t>
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
@@ -4305,7 +4321,7 @@
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802953545?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5821302522?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4321,12 +4337,12 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (Projektmanagement &amp; Prozessoptimierung) (m/w/d)</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
@@ -4349,7 +4365,7 @@
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802984051?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802953545?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4365,7 +4381,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (Business Analyst/Automation Engineer/Applied AI Engineer) (m/w/d)</t>
+          <t>Praktikum im Business Development (Projektmanagement &amp; Prozessoptimierung) (m/w/d)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -4393,7 +4409,7 @@
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802977130?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802984051?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4404,17 +4420,17 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>REWE Group</t>
+          <t>Pflegia</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Praktikum im Business Development (Business Analyst/Automation Engineer/Applied AI Engineer) (m/w/d)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Wedding, Berlin</t>
         </is>
       </c>
       <c r="F87" t="inlineStr"/>
@@ -4437,7 +4453,7 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5712965755?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802977130?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4448,17 +4464,17 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>SHAVENT - ARA Sustainable Products</t>
+          <t>REWE Group</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Praktikum Business Development in nachhaltigem Start-Up (w/m/d) Remote in DE</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Sendling, München</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F88" t="inlineStr"/>
@@ -4481,7 +4497,7 @@
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802951937?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5712965755?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4492,17 +4508,17 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>SINN Power</t>
+          <t>SHAVENT - ARA Sustainable Products</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Praktikum im AI Business Development (m/w/d)</t>
+          <t>Praktikum Business Development in nachhaltigem Start-Up (w/m/d) Remote in DE</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Kasten, München (Kreis)</t>
+          <t>Sendling, München</t>
         </is>
       </c>
       <c r="F89" t="inlineStr"/>
@@ -4525,7 +4541,7 @@
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727348338?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802951937?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4536,17 +4552,17 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>SINN Power</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Praktikum Strategy &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im AI Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Kasten, München (Kreis)</t>
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
@@ -4569,7 +4585,7 @@
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5799516357?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5727348338?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4580,17 +4596,17 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Vitolus</t>
+          <t>Tchibo GmbH</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
+          <t>Praktikum Strategy &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F91" t="inlineStr"/>
@@ -4613,7 +4629,7 @@
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5785872138?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5799516357?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4624,17 +4640,17 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Vivanta Gmbh</t>
+          <t>Vitolus</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F92" t="inlineStr"/>
@@ -4657,7 +4673,7 @@
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802952325?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5785872138?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4678,7 +4694,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F93" t="inlineStr"/>
@@ -4701,7 +4717,7 @@
       <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804549349?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802952325?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4712,12 +4728,12 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Werkia</t>
+          <t>Vivanta Gmbh</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d) - Datenanalyse &amp; Automatisierung</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -4745,7 +4761,7 @@
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802974922?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804549349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4761,7 +4777,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d) - Berlin</t>
+          <t>Praktikum Business Development (m/w/d) - Datenanalyse &amp; Automatisierung</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4789,7 +4805,7 @@
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802950225?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802974922?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4800,17 +4816,17 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>innpuls</t>
+          <t>Werkia</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Praktikum im Business Development (m/w/d) - Berlin</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Wedding, Berlin</t>
         </is>
       </c>
       <c r="F96" t="inlineStr"/>
@@ -4833,7 +4849,7 @@
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5735591887?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802950225?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4844,17 +4860,17 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>paero</t>
+          <t>innpuls</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Ludwigsvorstadt-Isarvorstadt, München</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -4877,28 +4893,28 @@
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813846665?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5735591887?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr"/>
       <c r="B98" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>paero</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Ludwigsvorstadt-Isarvorstadt, München</t>
         </is>
       </c>
       <c r="F98" t="inlineStr"/>
@@ -4921,7 +4937,7 @@
       <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5813846665?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4942,7 +4958,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Altstadt-Nord, Köln</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F99" t="inlineStr"/>
@@ -4965,28 +4981,28 @@
       <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr"/>
       <c r="B100" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Devoteam G Cloud Germany</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt-Nord, Köln</t>
         </is>
       </c>
       <c r="F100" t="inlineStr"/>
@@ -5009,7 +5025,7 @@
       <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811135653?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5020,12 +5036,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>Devoteam G Cloud Germany</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -5053,7 +5069,7 @@
       <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5811135653?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5069,7 +5085,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -5097,7 +5113,7 @@
       <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5113,12 +5129,12 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F103" t="inlineStr"/>
@@ -5141,7 +5157,7 @@
       <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5157,7 +5173,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -5185,7 +5201,7 @@
       <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5196,17 +5212,17 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>sailwithus</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F105" t="inlineStr"/>
@@ -5229,7 +5245,7 @@
       <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5250,7 +5266,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F106" t="inlineStr"/>
@@ -5273,12 +5289,56 @@
       <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr"/>
+      <c r="B107" t="n">
+        <v>45</v>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>sailwithus</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr"/>
+      <c r="G107" t="inlineStr"/>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr"/>
+      <c r="L107" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5804544237?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L106"/>
+  <autoFilter ref="A1:L107"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5302,37 +5362,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Unternehmen</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Treffer</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Bester Score</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Beispielrolle</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Wird überwacht</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>System</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Zuerst gesehen</t>
         </is>
@@ -5345,7 +5405,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C2" t="n">
         <v>107</v>
@@ -5370,7 +5430,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C3" t="n">
         <v>91</v>
@@ -5395,7 +5455,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C4" t="n">
         <v>89</v>
@@ -5420,7 +5480,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C5" t="n">
         <v>84</v>
@@ -5445,7 +5505,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C6" t="n">
         <v>84</v>
@@ -5470,7 +5530,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C7" t="n">
         <v>84</v>
@@ -5503,7 +5563,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C8" t="n">
         <v>84</v>
@@ -5528,7 +5588,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C9" t="n">
         <v>84</v>
@@ -5553,7 +5613,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
@@ -5578,7 +5638,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C11" t="n">
         <v>84</v>
@@ -5603,7 +5663,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C12" t="n">
         <v>80</v>
@@ -5678,7 +5738,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C15" t="n">
         <v>78</v>
@@ -5711,7 +5771,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C16" t="n">
         <v>78</v>
@@ -5736,7 +5796,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C17" t="n">
         <v>74</v>
@@ -5761,7 +5821,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C18" t="n">
         <v>74</v>
@@ -5786,7 +5846,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C19" t="n">
         <v>73</v>
@@ -5844,7 +5904,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C21" t="n">
         <v>73</v>
@@ -5869,7 +5929,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C22" t="n">
         <v>72</v>
@@ -5894,7 +5954,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C23" t="n">
         <v>72</v>
@@ -5944,7 +6004,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C25" t="n">
         <v>69</v>
@@ -5969,7 +6029,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C26" t="n">
         <v>68</v>
@@ -6002,7 +6062,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C27" t="n">
         <v>68</v>
@@ -6027,7 +6087,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C28" t="n">
         <v>68</v>
@@ -6077,7 +6137,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C30" t="n">
         <v>66</v>
@@ -6102,7 +6162,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C31" t="n">
         <v>65</v>
@@ -6127,7 +6187,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C32" t="n">
         <v>62</v>
@@ -6152,7 +6212,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C33" t="n">
         <v>57</v>
@@ -6185,7 +6245,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C34" t="n">
         <v>56</v>
@@ -6235,7 +6295,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C36" t="n">
         <v>54</v>
@@ -6260,7 +6320,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C37" t="n">
         <v>53</v>
@@ -6285,7 +6345,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C38" t="n">
         <v>53</v>
@@ -6310,7 +6370,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C39" t="n">
         <v>53</v>
@@ -6360,7 +6420,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C41" t="n">
         <v>51</v>
@@ -6385,7 +6445,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C42" t="n">
         <v>51</v>
@@ -6410,7 +6470,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C43" t="n">
         <v>51</v>
@@ -6435,7 +6495,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C44" t="n">
         <v>51</v>
@@ -6460,7 +6520,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C45" t="n">
         <v>51</v>
@@ -6485,7 +6545,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C46" t="n">
         <v>49</v>
@@ -6510,7 +6570,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C47" t="n">
         <v>49</v>
@@ -6535,7 +6595,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C48" t="n">
         <v>49</v>
@@ -6560,7 +6620,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C49" t="n">
         <v>49</v>
@@ -6585,7 +6645,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C50" t="n">
         <v>49</v>
@@ -6610,7 +6670,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C51" t="n">
         <v>48</v>
@@ -6985,7 +7045,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C66" t="n">
         <v>46</v>

</xml_diff>

<commit_message>
Lauf 2026-08-12 07:32 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firmen entdeckt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$107</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$108</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$84</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L107"/>
+  <dimension ref="A1:L108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5074,46 +5074,50 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" t="inlineStr"/>
-      <c r="B102" t="n">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>prepmymeal GmbH</t>
-        </is>
-      </c>
-      <c r="D102" t="inlineStr">
-        <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F102" t="inlineStr"/>
-      <c r="G102" t="inlineStr"/>
-      <c r="H102" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I102" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J102" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K102" t="inlineStr"/>
-      <c r="L102" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>freudio</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>Wien, Österreich</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr"/>
+      <c r="G102" s="2" t="inlineStr"/>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I102" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="J102" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K102" s="2" t="inlineStr"/>
+      <c r="L102" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.at/details/5836667156?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5129,7 +5133,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -5157,7 +5161,7 @@
       <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5173,12 +5177,12 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F104" t="inlineStr"/>
@@ -5201,7 +5205,7 @@
       <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5221,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -5245,7 +5249,7 @@
       <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5256,17 +5260,17 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>sailwithus</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F106" t="inlineStr"/>
@@ -5289,7 +5293,7 @@
       <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5310,7 +5314,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F107" t="inlineStr"/>
@@ -5333,12 +5337,56 @@
       <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr"/>
+      <c r="B108" t="n">
+        <v>45</v>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>sailwithus</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr"/>
+      <c r="G108" t="inlineStr"/>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr"/>
+      <c r="L108" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5804544237?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L107"/>
+  <autoFilter ref="A1:L108"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5349,7 +5397,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G83"/>
+  <dimension ref="A1:G84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -5405,7 +5453,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C2" t="n">
         <v>107</v>
@@ -5455,7 +5503,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C4" t="n">
         <v>89</v>
@@ -5480,7 +5528,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C5" t="n">
         <v>84</v>
@@ -5505,7 +5553,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C6" t="n">
         <v>84</v>
@@ -5530,7 +5578,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C7" t="n">
         <v>84</v>
@@ -5563,7 +5611,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C8" t="n">
         <v>84</v>
@@ -5588,7 +5636,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C9" t="n">
         <v>84</v>
@@ -5613,7 +5661,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
@@ -5638,7 +5686,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C11" t="n">
         <v>84</v>
@@ -5663,7 +5711,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C12" t="n">
         <v>80</v>
@@ -5738,7 +5786,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C15" t="n">
         <v>78</v>
@@ -5771,7 +5819,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C16" t="n">
         <v>78</v>
@@ -5796,7 +5844,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C17" t="n">
         <v>74</v>
@@ -5821,7 +5869,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C18" t="n">
         <v>74</v>
@@ -5846,7 +5894,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C19" t="n">
         <v>73</v>
@@ -5904,7 +5952,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C21" t="n">
         <v>73</v>
@@ -5929,7 +5977,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C22" t="n">
         <v>72</v>
@@ -5954,7 +6002,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C23" t="n">
         <v>72</v>
@@ -6004,7 +6052,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C25" t="n">
         <v>69</v>
@@ -6029,7 +6077,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C26" t="n">
         <v>68</v>
@@ -6062,7 +6110,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C27" t="n">
         <v>68</v>
@@ -6087,7 +6135,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C28" t="n">
         <v>68</v>
@@ -6137,7 +6185,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C30" t="n">
         <v>66</v>
@@ -6162,7 +6210,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C31" t="n">
         <v>65</v>
@@ -6187,7 +6235,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C32" t="n">
         <v>62</v>
@@ -6212,7 +6260,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C33" t="n">
         <v>57</v>
@@ -6245,7 +6293,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C34" t="n">
         <v>56</v>
@@ -6320,7 +6368,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C37" t="n">
         <v>53</v>
@@ -6345,7 +6393,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C38" t="n">
         <v>53</v>
@@ -6370,7 +6418,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C39" t="n">
         <v>53</v>
@@ -6420,7 +6468,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C41" t="n">
         <v>51</v>
@@ -6445,7 +6493,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C42" t="n">
         <v>51</v>
@@ -6470,7 +6518,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C43" t="n">
         <v>51</v>
@@ -6495,7 +6543,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C44" t="n">
         <v>51</v>
@@ -6520,7 +6568,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C45" t="n">
         <v>51</v>
@@ -6545,7 +6593,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C46" t="n">
         <v>49</v>
@@ -6570,7 +6618,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C47" t="n">
         <v>49</v>
@@ -6595,7 +6643,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C48" t="n">
         <v>49</v>
@@ -6620,7 +6668,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C49" t="n">
         <v>49</v>
@@ -6645,7 +6693,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C50" t="n">
         <v>49</v>
@@ -6670,7 +6718,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C51" t="n">
         <v>48</v>
@@ -7045,7 +7093,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C66" t="n">
         <v>46</v>
@@ -7066,32 +7114,32 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>STARTPLATZ Gruppe</t>
+          <t>freudio</t>
         </is>
       </c>
       <c r="B67" t="n">
         <v>1</v>
       </c>
       <c r="C67" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Sales (m/w/d) – STARTPLATZ</t>
+          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>spring.gate business consulting UG</t>
+          <t>STARTPLATZ Gruppe</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -7102,7 +7150,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development &amp; B2B Akquise (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Sales (m/w/d) – STARTPLATZ</t>
         </is>
       </c>
       <c r="E68" t="inlineStr"/>
@@ -7116,7 +7164,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>specter automation</t>
+          <t>spring.gate business consulting UG</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -7127,7 +7175,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Praktikum (M/W/D) im Business Development</t>
+          <t>Praktikum im Business Development &amp; B2B Akquise (m/w/d)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
@@ -7141,18 +7189,18 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Closd Kunststoffprodukte GmbH</t>
+          <t>specter automation</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C70" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Praktikum beim E-Commerce Startup Closd als Founders Associate (m/w/d)</t>
+          <t>Praktikum (M/W/D) im Business Development</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
@@ -7166,18 +7214,18 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Bosch Rexroth AG</t>
+          <t>Closd Kunststoffprodukte GmbH</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C71" t="n">
         <v>38</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Praktikum Business Development – Software Defined Business</t>
+          <t>Praktikum beim E-Commerce Startup Closd als Founders Associate (m/w/d)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr"/>
@@ -7191,7 +7239,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Weenect</t>
+          <t>Bosch Rexroth AG</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -7202,7 +7250,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d) – Markt DACH – Standort Brüssel</t>
+          <t>Praktikum Business Development – Software Defined Business</t>
         </is>
       </c>
       <c r="E72" t="inlineStr"/>
@@ -7216,18 +7264,18 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Lidl Dienstleistung GmbH &amp; Co. KG</t>
+          <t>Weenect</t>
         </is>
       </c>
       <c r="B73" t="n">
         <v>1</v>
       </c>
       <c r="C73" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Praktikum Business Development (m/w/d) – Markt DACH – Standort Brüssel</t>
         </is>
       </c>
       <c r="E73" t="inlineStr"/>
@@ -7241,18 +7289,18 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Drägerwerk AG &amp; Co. KGaA</t>
+          <t>Lidl Dienstleistung GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C74" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Praktikum New Business Development</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E74" t="inlineStr"/>
@@ -7266,18 +7314,18 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Arteus Energy</t>
+          <t>Drägerwerk AG &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C75" t="n">
         <v>28</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Praktikum Business Development und Marketing Photovoltaik</t>
+          <t>Praktikum New Business Development</t>
         </is>
       </c>
       <c r="E75" t="inlineStr"/>
@@ -7291,7 +7339,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>aramido</t>
+          <t>Arteus Energy</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -7302,7 +7350,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/x)</t>
+          <t>Praktikum Business Development und Marketing Photovoltaik</t>
         </is>
       </c>
       <c r="E76" t="inlineStr"/>
@@ -7316,7 +7364,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>pacemaker.ai by thyssenkrupp</t>
+          <t>aramido</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -7327,7 +7375,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/x)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr"/>
@@ -7341,7 +7389,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Wonder Natural GmbH</t>
+          <t>pacemaker.ai by thyssenkrupp</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -7352,7 +7400,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E78" t="inlineStr"/>
@@ -7366,7 +7414,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Molly Suh GmbH</t>
+          <t>Wonder Natural GmbH</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -7377,7 +7425,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; B2B Sales (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
         </is>
       </c>
       <c r="E79" t="inlineStr"/>
@@ -7391,7 +7439,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>homewise</t>
+          <t>Molly Suh GmbH</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -7402,7 +7450,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development &amp; Strategie (m/w/d)</t>
+          <t>Praktikum Business Development &amp; B2B Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E80" t="inlineStr"/>
@@ -7416,7 +7464,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ClipMyHorse.TV</t>
+          <t>homewise</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -7427,7 +7475,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Praktikum HR &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im Business Development &amp; Strategie (m/w/d)</t>
         </is>
       </c>
       <c r="E81" t="inlineStr"/>
@@ -7441,7 +7489,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>AUMOVIO</t>
+          <t>ClipMyHorse.TV</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -7452,7 +7500,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Praktikum - Administration/Assistenz &amp; Business Development</t>
+          <t>Praktikum HR &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E82" t="inlineStr"/>
@@ -7466,7 +7514,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>TRUMPF Group</t>
+          <t>AUMOVIO</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -7477,7 +7525,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich Business Development für Smart Factory Solutions (WS26/27)</t>
+          <t>Praktikum - Administration/Assistenz &amp; Business Development</t>
         </is>
       </c>
       <c r="E83" t="inlineStr"/>
@@ -7488,8 +7536,33 @@
         </is>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>TRUMPF Group</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>1</v>
+      </c>
+      <c r="C84" t="n">
+        <v>28</v>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Praktikum im Bereich Business Development für Smart Factory Solutions (WS26/27)</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr"/>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G83"/>
+  <autoFilter ref="A1:G84"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Lauf 2026-08-14 07:32 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firmen entdeckt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$109</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$110</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$85</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L109"/>
+  <dimension ref="A1:L110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2868,50 +2868,56 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr"/>
-      <c r="B52" t="n">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="n">
         <v>64</v>
       </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>PENNY International</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>Köln, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5822943276?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=580C236799B96DFD395A1EC1CBBF7474C7F58435</t>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Nestle Deutschland</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum Marketing &amp; Sales (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main, DE, 60329</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>fmcg</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr"/>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-&amp;-Sales-%28mwd%29-60329/1425985633/</t>
         </is>
       </c>
     </row>
@@ -2922,21 +2928,25 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>WirWinzer</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Praktikum Business Development Weinhandel (all genders)</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr"/>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H53" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2955,28 +2965,28 @@
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5822943276?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=580C236799B96DFD395A1EC1CBBF7474C7F58435</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr"/>
       <c r="B54" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Calypso Ventures GmbH</t>
+          <t>WirWinzer</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
+          <t>Praktikum Business Development Weinhandel (all genders)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F54" t="inlineStr"/>
@@ -2999,35 +3009,35 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr"/>
       <c r="B55" t="n">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Calypso Ventures GmbH</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
+          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3043,35 +3053,35 @@
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
+          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr"/>
       <c r="B56" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -3087,7 +3097,7 @@
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
         </is>
       </c>
     </row>
@@ -3108,7 +3118,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F57" t="inlineStr"/>
@@ -3131,36 +3141,32 @@
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr"/>
       <c r="B58" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Sayano Deutschland GmbH</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3179,7 +3185,7 @@
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816572451?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3190,23 +3196,25 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>THE VERSE Ventures</t>
+          <t>Sayano Deutschland GmbH</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
-        </is>
-      </c>
-      <c r="F59" t="n">
-        <v>6</v>
-      </c>
-      <c r="G59" t="inlineStr"/>
+          <t>Mitte, Stuttgart</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H59" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3225,31 +3233,33 @@
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5816572451?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr"/>
       <c r="B60" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>THE VERSE Ventures</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Internship International Marketing Schwarzkopf Coloration - Legacy Brands</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Benrath, Düsseldorf</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr"/>
+          <t>Berlin, Deutschland</t>
+        </is>
+      </c>
+      <c r="F60" t="n">
+        <v>6</v>
+      </c>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
@@ -3269,7 +3279,7 @@
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5819890143?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3280,17 +3290,17 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Lidl Stiftung &amp; Co. KG</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Internship International Marketing Schwarzkopf Coloration - Legacy Brands</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Benrath, Düsseldorf</t>
         </is>
       </c>
       <c r="F61" t="inlineStr"/>
@@ -3313,38 +3323,32 @@
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
+          <t>https://www.adzuna.de/details/5819890143?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr"/>
       <c r="B62" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>LIGANOVA I Karriere</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Praktikum Buying (all genders) – August/September 2026</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
-        </is>
-      </c>
-      <c r="F62" t="n">
-        <v>6</v>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3363,7 +3367,7 @@
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805407495?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
         </is>
       </c>
     </row>
@@ -3374,24 +3378,30 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>LIGANOVA I Karriere</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Marketing &amp; Merchandising Assistant Trainee</t>
+          <t>Praktikum Buying (all genders) – August/September 2026</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>MILAN</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
+          <t>Mitte, Stuttgart</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>6</v>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -3407,7 +3417,7 @@
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
+          <t>https://www.adzuna.de/details/5805407495?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3423,7 +3433,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Marketing and Merchandising Assistant Trainee</t>
+          <t>Marketing &amp; Merchandising Assistant Trainee</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -3451,35 +3461,35 @@
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing-and-Merchandising-Assistant-Trainee_JR128690</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr"/>
       <c r="B65" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Digitalagenten</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
+          <t>Marketing and Merchandising Assistant Trainee</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Charlottenburg, Berlin</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -3495,103 +3505,103 @@
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing-and-Merchandising-Assistant-Trainee_JR128690</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr"/>
+      <c r="B66" t="n">
+        <v>51</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Digitalagenten</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Charlottenburg, Berlin</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5804948828?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="2" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
         <is>
           <t>NEU</t>
         </is>
       </c>
-      <c r="B66" s="2" t="n">
+      <c r="B67" s="2" t="n">
         <v>51</v>
       </c>
-      <c r="C66" s="2" t="inlineStr">
+      <c r="C67" s="2" t="inlineStr">
         <is>
           <t>SERVICEPLAN Gruppe</t>
         </is>
       </c>
-      <c r="D66" s="2" t="inlineStr">
+      <c r="D67" s="2" t="inlineStr">
         <is>
           <t>Praktikum Business Development &amp; Sales (Marketing / New Business) (all genders)</t>
         </is>
       </c>
-      <c r="E66" s="2" t="inlineStr">
+      <c r="E67" s="2" t="inlineStr">
         <is>
           <t>München, München (Kreis)</t>
         </is>
       </c>
-      <c r="F66" s="2" t="inlineStr"/>
-      <c r="G66" s="2" t="inlineStr">
+      <c r="F67" s="2" t="inlineStr"/>
+      <c r="G67" s="2" t="inlineStr">
         <is>
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="H66" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I66" s="2" t="inlineStr">
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="J66" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K66" s="2" t="inlineStr"/>
-      <c r="L66" s="2" t="inlineStr">
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K67" s="2" t="inlineStr"/>
+      <c r="L67" s="2" t="inlineStr">
         <is>
           <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr"/>
-      <c r="B67" t="n">
-        <v>49</v>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>Brand Trust</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>Gleißbühl, Nürnberg</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr"/>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K67" t="inlineStr"/>
-      <c r="L67" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5669847401?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3602,15 +3612,19 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Brand Trust</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr"/>
+          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Gleißbühl, Nürnberg</t>
+        </is>
+      </c>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr">
@@ -3631,7 +3645,7 @@
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
+          <t>https://www.adzuna.de/details/5669847401?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3647,7 +3661,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Operational Trade Marketing Intern</t>
+          <t>Marketing Intern - Trade Marketing</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
@@ -3671,7 +3685,7 @@
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Toronto-Operational-Trade-Marketing-Intern-ON-M5H4H2/1397938633/</t>
+          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
         </is>
       </c>
     </row>
@@ -3682,19 +3696,15 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>Benrath, Düsseldorf</t>
-        </is>
-      </c>
+          <t>Operational Trade Marketing Intern</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
@@ -3704,7 +3714,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -3715,7 +3725,7 @@
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://careers.coty.com/job/Toronto-Operational-Trade-Marketing-Intern-ON-M5H4H2/1397938633/</t>
         </is>
       </c>
     </row>
@@ -3726,17 +3736,17 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
+          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Schwabing-Freimann, München</t>
+          <t>Benrath, Düsseldorf</t>
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
@@ -3748,7 +3758,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
@@ -3759,7 +3769,7 @@
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3770,24 +3780,24 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>DEU-Bayern-Unterhaching</t>
+          <t>Schwabing-Freimann, München</t>
         </is>
       </c>
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -3803,7 +3813,7 @@
       <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
+          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3814,24 +3824,24 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>DEU-Bayern-Unterhaching</t>
         </is>
       </c>
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -3847,7 +3857,7 @@
       <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
         </is>
       </c>
     </row>
@@ -3858,17 +3868,17 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F74" t="inlineStr"/>
@@ -3891,7 +3901,7 @@
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
+          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3907,7 +3917,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3935,7 +3945,7 @@
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
+          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
         </is>
       </c>
     </row>
@@ -3951,7 +3961,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -3979,7 +3989,7 @@
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
+          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
         </is>
       </c>
     </row>
@@ -3990,17 +4000,17 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F77" t="inlineStr"/>
@@ -4023,28 +4033,28 @@
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr"/>
       <c r="B78" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>AUTO1 Global Services SE &amp; Co. KG</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (d/m/w)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
         </is>
       </c>
       <c r="F78" t="inlineStr"/>
@@ -4067,7 +4077,7 @@
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5789927805?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4078,17 +4088,17 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Amolina</t>
+          <t>AUTO1 Global Services SE &amp; Co. KG</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
+          <t>Praktikum Business Development (d/m/w)</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F79" t="inlineStr"/>
@@ -4111,7 +4121,7 @@
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727292709?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5789927805?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4122,17 +4132,17 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>CTG Consulting</t>
+          <t>Amolina</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Praktikum Sales/Business Development // Hamburg oder Berlin</t>
+          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F80" t="inlineStr"/>
@@ -4155,7 +4165,7 @@
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5694221323?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5727292709?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4166,17 +4176,17 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Dronesperhour</t>
+          <t>CTG Consulting</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development eines Startups (m/w/d)</t>
+          <t>Praktikum Sales/Business Development // Hamburg oder Berlin</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Mitte, Berlin</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F81" t="inlineStr"/>
@@ -4199,7 +4209,7 @@
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5669955732?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5694221323?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4210,17 +4220,17 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>GrantLift GmbH</t>
+          <t>Dronesperhour</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
+          <t>Praktikum im Business Development eines Startups (m/w/d)</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Mitte, Berlin</t>
         </is>
       </c>
       <c r="F82" t="inlineStr"/>
@@ -4243,7 +4253,7 @@
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5803032426?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5669955732?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4264,7 +4274,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F83" t="inlineStr"/>
@@ -4287,7 +4297,7 @@
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804575149?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5803032426?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4298,17 +4308,17 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Otto Group one.O GmbH</t>
+          <t>GrantLift GmbH</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Praktikum im Knowledge Management - Corporate Strategy (w/m/d)</t>
+          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
@@ -4331,7 +4341,7 @@
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5809516963?se=mrUvpGeQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=7970F7260CB99374DD6661F2025E46043B457CE4</t>
+          <t>https://www.adzuna.de/details/5804575149?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4342,17 +4352,17 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Pflegia</t>
+          <t>Otto Group one.O GmbH</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Praktikum im Knowledge Management - Corporate Strategy (w/m/d)</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
@@ -4375,7 +4385,7 @@
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5821302522?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5809516963?se=mrUvpGeQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=7970F7260CB99374DD6661F2025E46043B457CE4</t>
         </is>
       </c>
     </row>
@@ -4396,7 +4406,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Wedding, Berlin</t>
         </is>
       </c>
       <c r="F86" t="inlineStr"/>
@@ -4419,7 +4429,7 @@
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802953545?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5821302522?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4435,12 +4445,12 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (Projektmanagement &amp; Prozessoptimierung) (m/w/d)</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F87" t="inlineStr"/>
@@ -4463,7 +4473,7 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802984051?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802953545?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4479,7 +4489,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (Business Analyst/Automation Engineer/Applied AI Engineer) (m/w/d)</t>
+          <t>Praktikum im Business Development (Projektmanagement &amp; Prozessoptimierung) (m/w/d)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -4507,7 +4517,7 @@
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802977130?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802984051?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4518,17 +4528,17 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>REWE Group</t>
+          <t>Pflegia</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Praktikum im Business Development (Business Analyst/Automation Engineer/Applied AI Engineer) (m/w/d)</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Wedding, Berlin</t>
         </is>
       </c>
       <c r="F89" t="inlineStr"/>
@@ -4551,7 +4561,7 @@
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5712965755?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802977130?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4562,17 +4572,17 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>SHAVENT - ARA Sustainable Products</t>
+          <t>REWE Group</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Praktikum Business Development in nachhaltigem Start-Up (w/m/d) Remote in DE</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Sendling, München</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
@@ -4595,7 +4605,7 @@
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802951937?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5712965755?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4606,17 +4616,17 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>SINN Power</t>
+          <t>SHAVENT - ARA Sustainable Products</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Praktikum im AI Business Development (m/w/d)</t>
+          <t>Praktikum Business Development in nachhaltigem Start-Up (w/m/d) Remote in DE</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Kasten, München (Kreis)</t>
+          <t>Sendling, München</t>
         </is>
       </c>
       <c r="F91" t="inlineStr"/>
@@ -4639,7 +4649,7 @@
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727348338?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802951937?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4650,17 +4660,17 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>SINN Power</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Praktikum Strategy &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im AI Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Kasten, München (Kreis)</t>
         </is>
       </c>
       <c r="F92" t="inlineStr"/>
@@ -4683,7 +4693,7 @@
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5799516357?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5727348338?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4694,17 +4704,17 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Vitolus</t>
+          <t>Tchibo GmbH</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
+          <t>Praktikum Strategy &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F93" t="inlineStr"/>
@@ -4727,7 +4737,7 @@
       <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5785872138?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5799516357?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4738,17 +4748,17 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Vivanta Gmbh</t>
+          <t>Vitolus</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F94" t="inlineStr"/>
@@ -4771,7 +4781,7 @@
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802952325?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5785872138?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4792,7 +4802,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F95" t="inlineStr"/>
@@ -4815,7 +4825,7 @@
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804549349?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802952325?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4826,12 +4836,12 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Werkia</t>
+          <t>Vivanta Gmbh</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d) - Datenanalyse &amp; Automatisierung</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -4859,7 +4869,7 @@
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802974922?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804549349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4875,7 +4885,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d) - Berlin</t>
+          <t>Praktikum Business Development (m/w/d) - Datenanalyse &amp; Automatisierung</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4903,7 +4913,7 @@
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802950225?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802974922?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4914,17 +4924,17 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>innpuls</t>
+          <t>Werkia</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Praktikum im Business Development (m/w/d) - Berlin</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Wedding, Berlin</t>
         </is>
       </c>
       <c r="F98" t="inlineStr"/>
@@ -4947,7 +4957,7 @@
       <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5735591887?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802950225?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4958,17 +4968,17 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>paero</t>
+          <t>innpuls</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Ludwigsvorstadt-Isarvorstadt, München</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F99" t="inlineStr"/>
@@ -4991,28 +5001,28 @@
       <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813846665?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5735591887?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr"/>
       <c r="B100" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>paero</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Ludwigsvorstadt-Isarvorstadt, München</t>
         </is>
       </c>
       <c r="F100" t="inlineStr"/>
@@ -5035,7 +5045,7 @@
       <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5813846665?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5056,7 +5066,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Altstadt-Nord, Köln</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F101" t="inlineStr"/>
@@ -5079,28 +5089,28 @@
       <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr"/>
       <c r="B102" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Devoteam G Cloud Germany</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt-Nord, Köln</t>
         </is>
       </c>
       <c r="F102" t="inlineStr"/>
@@ -5123,55 +5133,51 @@
       <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr"/>
+      <c r="B103" t="n">
+        <v>45</v>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Devoteam G Cloud Germany</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Praktikum im Business Development (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr"/>
+      <c r="G103" t="inlineStr"/>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr"/>
+      <c r="L103" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5811135653?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B103" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="C103" s="2" t="inlineStr">
-        <is>
-          <t>freudio</t>
-        </is>
-      </c>
-      <c r="D103" s="2" t="inlineStr">
-        <is>
-          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
-        </is>
-      </c>
-      <c r="E103" s="2" t="inlineStr">
-        <is>
-          <t>Wien, Österreich</t>
-        </is>
-      </c>
-      <c r="F103" s="2" t="inlineStr"/>
-      <c r="G103" s="2" t="inlineStr"/>
-      <c r="H103" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I103" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="J103" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K103" s="2" t="inlineStr"/>
-      <c r="L103" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.at/details/5836667156?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5182,17 +5188,17 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>freudio</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Wien, Österreich</t>
         </is>
       </c>
       <c r="F104" t="inlineStr"/>
@@ -5204,7 +5210,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -5215,7 +5221,7 @@
       <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/details/5836667156?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5231,7 +5237,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -5259,7 +5265,7 @@
       <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5275,12 +5281,12 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F106" t="inlineStr"/>
@@ -5303,7 +5309,7 @@
       <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5319,7 +5325,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -5347,7 +5353,7 @@
       <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5358,17 +5364,17 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>sailwithus</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F108" t="inlineStr"/>
@@ -5391,7 +5397,7 @@
       <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5412,7 +5418,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F109" t="inlineStr"/>
@@ -5435,12 +5441,56 @@
       <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr"/>
+      <c r="B110" t="n">
+        <v>45</v>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>sailwithus</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr"/>
+      <c r="G110" t="inlineStr"/>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr"/>
+      <c r="L110" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5804544237?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L109"/>
+  <autoFilter ref="A1:L110"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5532,7 +5582,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C3" t="n">
         <v>91</v>
@@ -5557,7 +5607,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C4" t="n">
         <v>89</v>
@@ -5582,7 +5632,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C5" t="n">
         <v>84</v>
@@ -5607,7 +5657,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C6" t="n">
         <v>84</v>
@@ -5632,7 +5682,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C7" t="n">
         <v>84</v>
@@ -5665,7 +5715,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C8" t="n">
         <v>84</v>
@@ -5690,7 +5740,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C9" t="n">
         <v>84</v>
@@ -5715,7 +5765,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
@@ -5740,7 +5790,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C11" t="n">
         <v>84</v>
@@ -5765,7 +5815,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C12" t="n">
         <v>84</v>
@@ -5790,7 +5840,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C13" t="n">
         <v>84</v>
@@ -5815,7 +5865,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C14" t="n">
         <v>80</v>
@@ -5890,7 +5940,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C17" t="n">
         <v>78</v>
@@ -5923,7 +5973,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C18" t="n">
         <v>78</v>
@@ -5948,7 +5998,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C19" t="n">
         <v>74</v>
@@ -5973,7 +6023,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C20" t="n">
         <v>74</v>
@@ -5998,7 +6048,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C21" t="n">
         <v>73</v>
@@ -6027,18 +6077,18 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>P&amp;G</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C22" t="n">
         <v>73</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr"/>
@@ -6052,7 +6102,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>P&amp;G</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -6063,7 +6113,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
         </is>
       </c>
       <c r="E23" t="inlineStr"/>
@@ -6081,7 +6131,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C24" t="n">
         <v>72</v>
@@ -6106,7 +6156,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C25" t="n">
         <v>72</v>
@@ -6156,7 +6206,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C27" t="n">
         <v>69</v>
@@ -6181,7 +6231,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C28" t="n">
         <v>68</v>
@@ -6214,7 +6264,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C29" t="n">
         <v>68</v>
@@ -6239,7 +6289,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C30" t="n">
         <v>68</v>
@@ -6289,7 +6339,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C32" t="n">
         <v>66</v>
@@ -6314,7 +6364,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C33" t="n">
         <v>65</v>
@@ -6339,7 +6389,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C34" t="n">
         <v>64</v>
@@ -6364,7 +6414,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C35" t="n">
         <v>62</v>
@@ -6389,7 +6439,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C36" t="n">
         <v>57</v>
@@ -6422,7 +6472,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C37" t="n">
         <v>56</v>
@@ -6447,7 +6497,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C38" t="n">
         <v>55</v>
@@ -6522,7 +6572,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="C41" t="n">
         <v>53</v>
@@ -6547,7 +6597,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C42" t="n">
         <v>53</v>
@@ -6572,7 +6622,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C43" t="n">
         <v>53</v>
@@ -6622,7 +6672,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C45" t="n">
         <v>51</v>
@@ -6647,7 +6697,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C46" t="n">
         <v>51</v>
@@ -6672,7 +6722,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C47" t="n">
         <v>49</v>
@@ -6697,7 +6747,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C48" t="n">
         <v>49</v>
@@ -6722,7 +6772,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C49" t="n">
         <v>49</v>
@@ -6747,7 +6797,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C50" t="n">
         <v>49</v>
@@ -6772,7 +6822,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C51" t="n">
         <v>49</v>
@@ -6797,7 +6847,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C52" t="n">
         <v>48</v>
@@ -7172,7 +7222,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C67" t="n">
         <v>46</v>
@@ -7197,7 +7247,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C68" t="n">
         <v>45</v>

</xml_diff>

<commit_message>
Lauf 2026-08-17 07:01 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -1176,50 +1176,46 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="n">
+      <c r="A16" t="inlineStr"/>
+      <c r="B16" t="n">
         <v>84</v>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>Wonder Natural GmbH</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="F16" s="2" t="n">
+      <c r="F16" t="n">
         <v>3</v>
       </c>
-      <c r="G16" s="2" t="inlineStr"/>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
         <is>
           <t>2026-08-15</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr"/>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr">
         <is>
           <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
@@ -5760,7 +5756,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C3" t="n">
         <v>91</v>
@@ -5785,7 +5781,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C4" t="n">
         <v>89</v>
@@ -5810,7 +5806,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="C5" t="n">
         <v>84</v>
@@ -5835,7 +5831,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C6" t="n">
         <v>84</v>
@@ -5860,7 +5856,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C7" t="n">
         <v>84</v>
@@ -5893,7 +5889,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C8" t="n">
         <v>84</v>
@@ -5918,7 +5914,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C9" t="n">
         <v>84</v>
@@ -5943,7 +5939,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
@@ -5968,7 +5964,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C11" t="n">
         <v>84</v>
@@ -5993,7 +5989,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C12" t="n">
         <v>84</v>
@@ -6018,7 +6014,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C13" t="n">
         <v>84</v>
@@ -6043,7 +6039,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C14" t="n">
         <v>84</v>
@@ -6068,7 +6064,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C15" t="n">
         <v>84</v>
@@ -6093,7 +6089,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C16" t="n">
         <v>80</v>
@@ -6168,7 +6164,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C19" t="n">
         <v>78</v>
@@ -6201,7 +6197,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C20" t="n">
         <v>78</v>
@@ -6251,7 +6247,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C22" t="n">
         <v>74</v>
@@ -6276,7 +6272,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C23" t="n">
         <v>74</v>
@@ -6301,7 +6297,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C24" t="n">
         <v>73</v>
@@ -6334,7 +6330,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C25" t="n">
         <v>73</v>
@@ -6384,7 +6380,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C27" t="n">
         <v>72</v>
@@ -6409,7 +6405,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C28" t="n">
         <v>72</v>
@@ -6434,7 +6430,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C29" t="n">
         <v>69</v>
@@ -6459,7 +6455,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C30" t="n">
         <v>68</v>
@@ -6492,7 +6488,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C31" t="n">
         <v>68</v>
@@ -6517,7 +6513,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C32" t="n">
         <v>68</v>
@@ -6567,7 +6563,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C34" t="n">
         <v>66</v>
@@ -6592,7 +6588,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C35" t="n">
         <v>65</v>
@@ -6617,7 +6613,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C36" t="n">
         <v>64</v>
@@ -6642,7 +6638,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C37" t="n">
         <v>62</v>
@@ -6667,7 +6663,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C38" t="n">
         <v>62</v>
@@ -6700,7 +6696,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C39" t="n">
         <v>57</v>
@@ -6733,7 +6729,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C40" t="n">
         <v>56</v>
@@ -6758,7 +6754,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C41" t="n">
         <v>55</v>
@@ -6833,7 +6829,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C44" t="n">
         <v>53</v>
@@ -6858,7 +6854,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C45" t="n">
         <v>53</v>
@@ -6883,7 +6879,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C46" t="n">
         <v>53</v>
@@ -6933,7 +6929,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C48" t="n">
         <v>51</v>
@@ -6958,7 +6954,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C49" t="n">
         <v>49</v>
@@ -6983,7 +6979,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C50" t="n">
         <v>49</v>
@@ -7008,7 +7004,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C51" t="n">
         <v>49</v>
@@ -7033,7 +7029,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C52" t="n">
         <v>49</v>
@@ -7058,7 +7054,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C53" t="n">
         <v>49</v>
@@ -7083,7 +7079,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C54" t="n">
         <v>48</v>
@@ -7458,7 +7454,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C69" t="n">
         <v>46</v>
@@ -7483,7 +7479,7 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C70" t="n">
         <v>45</v>

</xml_diff>

<commit_message>
Lauf 2026-08-18 06:49 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -34,7 +34,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -44,11 +44,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F3864"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D8F3DC"/>
       </patternFill>
     </fill>
   </fills>
@@ -64,12 +59,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1044,17 +1038,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>PARSA Haar- und Modeartikel GmbH</t>
+          <t>Picnic</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
+          <t>Category Management Praktikum (m/w/d)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -1068,7 +1062,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1079,7 +1073,7 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
+          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1094,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F14" t="n">
@@ -1125,34 +1119,36 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759088383?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="n">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Picnic</t>
+          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Category Management Praktikum (m/w/d)</t>
+          <t>Praktikum Brand Management National</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F15" t="n">
-        <v>6</v>
-      </c>
-      <c r="G15" t="inlineStr"/>
+          <t>Au-Haidhausen, München</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1171,42 +1167,38 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759088383?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805399065?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="n">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Wonder Natural GmbH</t>
+          <t>EAT HAPPY GROUP</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
+          <t>Praktikum Brand Marketing (m/w/d) Marketing · Köln</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
       <c r="F16" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1217,34 +1209,36 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://eathappygroup.teamtailor.com/jobs/7902845-praktikum-brand-marketing-m-w-d</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
+          <t>Marc O'Polo</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management National</t>
+          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Au-Haidhausen, München</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr"/>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>6</v>
+      </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1265,7 +1259,7 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805399065?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1276,22 +1270,26 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>EAT HAPPY GROUP</t>
+          <t>Yogi Tea</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Praktikum Brand Marketing (m/w/d) Marketing · Köln</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
+          <t>Praktikum im Marketing - Brand &amp; Product / mindestens 5 Monate</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Hamburg, Deutschland</t>
+        </is>
+      </c>
       <c r="F18" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1307,34 +1305,38 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://eathappygroup.teamtailor.com/jobs/7902845-praktikum-brand-marketing-m-w-d</t>
+          <t>https://www.adzuna.de/details/5744980745?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
       <c r="B19" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Yogi Tea</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Praktikum im Marketing - Brand &amp; Product / mindestens 5 Monate</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>5</v>
-      </c>
-      <c r="G19" t="inlineStr"/>
+        <v>6</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1353,7 +1355,7 @@
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5744980745?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1369,7 +1371,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1382,7 +1384,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1403,7 +1405,7 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5799961458?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1419,7 +1421,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1430,11 +1432,7 @@
       <c r="F21" t="n">
         <v>6</v>
       </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1453,7 +1451,7 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5799961458?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1464,17 +1462,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Ferrero</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikum im Bereich Marketing für die Marke BE-KIND DACH</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F22" t="n">
@@ -1499,7 +1497,7 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5753617280?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1510,23 +1508,27 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich Marketing für die Marke BE-KIND DACH</t>
+          <t>Praktikum Brand Management (m/w/d)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F23" t="n">
         <v>6</v>
       </c>
-      <c r="G23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="H23" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1545,38 +1547,32 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5753617280?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802899675?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d)</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F24" t="n">
-        <v>6</v>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1584,7 +1580,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -1595,151 +1591,139 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899675?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5843630960?se=znNqlDyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=875B574D03DFD36B16B3A3ABE0AA46F858215182</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="n">
+      <c r="A25" t="inlineStr"/>
+      <c r="B25" t="n">
         <v>74</v>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr"/>
-      <c r="G25" s="2" t="inlineStr"/>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I25" s="2" t="inlineStr">
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
         <is>
           <t>2026-08-16</t>
         </is>
       </c>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K25" s="2" t="inlineStr"/>
-      <c r="L25" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5843630960?se=znNqlDyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=875B574D03DFD36B16B3A3ABE0AA46F858215182</t>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/land/ad/5843628966?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=3DAF9A0A7032477BEFBE4DD229577F81F1D32CF0</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="n">
+      <c r="A26" t="inlineStr"/>
+      <c r="B26" t="n">
         <v>74</v>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
         <is>
           <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr"/>
-      <c r="G26" s="2" t="inlineStr"/>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
         <is>
           <t>2026-08-16</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr"/>
-      <c r="L26" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5843628966?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=3DAF9A0A7032477BEFBE4DD229577F81F1D32CF0</t>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/land/ad/5843628932?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=65C46D18FCDB11FD2E933BD305E494E07D043D72</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="n">
+      <c r="A27" t="inlineStr"/>
+      <c r="B27" t="n">
         <v>74</v>
       </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr"/>
-      <c r="G27" s="2" t="inlineStr"/>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I27" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-16</t>
-        </is>
-      </c>
-      <c r="J27" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K27" s="2" t="inlineStr"/>
-      <c r="L27" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5843628932?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=65C46D18FCDB11FD2E933BD305E494E07D043D72</t>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Miles &amp; More GmbH</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Internship Marketing Strategy &amp; Delivery</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Flughafen, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5828674997?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1750,27 +1734,21 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Marc O'Polo</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
+          <t>Praktikum Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F28" t="n">
-        <v>6</v>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1789,32 +1767,38 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802899691?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Miles &amp; More GmbH</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Internship Marketing Strategy &amp; Delivery</t>
+          <t>Praktikum Digital Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Flughafen, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
+          <t>Benrath, Düsseldorf</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>6</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
       <c r="H29" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1833,31 +1817,33 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5828674997?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5816415884?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Praktikum Marketing (m/w/d)</t>
+          <t>Praktikum im Bereich Marketing für die Marke BE-KIND DACH</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr"/>
+          <t>Unterhaching, München (Kreis)</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>6</v>
+      </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
@@ -1877,7 +1863,7 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899691?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5752932983?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1888,17 +1874,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>P&amp;G</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F31" t="n">
@@ -1923,7 +1909,7 @@
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1934,27 +1920,23 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>Tchibo GmbH</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Praktikum Digital Marketing &amp; Category Management</t>
+          <t>Praktikum Category Management Non Food Vertrieb (m/w/d)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Benrath, Düsseldorf</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F32" t="n">
         <v>6</v>
       </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
+      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1973,7 +1955,7 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816415884?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5795118484?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1984,17 +1966,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Tchibo GmbH</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich Marketing für die Marke BE-KIND DACH</t>
+          <t>Praktikum CNX Category Management Home &amp; Living (m/w/d)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Unterhaching, München (Kreis)</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F33" t="n">
@@ -2019,7 +2001,7 @@
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5752932983?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5765078175?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2030,17 +2012,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>P&amp;G</t>
+          <t>Tchibo GmbH</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum Trade Marketing Tchibo (m/w/d)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F34" t="n">
@@ -2065,7 +2047,7 @@
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5744245447?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2081,7 +2063,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Praktikum Category Management Non Food Vertrieb (m/w/d)</t>
+          <t>Praktikum Trade Marketing Eduscho (m/w/d)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2111,32 +2093,32 @@
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5795118484?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5773205889?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Praktikum CNX Category Management Home &amp; Living (m/w/d)</t>
+          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
@@ -2157,32 +2139,32 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5765078175?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>markenbaumarkt24</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing Tchibo (m/w/d)</t>
+          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Feuersbach, Siegen</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
@@ -2203,33 +2185,31 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5744245447?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="n">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>PARSA Haar- und Modeartikel GmbH</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing Eduscho (m/w/d)</t>
+          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
-        </is>
-      </c>
-      <c r="F38" t="n">
-        <v>6</v>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
@@ -2238,7 +2218,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -2249,32 +2229,32 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5773205889?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr"/>
       <c r="B39" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>Lidl Stiftung</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food in Neckarsulm</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
@@ -2295,33 +2275,31 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5813494719?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr"/>
       <c r="B40" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>markenbaumarkt24</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Feuersbach, Siegen</t>
-        </is>
-      </c>
-      <c r="F40" t="n">
-        <v>2</v>
-      </c>
+          <t>Hamburg, Deutschland</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
@@ -2341,28 +2319,28 @@
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr"/>
       <c r="B41" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Lidl Stiftung</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food in Neckarsulm</t>
+          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F41" t="n">
@@ -2387,31 +2365,33 @@
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813494719?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr"/>
       <c r="B42" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr"/>
+          <t>Köln, Nordrhein-Westfalen</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>6</v>
+      </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
@@ -2431,7 +2411,7 @@
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
+          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2447,7 +2427,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
+          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2458,7 +2438,11 @@
       <c r="F43" t="n">
         <v>6</v>
       </c>
-      <c r="G43" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H43" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2477,7 +2461,7 @@
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2488,17 +2472,17 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>Bosch Thermotechnik GmbH</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
+          <t>Praktikum im internationalen Brand Management</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Wernau (Neckar), Esslingen (Kreis)</t>
         </is>
       </c>
       <c r="F44" t="n">
@@ -2506,7 +2490,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -2527,7 +2511,7 @@
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5799981240?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2538,27 +2522,23 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Bosch Thermotechnik GmbH</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Praktikum im internationalen Brand Management</t>
+          <t>Intern Category Growth</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Wernau (Neckar), Esslingen (Kreis)</t>
+          <t>Darmstadt, Hessen</t>
         </is>
       </c>
       <c r="F45" t="n">
         <v>6</v>
       </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2577,7 +2557,7 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5799981240?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5754086625?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2588,23 +2568,27 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>L’ORÉAL</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Intern Category Growth</t>
+          <t>PRAKTIKUM (M/W/D) Product Marketing - Start ab August/September/Oktober für 6 Monate</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Darmstadt, Hessen</t>
+          <t>Nordrhein-Westfalen, Deutschland</t>
         </is>
       </c>
       <c r="F46" t="n">
         <v>6</v>
       </c>
-      <c r="G46" t="inlineStr"/>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H46" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2623,7 +2607,7 @@
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5754086625?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5754061318?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2634,17 +2618,17 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>L’ORÉAL</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>PRAKTIKUM (M/W/D) Product Marketing - Start ab August/September/Oktober für 6 Monate</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Nordrhein-Westfalen, Deutschland</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F47" t="n">
@@ -2673,7 +2657,7 @@
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5754061318?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2684,27 +2668,23 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>coty</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>Marketing Intern - Trade Marketing</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Darmstadt, Hessen</t>
         </is>
       </c>
       <c r="F48" t="n">
         <v>6</v>
       </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2723,28 +2703,28 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr"/>
       <c r="B49" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>coty</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Darmstadt, Hessen</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F49" t="n">
@@ -2769,7 +2749,7 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2790,7 +2770,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
+          <t>Altstadt, Düsseldorf</t>
         </is>
       </c>
       <c r="F50" t="n">
@@ -2815,33 +2795,31 @@
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr"/>
       <c r="B51" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>Abrio</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Altstadt, Düsseldorf</t>
-        </is>
-      </c>
-      <c r="F51" t="n">
-        <v>6</v>
-      </c>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr">
         <is>
@@ -2861,35 +2839,41 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr"/>
       <c r="B52" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Abrio</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
+          <t>Praktikum Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr"/>
+          <t>Frankfurt am Main, DE, 60329</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>5</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -2905,7 +2889,7 @@
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
         </is>
       </c>
     </row>
@@ -2916,30 +2900,28 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Praktikum Marketing (m/w/d)</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
-        </is>
-      </c>
-      <c r="F53" t="n">
-        <v>5</v>
-      </c>
+          <t>Köln, Nordrhein-Westfalen</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -2955,46 +2937,40 @@
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
+          <t>https://www.adzuna.de/land/ad/5822943276?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=580C236799B96DFD395A1EC1CBBF7474C7F58435</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr"/>
       <c r="B54" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Calypso Ventures GmbH</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Sales (m/w/d)</t>
+          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
-        </is>
-      </c>
-      <c r="F54" t="n">
-        <v>5</v>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>2026-11-01</t>
-        </is>
-      </c>
+          <t>Berlin, Deutschland</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -3005,39 +2981,35 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-&amp;-Sales-%28mwd%29-60329/1425985633/</t>
+          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr"/>
       <c r="B55" t="n">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3053,28 +3025,28 @@
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5822943276?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=580C236799B96DFD395A1EC1CBBF7474C7F58435</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr"/>
       <c r="B56" t="n">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Calypso Ventures GmbH</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F56" t="inlineStr"/>
@@ -3097,35 +3069,35 @@
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr"/>
       <c r="B57" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -3141,32 +3113,36 @@
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
+          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr"/>
       <c r="B58" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>Sayano Deutschland GmbH</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Mitte, Stuttgart</t>
         </is>
       </c>
       <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr"/>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H58" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3185,28 +3161,28 @@
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5816572451?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr"/>
       <c r="B59" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>Internship International Marketing Schwarzkopf Coloration - Legacy Brands</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Benrath, Düsseldorf</t>
         </is>
       </c>
       <c r="F59" t="inlineStr"/>
@@ -3229,36 +3205,32 @@
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5819890143?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr"/>
       <c r="B60" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Sayano Deutschland GmbH</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3277,7 +3249,7 @@
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816572451?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
         </is>
       </c>
     </row>
@@ -3288,29 +3260,29 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Internship International Marketing Schwarzkopf Coloration - Legacy Brands</t>
+          <t>Praktikum Marketing &amp; Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Benrath, Düsseldorf</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -3321,32 +3293,38 @@
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5819890143?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-&amp;-Sales-%28mwd%29-60329/1425985633/</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr"/>
       <c r="B62" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Lidl Stiftung &amp; Co. KG</t>
+          <t>LIGANOVA I Karriere</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Praktikum Buying (all genders) – August/September 2026</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
+          <t>Mitte, Stuttgart</t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v>6</v>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="H62" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3365,7 +3343,7 @@
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
+          <t>https://www.adzuna.de/details/5805407495?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3376,30 +3354,24 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>LIGANOVA I Karriere</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Praktikum Buying (all genders) – August/September 2026</t>
+          <t>Marketing &amp; Merchandising Assistant Trainee</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
-        </is>
-      </c>
-      <c r="F63" t="n">
-        <v>6</v>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+          <t>MILAN</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -3415,7 +3387,7 @@
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805407495?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
         </is>
       </c>
     </row>
@@ -3431,7 +3403,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Marketing &amp; Merchandising Assistant Trainee</t>
+          <t>Marketing and Merchandising Assistant Trainee</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -3459,7 +3431,7 @@
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing-and-Merchandising-Assistant-Trainee_JR128690</t>
         </is>
       </c>
     </row>
@@ -3470,29 +3442,29 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Wonder Natural GmbH</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Marketing and Merchandising Assistant Trainee</t>
+          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -3503,7 +3475,7 @@
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing-and-Merchandising-Assistant-Trainee_JR128690</t>
+          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5688,37 +5660,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Unternehmen</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Treffer</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Bester Score</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Beispielrolle</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Wird überwacht</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>System</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Zuerst gesehen</t>
         </is>
@@ -5756,7 +5728,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C3" t="n">
         <v>91</v>
@@ -5781,7 +5753,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C4" t="n">
         <v>89</v>
@@ -5806,7 +5778,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="C5" t="n">
         <v>84</v>
@@ -5831,7 +5803,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C6" t="n">
         <v>84</v>
@@ -5856,7 +5828,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C7" t="n">
         <v>84</v>
@@ -5889,7 +5861,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C8" t="n">
         <v>84</v>
@@ -5914,7 +5886,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C9" t="n">
         <v>84</v>
@@ -5939,7 +5911,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
@@ -5964,7 +5936,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C11" t="n">
         <v>84</v>
@@ -5989,7 +5961,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C12" t="n">
         <v>84</v>
@@ -6014,7 +5986,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C13" t="n">
         <v>84</v>
@@ -6039,7 +6011,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C14" t="n">
         <v>84</v>
@@ -6064,7 +6036,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C15" t="n">
         <v>84</v>
@@ -6089,7 +6061,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C16" t="n">
         <v>80</v>
@@ -6110,18 +6082,18 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>EAT HAPPY GROUP</t>
+          <t>Marc O'Polo</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="C17" t="n">
         <v>79</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Praktikum Brand Marketing (m/w/d) Marketing · Köln</t>
+          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
@@ -6135,18 +6107,18 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Yogi Tea</t>
+          <t>EAT HAPPY GROUP</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C18" t="n">
         <v>79</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Praktikum im Marketing - Brand &amp; Product / mindestens 5 Monate</t>
+          <t>Praktikum Brand Marketing (m/w/d) Marketing · Köln</t>
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
@@ -6160,30 +6132,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Ferrero</t>
+          <t>Yogi Tea</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="C19" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>successfactors</t>
-        </is>
-      </c>
+          <t>Praktikum im Marketing - Brand &amp; Product / mindestens 5 Monate</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -6193,22 +6157,30 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="C20" t="n">
         <v>78</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich Marketing für die Marke BE-KIND DACH</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>successfactors</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -6218,18 +6190,18 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Marc O'Polo</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="C21" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
+          <t>Praktikum im Bereich Marketing für die Marke BE-KIND DACH</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
@@ -6247,7 +6219,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C22" t="n">
         <v>74</v>
@@ -6272,7 +6244,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C23" t="n">
         <v>74</v>
@@ -6330,7 +6302,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C25" t="n">
         <v>73</v>
@@ -6355,7 +6327,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C26" t="n">
         <v>73</v>
@@ -6380,7 +6352,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C27" t="n">
         <v>72</v>
@@ -6405,7 +6377,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C28" t="n">
         <v>72</v>
@@ -6430,7 +6402,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C29" t="n">
         <v>69</v>
@@ -6455,7 +6427,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C30" t="n">
         <v>68</v>
@@ -6488,7 +6460,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C31" t="n">
         <v>68</v>
@@ -6513,7 +6485,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C32" t="n">
         <v>68</v>
@@ -6563,7 +6535,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C34" t="n">
         <v>66</v>
@@ -6588,7 +6560,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C35" t="n">
         <v>65</v>
@@ -6613,7 +6585,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C36" t="n">
         <v>64</v>
@@ -6638,7 +6610,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C37" t="n">
         <v>62</v>
@@ -6663,7 +6635,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C38" t="n">
         <v>62</v>
@@ -6696,7 +6668,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C39" t="n">
         <v>57</v>
@@ -6729,7 +6701,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C40" t="n">
         <v>56</v>
@@ -6754,7 +6726,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C41" t="n">
         <v>55</v>
@@ -6829,7 +6801,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C44" t="n">
         <v>53</v>
@@ -6854,7 +6826,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C45" t="n">
         <v>53</v>
@@ -6879,7 +6851,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C46" t="n">
         <v>53</v>
@@ -6929,7 +6901,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C48" t="n">
         <v>51</v>
@@ -6954,7 +6926,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C49" t="n">
         <v>49</v>
@@ -6979,7 +6951,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C50" t="n">
         <v>49</v>
@@ -7004,7 +6976,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C51" t="n">
         <v>49</v>
@@ -7029,7 +7001,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C52" t="n">
         <v>49</v>
@@ -7054,7 +7026,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C53" t="n">
         <v>49</v>
@@ -7079,7 +7051,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C54" t="n">
         <v>48</v>
@@ -7454,7 +7426,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C69" t="n">
         <v>46</v>
@@ -7479,7 +7451,7 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C70" t="n">
         <v>45</v>

</xml_diff>

<commit_message>
Lauf 2026-08-19 06:50 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firmen entdeckt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$114</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$96</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$86</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -34,7 +34,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -44,6 +44,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D8F3DC"/>
       </patternFill>
     </fill>
   </fills>
@@ -59,11 +64,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -430,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L114"/>
+  <dimension ref="A1:L96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1774,31 +1780,27 @@
     <row r="29">
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>coty</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Praktikum Digital Marketing &amp; Category Management</t>
+          <t>Marketing Intern - Trade Marketing</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Benrath, Düsseldorf</t>
+          <t>Darmstadt, Hessen</t>
         </is>
       </c>
       <c r="F29" t="n">
         <v>6</v>
       </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
+      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1817,7 +1819,7 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816415884?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1828,23 +1830,27 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich Marketing für die Marke BE-KIND DACH</t>
+          <t>Praktikum Digital Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Unterhaching, München (Kreis)</t>
+          <t>Benrath, Düsseldorf</t>
         </is>
       </c>
       <c r="F30" t="n">
         <v>6</v>
       </c>
-      <c r="G30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
       <c r="H30" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1863,7 +1869,7 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5752932983?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5816415884?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1874,17 +1880,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>P&amp;G</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum im Bereich Marketing für die Marke BE-KIND DACH</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Unterhaching, München (Kreis)</t>
         </is>
       </c>
       <c r="F31" t="n">
@@ -1909,7 +1915,7 @@
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5752932983?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1920,17 +1926,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>P&amp;G</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Praktikum Category Management Non Food Vertrieb (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F32" t="n">
@@ -1955,7 +1961,7 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5795118484?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1971,7 +1977,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Praktikum CNX Category Management Home &amp; Living (m/w/d)</t>
+          <t>Praktikum Category Management Non Food Vertrieb (m/w/d)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2001,7 +2007,7 @@
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5765078175?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5795118484?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2017,7 +2023,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing Tchibo (m/w/d)</t>
+          <t>Praktikum CNX Category Management Home &amp; Living (m/w/d)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2047,7 +2053,7 @@
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5744245447?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5765078175?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2063,7 +2069,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing Eduscho (m/w/d)</t>
+          <t>Praktikum Trade Marketing Tchibo (m/w/d)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2093,32 +2099,32 @@
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5773205889?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5744245447?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>Tchibo GmbH</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Trade Marketing Eduscho (m/w/d)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
@@ -2139,7 +2145,7 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5773205889?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2150,21 +2156,21 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>markenbaumarkt24</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
+          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Feuersbach, Siegen</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
@@ -2185,31 +2191,33 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>PARSA Haar- und Modeartikel GmbH</t>
+          <t>markenbaumarkt24</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
+          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr"/>
+          <t>Feuersbach, Siegen</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>2</v>
+      </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
@@ -2218,7 +2226,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -2229,23 +2237,23 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
+          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr"/>
       <c r="B39" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Lidl Stiftung</t>
+          <t>PARSA Haar- und Modeartikel GmbH</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food in Neckarsulm</t>
+          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2253,9 +2261,7 @@
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="F39" t="n">
-        <v>6</v>
-      </c>
+      <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
@@ -2264,7 +2270,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -2275,7 +2281,7 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813494719?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
         </is>
       </c>
     </row>
@@ -2286,20 +2292,22 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Lidl Stiftung</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food in Neckarsulm</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr"/>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>6</v>
+      </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
@@ -2319,33 +2327,31 @@
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
+          <t>https://www.adzuna.de/details/5813494719?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr"/>
       <c r="B41" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F41" t="n">
-        <v>6</v>
-      </c>
+          <t>Hamburg, Deutschland</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
@@ -2365,7 +2371,7 @@
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
         </is>
       </c>
     </row>
@@ -2381,7 +2387,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
+          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2411,7 +2417,7 @@
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2427,7 +2433,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
+          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2438,11 +2444,7 @@
       <c r="F43" t="n">
         <v>6</v>
       </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2461,7 +2463,7 @@
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2472,17 +2474,17 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Bosch Thermotechnik GmbH</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Praktikum im internationalen Brand Management</t>
+          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Wernau (Neckar), Esslingen (Kreis)</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F44" t="n">
@@ -2490,7 +2492,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -2511,7 +2513,7 @@
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5799981240?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2522,23 +2524,27 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Bosch Thermotechnik GmbH</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Intern Category Growth</t>
+          <t>Praktikum im internationalen Brand Management</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Darmstadt, Hessen</t>
+          <t>Wernau (Neckar), Esslingen (Kreis)</t>
         </is>
       </c>
       <c r="F45" t="n">
         <v>6</v>
       </c>
-      <c r="G45" t="inlineStr"/>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="H45" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2557,7 +2563,7 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5754086625?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5799981240?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2568,27 +2574,23 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>L’ORÉAL</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>PRAKTIKUM (M/W/D) Product Marketing - Start ab August/September/Oktober für 6 Monate</t>
+          <t>Intern Category Growth</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Nordrhein-Westfalen, Deutschland</t>
+          <t>Darmstadt, Hessen</t>
         </is>
       </c>
       <c r="F46" t="n">
         <v>6</v>
       </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2607,7 +2609,7 @@
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5754061318?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5754086625?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2618,17 +2620,17 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>L’ORÉAL</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>PRAKTIKUM (M/W/D) Product Marketing - Start ab August/September/Oktober für 6 Monate</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Nordrhein-Westfalen, Deutschland</t>
         </is>
       </c>
       <c r="F47" t="n">
@@ -2657,7 +2659,7 @@
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5754061318?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2668,23 +2670,27 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>coty</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Darmstadt, Hessen</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F48" t="n">
         <v>6</v>
       </c>
-      <c r="G48" t="inlineStr"/>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H48" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2703,7 +2709,7 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2844,52 +2850,50 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr"/>
-      <c r="B52" t="n">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="n">
         <v>64</v>
       </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Nestle Deutschland</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>Praktikum Marketing (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>Frankfurt am Main, DE, 60329</t>
-        </is>
-      </c>
-      <c r="F52" t="n">
-        <v>5</v>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>2026-11-01</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Mars</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Internship in Trade Marketing</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>DEU-Nordrhein-Westfalen-Köln</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr"/>
+      <c r="G52" s="2" t="inlineStr"/>
+      <c r="H52" s="2" t="inlineStr">
         <is>
           <t>fmcg</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr"/>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
         </is>
       </c>
     </row>
@@ -2900,28 +2904,30 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>Praktikum Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr"/>
+          <t>Frankfurt am Main, DE, 60329</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>5</v>
+      </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -2937,40 +2943,46 @@
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5822943276?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=580C236799B96DFD395A1EC1CBBF7474C7F58435</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr"/>
       <c r="B54" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Calypso Ventures GmbH</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
+          <t>Praktikum Marketing &amp; Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
+          <t>Frankfurt am Main, DE, 60329</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>5</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -2981,35 +2993,39 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-&amp;-Sales-%28mwd%29-60329/1425985633/</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr"/>
       <c r="B55" t="n">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3025,28 +3041,28 @@
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
+          <t>https://www.adzuna.de/land/ad/5822943276?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=580C236799B96DFD395A1EC1CBBF7474C7F58435</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr"/>
       <c r="B56" t="n">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>Calypso Ventures GmbH</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F56" t="inlineStr"/>
@@ -3069,83 +3085,83 @@
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr"/>
-      <c r="B57" t="n">
-        <v>56</v>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>Upsters Energy GmbH</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>Altstadt, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Exclusive Associates</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>Düsseltal, Düsseldorf</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr"/>
+      <c r="G57" s="2" t="inlineStr"/>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K57" s="2" t="inlineStr"/>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr"/>
       <c r="B58" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Sayano Deutschland GmbH</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
+          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -3161,28 +3177,28 @@
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816572451?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr"/>
       <c r="B59" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Internship International Marketing Schwarzkopf Coloration - Legacy Brands</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Benrath, Düsseldorf</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F59" t="inlineStr"/>
@@ -3205,28 +3221,28 @@
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5819890143?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr"/>
       <c r="B60" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Lidl Stiftung &amp; Co. KG</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F60" t="inlineStr"/>
@@ -3249,40 +3265,44 @@
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
+          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr"/>
       <c r="B61" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Sayano Deutschland GmbH</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Sales (m/w/d)</t>
+          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Mitte, Stuttgart</t>
         </is>
       </c>
       <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr"/>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -3293,38 +3313,34 @@
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-&amp;-Sales-%28mwd%29-60329/1425985633/</t>
+          <t>https://www.adzuna.de/details/5816572451?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr"/>
       <c r="B62" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>LIGANOVA I Karriere</t>
+          <t>THE VERSE Ventures</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Praktikum Buying (all genders) – August/September 2026</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F62" t="n">
         <v>6</v>
       </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+      <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3343,35 +3359,35 @@
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805407495?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr"/>
       <c r="B63" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Marketing &amp; Merchandising Assistant Trainee</t>
+          <t>Internship International Marketing Schwarzkopf Coloration - Legacy Brands</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Benrath, Düsseldorf</t>
         </is>
       </c>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -3387,35 +3403,35 @@
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
+          <t>https://www.adzuna.de/details/5819890143?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr"/>
       <c r="B64" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Marketing and Merchandising Assistant Trainee</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -3431,7 +3447,7 @@
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing-and-Merchandising-Assistant-Trainee_JR128690</t>
+          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
         </is>
       </c>
     </row>
@@ -3442,21 +3458,27 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Wonder Natural GmbH</t>
+          <t>LIGANOVA I Karriere</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
+          <t>Praktikum Buying (all genders) – August/September 2026</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr"/>
-      <c r="G65" t="inlineStr"/>
+          <t>Mitte, Stuttgart</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>6</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="H65" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3464,7 +3486,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -3475,35 +3497,35 @@
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805407495?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr"/>
       <c r="B66" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Digitalagenten</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
+          <t>Marketing &amp; Merchandising Assistant Trainee</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Charlottenburg, Berlin</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -3519,35 +3541,35 @@
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804948828?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr"/>
       <c r="B67" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>LIMITD by Wunderproducts GmbH</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Marketing and Merchandising Assistant Trainee</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Kreuzberg, Berlin</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -3563,36 +3585,32 @@
       <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing-and-Merchandising-Assistant-Trainee_JR128690</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr"/>
       <c r="B68" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers GmbH WPG</t>
+          <t>Wonder Natural GmbH</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
+          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F68" t="inlineStr"/>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
+      <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3600,7 +3618,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -3611,7 +3629,7 @@
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3622,25 +3640,21 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>SERVICEPLAN Gruppe</t>
+          <t>Digitalagenten</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Sales (Marketing / New Business) (all genders)</t>
+          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Charlottenburg, Berlin</t>
         </is>
       </c>
       <c r="F69" t="inlineStr"/>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3648,7 +3662,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -3659,7 +3673,7 @@
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804948828?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3670,7 +3684,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>THE VERSE Ventures</t>
+          <t>LIMITD by Wunderproducts GmbH</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -3680,7 +3694,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Kreuzberg, Berlin</t>
         </is>
       </c>
       <c r="F70" t="inlineStr"/>
@@ -3703,7 +3717,7 @@
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3714,21 +3728,25 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>WirWinzer</t>
+          <t>PricewaterhouseCoopers GmbH WPG</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Praktikum Business Development Weinhandel (all genders)</t>
+          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
-      <c r="G71" t="inlineStr"/>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
       <c r="H71" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3747,32 +3765,36 @@
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr"/>
       <c r="B72" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Brand Trust</t>
+          <t>SERVICEPLAN Gruppe</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Sales (Marketing / New Business) (all genders)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Gleißbühl, Nürnberg</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F72" t="inlineStr"/>
-      <c r="G72" t="inlineStr"/>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H72" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3780,7 +3802,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -3791,26 +3813,30 @@
       <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5669847401?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr"/>
       <c r="B73" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>WirWinzer</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr"/>
+          <t>Praktikum Business Development Weinhandel (all genders)</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Altstadt-Lehel, München</t>
+        </is>
+      </c>
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr">
@@ -3831,47 +3857,55 @@
       <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
+          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr"/>
-      <c r="B74" t="n">
-        <v>49</v>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>Coty</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>Operational Trade Marketing Intern</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr"/>
-      <c r="F74" t="inlineStr"/>
-      <c r="G74" t="inlineStr"/>
-      <c r="H74" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J74" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K74" t="inlineStr"/>
-      <c r="L74" t="inlineStr">
-        <is>
-          <t>https://careers.coty.com/job/Toronto-Operational-Trade-Marketing-Intern-ON-M5H4H2/1397938633/</t>
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Richemont</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Internship - High Jewelry Business Development Assistant</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr"/>
+      <c r="G74" s="2" t="inlineStr"/>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>fashion</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K74" s="2" t="inlineStr"/>
+      <c r="L74" s="2" t="inlineStr">
+        <is>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
         </is>
       </c>
     </row>
@@ -3882,17 +3916,17 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>Brand Trust</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
+          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Benrath, Düsseldorf</t>
+          <t>Gleißbühl, Nürnberg</t>
         </is>
       </c>
       <c r="F75" t="inlineStr"/>
@@ -3904,7 +3938,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
@@ -3915,7 +3949,7 @@
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5669847401?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3926,19 +3960,15 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>Schwabing-Freimann, München</t>
-        </is>
-      </c>
+          <t>Marketing Intern - Trade Marketing</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
@@ -3959,7 +3989,7 @@
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
         </is>
       </c>
     </row>
@@ -3970,24 +4000,20 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>DEU-Bayern-Unterhaching</t>
-        </is>
-      </c>
+          <t>Operational Trade Marketing Intern</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -4003,7 +4029,7 @@
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
+          <t>https://careers.coty.com/job/Toronto-Operational-Trade-Marketing-Intern-ON-M5H4H2/1397938633/</t>
         </is>
       </c>
     </row>
@@ -4014,17 +4040,17 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>Benrath, Düsseldorf</t>
         </is>
       </c>
       <c r="F78" t="inlineStr"/>
@@ -4036,7 +4062,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -4047,7 +4073,7 @@
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4058,17 +4084,17 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Schwabing-Freimann, München</t>
         </is>
       </c>
       <c r="F79" t="inlineStr"/>
@@ -4091,7 +4117,7 @@
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
+          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4102,24 +4128,24 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>DEU-Bayern-Unterhaching</t>
         </is>
       </c>
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -4135,7 +4161,7 @@
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
         </is>
       </c>
     </row>
@@ -4146,17 +4172,17 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F81" t="inlineStr"/>
@@ -4179,7 +4205,7 @@
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
+          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4190,17 +4216,17 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F82" t="inlineStr"/>
@@ -4223,28 +4249,28 @@
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr"/>
       <c r="B83" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>AUTO1 Global Services SE &amp; Co. KG</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (d/m/w)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F83" t="inlineStr"/>
@@ -4267,28 +4293,28 @@
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5789927805?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr"/>
       <c r="B84" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Amolina</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
@@ -4311,28 +4337,28 @@
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727292709?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr"/>
       <c r="B85" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>CTG Consulting</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Praktikum Sales/Business Development // Hamburg oder Berlin</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
@@ -4355,7 +4381,7 @@
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5694221323?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4366,17 +4392,17 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Dronesperhour</t>
+          <t>REWE Group</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development eines Startups (m/w/d)</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Mitte, Berlin</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F86" t="inlineStr"/>
@@ -4399,28 +4425,28 @@
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5669955732?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5712965755?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr"/>
       <c r="B87" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>GrantLift GmbH</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F87" t="inlineStr"/>
@@ -4443,28 +4469,28 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5803032426?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr"/>
       <c r="B88" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>GrantLift GmbH</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Altstadt-Nord, Köln</t>
         </is>
       </c>
       <c r="F88" t="inlineStr"/>
@@ -4487,28 +4513,28 @@
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804575149?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr"/>
       <c r="B89" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Otto Group one.O GmbH</t>
+          <t>Devoteam G Cloud Germany</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Praktikum im Knowledge Management - Corporate Strategy (w/m/d)</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F89" t="inlineStr"/>
@@ -4531,28 +4557,28 @@
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5809516963?se=mrUvpGeQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=7970F7260CB99374DD6661F2025E46043B457CE4</t>
+          <t>https://www.adzuna.de/details/5811135653?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr"/>
       <c r="B90" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Pflegia</t>
+          <t>freudio</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Wien, Österreich</t>
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
@@ -4564,7 +4590,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -4575,28 +4601,28 @@
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5821302522?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/details/5836667156?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr"/>
       <c r="B91" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Pflegia</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F91" t="inlineStr"/>
@@ -4619,28 +4645,28 @@
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802953545?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr"/>
       <c r="B92" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Pflegia</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (Projektmanagement &amp; Prozessoptimierung) (m/w/d)</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F92" t="inlineStr"/>
@@ -4663,28 +4689,28 @@
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802984051?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr"/>
       <c r="B93" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Pflegia</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (Business Analyst/Automation Engineer/Applied AI Engineer) (m/w/d)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F93" t="inlineStr"/>
@@ -4707,28 +4733,28 @@
       <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802977130?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr"/>
       <c r="B94" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>REWE Group</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F94" t="inlineStr"/>
@@ -4751,28 +4777,28 @@
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5712965755?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr"/>
       <c r="B95" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>SHAVENT - ARA Sustainable Products</t>
+          <t>sailwithus</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Praktikum Business Development in nachhaltigem Start-Up (w/m/d) Remote in DE</t>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Sendling, München</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F95" t="inlineStr"/>
@@ -4795,28 +4821,28 @@
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802951937?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr"/>
       <c r="B96" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>SINN Power</t>
+          <t>sailwithus</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Praktikum im AI Business Development (m/w/d)</t>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Kasten, München (Kreis)</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F96" t="inlineStr"/>
@@ -4839,804 +4865,12 @@
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727348338?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr"/>
-      <c r="B97" t="n">
-        <v>48</v>
-      </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>Tchibo GmbH</t>
-        </is>
-      </c>
-      <c r="D97" t="inlineStr">
-        <is>
-          <t>Praktikum Strategy &amp; Business Development (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E97" t="inlineStr">
-        <is>
-          <t>Hamburg, Deutschland</t>
-        </is>
-      </c>
-      <c r="F97" t="inlineStr"/>
-      <c r="G97" t="inlineStr"/>
-      <c r="H97" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I97" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J97" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K97" t="inlineStr"/>
-      <c r="L97" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5799516357?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr"/>
-      <c r="B98" t="n">
-        <v>48</v>
-      </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>Vitolus</t>
-        </is>
-      </c>
-      <c r="D98" t="inlineStr">
-        <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>Altstadt-Lehel, München</t>
-        </is>
-      </c>
-      <c r="F98" t="inlineStr"/>
-      <c r="G98" t="inlineStr"/>
-      <c r="H98" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I98" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J98" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K98" t="inlineStr"/>
-      <c r="L98" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5785872138?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr"/>
-      <c r="B99" t="n">
-        <v>48</v>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>Vivanta Gmbh</t>
-        </is>
-      </c>
-      <c r="D99" t="inlineStr">
-        <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>Berlin, Deutschland</t>
-        </is>
-      </c>
-      <c r="F99" t="inlineStr"/>
-      <c r="G99" t="inlineStr"/>
-      <c r="H99" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I99" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J99" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K99" t="inlineStr"/>
-      <c r="L99" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5802952325?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr"/>
-      <c r="B100" t="n">
-        <v>48</v>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>Vivanta Gmbh</t>
-        </is>
-      </c>
-      <c r="D100" t="inlineStr">
-        <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>Wedding, Berlin</t>
-        </is>
-      </c>
-      <c r="F100" t="inlineStr"/>
-      <c r="G100" t="inlineStr"/>
-      <c r="H100" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I100" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J100" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K100" t="inlineStr"/>
-      <c r="L100" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5804549349?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr"/>
-      <c r="B101" t="n">
-        <v>48</v>
-      </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>Werkia</t>
-        </is>
-      </c>
-      <c r="D101" t="inlineStr">
-        <is>
-          <t>Praktikum Business Development (m/w/d) - Datenanalyse &amp; Automatisierung</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>Wedding, Berlin</t>
-        </is>
-      </c>
-      <c r="F101" t="inlineStr"/>
-      <c r="G101" t="inlineStr"/>
-      <c r="H101" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I101" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J101" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K101" t="inlineStr"/>
-      <c r="L101" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5802974922?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr"/>
-      <c r="B102" t="n">
-        <v>48</v>
-      </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>Werkia</t>
-        </is>
-      </c>
-      <c r="D102" t="inlineStr">
-        <is>
-          <t>Praktikum im Business Development (m/w/d) - Berlin</t>
-        </is>
-      </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>Wedding, Berlin</t>
-        </is>
-      </c>
-      <c r="F102" t="inlineStr"/>
-      <c r="G102" t="inlineStr"/>
-      <c r="H102" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I102" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J102" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K102" t="inlineStr"/>
-      <c r="L102" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5802950225?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr"/>
-      <c r="B103" t="n">
-        <v>48</v>
-      </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>innpuls</t>
-        </is>
-      </c>
-      <c r="D103" t="inlineStr">
-        <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E103" t="inlineStr">
-        <is>
-          <t>Altstadt-Lehel, München</t>
-        </is>
-      </c>
-      <c r="F103" t="inlineStr"/>
-      <c r="G103" t="inlineStr"/>
-      <c r="H103" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I103" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J103" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K103" t="inlineStr"/>
-      <c r="L103" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5735591887?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="inlineStr"/>
-      <c r="B104" t="n">
-        <v>48</v>
-      </c>
-      <c r="C104" t="inlineStr">
-        <is>
-          <t>paero</t>
-        </is>
-      </c>
-      <c r="D104" t="inlineStr">
-        <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E104" t="inlineStr">
-        <is>
-          <t>Ludwigsvorstadt-Isarvorstadt, München</t>
-        </is>
-      </c>
-      <c r="F104" t="inlineStr"/>
-      <c r="G104" t="inlineStr"/>
-      <c r="H104" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I104" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J104" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K104" t="inlineStr"/>
-      <c r="L104" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5813846665?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="inlineStr"/>
-      <c r="B105" t="n">
-        <v>46</v>
-      </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>SUPA - Sport Und Party App</t>
-        </is>
-      </c>
-      <c r="D105" t="inlineStr">
-        <is>
-          <t>Business Development Praktikum</t>
-        </is>
-      </c>
-      <c r="E105" t="inlineStr">
-        <is>
-          <t>Köln, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F105" t="inlineStr"/>
-      <c r="G105" t="inlineStr"/>
-      <c r="H105" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I105" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J105" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K105" t="inlineStr"/>
-      <c r="L105" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="inlineStr"/>
-      <c r="B106" t="n">
-        <v>46</v>
-      </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>SUPA - Sport Und Party App</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr">
-        <is>
-          <t>Business Development Praktikum</t>
-        </is>
-      </c>
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>Altstadt-Nord, Köln</t>
-        </is>
-      </c>
-      <c r="F106" t="inlineStr"/>
-      <c r="G106" t="inlineStr"/>
-      <c r="H106" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I106" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J106" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K106" t="inlineStr"/>
-      <c r="L106" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="inlineStr"/>
-      <c r="B107" t="n">
-        <v>45</v>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>Devoteam G Cloud Germany</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr">
-        <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F107" t="inlineStr"/>
-      <c r="G107" t="inlineStr"/>
-      <c r="H107" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I107" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J107" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K107" t="inlineStr"/>
-      <c r="L107" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5811135653?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="inlineStr"/>
-      <c r="B108" t="n">
-        <v>45</v>
-      </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>freudio</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr">
-        <is>
-          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
-        </is>
-      </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t>Wien, Österreich</t>
-        </is>
-      </c>
-      <c r="F108" t="inlineStr"/>
-      <c r="G108" t="inlineStr"/>
-      <c r="H108" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I108" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="J108" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K108" t="inlineStr"/>
-      <c r="L108" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.at/details/5836667156?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="inlineStr"/>
-      <c r="B109" t="n">
-        <v>45</v>
-      </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>prepmymeal GmbH</t>
-        </is>
-      </c>
-      <c r="D109" t="inlineStr">
-        <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E109" t="inlineStr">
-        <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F109" t="inlineStr"/>
-      <c r="G109" t="inlineStr"/>
-      <c r="H109" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I109" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J109" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K109" t="inlineStr"/>
-      <c r="L109" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="inlineStr"/>
-      <c r="B110" t="n">
-        <v>45</v>
-      </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>prepmymeal GmbH</t>
-        </is>
-      </c>
-      <c r="D110" t="inlineStr">
-        <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E110" t="inlineStr">
-        <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F110" t="inlineStr"/>
-      <c r="G110" t="inlineStr"/>
-      <c r="H110" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I110" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J110" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K110" t="inlineStr"/>
-      <c r="L110" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="inlineStr"/>
-      <c r="B111" t="n">
-        <v>45</v>
-      </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>prepmymeal GmbH</t>
-        </is>
-      </c>
-      <c r="D111" t="inlineStr">
-        <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E111" t="inlineStr">
-        <is>
-          <t>Altstadt, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F111" t="inlineStr"/>
-      <c r="G111" t="inlineStr"/>
-      <c r="H111" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I111" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J111" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K111" t="inlineStr"/>
-      <c r="L111" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="inlineStr"/>
-      <c r="B112" t="n">
-        <v>45</v>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>prepmymeal GmbH</t>
-        </is>
-      </c>
-      <c r="D112" t="inlineStr">
-        <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E112" t="inlineStr">
-        <is>
-          <t>Altstadt, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F112" t="inlineStr"/>
-      <c r="G112" t="inlineStr"/>
-      <c r="H112" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I112" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J112" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K112" t="inlineStr"/>
-      <c r="L112" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="inlineStr"/>
-      <c r="B113" t="n">
-        <v>45</v>
-      </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>sailwithus</t>
-        </is>
-      </c>
-      <c r="D113" t="inlineStr">
-        <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
-        </is>
-      </c>
-      <c r="E113" t="inlineStr">
-        <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F113" t="inlineStr"/>
-      <c r="G113" t="inlineStr"/>
-      <c r="H113" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I113" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J113" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K113" t="inlineStr"/>
-      <c r="L113" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="inlineStr"/>
-      <c r="B114" t="n">
-        <v>45</v>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>sailwithus</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
-        </is>
-      </c>
-      <c r="E114" t="inlineStr">
-        <is>
-          <t>Altstadt, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F114" t="inlineStr"/>
-      <c r="G114" t="inlineStr"/>
-      <c r="H114" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I114" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J114" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K114" t="inlineStr"/>
-      <c r="L114" t="inlineStr">
-        <is>
           <t>https://www.adzuna.de/details/5804544237?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L114"/>
+  <autoFilter ref="A1:L96"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5660,37 +4894,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Unternehmen</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Treffer</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Bester Score</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Beispielrolle</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Wird überwacht</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>System</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Zuerst gesehen</t>
         </is>
@@ -5728,7 +4962,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C3" t="n">
         <v>91</v>
@@ -5778,7 +5012,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="C5" t="n">
         <v>84</v>
@@ -5803,7 +5037,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C6" t="n">
         <v>84</v>
@@ -5828,7 +5062,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C7" t="n">
         <v>84</v>
@@ -5861,7 +5095,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C8" t="n">
         <v>84</v>
@@ -5886,7 +5120,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C9" t="n">
         <v>84</v>
@@ -5911,7 +5145,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
@@ -5936,7 +5170,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C11" t="n">
         <v>84</v>
@@ -5961,7 +5195,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C12" t="n">
         <v>84</v>
@@ -5986,7 +5220,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C13" t="n">
         <v>84</v>
@@ -6007,32 +5241,32 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Wonder Natural GmbH</t>
+          <t>PARSA Haar- und Modeartikel GmbH</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C14" t="n">
         <v>84</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
+          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-08</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PARSA Haar- und Modeartikel GmbH</t>
+          <t>Wonder Natural GmbH</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -6043,14 +5277,14 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
@@ -6061,7 +5295,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C16" t="n">
         <v>80</v>
@@ -6161,7 +5395,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C20" t="n">
         <v>78</v>
@@ -6194,7 +5428,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C21" t="n">
         <v>78</v>
@@ -6215,22 +5449,30 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Miles &amp; More GmbH</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>14</v>
+        <v>49</v>
       </c>
       <c r="C22" t="n">
         <v>74</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Internship Marketing Strategy &amp; Delivery</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
+          <t>Marketing Intern - Trade Marketing</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>successfactors</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -6240,80 +5482,80 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>Miles &amp; More GmbH</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="C23" t="n">
         <v>74</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Internship Marketing Strategy &amp; Delivery</t>
         </is>
       </c>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="C24" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Praktikum Category Management Non Food Vertrieb (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>successfactors</t>
-        </is>
-      </c>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>P&amp;G</t>
+          <t>Tchibo GmbH</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="C25" t="n">
         <v>73</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
+          <t>Praktikum Category Management Non Food Vertrieb (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>successfactors</t>
+        </is>
+      </c>
       <c r="G25" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -6327,7 +5569,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C26" t="n">
         <v>73</v>
@@ -6348,18 +5590,18 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>markenbaumarkt24</t>
+          <t>P&amp;G</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C27" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr"/>
@@ -6377,7 +5619,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C28" t="n">
         <v>72</v>
@@ -6398,18 +5640,18 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Lidl Stiftung</t>
+          <t>markenbaumarkt24</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C29" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food in Neckarsulm</t>
+          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
@@ -6423,30 +5665,22 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Lidl Stiftung</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="C30" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Intern Category Growth</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>successfactors</t>
-        </is>
-      </c>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food in Neckarsulm</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -6485,7 +5719,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C32" t="n">
         <v>68</v>
@@ -6535,7 +5769,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C34" t="n">
         <v>66</v>
@@ -6560,7 +5794,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C35" t="n">
         <v>65</v>
@@ -6585,7 +5819,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C36" t="n">
         <v>64</v>
@@ -6610,7 +5844,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C37" t="n">
         <v>62</v>
@@ -6635,7 +5869,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C38" t="n">
         <v>62</v>
@@ -6668,7 +5902,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C39" t="n">
         <v>57</v>
@@ -6701,7 +5935,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C40" t="n">
         <v>56</v>
@@ -6726,7 +5960,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C41" t="n">
         <v>55</v>
@@ -6801,7 +6035,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C44" t="n">
         <v>53</v>
@@ -6826,7 +6060,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C45" t="n">
         <v>53</v>
@@ -6851,7 +6085,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C46" t="n">
         <v>53</v>
@@ -6901,7 +6135,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C48" t="n">
         <v>51</v>
@@ -6926,7 +6160,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C49" t="n">
         <v>49</v>
@@ -6951,7 +6185,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C50" t="n">
         <v>49</v>
@@ -6976,7 +6210,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C51" t="n">
         <v>49</v>
@@ -7001,7 +6235,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C52" t="n">
         <v>49</v>
@@ -7026,7 +6260,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C53" t="n">
         <v>49</v>
@@ -7051,7 +6285,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C54" t="n">
         <v>48</v>
@@ -7426,7 +6660,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C69" t="n">
         <v>46</v>
@@ -7451,7 +6685,7 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C70" t="n">
         <v>45</v>

</xml_diff>

<commit_message>
Lauf 2026-08-20 06:53 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firmen entdeckt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$96</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$100</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$86</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L96"/>
+  <dimension ref="A1:L100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -992,48 +992,56 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" t="n">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
         <v>84</v>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Hamburg-Altstadt, Hamburg</t>
-        </is>
-      </c>
-      <c r="F12" t="n">
-        <v>6</v>
-      </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5829732882?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Nestle Deutschland</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main, DE, 60329</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>fmcg</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Category-Management%2C-Brand-Activation-und-Sales-%28mwd%29-60329/1427883433/</t>
         </is>
       </c>
     </row>
@@ -1044,17 +1052,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Picnic</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Category Management Praktikum (m/w/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Hamburg-Altstadt, Hamburg</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -1068,7 +1076,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1079,7 +1087,7 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5829732882?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1108,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F14" t="n">
@@ -1125,36 +1133,34 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759088383?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="n">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
+          <t>Picnic</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management National</t>
+          <t>Category Management Praktikum (m/w/d)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Au-Haidhausen, München</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>6</v>
+      </c>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1173,33 +1179,39 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805399065?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759088383?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>EAT HAPPY GROUP</t>
+          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Praktikum Brand Marketing (m/w/d) Marketing · Köln</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="n">
-        <v>6</v>
-      </c>
-      <c r="G16" t="inlineStr"/>
+          <t>Praktikum Brand Management National</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Au-Haidhausen, München</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1215,7 +1227,7 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://eathappygroup.teamtailor.com/jobs/7902845-praktikum-brand-marketing-m-w-d</t>
+          <t>https://www.adzuna.de/details/5805399065?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1226,30 +1238,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Marc O'Polo</t>
+          <t>EAT HAPPY GROUP</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
+          <t>Praktikum Brand Marketing (m/w/d) Marketing · Köln</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
       <c r="F17" t="n">
         <v>6</v>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1265,7 +1269,7 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://eathappygroup.teamtailor.com/jobs/7902845-praktikum-brand-marketing-m-w-d</t>
         </is>
       </c>
     </row>
@@ -1276,23 +1280,27 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Yogi Tea</t>
+          <t>Marc O'Polo</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Praktikum im Marketing - Brand &amp; Product / mindestens 5 Monate</t>
+          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>5</v>
-      </c>
-      <c r="G18" t="inlineStr"/>
+        <v>6</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1311,7 +1319,7 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5744980745?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2376,48 +2384,50 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr"/>
-      <c r="B42" t="n">
-        <v>68</v>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Barilla</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Köln, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F42" t="n">
-        <v>6</v>
-      </c>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Otto GmbH &amp; Co. KGaA</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr"/>
+      <c r="G42" s="2" t="inlineStr"/>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr"/>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/land/ad/5849209692?se=qJaID2Kc8RGlrvMe-VN8Yg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B8E6A551D4E75B7916A5994DC13A8DA3451895D</t>
         </is>
       </c>
     </row>
@@ -2433,7 +2443,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
+          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2463,7 +2473,7 @@
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2479,7 +2489,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
+          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2490,11 +2500,7 @@
       <c r="F44" t="n">
         <v>6</v>
       </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2513,7 +2519,7 @@
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2524,17 +2530,17 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Bosch Thermotechnik GmbH</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Praktikum im internationalen Brand Management</t>
+          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Wernau (Neckar), Esslingen (Kreis)</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F45" t="n">
@@ -2542,7 +2548,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2563,7 +2569,7 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5799981240?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2574,23 +2580,27 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Bosch Thermotechnik GmbH</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Intern Category Growth</t>
+          <t>Praktikum im internationalen Brand Management</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Darmstadt, Hessen</t>
+          <t>Wernau (Neckar), Esslingen (Kreis)</t>
         </is>
       </c>
       <c r="F46" t="n">
         <v>6</v>
       </c>
-      <c r="G46" t="inlineStr"/>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="H46" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2609,7 +2619,7 @@
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5754086625?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5799981240?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2620,27 +2630,23 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>L’ORÉAL</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>PRAKTIKUM (M/W/D) Product Marketing - Start ab August/September/Oktober für 6 Monate</t>
+          <t>Intern Category Growth</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Nordrhein-Westfalen, Deutschland</t>
+          <t>Darmstadt, Hessen</t>
         </is>
       </c>
       <c r="F47" t="n">
         <v>6</v>
       </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2659,7 +2665,7 @@
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5754061318?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5754086625?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2670,17 +2676,17 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>L’ORÉAL</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>PRAKTIKUM (M/W/D) Product Marketing - Start ab August/September/Oktober für 6 Monate</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Nordrhein-Westfalen, Deutschland</t>
         </is>
       </c>
       <c r="F48" t="n">
@@ -2709,34 +2715,38 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5754061318?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr"/>
       <c r="B49" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F49" t="n">
         <v>6</v>
       </c>
-      <c r="G49" t="inlineStr"/>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H49" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2755,7 +2765,7 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2776,7 +2786,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Altstadt, Düsseldorf</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F50" t="n">
@@ -2801,31 +2811,33 @@
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr"/>
       <c r="B51" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Abrio</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr"/>
+          <t>Altstadt, Düsseldorf</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>6</v>
+      </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr">
         <is>
@@ -2845,7 +2857,7 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2904,30 +2916,28 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Praktikum Marketing (m/w/d)</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
-        </is>
-      </c>
-      <c r="F53" t="n">
-        <v>5</v>
-      </c>
+          <t>Köln, Nordrhein-Westfalen</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -2943,46 +2953,40 @@
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
+          <t>https://www.adzuna.de/land/ad/5822943276?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=580C236799B96DFD395A1EC1CBBF7474C7F58435</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr"/>
       <c r="B54" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Calypso Ventures GmbH</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Sales (m/w/d)</t>
+          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
-        </is>
-      </c>
-      <c r="F54" t="n">
-        <v>5</v>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>2026-11-01</t>
-        </is>
-      </c>
+          <t>Berlin, Deutschland</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -2993,99 +2997,103 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-&amp;-Sales-%28mwd%29-60329/1425985633/</t>
+          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr"/>
-      <c r="B55" t="n">
-        <v>64</v>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>PENNY International</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>Köln, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5822943276?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=580C236799B96DFD395A1EC1CBBF7474C7F58435</t>
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Exclusive Associates</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Düsseltal, Düsseldorf</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr"/>
+      <c r="G55" s="2" t="inlineStr"/>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K55" s="2" t="inlineStr"/>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr"/>
-      <c r="B56" t="n">
-        <v>62</v>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>Calypso Ventures GmbH</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Berlin, Deutschland</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr"/>
+      <c r="G56" s="2" t="inlineStr"/>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr"/>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/land/ad/5848400955?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=4E59A334AC360616EAEAAC474F72A07451A7C624</t>
         </is>
       </c>
     </row>
@@ -3096,21 +3104,21 @@
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr"/>
@@ -3122,7 +3130,7 @@
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr">
@@ -3133,79 +3141,83 @@
       <c r="K57" s="2" t="inlineStr"/>
       <c r="L57" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5848409009?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5C62DDCDA5E03F77D6089CD03CFA1D966DF15C96</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr"/>
-      <c r="B58" t="n">
-        <v>57</v>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>Richemont</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>MILAN</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>fashion</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr">
-        <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr"/>
+      <c r="G58" s="2" t="inlineStr"/>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr"/>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/land/ad/5848363308?se=OLEhDWKc8RGNPOjEPgN71g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=60107C204BD9BC811A91BB2CBB46D624738C18B4</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr"/>
       <c r="B59" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -3221,7 +3233,7 @@
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3254,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F60" t="inlineStr"/>
@@ -3265,36 +3277,32 @@
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr"/>
       <c r="B61" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Sayano Deutschland GmbH</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3313,7 +3321,7 @@
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816572451?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3324,23 +3332,25 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>THE VERSE Ventures</t>
+          <t>Sayano Deutschland GmbH</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
-        </is>
-      </c>
-      <c r="F62" t="n">
-        <v>6</v>
-      </c>
-      <c r="G62" t="inlineStr"/>
+          <t>Mitte, Stuttgart</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H62" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3359,31 +3369,33 @@
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5816572451?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr"/>
       <c r="B63" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>THE VERSE Ventures</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Internship International Marketing Schwarzkopf Coloration - Legacy Brands</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Benrath, Düsseldorf</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr"/>
+          <t>Berlin, Deutschland</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>6</v>
+      </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
@@ -3403,7 +3415,7 @@
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5819890143?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3414,17 +3426,17 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Lidl Stiftung &amp; Co. KG</t>
+          <t>Abrio</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F64" t="inlineStr"/>
@@ -3447,38 +3459,32 @@
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
+          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr"/>
       <c r="B65" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>LIGANOVA I Karriere</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Praktikum Buying (all genders) – August/September 2026</t>
+          <t>Internship International Marketing Schwarzkopf Coloration - Legacy Brands</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
-        </is>
-      </c>
-      <c r="F65" t="n">
-        <v>6</v>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+          <t>Benrath, Düsseldorf</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3497,35 +3503,35 @@
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805407495?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5819890143?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr"/>
       <c r="B66" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Marketing &amp; Merchandising Assistant Trainee</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -3541,35 +3547,35 @@
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
+          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr"/>
       <c r="B67" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Marketing and Merchandising Assistant Trainee</t>
+          <t>Praktikum Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -3585,40 +3591,40 @@
       <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing-and-Merchandising-Assistant-Trainee_JR128690</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr"/>
       <c r="B68" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Wonder Natural GmbH</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
+          <t>Praktikum Marketing &amp; Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -3629,32 +3635,38 @@
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-&amp;-Sales-%28mwd%29-60329/1425985633/</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr"/>
       <c r="B69" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Digitalagenten</t>
+          <t>LIGANOVA I Karriere</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
+          <t>Praktikum Buying (all genders) – August/September 2026</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Charlottenburg, Berlin</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr"/>
-      <c r="G69" t="inlineStr"/>
+          <t>Mitte, Stuttgart</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>6</v>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="H69" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3673,35 +3685,35 @@
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804948828?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805407495?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr"/>
       <c r="B70" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>LIMITD by Wunderproducts GmbH</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Marketing &amp; Merchandising Assistant Trainee</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Kreuzberg, Berlin</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -3717,39 +3729,35 @@
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr"/>
       <c r="B71" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers GmbH WPG</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
+          <t>Marketing and Merchandising Assistant Trainee</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
+      <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -3765,36 +3773,32 @@
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing-and-Merchandising-Assistant-Trainee_JR128690</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr"/>
       <c r="B72" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>SERVICEPLAN Gruppe</t>
+          <t>Wonder Natural GmbH</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Sales (Marketing / New Business) (all genders)</t>
+          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F72" t="inlineStr"/>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3802,7 +3806,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -3813,7 +3817,7 @@
       <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3824,17 +3828,17 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>WirWinzer</t>
+          <t>Digitalagenten</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Praktikum Business Development Weinhandel (all genders)</t>
+          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Charlottenburg, Berlin</t>
         </is>
       </c>
       <c r="F73" t="inlineStr"/>
@@ -3857,80 +3861,80 @@
       <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804948828?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B74" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="C74" s="2" t="inlineStr">
-        <is>
-          <t>Richemont</t>
-        </is>
-      </c>
-      <c r="D74" s="2" t="inlineStr">
-        <is>
-          <t>Internship - High Jewelry Business Development Assistant</t>
-        </is>
-      </c>
-      <c r="E74" s="2" t="inlineStr">
-        <is>
-          <t>PARIS</t>
-        </is>
-      </c>
-      <c r="F74" s="2" t="inlineStr"/>
-      <c r="G74" s="2" t="inlineStr"/>
-      <c r="H74" s="2" t="inlineStr">
-        <is>
-          <t>fashion</t>
-        </is>
-      </c>
-      <c r="I74" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="J74" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K74" s="2" t="inlineStr"/>
-      <c r="L74" s="2" t="inlineStr">
-        <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
+      <c r="A74" t="inlineStr"/>
+      <c r="B74" t="n">
+        <v>51</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>LIMITD by Wunderproducts GmbH</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Praktikum - Business Development (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Kreuzberg, Berlin</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr"/>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr"/>
       <c r="B75" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Brand Trust</t>
+          <t>PricewaterhouseCoopers GmbH WPG</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Gleißbühl, Nürnberg</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F75" t="inlineStr"/>
-      <c r="G75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
       <c r="H75" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3949,28 +3953,36 @@
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5669847401?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr"/>
       <c r="B76" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>SERVICEPLAN Gruppe</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr"/>
+          <t>Praktikum Business Development &amp; Sales (Marketing / New Business) (all genders)</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>München, München (Kreis)</t>
+        </is>
+      </c>
       <c r="F76" t="inlineStr"/>
-      <c r="G76" t="inlineStr"/>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H76" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3978,7 +3990,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -3989,26 +4001,30 @@
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
+          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr"/>
       <c r="B77" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>WirWinzer</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Operational Trade Marketing Intern</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr"/>
+          <t>Praktikum Business Development Weinhandel (all genders)</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Altstadt-Lehel, München</t>
+        </is>
+      </c>
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
@@ -4029,51 +4045,55 @@
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Toronto-Operational-Trade-Marketing-Intern-ON-M5H4H2/1397938633/</t>
+          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr"/>
-      <c r="B78" t="n">
-        <v>49</v>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>Henkel</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
-        </is>
-      </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>Benrath, Düsseldorf</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr"/>
-      <c r="G78" t="inlineStr"/>
-      <c r="H78" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I78" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="J78" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K78" t="inlineStr"/>
-      <c r="L78" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>Richemont</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>Internship - High Jewelry Business Development Assistant</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr"/>
+      <c r="G78" s="2" t="inlineStr"/>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>fashion</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K78" s="2" t="inlineStr"/>
+      <c r="L78" s="2" t="inlineStr">
+        <is>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
         </is>
       </c>
     </row>
@@ -4084,17 +4104,17 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Brand Trust</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
+          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Schwabing-Freimann, München</t>
+          <t>Gleißbühl, Nürnberg</t>
         </is>
       </c>
       <c r="F79" t="inlineStr"/>
@@ -4117,7 +4137,7 @@
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5669847401?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4128,24 +4148,20 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>DEU-Bayern-Unterhaching</t>
-        </is>
-      </c>
+          <t>Marketing Intern - Trade Marketing</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -4161,7 +4177,7 @@
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
+          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
         </is>
       </c>
     </row>
@@ -4172,19 +4188,15 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>Fischach, Augsburg (Kreis)</t>
-        </is>
-      </c>
+          <t>Operational Trade Marketing Intern</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
@@ -4205,7 +4217,7 @@
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://careers.coty.com/job/Toronto-Operational-Trade-Marketing-Intern-ON-M5H4H2/1397938633/</t>
         </is>
       </c>
     </row>
@@ -4216,17 +4228,17 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
+          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Benrath, Düsseldorf</t>
         </is>
       </c>
       <c r="F82" t="inlineStr"/>
@@ -4238,7 +4250,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -4249,7 +4261,7 @@
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
+          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4260,17 +4272,17 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Schwabing-Freimann, München</t>
         </is>
       </c>
       <c r="F83" t="inlineStr"/>
@@ -4293,7 +4305,7 @@
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
+          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4304,24 +4316,24 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>DEU-Bayern-Unterhaching</t>
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -4337,7 +4349,7 @@
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
         </is>
       </c>
     </row>
@@ -4348,17 +4360,17 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
@@ -4381,28 +4393,28 @@
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr"/>
       <c r="B86" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>REWE Group</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F86" t="inlineStr"/>
@@ -4425,28 +4437,28 @@
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5712965755?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr"/>
       <c r="B87" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F87" t="inlineStr"/>
@@ -4469,28 +4481,28 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr"/>
       <c r="B88" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Altstadt-Nord, Köln</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F88" t="inlineStr"/>
@@ -4513,28 +4525,28 @@
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr"/>
       <c r="B89" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Devoteam G Cloud Germany</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
         </is>
       </c>
       <c r="F89" t="inlineStr"/>
@@ -4557,28 +4569,28 @@
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811135653?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr"/>
       <c r="B90" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>freudio</t>
+          <t>REWE Group</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Wien, Österreich</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
@@ -4590,7 +4602,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -4601,28 +4613,28 @@
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/details/5836667156?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5712965755?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr"/>
       <c r="B91" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F91" t="inlineStr"/>
@@ -4645,28 +4657,28 @@
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr"/>
       <c r="B92" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt-Nord, Köln</t>
         </is>
       </c>
       <c r="F92" t="inlineStr"/>
@@ -4689,7 +4701,7 @@
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4700,17 +4712,17 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>Devoteam G Cloud Germany</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F93" t="inlineStr"/>
@@ -4733,7 +4745,7 @@
       <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5811135653?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4744,17 +4756,17 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>freudio</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Wien, Österreich</t>
         </is>
       </c>
       <c r="F94" t="inlineStr"/>
@@ -4766,7 +4778,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
@@ -4777,7 +4789,7 @@
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/details/5836667156?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4788,12 +4800,12 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>sailwithus</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4821,7 +4833,7 @@
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4832,17 +4844,17 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>sailwithus</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F96" t="inlineStr"/>
@@ -4865,12 +4877,188 @@
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr"/>
+      <c r="B97" t="n">
+        <v>45</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>prepmymeal GmbH</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" t="inlineStr"/>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr"/>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr"/>
+      <c r="B98" t="n">
+        <v>45</v>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>prepmymeal GmbH</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr"/>
+      <c r="G98" t="inlineStr"/>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr"/>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr"/>
+      <c r="B99" t="n">
+        <v>45</v>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>sailwithus</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr"/>
+      <c r="G99" t="inlineStr"/>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr"/>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr"/>
+      <c r="B100" t="n">
+        <v>45</v>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>sailwithus</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr"/>
+      <c r="G100" t="inlineStr"/>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr"/>
+      <c r="L100" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5804544237?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L96"/>
+  <autoFilter ref="A1:L100"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4962,7 +5150,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C3" t="n">
         <v>91</v>
@@ -5012,7 +5200,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C5" t="n">
         <v>84</v>
@@ -5037,7 +5225,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C6" t="n">
         <v>84</v>
@@ -5062,7 +5250,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C7" t="n">
         <v>84</v>
@@ -5095,7 +5283,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C8" t="n">
         <v>84</v>
@@ -5120,7 +5308,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C9" t="n">
         <v>84</v>
@@ -5145,7 +5333,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
@@ -5170,7 +5358,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C11" t="n">
         <v>84</v>
@@ -5195,7 +5383,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C12" t="n">
         <v>84</v>
@@ -5220,7 +5408,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C13" t="n">
         <v>84</v>
@@ -5295,7 +5483,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C16" t="n">
         <v>80</v>
@@ -5320,7 +5508,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C17" t="n">
         <v>79</v>
@@ -5395,7 +5583,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C20" t="n">
         <v>78</v>
@@ -5428,7 +5616,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C21" t="n">
         <v>78</v>
@@ -5453,7 +5641,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C22" t="n">
         <v>74</v>
@@ -5482,50 +5670,50 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Miles &amp; More GmbH</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C23" t="n">
         <v>74</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Internship Marketing Strategy &amp; Delivery</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>Miles &amp; More GmbH</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C24" t="n">
         <v>74</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Internship Marketing Strategy &amp; Delivery</t>
         </is>
       </c>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
@@ -5569,7 +5757,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C26" t="n">
         <v>73</v>
@@ -5594,7 +5782,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C27" t="n">
         <v>73</v>
@@ -5619,7 +5807,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C28" t="n">
         <v>72</v>
@@ -5644,7 +5832,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C29" t="n">
         <v>72</v>
@@ -5769,7 +5957,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C34" t="n">
         <v>66</v>
@@ -5794,7 +5982,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C35" t="n">
         <v>65</v>
@@ -5819,7 +6007,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C36" t="n">
         <v>64</v>
@@ -5844,7 +6032,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C37" t="n">
         <v>62</v>
@@ -5869,7 +6057,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C38" t="n">
         <v>62</v>
@@ -5898,30 +6086,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="C39" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>workday</t>
-        </is>
-      </c>
+          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -5931,22 +6111,30 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="C40" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
+          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>workday</t>
+        </is>
+      </c>
       <c r="G40" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -5956,18 +6144,18 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>THE VERSE Ventures</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="C41" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E41" t="inlineStr"/>
@@ -5981,18 +6169,18 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Sayano Deutschland GmbH</t>
+          <t>THE VERSE Ventures</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="C42" t="n">
         <v>55</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E42" t="inlineStr"/>
@@ -6006,18 +6194,18 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Lidl Stiftung &amp; Co. KG</t>
+          <t>Sayano Deutschland GmbH</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C43" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr"/>
@@ -6031,18 +6219,18 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>72</v>
+        <v>11</v>
       </c>
       <c r="C44" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E44" t="inlineStr"/>
@@ -6056,18 +6244,18 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>sailwithus</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>36</v>
+        <v>76</v>
       </c>
       <c r="C45" t="n">
         <v>53</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr"/>
@@ -6081,18 +6269,18 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Devoteam G Cloud Germany</t>
+          <t>sailwithus</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="C46" t="n">
         <v>53</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
         </is>
       </c>
       <c r="E46" t="inlineStr"/>
@@ -6106,18 +6294,18 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>LIGANOVA I Karriere</t>
+          <t>Devoteam G Cloud Germany</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="C47" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Praktikum Buying (all genders) – August/September 2026</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
@@ -6131,18 +6319,18 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Digitalagenten</t>
+          <t>LIGANOVA I Karriere</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="C48" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
+          <t>Praktikum Buying (all genders) – August/September 2026</t>
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
@@ -6156,18 +6344,18 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Digitalagenten</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>50</v>
+        <v>19</v>
       </c>
       <c r="C49" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
+          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr"/>
@@ -6185,7 +6373,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C50" t="n">
         <v>49</v>
@@ -6210,7 +6398,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C51" t="n">
         <v>49</v>
@@ -6235,7 +6423,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C52" t="n">
         <v>49</v>
@@ -6260,7 +6448,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C53" t="n">
         <v>49</v>
@@ -6660,7 +6848,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C69" t="n">
         <v>46</v>
@@ -6685,7 +6873,7 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C70" t="n">
         <v>45</v>

</xml_diff>

<commit_message>
Lauf 2026-08-21 06:52 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firmen entdeckt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$100</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$98</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$87</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L100"/>
+  <dimension ref="A1:L98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1276,21 +1276,21 @@
     <row r="18">
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Marc O'Polo</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F18" t="n">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1319,7 +1319,7 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1335,7 +1335,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1369,7 +1369,7 @@
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5799961458?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1385,7 +1385,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1396,11 +1396,7 @@
       <c r="F20" t="n">
         <v>6</v>
       </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1419,7 +1415,7 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5799961458?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1430,17 +1426,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Ferrero</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikum im Bereich Marketing für die Marke BE-KIND DACH</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F21" t="n">
@@ -1465,7 +1461,7 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5753617280?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1476,23 +1472,27 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich Marketing für die Marke BE-KIND DACH</t>
+          <t>Praktikum Brand Management (m/w/d)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F22" t="n">
         <v>6</v>
       </c>
-      <c r="G22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1511,38 +1511,32 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5753617280?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802899675?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d)</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F23" t="n">
-        <v>6</v>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1550,7 +1544,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1561,7 +1555,7 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899675?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5843630960?se=znNqlDyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=875B574D03DFD36B16B3A3ABE0AA46F858215182</t>
         </is>
       </c>
     </row>
@@ -1577,7 +1571,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1605,7 +1599,7 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5843630960?se=znNqlDyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=875B574D03DFD36B16B3A3ABE0AA46F858215182</t>
+          <t>https://www.adzuna.de/land/ad/5843628966?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=3DAF9A0A7032477BEFBE4DD229577F81F1D32CF0</t>
         </is>
       </c>
     </row>
@@ -1621,7 +1615,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1649,7 +1643,7 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5843628966?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=3DAF9A0A7032477BEFBE4DD229577F81F1D32CF0</t>
+          <t>https://www.adzuna.de/land/ad/5843628932?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=65C46D18FCDB11FD2E933BD305E494E07D043D72</t>
         </is>
       </c>
     </row>
@@ -1660,21 +1654,27 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>Marc O'Polo</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>6</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
       <c r="H26" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -1693,7 +1693,7 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5843628932?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=65C46D18FCDB11FD2E933BD305E494E07D043D72</t>
+          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Praktikum CNX Category Management Home &amp; Living (m/w/d)</t>
+          <t>Praktikum Trade Marketing Tchibo (m/w/d)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2061,7 +2061,7 @@
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5765078175?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5744245447?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2077,7 +2077,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing Tchibo (m/w/d)</t>
+          <t>Praktikum Trade Marketing Eduscho (m/w/d)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2107,32 +2107,32 @@
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5744245447?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5773205889?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing Eduscho (m/w/d)</t>
+          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
@@ -2153,7 +2153,7 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5773205889?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2164,21 +2164,21 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>markenbaumarkt24</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Feuersbach, Siegen</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
@@ -2199,33 +2199,31 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>markenbaumarkt24</t>
+          <t>PARSA Haar- und Modeartikel GmbH</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
+          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Feuersbach, Siegen</t>
-        </is>
-      </c>
-      <c r="F38" t="n">
-        <v>2</v>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
@@ -2234,7 +2232,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -2245,23 +2243,23 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr"/>
       <c r="B39" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>PARSA Haar- und Modeartikel GmbH</t>
+          <t>Lidl Stiftung</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food in Neckarsulm</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2269,7 +2267,9 @@
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr"/>
+      <c r="F39" t="n">
+        <v>6</v>
+      </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
@@ -2278,7 +2278,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -2289,7 +2289,7 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
+          <t>https://www.adzuna.de/details/5813494719?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2300,22 +2300,20 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Lidl Stiftung</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food in Neckarsulm</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F40" t="n">
-        <v>6</v>
-      </c>
+          <t>Hamburg, Deutschland</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
@@ -2335,99 +2333,101 @@
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813494719?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr"/>
-      <c r="B41" t="n">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="n">
         <v>69</v>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Hamburg, Deutschland</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr"/>
+      <c r="G41" s="2" t="inlineStr"/>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr"/>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/land/ad/5849209692?se=qJaID2Kc8RGlrvMe-VN8Yg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B8E6A551D4E75B7916A5994DC13A8DA3451895D</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="n">
-        <v>69</v>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr"/>
-      <c r="G42" s="2" t="inlineStr"/>
-      <c r="H42" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="J42" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K42" s="2" t="inlineStr"/>
-      <c r="L42" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5849209692?se=qJaID2Kc8RGlrvMe-VN8Yg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B8E6A551D4E75B7916A5994DC13A8DA3451895D</t>
+      <c r="A42" t="inlineStr"/>
+      <c r="B42" t="n">
+        <v>68</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Barilla</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Köln, Nordrhein-Westfalen</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>6</v>
+      </c>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2443,7 +2443,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
+          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2473,7 +2473,7 @@
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2489,7 +2489,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
+          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2500,7 +2500,11 @@
       <c r="F44" t="n">
         <v>6</v>
       </c>
-      <c r="G44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H44" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2519,7 +2523,7 @@
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2530,17 +2534,17 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>Bosch Thermotechnik GmbH</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
+          <t>Praktikum im internationalen Brand Management</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Wernau (Neckar), Esslingen (Kreis)</t>
         </is>
       </c>
       <c r="F45" t="n">
@@ -2548,7 +2552,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2569,7 +2573,7 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5799981240?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2580,27 +2584,23 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Bosch Thermotechnik GmbH</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Praktikum im internationalen Brand Management</t>
+          <t>Intern Category Growth</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Wernau (Neckar), Esslingen (Kreis)</t>
+          <t>Darmstadt, Hessen</t>
         </is>
       </c>
       <c r="F46" t="n">
         <v>6</v>
       </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2619,7 +2619,7 @@
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5799981240?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5754086625?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2630,23 +2630,27 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>L’ORÉAL</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Intern Category Growth</t>
+          <t>PRAKTIKUM (M/W/D) Product Marketing - Start ab August/September/Oktober für 6 Monate</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Darmstadt, Hessen</t>
+          <t>Nordrhein-Westfalen, Deutschland</t>
         </is>
       </c>
       <c r="F47" t="n">
         <v>6</v>
       </c>
-      <c r="G47" t="inlineStr"/>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H47" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2665,7 +2669,7 @@
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5754086625?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5754061318?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2676,17 +2680,17 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>L’ORÉAL</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>PRAKTIKUM (M/W/D) Product Marketing - Start ab August/September/Oktober für 6 Monate</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Nordrhein-Westfalen, Deutschland</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F48" t="n">
@@ -2715,38 +2719,34 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5754061318?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr"/>
       <c r="B49" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F49" t="n">
         <v>6</v>
       </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2765,7 +2765,7 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2786,7 +2786,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
+          <t>Altstadt, Düsseldorf</t>
         </is>
       </c>
       <c r="F50" t="n">
@@ -2811,33 +2811,31 @@
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr"/>
       <c r="B51" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>Abrio</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Altstadt, Düsseldorf</t>
-        </is>
-      </c>
-      <c r="F51" t="n">
-        <v>6</v>
-      </c>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr">
         <is>
@@ -2857,53 +2855,49 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="n">
+      <c r="A52" t="inlineStr"/>
+      <c r="B52" t="n">
         <v>64</v>
       </c>
-      <c r="C52" s="2" t="inlineStr">
+      <c r="C52" t="inlineStr">
         <is>
           <t>Mars</t>
         </is>
       </c>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="D52" t="inlineStr">
         <is>
           <t>Internship in Trade Marketing</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="E52" t="inlineStr">
         <is>
           <t>DEU-Nordrhein-Westfalen-Köln</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr"/>
-      <c r="G52" s="2" t="inlineStr"/>
-      <c r="H52" s="2" t="inlineStr">
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr">
         <is>
           <t>fmcg</t>
         </is>
       </c>
-      <c r="I52" s="2" t="inlineStr">
+      <c r="I52" t="inlineStr">
         <is>
           <t>2026-08-19</t>
         </is>
       </c>
-      <c r="J52" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K52" s="2" t="inlineStr"/>
-      <c r="L52" s="2" t="inlineStr">
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr">
         <is>
           <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
         </is>
@@ -3002,48 +2996,44 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B55" s="2" t="n">
+      <c r="A55" t="inlineStr"/>
+      <c r="B55" t="n">
         <v>62</v>
       </c>
-      <c r="C55" s="2" t="inlineStr">
+      <c r="C55" t="inlineStr">
         <is>
           <t>Exclusive Associates</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="D55" t="inlineStr">
         <is>
           <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr">
+      <c r="E55" t="inlineStr">
         <is>
           <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
-      <c r="F55" s="2" t="inlineStr"/>
-      <c r="G55" s="2" t="inlineStr"/>
-      <c r="H55" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I55" s="2" t="inlineStr">
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
         <is>
           <t>2026-08-19</t>
         </is>
       </c>
-      <c r="J55" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K55" s="2" t="inlineStr"/>
-      <c r="L55" s="2" t="inlineStr">
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr">
         <is>
           <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
@@ -3426,17 +3416,17 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Abrio</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F64" t="inlineStr"/>
@@ -3459,7 +3449,7 @@
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
         </is>
       </c>
     </row>
@@ -3470,24 +3460,24 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Internship International Marketing Schwarzkopf Coloration - Legacy Brands</t>
+          <t>Praktikum Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Benrath, Düsseldorf</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -3503,7 +3493,7 @@
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5819890143?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
         </is>
       </c>
     </row>
@@ -3514,29 +3504,29 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Lidl Stiftung &amp; Co. KG</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Praktikum Marketing &amp; Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -3547,84 +3537,94 @@
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-&amp;-Sales-%28mwd%29-60329/1425985633/</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr"/>
-      <c r="B67" t="n">
-        <v>54</v>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>Nestle Deutschland</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>Praktikum Marketing (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>Frankfurt am Main, DE, 60329</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr"/>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>fmcg</t>
-        </is>
-      </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K67" t="inlineStr"/>
-      <c r="L67" t="inlineStr">
-        <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>LIGANOVA GmbH</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum Buying (all genders) – September 2026</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>Mitte, Stuttgart</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K67" s="2" t="inlineStr"/>
+      <c r="L67" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5849630691?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr"/>
       <c r="B68" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Sales (m/w/d)</t>
+          <t>Marketing &amp; Merchandising Assistant Trainee</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -3635,7 +3635,7 @@
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-&amp;-Sales-%28mwd%29-60329/1425985633/</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
         </is>
       </c>
     </row>
@@ -3646,30 +3646,24 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>LIGANOVA I Karriere</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Praktikum Buying (all genders) – August/September 2026</t>
+          <t>Marketing and Merchandising Assistant Trainee</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
-        </is>
-      </c>
-      <c r="F69" t="n">
-        <v>6</v>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+          <t>MILAN</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -3685,7 +3679,7 @@
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805407495?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing-and-Merchandising-Assistant-Trainee_JR128690</t>
         </is>
       </c>
     </row>
@@ -3696,29 +3690,29 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Wonder Natural GmbH</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Marketing &amp; Merchandising Assistant Trainee</t>
+          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -3729,35 +3723,35 @@
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
+          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr"/>
       <c r="B71" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Digitalagenten</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Marketing and Merchandising Assistant Trainee</t>
+          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Charlottenburg, Berlin</t>
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -3773,28 +3767,28 @@
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing-and-Merchandising-Assistant-Trainee_JR128690</t>
+          <t>https://www.adzuna.de/details/5804948828?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr"/>
       <c r="B72" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Wonder Natural GmbH</t>
+          <t>LIMITD by Wunderproducts GmbH</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Kreuzberg, Berlin</t>
         </is>
       </c>
       <c r="F72" t="inlineStr"/>
@@ -3806,7 +3800,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -3817,7 +3811,7 @@
       <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3828,21 +3822,25 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Digitalagenten</t>
+          <t>PricewaterhouseCoopers GmbH WPG</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Charlottenburg, Berlin</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F73" t="inlineStr"/>
-      <c r="G73" t="inlineStr"/>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
       <c r="H73" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3861,7 +3859,7 @@
       <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804948828?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3872,21 +3870,25 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>LIMITD by Wunderproducts GmbH</t>
+          <t>SERVICEPLAN Gruppe</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Sales (Marketing / New Business) (all genders)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Kreuzberg, Berlin</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F74" t="inlineStr"/>
-      <c r="G74" t="inlineStr"/>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H74" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3894,7 +3896,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -3905,7 +3907,7 @@
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3916,25 +3918,21 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers GmbH WPG</t>
+          <t>WirWinzer</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
+          <t>Praktikum Business Development Weinhandel (all genders)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F75" t="inlineStr"/>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
+      <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3953,44 +3951,40 @@
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr"/>
       <c r="B76" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>SERVICEPLAN Gruppe</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Sales (Marketing / New Business) (all genders)</t>
+          <t>Internship - High Jewelry Business Development Assistant</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>PARIS</t>
         </is>
       </c>
       <c r="F76" t="inlineStr"/>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -4001,28 +3995,28 @@
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr"/>
       <c r="B77" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>WirWinzer</t>
+          <t>Brand Trust</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Praktikum Business Development Weinhandel (all genders)</t>
+          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Gleißbühl, Nürnberg</t>
         </is>
       </c>
       <c r="F77" t="inlineStr"/>
@@ -4045,55 +4039,47 @@
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5669847401?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B78" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="C78" s="2" t="inlineStr">
-        <is>
-          <t>Richemont</t>
-        </is>
-      </c>
-      <c r="D78" s="2" t="inlineStr">
-        <is>
-          <t>Internship - High Jewelry Business Development Assistant</t>
-        </is>
-      </c>
-      <c r="E78" s="2" t="inlineStr">
-        <is>
-          <t>PARIS</t>
-        </is>
-      </c>
-      <c r="F78" s="2" t="inlineStr"/>
-      <c r="G78" s="2" t="inlineStr"/>
-      <c r="H78" s="2" t="inlineStr">
-        <is>
-          <t>fashion</t>
-        </is>
-      </c>
-      <c r="I78" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="J78" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K78" s="2" t="inlineStr"/>
-      <c r="L78" s="2" t="inlineStr">
-        <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
+      <c r="A78" t="inlineStr"/>
+      <c r="B78" t="n">
+        <v>49</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Coty</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Marketing Intern - Trade Marketing</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr"/>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
         </is>
       </c>
     </row>
@@ -4104,19 +4090,15 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Brand Trust</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>Gleißbühl, Nürnberg</t>
-        </is>
-      </c>
+          <t>Operational Trade Marketing Intern</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
@@ -4137,7 +4119,7 @@
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5669847401?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://careers.coty.com/job/Toronto-Operational-Trade-Marketing-Intern-ON-M5H4H2/1397938633/</t>
         </is>
       </c>
     </row>
@@ -4148,15 +4130,19 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr"/>
+          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Benrath, Düsseldorf</t>
+        </is>
+      </c>
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
@@ -4166,7 +4152,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -4177,7 +4163,7 @@
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
+          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4188,15 +4174,19 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Operational Trade Marketing Intern</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr"/>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Schwabing-Freimann, München</t>
+        </is>
+      </c>
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
@@ -4217,7 +4207,7 @@
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Toronto-Operational-Trade-Marketing-Intern-ON-M5H4H2/1397938633/</t>
+          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4228,29 +4218,29 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
+          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Benrath, Düsseldorf</t>
+          <t>DEU-Bayern-Unterhaching</t>
         </is>
       </c>
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -4261,7 +4251,7 @@
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
         </is>
       </c>
     </row>
@@ -4272,17 +4262,17 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Schwabing-Freimann, München</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F83" t="inlineStr"/>
@@ -4305,7 +4295,7 @@
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4316,24 +4306,24 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
+          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>DEU-Bayern-Unterhaching</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -4349,7 +4339,7 @@
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
+          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
         </is>
       </c>
     </row>
@@ -4360,17 +4350,17 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
@@ -4393,7 +4383,7 @@
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
         </is>
       </c>
     </row>
@@ -4409,7 +4399,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -4437,7 +4427,7 @@
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
+          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
         </is>
       </c>
     </row>
@@ -4448,17 +4438,17 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
         </is>
       </c>
       <c r="F87" t="inlineStr"/>
@@ -4481,28 +4471,28 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
+          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr"/>
       <c r="B88" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>REWE Group</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F88" t="inlineStr"/>
@@ -4525,28 +4515,28 @@
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
+          <t>https://www.adzuna.de/details/5712965755?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr"/>
       <c r="B89" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F89" t="inlineStr"/>
@@ -4569,28 +4559,28 @@
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr"/>
       <c r="B90" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>REWE Group</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Altstadt-Nord, Köln</t>
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
@@ -4613,28 +4603,28 @@
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5712965755?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr"/>
       <c r="B91" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>Devoteam G Cloud Germany</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F91" t="inlineStr"/>
@@ -4657,28 +4647,28 @@
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5811135653?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr"/>
       <c r="B92" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>freudio</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Altstadt-Nord, Köln</t>
+          <t>Wien, Österreich</t>
         </is>
       </c>
       <c r="F92" t="inlineStr"/>
@@ -4690,7 +4680,7 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
@@ -4701,7 +4691,7 @@
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/details/5836667156?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4712,12 +4702,12 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Devoteam G Cloud Germany</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -4745,7 +4735,7 @@
       <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811135653?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4756,17 +4746,17 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>freudio</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Wien, Österreich</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F94" t="inlineStr"/>
@@ -4778,7 +4768,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
@@ -4789,7 +4779,7 @@
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/details/5836667156?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4810,7 +4800,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F95" t="inlineStr"/>
@@ -4833,7 +4823,7 @@
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4854,7 +4844,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F96" t="inlineStr"/>
@@ -4877,7 +4867,7 @@
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4888,17 +4878,17 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>sailwithus</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -4921,7 +4911,7 @@
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4932,12 +4922,12 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>sailwithus</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -4965,100 +4955,12 @@
       <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr"/>
-      <c r="B99" t="n">
-        <v>45</v>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>sailwithus</t>
-        </is>
-      </c>
-      <c r="D99" t="inlineStr">
-        <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
-        </is>
-      </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F99" t="inlineStr"/>
-      <c r="G99" t="inlineStr"/>
-      <c r="H99" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I99" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J99" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K99" t="inlineStr"/>
-      <c r="L99" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr"/>
-      <c r="B100" t="n">
-        <v>45</v>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>sailwithus</t>
-        </is>
-      </c>
-      <c r="D100" t="inlineStr">
-        <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
-        </is>
-      </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>Altstadt, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F100" t="inlineStr"/>
-      <c r="G100" t="inlineStr"/>
-      <c r="H100" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I100" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J100" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K100" t="inlineStr"/>
-      <c r="L100" t="inlineStr">
-        <is>
           <t>https://www.adzuna.de/details/5804544237?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L100"/>
+  <autoFilter ref="A1:L98"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5069,7 +4971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G86"/>
+  <dimension ref="A1:G87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -5150,7 +5052,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C3" t="n">
         <v>91</v>
@@ -5200,7 +5102,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="C5" t="n">
         <v>84</v>
@@ -5225,7 +5127,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C6" t="n">
         <v>84</v>
@@ -5250,7 +5152,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C7" t="n">
         <v>84</v>
@@ -5283,7 +5185,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C8" t="n">
         <v>84</v>
@@ -5308,7 +5210,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C9" t="n">
         <v>84</v>
@@ -5333,7 +5235,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
@@ -5358,7 +5260,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C11" t="n">
         <v>84</v>
@@ -5383,7 +5285,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C12" t="n">
         <v>84</v>
@@ -5408,7 +5310,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C13" t="n">
         <v>84</v>
@@ -5483,7 +5385,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C16" t="n">
         <v>80</v>
@@ -5508,7 +5410,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C17" t="n">
         <v>79</v>
@@ -5583,7 +5485,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C20" t="n">
         <v>78</v>
@@ -5616,7 +5518,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C21" t="n">
         <v>78</v>
@@ -5641,7 +5543,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C22" t="n">
         <v>74</v>
@@ -5674,7 +5576,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C23" t="n">
         <v>74</v>
@@ -5699,7 +5601,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C24" t="n">
         <v>74</v>
@@ -5757,7 +5659,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C26" t="n">
         <v>73</v>
@@ -5782,7 +5684,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C27" t="n">
         <v>73</v>
@@ -5807,7 +5709,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C28" t="n">
         <v>72</v>
@@ -5832,7 +5734,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C29" t="n">
         <v>72</v>
@@ -5957,7 +5859,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C34" t="n">
         <v>66</v>
@@ -5982,7 +5884,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C35" t="n">
         <v>65</v>
@@ -6007,7 +5909,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C36" t="n">
         <v>64</v>
@@ -6032,7 +5934,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C37" t="n">
         <v>62</v>
@@ -6057,7 +5959,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C38" t="n">
         <v>62</v>
@@ -6090,7 +5992,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C39" t="n">
         <v>59</v>
@@ -6115,7 +6017,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C40" t="n">
         <v>57</v>
@@ -6148,7 +6050,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C41" t="n">
         <v>56</v>
@@ -6173,7 +6075,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C42" t="n">
         <v>55</v>
@@ -6248,7 +6150,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C45" t="n">
         <v>53</v>
@@ -6273,7 +6175,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C46" t="n">
         <v>53</v>
@@ -6344,43 +6246,43 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Digitalagenten</t>
+          <t>LIGANOVA GmbH</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="C49" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
+          <t>Praktikum Buying (all genders) – September 2026</t>
         </is>
       </c>
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Brand Trust</t>
+          <t>Digitalagenten</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C50" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
+          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
@@ -6394,18 +6296,18 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>Brand Trust</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C51" t="n">
         <v>49</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr"/>
@@ -6419,18 +6321,18 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C52" t="n">
         <v>49</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E52" t="inlineStr"/>
@@ -6444,18 +6346,18 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C53" t="n">
         <v>49</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
@@ -6469,18 +6371,18 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>REWE Group</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C54" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr"/>
@@ -6494,18 +6396,18 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Pflegia</t>
+          <t>REWE Group</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="C55" t="n">
         <v>48</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr"/>
@@ -6519,18 +6421,18 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Werkia</t>
+          <t>Pflegia</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C56" t="n">
         <v>48</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d) - Datenanalyse &amp; Automatisierung</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr"/>
@@ -6544,7 +6446,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>paero</t>
+          <t>Werkia</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -6555,7 +6457,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/d) - Datenanalyse &amp; Automatisierung</t>
         </is>
       </c>
       <c r="E57" t="inlineStr"/>
@@ -6569,7 +6471,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Vivanta Gmbh</t>
+          <t>paero</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -6580,7 +6482,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
@@ -6594,7 +6496,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Vitolus</t>
+          <t>Vivanta Gmbh</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -6605,7 +6507,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
@@ -6619,7 +6521,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>GrantLift GmbH</t>
+          <t>Vitolus</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -6630,7 +6532,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
+          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
         </is>
       </c>
       <c r="E60" t="inlineStr"/>
@@ -6644,7 +6546,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Otto Group one.O GmbH</t>
+          <t>GrantLift GmbH</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -6655,7 +6557,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Praktikum im Knowledge Management - Corporate Strategy (w/m/d)</t>
+          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E61" t="inlineStr"/>
@@ -6669,18 +6571,18 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>AUTO1 Global Services SE &amp; Co. KG</t>
+          <t>Otto Group one.O GmbH</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C62" t="n">
         <v>48</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (d/m/w)</t>
+          <t>Praktikum im Knowledge Management - Corporate Strategy (w/m/d)</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
@@ -6694,7 +6596,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>SHAVENT - ARA Sustainable Products</t>
+          <t>AUTO1 Global Services SE &amp; Co. KG</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -6705,7 +6607,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Praktikum Business Development in nachhaltigem Start-Up (w/m/d) Remote in DE</t>
+          <t>Praktikum Business Development (d/m/w)</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
@@ -6719,7 +6621,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CTG Consulting</t>
+          <t>SHAVENT - ARA Sustainable Products</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -6730,7 +6632,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Praktikum Sales/Business Development // Hamburg oder Berlin</t>
+          <t>Praktikum Business Development in nachhaltigem Start-Up (w/m/d) Remote in DE</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
@@ -6744,7 +6646,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Dronesperhour</t>
+          <t>CTG Consulting</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -6755,7 +6657,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development eines Startups (m/w/d)</t>
+          <t>Praktikum Sales/Business Development // Hamburg oder Berlin</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
@@ -6769,7 +6671,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>SINN Power</t>
+          <t>Dronesperhour</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -6780,7 +6682,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Praktikum im AI Business Development (m/w/d)</t>
+          <t>Praktikum im Business Development eines Startups (m/w/d)</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
@@ -6794,7 +6696,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>innpuls</t>
+          <t>SINN Power</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -6805,7 +6707,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Praktikum im AI Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
@@ -6819,7 +6721,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Amolina</t>
+          <t>innpuls</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -6830,7 +6732,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr"/>
@@ -6844,18 +6746,18 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>Amolina</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>38</v>
+        <v>1</v>
       </c>
       <c r="C69" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
@@ -6869,57 +6771,57 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>freudio</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>9</v>
+        <v>40</v>
       </c>
       <c r="C70" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>STARTPLATZ Gruppe</t>
+          <t>freudio</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C71" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Sales (m/w/d) – STARTPLATZ</t>
+          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>spring.gate business consulting UG</t>
+          <t>STARTPLATZ Gruppe</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -6930,7 +6832,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development &amp; B2B Akquise (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Sales (m/w/d) – STARTPLATZ</t>
         </is>
       </c>
       <c r="E72" t="inlineStr"/>
@@ -6944,7 +6846,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>specter automation</t>
+          <t>spring.gate business consulting UG</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -6955,7 +6857,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Praktikum (M/W/D) im Business Development</t>
+          <t>Praktikum im Business Development &amp; B2B Akquise (m/w/d)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr"/>
@@ -6969,18 +6871,18 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Closd Kunststoffprodukte GmbH</t>
+          <t>specter automation</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C74" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Praktikum beim E-Commerce Startup Closd als Founders Associate (m/w/d)</t>
+          <t>Praktikum (M/W/D) im Business Development</t>
         </is>
       </c>
       <c r="E74" t="inlineStr"/>
@@ -6994,18 +6896,18 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Bosch Rexroth AG</t>
+          <t>Closd Kunststoffprodukte GmbH</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C75" t="n">
         <v>38</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Praktikum Business Development – Software Defined Business</t>
+          <t>Praktikum beim E-Commerce Startup Closd als Founders Associate (m/w/d)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr"/>
@@ -7019,7 +6921,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Weenect</t>
+          <t>Bosch Rexroth AG</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -7030,7 +6932,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d) – Markt DACH – Standort Brüssel</t>
+          <t>Praktikum Business Development – Software Defined Business</t>
         </is>
       </c>
       <c r="E76" t="inlineStr"/>
@@ -7044,18 +6946,18 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Lidl Dienstleistung GmbH &amp; Co. KG</t>
+          <t>Weenect</t>
         </is>
       </c>
       <c r="B77" t="n">
         <v>1</v>
       </c>
       <c r="C77" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Praktikum Business Development (m/w/d) – Markt DACH – Standort Brüssel</t>
         </is>
       </c>
       <c r="E77" t="inlineStr"/>
@@ -7069,18 +6971,18 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Drägerwerk AG &amp; Co. KGaA</t>
+          <t>Lidl Dienstleistung GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C78" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Praktikum New Business Development</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E78" t="inlineStr"/>
@@ -7094,18 +6996,18 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Arteus Energy</t>
+          <t>Drägerwerk AG &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C79" t="n">
         <v>28</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Praktikum Business Development und Marketing Photovoltaik</t>
+          <t>Praktikum New Business Development</t>
         </is>
       </c>
       <c r="E79" t="inlineStr"/>
@@ -7119,7 +7021,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>aramido</t>
+          <t>Arteus Energy</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -7130,7 +7032,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/x)</t>
+          <t>Praktikum Business Development und Marketing Photovoltaik</t>
         </is>
       </c>
       <c r="E80" t="inlineStr"/>
@@ -7144,7 +7046,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>pacemaker.ai by thyssenkrupp</t>
+          <t>aramido</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -7155,7 +7057,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/x)</t>
         </is>
       </c>
       <c r="E81" t="inlineStr"/>
@@ -7169,7 +7071,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Molly Suh GmbH</t>
+          <t>pacemaker.ai by thyssenkrupp</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -7180,7 +7082,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; B2B Sales (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E82" t="inlineStr"/>
@@ -7194,7 +7096,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>homewise</t>
+          <t>Molly Suh GmbH</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -7205,7 +7107,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development &amp; Strategie (m/w/d)</t>
+          <t>Praktikum Business Development &amp; B2B Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E83" t="inlineStr"/>
@@ -7219,7 +7121,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>ClipMyHorse.TV</t>
+          <t>homewise</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -7230,7 +7132,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Praktikum HR &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im Business Development &amp; Strategie (m/w/d)</t>
         </is>
       </c>
       <c r="E84" t="inlineStr"/>
@@ -7244,7 +7146,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>AUMOVIO</t>
+          <t>ClipMyHorse.TV</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -7255,7 +7157,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Praktikum - Administration/Assistenz &amp; Business Development</t>
+          <t>Praktikum HR &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E85" t="inlineStr"/>
@@ -7269,7 +7171,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>TRUMPF Group</t>
+          <t>AUMOVIO</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -7280,7 +7182,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich Business Development für Smart Factory Solutions (WS26/27)</t>
+          <t>Praktikum - Administration/Assistenz &amp; Business Development</t>
         </is>
       </c>
       <c r="E86" t="inlineStr"/>
@@ -7291,8 +7193,33 @@
         </is>
       </c>
     </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>TRUMPF Group</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>1</v>
+      </c>
+      <c r="C87" t="n">
+        <v>28</v>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Praktikum im Bereich Business Development für Smart Factory Solutions (WS26/27)</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G86"/>
+  <autoFilter ref="A1:G87"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Lauf 2026-08-22 06:46 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firmen entdeckt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$98</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$97</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$87</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L98"/>
+  <dimension ref="A1:L97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -610,31 +610,27 @@
     <row r="4">
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="n">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>VEYNOU GmbH</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management &amp; Shopper Marketing</t>
+          <t>Praktikum Business Development (m/w/d) 3-6 Monate</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Benrath, Düsseldorf</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>4</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -653,28 +649,28 @@
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816411046?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5646645887?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="n">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>VEYNOU GmbH</t>
+          <t>Carwow</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d) 3-6 Monate</t>
+          <t>Praktikum Business Development &amp; Media (m/w/d) - OEM Partnerships @ Carwow</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -699,7 +695,7 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5646645887?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5822522402?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -710,17 +706,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Carwow</t>
+          <t>FC Viktoria 1889 Berlin Frauen-Fußball GmbH</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Media (m/w/d) - OEM Partnerships @ Carwow</t>
+          <t>PRAKTIKUM // Business Development</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Mitte, Berlin</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -745,7 +741,7 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5822522402?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802962068?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -756,21 +752,21 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>FC Viktoria 1889 Berlin Frauen-Fußball GmbH</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>PRAKTIKUM // Business Development</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Mitte, Berlin</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
@@ -791,7 +787,7 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802962068?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -802,25 +798,25 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>Nestle</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Internship Digital Brand Marketing</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Benrath, Düsseldorf</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -841,7 +837,7 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816488136?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -852,35 +848,35 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Internship Digital Brand Marketing Schwarzkopf</t>
+          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Benrath, Düsseldorf</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -891,7 +887,7 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816486591?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Category-Management%2C-Brand-Activation-und-Sales-%28mwd%29-60329/1427883433/</t>
         </is>
       </c>
     </row>
@@ -902,21 +898,21 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Hamburg-Altstadt, Hamburg</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
@@ -926,7 +922,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -937,7 +933,7 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5829732882?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -948,27 +944,23 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Nestle</t>
+          <t>Picnic</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Category Management Praktikum (m/w/d)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>5</v>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>2026-11-01</t>
-        </is>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -987,88 +979,82 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="n">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="n">
         <v>84</v>
       </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Nestle Deutschland</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Frankfurt am Main, DE, 60329</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>fmcg</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Category-Management%2C-Brand-Activation-und-Sales-%28mwd%29-60329/1427883433/</t>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Picnic</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Category Management Praktikum (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>6</v>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5759088383?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="n">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Brand Management National</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Hamburg-Altstadt, Hamburg</t>
-        </is>
-      </c>
-      <c r="F13" t="n">
-        <v>6</v>
-      </c>
-      <c r="G13" t="inlineStr"/>
+          <t>Au-Haidhausen, München</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1076,7 +1062,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1087,37 +1073,33 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5829732882?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805399065?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="n">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Picnic</t>
+          <t>EAT HAPPY GROUP</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Category Management Praktikum (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Hamburg, Deutschland</t>
-        </is>
-      </c>
+          <t>Praktikum Brand Marketing (m/w/d) Marketing · Köln</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="n">
         <v>6</v>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1133,34 +1115,38 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://eathappygroup.teamtailor.com/jobs/7902845-praktikum-brand-marketing-m-w-d</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="n">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Picnic</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Category Management Praktikum (m/w/d)</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F15" t="n">
         <v>6</v>
       </c>
-      <c r="G15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1179,34 +1165,36 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759088383?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management National</t>
+          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Au-Haidhausen, München</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr"/>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>6</v>
+      </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1227,33 +1215,37 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805399065?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5799961458?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>EAT HAPPY GROUP</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Praktikum Brand Marketing (m/w/d) Marketing · Köln</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
       <c r="F17" t="n">
         <v>6</v>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1269,7 +1261,7 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://eathappygroup.teamtailor.com/jobs/7902845-praktikum-brand-marketing-m-w-d</t>
+          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1280,27 +1272,23 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Ferrero</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikum im Bereich Marketing für die Marke BE-KIND DACH</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F18" t="n">
         <v>6</v>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1319,7 +1307,7 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5753617280?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1330,17 +1318,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Ferrero</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikum Brand Management (m/w/d)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F19" t="n">
@@ -1348,7 +1336,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1369,23 +1357,23 @@
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5799961458?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802899675?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Ferrero</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1393,9 +1381,7 @@
           <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
-      <c r="F20" t="n">
-        <v>6</v>
-      </c>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
@@ -1404,7 +1390,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1415,33 +1401,31 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5843630960?se=znNqlDyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=875B574D03DFD36B16B3A3ABE0AA46F858215182</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
       <c r="B21" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich Marketing für die Marke BE-KIND DACH</t>
+          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F21" t="n">
-        <v>6</v>
-      </c>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
@@ -1450,7 +1434,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -1461,38 +1445,32 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5753617280?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5843628966?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=3DAF9A0A7032477BEFBE4DD229577F81F1D32CF0</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr"/>
       <c r="B22" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F22" t="n">
-        <v>6</v>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1500,7 +1478,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1511,7 +1489,7 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899675?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5843628932?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=65C46D18FCDB11FD2E933BD305E494E07D043D72</t>
         </is>
       </c>
     </row>
@@ -1522,17 +1500,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>Miles &amp; More GmbH</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Internship Marketing Strategy &amp; Delivery</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Flughafen, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F23" t="inlineStr"/>
@@ -1544,7 +1522,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1555,7 +1533,7 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5843630960?se=znNqlDyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=875B574D03DFD36B16B3A3ABE0AA46F858215182</t>
+          <t>https://www.adzuna.de/details/5828674997?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1566,12 +1544,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikum Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1588,7 +1566,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -1599,7 +1577,7 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5843628966?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=3DAF9A0A7032477BEFBE4DD229577F81F1D32CF0</t>
+          <t>https://www.adzuna.de/details/5802899691?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1610,20 +1588,22 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>coty</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Marketing Intern - Trade Marketing</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr"/>
+          <t>Darmstadt, Hessen</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>6</v>
+      </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
@@ -1632,7 +1612,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -1643,38 +1623,34 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5843628932?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=65C46D18FCDB11FD2E933BD305E494E07D043D72</t>
+          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
       <c r="B26" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Marc O'Polo</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
+          <t>Praktikum im Bereich Marketing für die Marke BE-KIND DACH</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Unterhaching, München (Kreis)</t>
         </is>
       </c>
       <c r="F26" t="n">
         <v>6</v>
       </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
+      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1693,31 +1669,33 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5752932983?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Miles &amp; More GmbH</t>
+          <t>P&amp;G</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Internship Marketing Strategy &amp; Delivery</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Flughafen, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr"/>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>6</v>
+      </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
@@ -1737,31 +1715,33 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5828674997?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>Tchibo GmbH</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Praktikum Marketing (m/w/d)</t>
+          <t>Praktikum Category Management Non Food Vertrieb (m/w/d)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr"/>
+          <t>Hamburg, Deutschland</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>6</v>
+      </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
@@ -1781,28 +1761,28 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899691?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5795118484?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>coty</t>
+          <t>Tchibo GmbH</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
+          <t>Praktikum Trade Marketing Tchibo (m/w/d)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Darmstadt, Hessen</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F29" t="n">
@@ -1827,7 +1807,7 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5744245447?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1838,27 +1818,23 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>Tchibo GmbH</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Praktikum Digital Marketing &amp; Category Management</t>
+          <t>Praktikum Trade Marketing Eduscho (m/w/d)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Benrath, Düsseldorf</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F30" t="n">
         <v>6</v>
       </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
+      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1877,32 +1853,32 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816415884?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5773205889?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr"/>
       <c r="B31" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich Marketing für die Marke BE-KIND DACH</t>
+          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Unterhaching, München (Kreis)</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
@@ -1923,124 +1899,132 @@
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5752932983?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr"/>
-      <c r="B32" t="n">
-        <v>73</v>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>P&amp;G</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F32" t="n">
-        <v>6</v>
-      </c>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Exclusive Associates</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum Business Development &amp; Talent Partnerships (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Düsseltal, Düsseldorf</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr"/>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5851100606?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr"/>
-      <c r="B33" t="n">
-        <v>73</v>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Tchibo GmbH</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Praktikum Category Management Non Food Vertrieb (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Hamburg, Deutschland</t>
-        </is>
-      </c>
-      <c r="F33" t="n">
-        <v>6</v>
-      </c>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5795118484?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Exclusive Associates</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum im B2B-Vertrieb &amp; Business Development (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Düsseltal, Düsseldorf</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G33" s="2" t="inlineStr"/>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr"/>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5851898375?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr"/>
       <c r="B34" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>markenbaumarkt24</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing Tchibo (m/w/d)</t>
+          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Feuersbach, Siegen</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
@@ -2061,33 +2045,31 @@
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5744245447?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr"/>
       <c r="B35" t="n">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>PARSA Haar- und Modeartikel GmbH</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing Eduscho (m/w/d)</t>
+          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
-        </is>
-      </c>
-      <c r="F35" t="n">
-        <v>6</v>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
@@ -2096,7 +2078,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -2107,32 +2089,32 @@
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5773205889?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>Lidl Stiftung</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food in Neckarsulm</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
@@ -2153,33 +2135,31 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5813494719?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>markenbaumarkt24</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Feuersbach, Siegen</t>
-        </is>
-      </c>
-      <c r="F37" t="n">
-        <v>2</v>
-      </c>
+          <t>Hamburg, Deutschland</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
@@ -2199,23 +2179,23 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>PARSA Haar- und Modeartikel GmbH</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2232,7 +2212,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -2243,28 +2223,28 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
+          <t>https://www.adzuna.de/land/ad/5849209692?se=qJaID2Kc8RGlrvMe-VN8Yg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B8E6A551D4E75B7916A5994DC13A8DA3451895D</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr"/>
       <c r="B39" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Lidl Stiftung</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food in Neckarsulm</t>
+          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F39" t="n">
@@ -2289,31 +2269,33 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813494719?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr"/>
       <c r="B40" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr"/>
+          <t>Köln, Nordrhein-Westfalen</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>6</v>
+      </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
@@ -2333,55 +2315,57 @@
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
+          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="n">
-        <v>69</v>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr"/>
-      <c r="G41" s="2" t="inlineStr"/>
-      <c r="H41" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I41" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="J41" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K41" s="2" t="inlineStr"/>
-      <c r="L41" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5849209692?se=qJaID2Kc8RGlrvMe-VN8Yg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B8E6A551D4E75B7916A5994DC13A8DA3451895D</t>
+      <c r="A41" t="inlineStr"/>
+      <c r="B41" t="n">
+        <v>68</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Barilla</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Köln, Nordrhein-Westfalen</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>6</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2392,23 +2376,27 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>Bosch Thermotechnik GmbH</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
+          <t>Praktikum im internationalen Brand Management</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Wernau (Neckar), Esslingen (Kreis)</t>
         </is>
       </c>
       <c r="F42" t="n">
         <v>6</v>
       </c>
-      <c r="G42" t="inlineStr"/>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="H42" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2427,7 +2415,7 @@
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5799981240?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2438,17 +2426,17 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
+          <t>Intern Category Growth</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Darmstadt, Hessen</t>
         </is>
       </c>
       <c r="F43" t="n">
@@ -2473,7 +2461,7 @@
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5754086625?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2484,17 +2472,17 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>L’ORÉAL</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
+          <t>PRAKTIKUM (M/W/D) Product Marketing - Start ab August/September/Oktober für 6 Monate</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Nordrhein-Westfalen, Deutschland</t>
         </is>
       </c>
       <c r="F44" t="n">
@@ -2523,7 +2511,7 @@
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5754061318?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2534,17 +2522,17 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Bosch Thermotechnik GmbH</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Praktikum im internationalen Brand Management</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Wernau (Neckar), Esslingen (Kreis)</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F45" t="n">
@@ -2552,7 +2540,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2573,28 +2561,28 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5799981240?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr"/>
       <c r="B46" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Intern Category Growth</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Darmstadt, Hessen</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F46" t="n">
@@ -2619,38 +2607,34 @@
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5754086625?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr"/>
       <c r="B47" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>L’ORÉAL</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>PRAKTIKUM (M/W/D) Product Marketing - Start ab August/September/Oktober für 6 Monate</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Nordrhein-Westfalen, Deutschland</t>
+          <t>Altstadt, Düsseldorf</t>
         </is>
       </c>
       <c r="F47" t="n">
         <v>6</v>
       </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2669,46 +2653,40 @@
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5754061318?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr"/>
       <c r="B48" t="n">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>Internship in Trade Marketing</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
-        </is>
-      </c>
-      <c r="F48" t="n">
-        <v>6</v>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>DEU-Nordrhein-Westfalen-Köln</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -2719,34 +2697,36 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr"/>
       <c r="B49" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F49" t="n">
-        <v>6</v>
-      </c>
-      <c r="G49" t="inlineStr"/>
+          <t>Köln, Nordrhein-Westfalen</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H49" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2765,33 +2745,31 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5822943276?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=580C236799B96DFD395A1EC1CBBF7474C7F58435</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr"/>
       <c r="B50" t="n">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>Calypso Ventures GmbH</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Altstadt, Düsseldorf</t>
-        </is>
-      </c>
-      <c r="F50" t="n">
-        <v>6</v>
-      </c>
+          <t>Berlin, Deutschland</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr">
         <is>
@@ -2811,28 +2789,28 @@
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr"/>
       <c r="B51" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Abrio</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
+          <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
@@ -2844,7 +2822,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -2855,40 +2833,40 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr"/>
       <c r="B52" t="n">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Internship in Trade Marketing</t>
+          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>DEU-Nordrhein-Westfalen-Köln</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -2899,36 +2877,32 @@
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
+          <t>https://www.adzuna.de/land/ad/5848400955?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=4E59A334AC360616EAEAAC474F72A07451A7C624</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr"/>
       <c r="B53" t="n">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2936,7 +2910,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -2947,28 +2921,28 @@
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5822943276?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=580C236799B96DFD395A1EC1CBBF7474C7F58435</t>
+          <t>https://www.adzuna.de/land/ad/5848409009?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5C62DDCDA5E03F77D6089CD03CFA1D966DF15C96</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr"/>
       <c r="B54" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Calypso Ventures GmbH</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
+          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F54" t="inlineStr"/>
@@ -2980,7 +2954,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -2991,40 +2965,40 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5848363308?se=OLEhDWKc8RGNPOjEPgN71g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=60107C204BD9BC811A91BB2CBB46D624738C18B4</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr"/>
       <c r="B55" t="n">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -3035,179 +3009,173 @@
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B56" s="2" t="n">
-        <v>59</v>
-      </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr">
-        <is>
-          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F56" s="2" t="inlineStr"/>
-      <c r="G56" s="2" t="inlineStr"/>
-      <c r="H56" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I56" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="J56" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K56" s="2" t="inlineStr"/>
-      <c r="L56" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5848400955?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=4E59A334AC360616EAEAAC474F72A07451A7C624</t>
+      <c r="A56" t="inlineStr"/>
+      <c r="B56" t="n">
+        <v>56</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Upsters Energy GmbH</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B57" s="2" t="n">
-        <v>59</v>
-      </c>
-      <c r="C57" s="2" t="inlineStr">
-        <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
-        </is>
-      </c>
-      <c r="D57" s="2" t="inlineStr">
-        <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E57" s="2" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F57" s="2" t="inlineStr"/>
-      <c r="G57" s="2" t="inlineStr"/>
-      <c r="H57" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I57" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="J57" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K57" s="2" t="inlineStr"/>
-      <c r="L57" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5848409009?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5C62DDCDA5E03F77D6089CD03CFA1D966DF15C96</t>
+      <c r="A57" t="inlineStr"/>
+      <c r="B57" t="n">
+        <v>56</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Upsters Energy GmbH</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B58" s="2" t="n">
-        <v>59</v>
-      </c>
-      <c r="C58" s="2" t="inlineStr">
-        <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
-        </is>
-      </c>
-      <c r="D58" s="2" t="inlineStr">
-        <is>
-          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F58" s="2" t="inlineStr"/>
-      <c r="G58" s="2" t="inlineStr"/>
-      <c r="H58" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I58" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="J58" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K58" s="2" t="inlineStr"/>
-      <c r="L58" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5848363308?se=OLEhDWKc8RGNPOjEPgN71g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=60107C204BD9BC811A91BB2CBB46D624738C18B4</t>
+      <c r="A58" t="inlineStr"/>
+      <c r="B58" t="n">
+        <v>55</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Sayano Deutschland GmbH</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Mitte, Stuttgart</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5816572451?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr"/>
       <c r="B59" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>THE VERSE Ventures</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>MILAN</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr"/>
+          <t>Berlin, Deutschland</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>6</v>
+      </c>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -3223,28 +3191,28 @@
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
+          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr"/>
       <c r="B60" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>Abrio</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F60" t="inlineStr"/>
@@ -3267,28 +3235,28 @@
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr"/>
       <c r="B61" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F61" t="inlineStr"/>
@@ -3311,82 +3279,84 @@
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr"/>
-      <c r="B62" t="n">
-        <v>55</v>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Sayano Deutschland GmbH</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>Mitte, Stuttgart</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5816572451?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Lidl Stiftung &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr"/>
+      <c r="G62" s="2" t="inlineStr"/>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr"/>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr"/>
       <c r="B63" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>THE VERSE Ventures</t>
+          <t>Marc O'Polo</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
-        </is>
-      </c>
-      <c r="F63" t="n">
-        <v>6</v>
-      </c>
-      <c r="G63" t="inlineStr"/>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
       <c r="H63" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3405,7 +3375,7 @@
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3416,24 +3386,24 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Lidl Stiftung &amp; Co. KG</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Praktikum Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -3449,7 +3419,7 @@
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
         </is>
       </c>
     </row>
@@ -3465,7 +3435,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Praktikum Marketing (m/w/d)</t>
+          <t>Praktikum Marketing &amp; Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -3482,7 +3452,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -3493,105 +3463,105 @@
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-&amp;-Sales-%28mwd%29-60329/1425985633/</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr"/>
-      <c r="B66" t="n">
-        <v>54</v>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>Nestle Deutschland</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>Praktikum Marketing &amp; Sales (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>Frankfurt am Main, DE, 60329</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr"/>
-      <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>fmcg</t>
-        </is>
-      </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="J66" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K66" t="inlineStr"/>
-      <c r="L66" t="inlineStr">
-        <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-&amp;-Sales-%28mwd%29-60329/1425985633/</t>
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>LIGANOVA GmbH</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum Buying (all genders) – September 2026</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>Mitte, Stuttgart</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K66" s="2" t="inlineStr"/>
+      <c r="L66" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5849630691?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B67" s="2" t="n">
+      <c r="A67" t="inlineStr"/>
+      <c r="B67" t="n">
         <v>52</v>
       </c>
-      <c r="C67" s="2" t="inlineStr">
-        <is>
-          <t>LIGANOVA GmbH</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="inlineStr">
-        <is>
-          <t>Praktikum Buying (all genders) – September 2026</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="inlineStr">
-        <is>
-          <t>Mitte, Stuttgart</t>
-        </is>
-      </c>
-      <c r="F67" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="G67" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="H67" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I67" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="J67" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K67" s="2" t="inlineStr"/>
-      <c r="L67" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5849630691?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Richemont</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Merchandising Assistant Trainee</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>MILAN</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>fashion</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
         </is>
       </c>
     </row>
@@ -3607,7 +3577,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Marketing &amp; Merchandising Assistant Trainee</t>
+          <t>Marketing and Merchandising Assistant Trainee</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3635,7 +3605,7 @@
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing-and-Merchandising-Assistant-Trainee_JR128690</t>
         </is>
       </c>
     </row>
@@ -3646,29 +3616,29 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Wonder Natural GmbH</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Marketing and Merchandising Assistant Trainee</t>
+          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -3679,28 +3649,28 @@
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing-and-Merchandising-Assistant-Trainee_JR128690</t>
+          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr"/>
       <c r="B70" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Wonder Natural GmbH</t>
+          <t>Digitalagenten</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
+          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Charlottenburg, Berlin</t>
         </is>
       </c>
       <c r="F70" t="inlineStr"/>
@@ -3712,7 +3682,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -3723,7 +3693,7 @@
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804948828?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3734,17 +3704,17 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Digitalagenten</t>
+          <t>LIMITD by Wunderproducts GmbH</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Charlottenburg, Berlin</t>
+          <t>Kreuzberg, Berlin</t>
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
@@ -3767,7 +3737,7 @@
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804948828?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3778,21 +3748,25 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>LIMITD by Wunderproducts GmbH</t>
+          <t>PricewaterhouseCoopers GmbH WPG</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Kreuzberg, Berlin</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F72" t="inlineStr"/>
-      <c r="G72" t="inlineStr"/>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
       <c r="H72" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3811,7 +3785,7 @@
       <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3822,12 +3796,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers GmbH WPG</t>
+          <t>SERVICEPLAN Gruppe</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
+          <t>Praktikum Business Development &amp; Sales (Marketing / New Business) (all genders)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3838,7 +3812,7 @@
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -3848,7 +3822,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -3859,7 +3833,7 @@
       <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3870,25 +3844,21 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>SERVICEPLAN Gruppe</t>
+          <t>WirWinzer</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Sales (Marketing / New Business) (all genders)</t>
+          <t>Praktikum Business Development Weinhandel (all genders)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F74" t="inlineStr"/>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3896,7 +3866,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -3907,40 +3877,40 @@
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr"/>
       <c r="B75" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>WirWinzer</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Praktikum Business Development Weinhandel (all genders)</t>
+          <t>Internship - High Jewelry Business Development Assistant</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>PARIS</t>
         </is>
       </c>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
@@ -3951,40 +3921,40 @@
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr"/>
       <c r="B76" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Brand Trust</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Internship - High Jewelry Business Development Assistant</t>
+          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Gleißbühl, Nürnberg</t>
         </is>
       </c>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -3995,7 +3965,7 @@
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
+          <t>https://www.adzuna.de/details/5669847401?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4006,19 +3976,15 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Brand Trust</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>Gleißbühl, Nürnberg</t>
-        </is>
-      </c>
+          <t>Marketing Intern - Trade Marketing</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
@@ -4039,7 +4005,7 @@
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5669847401?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
         </is>
       </c>
     </row>
@@ -4055,7 +4021,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
+          <t>Operational Trade Marketing Intern</t>
         </is>
       </c>
       <c r="E78" t="inlineStr"/>
@@ -4079,7 +4045,7 @@
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
+          <t>https://careers.coty.com/job/Toronto-Operational-Trade-Marketing-Intern-ON-M5H4H2/1397938633/</t>
         </is>
       </c>
     </row>
@@ -4090,15 +4056,19 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Operational Trade Marketing Intern</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr"/>
+          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Benrath, Düsseldorf</t>
+        </is>
+      </c>
       <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
@@ -4108,7 +4078,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -4119,7 +4089,7 @@
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Toronto-Operational-Trade-Marketing-Intern-ON-M5H4H2/1397938633/</t>
+          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4130,17 +4100,17 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Benrath, Düsseldorf</t>
+          <t>Schwabing-Freimann, München</t>
         </is>
       </c>
       <c r="F80" t="inlineStr"/>
@@ -4152,7 +4122,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -4163,7 +4133,7 @@
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4174,24 +4144,24 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
+          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Schwabing-Freimann, München</t>
+          <t>DEU-Bayern-Unterhaching</t>
         </is>
       </c>
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -4207,7 +4177,7 @@
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
         </is>
       </c>
     </row>
@@ -4218,24 +4188,24 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>DEU-Bayern-Unterhaching</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -4251,7 +4221,7 @@
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
+          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4262,17 +4232,17 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F83" t="inlineStr"/>
@@ -4295,7 +4265,7 @@
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
         </is>
       </c>
     </row>
@@ -4311,7 +4281,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -4339,7 +4309,7 @@
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
+          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
         </is>
       </c>
     </row>
@@ -4355,7 +4325,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4383,7 +4353,7 @@
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
+          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
         </is>
       </c>
     </row>
@@ -4394,17 +4364,17 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
         </is>
       </c>
       <c r="F86" t="inlineStr"/>
@@ -4427,28 +4397,28 @@
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
+          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr"/>
       <c r="B87" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>REWE Group</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F87" t="inlineStr"/>
@@ -4471,28 +4441,28 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5712965755?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr"/>
       <c r="B88" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>REWE Group</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F88" t="inlineStr"/>
@@ -4515,7 +4485,7 @@
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5712965755?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4536,7 +4506,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Altstadt-Nord, Köln</t>
         </is>
       </c>
       <c r="F89" t="inlineStr"/>
@@ -4559,28 +4529,28 @@
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr"/>
       <c r="B90" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>Devoteam G Cloud Germany</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Altstadt-Nord, Köln</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
@@ -4603,7 +4573,7 @@
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5811135653?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4614,17 +4584,17 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Devoteam G Cloud Germany</t>
+          <t>freudio</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Wien, Österreich</t>
         </is>
       </c>
       <c r="F91" t="inlineStr"/>
@@ -4636,7 +4606,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -4647,7 +4617,7 @@
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811135653?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/details/5836667156?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4658,17 +4628,17 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>freudio</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Wien, Österreich</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F92" t="inlineStr"/>
@@ -4680,7 +4650,7 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
@@ -4691,7 +4661,7 @@
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/details/5836667156?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4707,7 +4677,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -4735,7 +4705,7 @@
       <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4751,12 +4721,12 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F94" t="inlineStr"/>
@@ -4779,7 +4749,7 @@
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4795,7 +4765,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4823,7 +4793,7 @@
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4834,17 +4804,17 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>sailwithus</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F96" t="inlineStr"/>
@@ -4867,7 +4837,7 @@
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4888,7 +4858,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -4911,56 +4881,12 @@
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr"/>
-      <c r="B98" t="n">
-        <v>45</v>
-      </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>sailwithus</t>
-        </is>
-      </c>
-      <c r="D98" t="inlineStr">
-        <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
-        </is>
-      </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>Altstadt, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F98" t="inlineStr"/>
-      <c r="G98" t="inlineStr"/>
-      <c r="H98" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I98" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J98" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K98" t="inlineStr"/>
-      <c r="L98" t="inlineStr">
-        <is>
           <t>https://www.adzuna.de/details/5804544237?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L98"/>
+  <autoFilter ref="A1:L97"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5052,7 +4978,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C3" t="n">
         <v>91</v>
@@ -5102,7 +5028,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="C5" t="n">
         <v>84</v>
@@ -5127,7 +5053,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C6" t="n">
         <v>84</v>
@@ -5152,7 +5078,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C7" t="n">
         <v>84</v>
@@ -5185,7 +5111,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C8" t="n">
         <v>84</v>
@@ -5210,7 +5136,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C9" t="n">
         <v>84</v>
@@ -5235,7 +5161,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
@@ -5260,7 +5186,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C11" t="n">
         <v>84</v>
@@ -5285,7 +5211,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C12" t="n">
         <v>84</v>
@@ -5310,7 +5236,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C13" t="n">
         <v>84</v>
@@ -5385,7 +5311,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C16" t="n">
         <v>80</v>
@@ -5410,7 +5336,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C17" t="n">
         <v>79</v>
@@ -5485,7 +5411,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C20" t="n">
         <v>78</v>
@@ -5543,7 +5469,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C22" t="n">
         <v>74</v>
@@ -5576,7 +5502,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C23" t="n">
         <v>74</v>
@@ -5601,7 +5527,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C24" t="n">
         <v>74</v>
@@ -5659,7 +5585,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C26" t="n">
         <v>73</v>
@@ -5684,7 +5610,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C27" t="n">
         <v>73</v>
@@ -5709,7 +5635,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C28" t="n">
         <v>72</v>
@@ -5734,7 +5660,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C29" t="n">
         <v>72</v>
@@ -5859,7 +5785,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C34" t="n">
         <v>66</v>
@@ -5884,7 +5810,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C35" t="n">
         <v>65</v>
@@ -5909,7 +5835,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C36" t="n">
         <v>64</v>
@@ -5934,7 +5860,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C37" t="n">
         <v>62</v>
@@ -5959,7 +5885,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C38" t="n">
         <v>62</v>
@@ -5992,7 +5918,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C39" t="n">
         <v>59</v>
@@ -6050,7 +5976,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C41" t="n">
         <v>56</v>
@@ -6075,7 +6001,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C42" t="n">
         <v>55</v>
@@ -6125,7 +6051,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C44" t="n">
         <v>54</v>
@@ -6150,7 +6076,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C45" t="n">
         <v>53</v>
@@ -6175,7 +6101,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C46" t="n">
         <v>53</v>
@@ -6250,7 +6176,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C49" t="n">
         <v>52</v>
@@ -6275,7 +6201,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C50" t="n">
         <v>51</v>
@@ -6300,7 +6226,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C51" t="n">
         <v>49</v>
@@ -6325,7 +6251,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C52" t="n">
         <v>49</v>
@@ -6350,7 +6276,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C53" t="n">
         <v>49</v>
@@ -6375,7 +6301,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C54" t="n">
         <v>49</v>
@@ -6775,7 +6701,7 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C70" t="n">
         <v>46</v>
@@ -6800,7 +6726,7 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C71" t="n">
         <v>45</v>

</xml_diff>

<commit_message>
Lauf 2026-08-24 07:05 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firmen entdeckt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$98</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$89</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$92</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L98"/>
+  <dimension ref="A1:L101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -858,13 +858,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F9" t="n">
         <v>5</v>
       </c>
-      <c r="G9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -904,7 +908,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -1596,27 +1600,21 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Marc O'Polo</t>
+          <t>Miles &amp; More GmbH</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
+          <t>Internship Marketing Strategy &amp; Delivery</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F25" t="n">
-        <v>6</v>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
+          <t>Flughafen, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1635,7 +1633,7 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5828674997?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1646,20 +1644,22 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Miles &amp; More GmbH</t>
+          <t>coty</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Internship Marketing Strategy &amp; Delivery</t>
+          <t>Marketing Intern - Trade Marketing</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Flughafen, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr"/>
+          <t>Darmstadt, Hessen</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>6</v>
+      </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
@@ -1679,31 +1679,33 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5828674997?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Praktikum Marketing (m/w/d)</t>
+          <t>Praktikum im Bereich Marketing für die Marke BE-KIND DACH</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr"/>
+          <t>Unterhaching, München (Kreis)</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>6</v>
+      </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
@@ -1723,28 +1725,28 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899691?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5752932983?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>coty</t>
+          <t>P&amp;G</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Darmstadt, Hessen</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F28" t="n">
@@ -1769,7 +1771,7 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1780,17 +1782,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Tchibo GmbH</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich Marketing für die Marke BE-KIND DACH</t>
+          <t>Praktikum Trade Marketing Tchibo (m/w/d)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Unterhaching, München (Kreis)</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F29" t="n">
@@ -1815,7 +1817,7 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5752932983?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5744245447?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1826,17 +1828,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>P&amp;G</t>
+          <t>Tchibo GmbH</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum Trade Marketing Eduscho (m/w/d)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F30" t="n">
@@ -1861,32 +1863,32 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5773205889?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr"/>
       <c r="B31" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing Tchibo (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Talent Partnerships (m/w/d)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
@@ -1896,7 +1898,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -1907,32 +1909,32 @@
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5744245447?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5851100606?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr"/>
       <c r="B32" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing Eduscho (m/w/d)</t>
+          <t>Praktikum im B2B-Vertrieb &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
@@ -1942,7 +1944,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -1953,7 +1955,7 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5773205889?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5851898375?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1964,21 +1966,21 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>markenbaumarkt24</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Feuersbach, Siegen</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
@@ -1999,133 +2001,121 @@
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="n">
-        <v>72</v>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>Exclusive Associates</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>Praktikum Business Development &amp; Talent Partnerships (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>Düsseltal, Düsseldorf</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="G34" s="2" t="inlineStr"/>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
-      </c>
-      <c r="J34" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K34" s="2" t="inlineStr"/>
-      <c r="L34" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5851100606?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="A34" t="inlineStr"/>
+      <c r="B34" t="n">
+        <v>70</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>PARSA Haar- und Modeartikel GmbH</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="n">
-        <v>72</v>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>Exclusive Associates</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>Praktikum im B2B-Vertrieb &amp; Business Development (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>Düsseltal, Düsseldorf</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="G35" s="2" t="inlineStr"/>
-      <c r="H35" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I35" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
-      </c>
-      <c r="J35" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K35" s="2" t="inlineStr"/>
-      <c r="L35" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5851898375?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="A35" t="inlineStr"/>
+      <c r="B35" t="n">
+        <v>69</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Lidl Stiftung</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food in Neckarsulm</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>6</v>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5813494719?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>markenbaumarkt24</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Feuersbach, Siegen</t>
-        </is>
-      </c>
-      <c r="F36" t="n">
-        <v>2</v>
-      </c>
+          <t>Hamburg, Deutschland</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
@@ -2145,23 +2135,23 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>PARSA Haar- und Modeartikel GmbH</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2178,7 +2168,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -2189,28 +2179,28 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
+          <t>https://www.adzuna.de/land/ad/5849209692?se=qJaID2Kc8RGlrvMe-VN8Yg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B8E6A551D4E75B7916A5994DC13A8DA3451895D</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Lidl Stiftung</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food in Neckarsulm</t>
+          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -2235,31 +2225,33 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813494719?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr"/>
       <c r="B39" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr"/>
+          <t>Köln, Nordrhein-Westfalen</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>6</v>
+      </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
@@ -2279,32 +2271,38 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
+          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr"/>
       <c r="B40" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
+          <t>Köln, Nordrhein-Westfalen</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>6</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H40" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2312,7 +2310,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -2323,7 +2321,7 @@
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5849209692?se=qJaID2Kc8RGlrvMe-VN8Yg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B8E6A551D4E75B7916A5994DC13A8DA3451895D</t>
+          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2334,23 +2332,27 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>Bosch Thermotechnik GmbH</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
+          <t>Praktikum im internationalen Brand Management</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Wernau (Neckar), Esslingen (Kreis)</t>
         </is>
       </c>
       <c r="F41" t="n">
         <v>6</v>
       </c>
-      <c r="G41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="H41" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2369,7 +2371,7 @@
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5799981240?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2380,23 +2382,27 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>L’ORÉAL</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
+          <t>PRAKTIKUM (M/W/D) Product Marketing - Start ab August/September/Oktober für 6 Monate</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Nordrhein-Westfalen, Deutschland</t>
         </is>
       </c>
       <c r="F42" t="n">
         <v>6</v>
       </c>
-      <c r="G42" t="inlineStr"/>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H42" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2415,7 +2421,7 @@
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5754061318?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2426,17 +2432,17 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F43" t="n">
@@ -2465,38 +2471,34 @@
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr"/>
       <c r="B44" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Bosch Thermotechnik GmbH</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Praktikum im internationalen Brand Management</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Wernau (Neckar), Esslingen (Kreis)</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F44" t="n">
         <v>6</v>
       </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2515,38 +2517,34 @@
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5799981240?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr"/>
       <c r="B45" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>L’ORÉAL</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>PRAKTIKUM (M/W/D) Product Marketing - Start ab August/September/Oktober für 6 Monate</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Nordrhein-Westfalen, Deutschland</t>
+          <t>Altstadt, Düsseldorf</t>
         </is>
       </c>
       <c r="F45" t="n">
         <v>6</v>
       </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2565,46 +2563,40 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5754061318?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr"/>
       <c r="B46" t="n">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>Internship in Trade Marketing</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
-        </is>
-      </c>
-      <c r="F46" t="n">
-        <v>6</v>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>DEU-Nordrhein-Westfalen-Köln</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -2615,34 +2607,36 @@
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr"/>
       <c r="B47" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F47" t="n">
-        <v>6</v>
-      </c>
-      <c r="G47" t="inlineStr"/>
+          <t>Köln, Nordrhein-Westfalen</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H47" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2661,33 +2655,31 @@
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5822943276?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=580C236799B96DFD395A1EC1CBBF7474C7F58435</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr"/>
       <c r="B48" t="n">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>Calypso Ventures GmbH</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Altstadt, Düsseldorf</t>
-        </is>
-      </c>
-      <c r="F48" t="n">
-        <v>6</v>
-      </c>
+          <t>Berlin, Deutschland</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
@@ -2707,40 +2699,40 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr"/>
       <c r="B49" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Internship in Trade Marketing</t>
+          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>DEU-Nordrhein-Westfalen-Köln</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -2751,36 +2743,32 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
+          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr"/>
       <c r="B50" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2788,7 +2776,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -2799,28 +2787,28 @@
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5822943276?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=580C236799B96DFD395A1EC1CBBF7474C7F58435</t>
+          <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr"/>
       <c r="B51" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Calypso Ventures GmbH</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
+          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
@@ -2832,7 +2820,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -2843,28 +2831,28 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5848400955?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=4E59A334AC360616EAEAAC474F72A07451A7C624</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr"/>
       <c r="B52" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F52" t="inlineStr"/>
@@ -2876,7 +2864,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -2887,7 +2875,7 @@
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5848409009?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5C62DDCDA5E03F77D6089CD03CFA1D966DF15C96</t>
         </is>
       </c>
     </row>
@@ -2898,12 +2886,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2931,40 +2919,40 @@
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848400955?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=4E59A334AC360616EAEAAC474F72A07451A7C624</t>
+          <t>https://www.adzuna.de/land/ad/5848363308?se=OLEhDWKc8RGNPOjEPgN71g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=60107C204BD9BC811A91BB2CBB46D624738C18B4</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr"/>
       <c r="B54" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -2975,28 +2963,28 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848409009?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5C62DDCDA5E03F77D6089CD03CFA1D966DF15C96</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr"/>
       <c r="B55" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
@@ -3008,7 +2996,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -3019,35 +3007,35 @@
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848363308?se=OLEhDWKc8RGNPOjEPgN71g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=60107C204BD9BC811A91BB2CBB46D624738C18B4</t>
+          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr"/>
       <c r="B56" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -3063,32 +3051,36 @@
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
+          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr"/>
       <c r="B57" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>Sayano Deutschland GmbH</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Mitte, Stuttgart</t>
         </is>
       </c>
       <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H57" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3107,31 +3099,33 @@
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5816572451?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr"/>
       <c r="B58" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>THE VERSE Ventures</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr"/>
+          <t>Berlin, Deutschland</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>6</v>
+      </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
         <is>
@@ -3151,36 +3145,32 @@
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr"/>
       <c r="B59" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Sayano Deutschland GmbH</t>
+          <t>Abrio</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Praktikum Amazon PPC &amp; Performance Marketing im E-Commerce Start-up (m/w/d)</t>
+          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3199,33 +3189,31 @@
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816572451?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr"/>
       <c r="B60" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>THE VERSE Ventures</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
-        </is>
-      </c>
-      <c r="F60" t="n">
-        <v>6</v>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr">
         <is>
@@ -3245,7 +3233,7 @@
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
         </is>
       </c>
     </row>
@@ -3256,17 +3244,17 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Abrio</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F61" t="inlineStr"/>
@@ -3278,7 +3266,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -3289,7 +3277,7 @@
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
         </is>
       </c>
     </row>
@@ -3300,12 +3288,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Lidl Stiftung &amp; Co. KG</t>
+          <t>Marc O'Polo</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -3314,7 +3302,11 @@
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
       <c r="H62" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3333,55 +3325,51 @@
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824556266?se=jJdvn2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=32CAAF75B08EB0A6F6B64E1794E8A158344FF4C9</t>
+          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B63" s="2" t="n">
+      <c r="A63" t="inlineStr"/>
+      <c r="B63" t="n">
         <v>54</v>
       </c>
-      <c r="C63" s="2" t="inlineStr">
-        <is>
-          <t>Lidl Stiftung &amp; Co. KG</t>
-        </is>
-      </c>
-      <c r="D63" s="2" t="inlineStr">
-        <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
-        </is>
-      </c>
-      <c r="E63" s="2" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F63" s="2" t="inlineStr"/>
-      <c r="G63" s="2" t="inlineStr"/>
-      <c r="H63" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I63" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
-      </c>
-      <c r="J63" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K63" s="2" t="inlineStr"/>
-      <c r="L63" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Nespresso Deutschland GmbH</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Praktikum Marketing (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5802899691?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3754,46 +3742,50 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr"/>
-      <c r="B72" t="n">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="n">
         <v>51</v>
       </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>LIMITD by Wunderproducts GmbH</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>Kreuzberg, Berlin</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr"/>
-      <c r="G72" t="inlineStr"/>
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J72" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K72" t="inlineStr"/>
-      <c r="L72" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>HardyTec Industries UG haftungsbeschränkt</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum Marketing &amp; Business Development</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>Büderich, Meerbusch</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr"/>
+      <c r="G72" s="2" t="inlineStr"/>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K72" s="2" t="inlineStr"/>
+      <c r="L72" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5848139968?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3804,25 +3796,21 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers GmbH WPG</t>
+          <t>LIMITD by Wunderproducts GmbH</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Kreuzberg, Berlin</t>
         </is>
       </c>
       <c r="F73" t="inlineStr"/>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
+      <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3841,7 +3829,7 @@
       <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3852,12 +3840,12 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>SERVICEPLAN Gruppe</t>
+          <t>PricewaterhouseCoopers GmbH WPG</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Sales (Marketing / New Business) (all genders)</t>
+          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3868,7 +3856,7 @@
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -3878,7 +3866,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -3889,7 +3877,7 @@
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3900,21 +3888,25 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>WirWinzer</t>
+          <t>SERVICEPLAN Gruppe</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Praktikum Business Development Weinhandel (all genders)</t>
+          <t>Praktikum Business Development &amp; Sales (Marketing / New Business) (all genders)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F75" t="inlineStr"/>
-      <c r="G75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H75" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3922,7 +3914,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
@@ -3933,40 +3925,40 @@
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr"/>
       <c r="B76" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>WirWinzer</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Internship - High Jewelry Business Development Assistant</t>
+          <t>Praktikum Business Development Weinhandel (all genders)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -3977,40 +3969,40 @@
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
+          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr"/>
       <c r="B77" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Brand Trust</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
+          <t>Internship - High Jewelry Business Development Assistant</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Gleißbühl, Nürnberg</t>
+          <t>PARIS</t>
         </is>
       </c>
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -4021,7 +4013,7 @@
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5669847401?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
         </is>
       </c>
     </row>
@@ -4032,15 +4024,19 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Brand Trust</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
-        </is>
-      </c>
-      <c r="E78" t="inlineStr"/>
+          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Gleißbühl, Nürnberg</t>
+        </is>
+      </c>
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr">
@@ -4061,7 +4057,7 @@
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
+          <t>https://www.adzuna.de/details/5669847401?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4077,7 +4073,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Operational Trade Marketing Intern</t>
+          <t>Marketing Intern - Trade Marketing</t>
         </is>
       </c>
       <c r="E79" t="inlineStr"/>
@@ -4101,7 +4097,7 @@
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Toronto-Operational-Trade-Marketing-Intern-ON-M5H4H2/1397938633/</t>
+          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
         </is>
       </c>
     </row>
@@ -4112,19 +4108,15 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>Benrath, Düsseldorf</t>
-        </is>
-      </c>
+          <t>Operational Trade Marketing Intern</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
@@ -4134,7 +4126,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -4145,51 +4137,55 @@
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://careers.coty.com/job/Toronto-Operational-Trade-Marketing-Intern-ON-M5H4H2/1397938633/</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" t="inlineStr"/>
-      <c r="B81" t="n">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="n">
         <v>49</v>
       </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>Honest Catch</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>Schwabing-Freimann, München</t>
-        </is>
-      </c>
-      <c r="F81" t="inlineStr"/>
-      <c r="G81" t="inlineStr"/>
-      <c r="H81" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I81" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J81" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K81" t="inlineStr"/>
-      <c r="L81" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>Genuine Parts Company</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum Category Management (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>Münster, Nordrhein-Westfalen</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr"/>
+      <c r="G81" s="2" t="inlineStr"/>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I81" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K81" s="2" t="inlineStr"/>
+      <c r="L81" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5853760166?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4200,29 +4196,29 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
+          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>DEU-Bayern-Unterhaching</t>
+          <t>Benrath, Düsseldorf</t>
         </is>
       </c>
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -4233,7 +4229,7 @@
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
+          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4244,17 +4240,17 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>Schwabing-Freimann, München</t>
         </is>
       </c>
       <c r="F83" t="inlineStr"/>
@@ -4277,7 +4273,7 @@
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4288,24 +4284,24 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
+          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>DEU-Bayern-Unterhaching</t>
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -4321,7 +4317,7 @@
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
         </is>
       </c>
     </row>
@@ -4332,17 +4328,17 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
@@ -4365,7 +4361,7 @@
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
+          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4381,7 +4377,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -4409,7 +4405,7 @@
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
+          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
         </is>
       </c>
     </row>
@@ -4420,17 +4416,17 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F87" t="inlineStr"/>
@@ -4453,28 +4449,28 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr"/>
       <c r="B88" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>REWE Group</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F88" t="inlineStr"/>
@@ -4497,28 +4493,28 @@
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5712965755?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr"/>
       <c r="B89" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
         </is>
       </c>
       <c r="F89" t="inlineStr"/>
@@ -4541,72 +4537,76 @@
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" t="inlineStr"/>
-      <c r="B90" t="n">
-        <v>46</v>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>SUPA - Sport Und Party App</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr">
-        <is>
-          <t>Business Development Praktikum</t>
-        </is>
-      </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>Altstadt-Nord, Köln</t>
-        </is>
-      </c>
-      <c r="F90" t="inlineStr"/>
-      <c r="G90" t="inlineStr"/>
-      <c r="H90" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I90" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J90" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K90" t="inlineStr"/>
-      <c r="L90" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>RAG</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>Gornhofen, Ravensburg</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr"/>
+      <c r="G90" s="2" t="inlineStr"/>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K90" s="2" t="inlineStr"/>
+      <c r="L90" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr"/>
       <c r="B91" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Devoteam G Cloud Germany</t>
+          <t>REWE Group</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F91" t="inlineStr"/>
@@ -4629,28 +4629,28 @@
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811135653?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5712965755?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr"/>
       <c r="B92" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>freudio</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Wien, Österreich</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F92" t="inlineStr"/>
@@ -4662,7 +4662,7 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
@@ -4673,28 +4673,28 @@
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/details/5836667156?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr"/>
       <c r="B93" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt-Nord, Köln</t>
         </is>
       </c>
       <c r="F93" t="inlineStr"/>
@@ -4717,7 +4717,7 @@
       <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4728,12 +4728,12 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>Devoteam G Cloud Germany</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -4761,7 +4761,7 @@
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5811135653?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4772,17 +4772,17 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>freudio</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Wien, Österreich</t>
         </is>
       </c>
       <c r="F95" t="inlineStr"/>
@@ -4794,7 +4794,7 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -4805,7 +4805,7 @@
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/details/5836667156?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4821,12 +4821,12 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F96" t="inlineStr"/>
@@ -4849,7 +4849,7 @@
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4860,12 +4860,12 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>sailwithus</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4893,7 +4893,7 @@
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4904,12 +4904,12 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>sailwithus</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -4937,12 +4937,144 @@
       <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr"/>
+      <c r="B99" t="n">
+        <v>45</v>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>prepmymeal GmbH</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr"/>
+      <c r="G99" t="inlineStr"/>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr"/>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr"/>
+      <c r="B100" t="n">
+        <v>45</v>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>sailwithus</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr"/>
+      <c r="G100" t="inlineStr"/>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr"/>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr"/>
+      <c r="B101" t="n">
+        <v>45</v>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>sailwithus</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr"/>
+      <c r="G101" t="inlineStr"/>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr"/>
+      <c r="L101" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5804544237?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L98"/>
+  <autoFilter ref="A1:L101"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4953,7 +5085,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G89"/>
+  <dimension ref="A1:G92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -5084,7 +5216,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="C5" t="n">
         <v>84</v>
@@ -5109,7 +5241,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C6" t="n">
         <v>84</v>
@@ -5134,7 +5266,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C7" t="n">
         <v>84</v>
@@ -5167,7 +5299,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C8" t="n">
         <v>84</v>
@@ -5192,7 +5324,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C9" t="n">
         <v>84</v>
@@ -5217,7 +5349,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
@@ -5242,7 +5374,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C11" t="n">
         <v>84</v>
@@ -5267,7 +5399,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C12" t="n">
         <v>84</v>
@@ -5292,7 +5424,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C13" t="n">
         <v>84</v>
@@ -5317,7 +5449,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C14" t="n">
         <v>84</v>
@@ -5367,7 +5499,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C16" t="n">
         <v>84</v>
@@ -5377,8 +5509,16 @@
           <t>Praktikum Product Marketing (x/f/m)</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>greenhouse</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr">
         <is>
           <t>2026-08-23</t>
@@ -5392,7 +5532,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C17" t="n">
         <v>80</v>
@@ -5417,7 +5557,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C18" t="n">
         <v>79</v>
@@ -5492,7 +5632,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C21" t="n">
         <v>78</v>
@@ -5525,7 +5665,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C22" t="n">
         <v>78</v>
@@ -5550,7 +5690,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C23" t="n">
         <v>78</v>
@@ -5608,7 +5748,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="C25" t="n">
         <v>74</v>
@@ -5633,7 +5773,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C26" t="n">
         <v>74</v>
@@ -5691,7 +5831,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C28" t="n">
         <v>73</v>
@@ -5741,7 +5881,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="C30" t="n">
         <v>72</v>
@@ -5766,7 +5906,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C31" t="n">
         <v>72</v>
@@ -5891,7 +6031,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C36" t="n">
         <v>66</v>
@@ -5916,7 +6056,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C37" t="n">
         <v>65</v>
@@ -5941,7 +6081,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C38" t="n">
         <v>64</v>
@@ -5966,7 +6106,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C39" t="n">
         <v>62</v>
@@ -5991,7 +6131,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C40" t="n">
         <v>62</v>
@@ -6024,7 +6164,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C41" t="n">
         <v>59</v>
@@ -6049,7 +6189,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C42" t="n">
         <v>57</v>
@@ -6082,7 +6222,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C43" t="n">
         <v>56</v>
@@ -6107,7 +6247,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C44" t="n">
         <v>55</v>
@@ -6182,7 +6322,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C47" t="n">
         <v>53</v>
@@ -6207,7 +6347,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C48" t="n">
         <v>53</v>
@@ -6257,7 +6397,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C50" t="n">
         <v>52</v>
@@ -6282,7 +6422,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C51" t="n">
         <v>52</v>
@@ -6307,7 +6447,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C52" t="n">
         <v>51</v>
@@ -6328,43 +6468,43 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Brand Trust</t>
+          <t>HardyTec Industries UG haftungsbeschränkt</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="C53" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
+          <t>Praktikum Marketing &amp; Business Development</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>Brand Trust</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C54" t="n">
         <v>49</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr"/>
@@ -6378,18 +6518,18 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C55" t="n">
         <v>49</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E55" t="inlineStr"/>
@@ -6403,18 +6543,18 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C56" t="n">
         <v>49</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr"/>
@@ -6428,18 +6568,18 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>REWE Group</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="C57" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E57" t="inlineStr"/>
@@ -6453,68 +6593,68 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Pflegia</t>
+          <t>Genuine Parts Company</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C58" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Praktikum Category Management (m/w/d)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Werkia</t>
+          <t>RAG</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C59" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d) - Datenanalyse &amp; Automatisierung</t>
+          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>paero</t>
+          <t>REWE Group</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="C60" t="n">
         <v>48</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E60" t="inlineStr"/>
@@ -6528,18 +6668,18 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Vivanta Gmbh</t>
+          <t>Pflegia</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C61" t="n">
         <v>48</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E61" t="inlineStr"/>
@@ -6553,7 +6693,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Vitolus</t>
+          <t>Werkia</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -6564,7 +6704,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/d) - Datenanalyse &amp; Automatisierung</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
@@ -6578,7 +6718,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>GrantLift GmbH</t>
+          <t>paero</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -6589,7 +6729,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
@@ -6603,7 +6743,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Otto Group one.O GmbH</t>
+          <t>Vivanta Gmbh</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -6614,7 +6754,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Praktikum im Knowledge Management - Corporate Strategy (w/m/d)</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
@@ -6628,18 +6768,18 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>AUTO1 Global Services SE &amp; Co. KG</t>
+          <t>Vitolus</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C65" t="n">
         <v>48</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (d/m/w)</t>
+          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
@@ -6653,18 +6793,18 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>SHAVENT - ARA Sustainable Products</t>
+          <t>GrantLift GmbH</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C66" t="n">
         <v>48</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Praktikum Business Development in nachhaltigem Start-Up (w/m/d) Remote in DE</t>
+          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
@@ -6678,18 +6818,18 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CTG Consulting</t>
+          <t>Otto Group one.O GmbH</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C67" t="n">
         <v>48</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Praktikum Sales/Business Development // Hamburg oder Berlin</t>
+          <t>Praktikum im Knowledge Management - Corporate Strategy (w/m/d)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
@@ -6703,7 +6843,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Dronesperhour</t>
+          <t>AUTO1 Global Services SE &amp; Co. KG</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -6714,7 +6854,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development eines Startups (m/w/d)</t>
+          <t>Praktikum Business Development (d/m/w)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr"/>
@@ -6728,7 +6868,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>SINN Power</t>
+          <t>SHAVENT - ARA Sustainable Products</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -6739,7 +6879,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Praktikum im AI Business Development (m/w/d)</t>
+          <t>Praktikum Business Development in nachhaltigem Start-Up (w/m/d) Remote in DE</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
@@ -6753,7 +6893,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>innpuls</t>
+          <t>CTG Consulting</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -6764,7 +6904,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Praktikum Sales/Business Development // Hamburg oder Berlin</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
@@ -6778,7 +6918,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Amolina</t>
+          <t>Dronesperhour</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -6789,7 +6929,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
+          <t>Praktikum im Business Development eines Startups (m/w/d)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr"/>
@@ -6803,18 +6943,18 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>SINN Power</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>44</v>
+        <v>1</v>
       </c>
       <c r="C72" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Praktikum im AI Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr"/>
@@ -6828,43 +6968,43 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>freudio</t>
+          <t>innpuls</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="C73" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>STARTPLATZ Gruppe</t>
+          <t>Amolina</t>
         </is>
       </c>
       <c r="B74" t="n">
         <v>1</v>
       </c>
       <c r="C74" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Sales (m/w/d) – STARTPLATZ</t>
+          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr"/>
@@ -6878,18 +7018,18 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>spring.gate business consulting UG</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>1</v>
+        <v>46</v>
       </c>
       <c r="C75" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development &amp; B2B Akquise (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E75" t="inlineStr"/>
@@ -6903,43 +7043,43 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>specter automation</t>
+          <t>freudio</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="C76" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Praktikum (M/W/D) im Business Development</t>
+          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Closd Kunststoffprodukte GmbH</t>
+          <t>STARTPLATZ Gruppe</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C77" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Praktikum beim E-Commerce Startup Closd als Founders Associate (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Sales (m/w/d) – STARTPLATZ</t>
         </is>
       </c>
       <c r="E77" t="inlineStr"/>
@@ -6953,18 +7093,18 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Bosch Rexroth AG</t>
+          <t>spring.gate business consulting UG</t>
         </is>
       </c>
       <c r="B78" t="n">
         <v>1</v>
       </c>
       <c r="C78" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Praktikum Business Development – Software Defined Business</t>
+          <t>Praktikum im Business Development &amp; B2B Akquise (m/w/d)</t>
         </is>
       </c>
       <c r="E78" t="inlineStr"/>
@@ -6978,18 +7118,18 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Weenect</t>
+          <t>specter automation</t>
         </is>
       </c>
       <c r="B79" t="n">
         <v>1</v>
       </c>
       <c r="C79" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d) – Markt DACH – Standort Brüssel</t>
+          <t>Praktikum (M/W/D) im Business Development</t>
         </is>
       </c>
       <c r="E79" t="inlineStr"/>
@@ -7003,18 +7143,18 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Lidl Dienstleistung GmbH &amp; Co. KG</t>
+          <t>Closd Kunststoffprodukte GmbH</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C80" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Praktikum beim E-Commerce Startup Closd als Founders Associate (m/w/d)</t>
         </is>
       </c>
       <c r="E80" t="inlineStr"/>
@@ -7028,18 +7168,18 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Drägerwerk AG &amp; Co. KGaA</t>
+          <t>Bosch Rexroth AG</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C81" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Praktikum New Business Development</t>
+          <t>Praktikum Business Development – Software Defined Business</t>
         </is>
       </c>
       <c r="E81" t="inlineStr"/>
@@ -7053,18 +7193,18 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Arteus Energy</t>
+          <t>Weenect</t>
         </is>
       </c>
       <c r="B82" t="n">
         <v>1</v>
       </c>
       <c r="C82" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Praktikum Business Development und Marketing Photovoltaik</t>
+          <t>Praktikum Business Development (m/w/d) – Markt DACH – Standort Brüssel</t>
         </is>
       </c>
       <c r="E82" t="inlineStr"/>
@@ -7078,18 +7218,18 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>aramido</t>
+          <t>Lidl Dienstleistung GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="B83" t="n">
         <v>1</v>
       </c>
       <c r="C83" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/x)</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E83" t="inlineStr"/>
@@ -7103,18 +7243,18 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>pacemaker.ai by thyssenkrupp</t>
+          <t>Drägerwerk AG &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C84" t="n">
         <v>28</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Praktikum New Business Development</t>
         </is>
       </c>
       <c r="E84" t="inlineStr"/>
@@ -7128,7 +7268,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Molly Suh GmbH</t>
+          <t>Arteus Energy</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -7139,7 +7279,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; B2B Sales (m/w/d)</t>
+          <t>Praktikum Business Development und Marketing Photovoltaik</t>
         </is>
       </c>
       <c r="E85" t="inlineStr"/>
@@ -7153,7 +7293,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>homewise</t>
+          <t>aramido</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -7164,7 +7304,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development &amp; Strategie (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/x)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr"/>
@@ -7178,7 +7318,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ClipMyHorse.TV</t>
+          <t>pacemaker.ai by thyssenkrupp</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -7189,7 +7329,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Praktikum HR &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr"/>
@@ -7203,7 +7343,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>AUMOVIO</t>
+          <t>Molly Suh GmbH</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -7214,7 +7354,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Praktikum - Administration/Assistenz &amp; Business Development</t>
+          <t>Praktikum Business Development &amp; B2B Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
@@ -7228,7 +7368,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>TRUMPF Group</t>
+          <t>homewise</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -7239,7 +7379,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich Business Development für Smart Factory Solutions (WS26/27)</t>
+          <t>Praktikum im Business Development &amp; Strategie (m/w/d)</t>
         </is>
       </c>
       <c r="E89" t="inlineStr"/>
@@ -7250,8 +7390,83 @@
         </is>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>ClipMyHorse.TV</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>1</v>
+      </c>
+      <c r="C90" t="n">
+        <v>28</v>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Praktikum HR &amp; Business Development (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>AUMOVIO</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>1</v>
+      </c>
+      <c r="C91" t="n">
+        <v>28</v>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Praktikum - Administration/Assistenz &amp; Business Development</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr"/>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>TRUMPF Group</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>1</v>
+      </c>
+      <c r="C92" t="n">
+        <v>28</v>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Praktikum im Bereich Business Development für Smart Factory Solutions (WS26/27)</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G89"/>
+  <autoFilter ref="A1:G92"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Lauf 2026-08-28 18:23 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firmen entdeckt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$113</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$97</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$116</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$99</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L113"/>
+  <dimension ref="A1:L116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1146,23 +1146,27 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich Marketing für die Marke BE-KIND DACH</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F15" t="n">
         <v>6</v>
       </c>
-      <c r="G15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1181,7 +1185,7 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5753617280?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1197,12 +1201,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Praktikum Brand Management (m/w/d)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -1210,7 +1214,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1231,38 +1235,32 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802899675?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d)</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F17" t="n">
-        <v>6</v>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1270,7 +1268,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1281,7 +1279,7 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899675?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5843630960?se=znNqlDyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=875B574D03DFD36B16B3A3ABE0AA46F858215182</t>
         </is>
       </c>
     </row>
@@ -1297,7 +1295,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1325,7 +1323,7 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5843630960?se=znNqlDyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=875B574D03DFD36B16B3A3ABE0AA46F858215182</t>
+          <t>https://www.adzuna.de/land/ad/5843628966?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=3DAF9A0A7032477BEFBE4DD229577F81F1D32CF0</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1339,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1369,7 +1367,7 @@
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5843628966?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=3DAF9A0A7032477BEFBE4DD229577F81F1D32CF0</t>
+          <t>https://www.adzuna.de/land/ad/5843628932?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=65C46D18FCDB11FD2E933BD305E494E07D043D72</t>
         </is>
       </c>
     </row>
@@ -1380,21 +1378,27 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>HUGO BOSS</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Internship Buying &amp; Planning - Global Merchandising (m/f/d)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
+          <t>Metzingen, Reutlingen (Kreis)</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>6</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H20" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1402,7 +1406,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1413,61 +1417,51 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5843628932?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=65C46D18FCDB11FD2E933BD305E494E07D043D72</t>
+          <t>https://www.adzuna.de/details/5856159470?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="n">
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" t="n">
         <v>74</v>
       </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>HUGO BOSS</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>Internship Buying &amp; Planning - Global Merchandising (m/f/d)</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>Metzingen, Reutlingen (Kreis)</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K21" s="2" t="inlineStr"/>
-      <c r="L21" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5856159470?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Miles &amp; More GmbH</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Internship Marketing Strategy &amp; Delivery</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Flughafen, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5828674997?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1478,20 +1472,22 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Miles &amp; More GmbH</t>
+          <t>coty</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Internship Marketing Strategy &amp; Delivery</t>
+          <t>Marketing Intern - Trade Marketing</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Flughafen, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr"/>
+          <t>Darmstadt, Hessen</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>6</v>
+      </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
@@ -1511,28 +1507,28 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5828674997?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>coty</t>
+          <t>Tchibo GmbH</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
+          <t>Praktikum Trade Marketing Eduscho (m/w/d)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Darmstadt, Hessen</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F23" t="n">
@@ -1557,32 +1553,32 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5773205889?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing Eduscho (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Talent Partnerships (m/w/d)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
@@ -1592,7 +1588,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -1603,7 +1599,7 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5773205889?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5851100606?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1619,7 +1615,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Talent Partnerships (m/w/d)</t>
+          <t>Praktikum im B2B-Vertrieb &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1649,7 +1645,7 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5851100606?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5851898375?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1660,21 +1656,21 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>markenbaumarkt24</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Praktikum im B2B-Vertrieb &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Feuersbach, Siegen</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
@@ -1684,7 +1680,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -1695,33 +1691,31 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5851898375?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>markenbaumarkt24</t>
+          <t>PARSA Haar- und Modeartikel GmbH</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
+          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Feuersbach, Siegen</t>
-        </is>
-      </c>
-      <c r="F27" t="n">
-        <v>2</v>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
@@ -1730,7 +1724,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -1741,28 +1735,28 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>PARSA Haar- und Modeartikel GmbH</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
+          <t>Praktikum Product Marketing (x/f/m)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F28" t="inlineStr"/>
@@ -1774,7 +1768,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -1785,99 +1779,101 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
+          <t>https://www.adzuna.de/details/5842051017?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr"/>
-      <c r="B29" t="n">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
         <v>69</v>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Doctolib</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Praktikum Product Marketing (x/f/m)</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Berlin, Berlin, Germany</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5842051017?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Groß- &amp; Einzelhandel Karriere</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr"/>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/land/ad/5848300231?se=1ucgSzui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=BF61BDCA3F28DD382163849647345A68CC617C45</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="n">
+      <c r="A30" t="inlineStr"/>
+      <c r="B30" t="n">
         <v>69</v>
       </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>Groß- &amp; Einzelhandel Karriere</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Lidl Stiftung</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food in Neckarsulm</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr"/>
-      <c r="G30" s="2" t="inlineStr"/>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I30" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-      <c r="J30" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K30" s="2" t="inlineStr"/>
-      <c r="L30" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5848300231?se=1ucgSzui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=BF61BDCA3F28DD382163849647345A68CC617C45</t>
+      <c r="F30" t="n">
+        <v>6</v>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5813494719?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1888,22 +1884,20 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Lidl Stiftung</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food in Neckarsulm</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F31" t="n">
-        <v>6</v>
-      </c>
+          <t>Hamburg, Deutschland</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
@@ -1923,7 +1917,7 @@
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813494719?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
         </is>
       </c>
     </row>
@@ -1944,7 +1938,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
@@ -1956,7 +1950,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -1967,51 +1961,55 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
+          <t>https://www.adzuna.de/land/ad/5849209692?se=qJaID2Kc8RGlrvMe-VN8Yg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B8E6A551D4E75B7916A5994DC13A8DA3451895D</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr"/>
-      <c r="B33" t="n">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="n">
         <v>69</v>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5849209692?se=qJaID2Kc8RGlrvMe-VN8Yg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B8E6A551D4E75B7916A5994DC13A8DA3451895D</t>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Hamburg, Deutschland</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr"/>
+      <c r="G33" s="2" t="inlineStr"/>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr"/>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/land/ad/5859954968?se=avT3yguj8RGEeLI7Dotn4Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FEC8C1664463BB6D76B4F51C80D7BE9A67B3E95</t>
         </is>
       </c>
     </row>
@@ -2526,50 +2524,46 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="n">
+      <c r="A45" t="inlineStr"/>
+      <c r="B45" t="n">
         <v>62</v>
       </c>
-      <c r="C45" s="2" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>FC Viktoria 1889 Berlin Frauen-Fußball GmbH</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>PRAKTIKUM // Business Development - In 3 Minuten erfolgreich bewerben</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="F45" s="2" t="n">
+      <c r="F45" t="n">
         <v>3</v>
       </c>
-      <c r="G45" s="2" t="inlineStr"/>
-      <c r="H45" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I45" s="2" t="inlineStr">
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="J45" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K45" s="2" t="inlineStr"/>
-      <c r="L45" s="2" t="inlineStr">
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr">
         <is>
           <t>https://www.adzuna.de/land/ad/5856283303?se=PMRjVxmh8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0E222C24DC5860DC4AEB24D8BB5E4CB04740A32C</t>
         </is>
@@ -3316,46 +3310,50 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr"/>
-      <c r="B62" t="n">
-        <v>56</v>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Upsters Energy GmbH</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Wonder Natural GmbH</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Köln, Nordrhein-Westfalen</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr"/>
+      <c r="G62" s="2" t="inlineStr"/>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr"/>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3376,7 +3374,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F63" t="inlineStr"/>
@@ -3399,33 +3397,31 @@
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr"/>
       <c r="B64" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>THE VERSE Ventures</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
-        </is>
-      </c>
-      <c r="F64" t="n">
-        <v>6</v>
-      </c>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
@@ -3445,31 +3441,33 @@
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr"/>
       <c r="B65" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Abrio</t>
+          <t>THE VERSE Ventures</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr"/>
+          <t>Berlin, Deutschland</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>6</v>
+      </c>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
@@ -3489,99 +3487,99 @@
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr"/>
+      <c r="B66" t="n">
+        <v>54</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Abrio</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="2" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
         <is>
           <t>NEU</t>
         </is>
       </c>
-      <c r="B66" s="2" t="n">
+      <c r="B67" s="2" t="n">
         <v>54</v>
       </c>
-      <c r="C66" s="2" t="inlineStr">
+      <c r="C67" s="2" t="inlineStr">
         <is>
           <t>Groß- &amp; Einzelhandel Karriere</t>
         </is>
       </c>
-      <c r="D66" s="2" t="inlineStr">
+      <c r="D67" s="2" t="inlineStr">
         <is>
           <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
         </is>
       </c>
-      <c r="E66" s="2" t="inlineStr">
+      <c r="E67" s="2" t="inlineStr">
         <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="F66" s="2" t="inlineStr"/>
-      <c r="G66" s="2" t="inlineStr"/>
-      <c r="H66" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I66" s="2" t="inlineStr">
+      <c r="F67" s="2" t="inlineStr"/>
+      <c r="G67" s="2" t="inlineStr"/>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="J66" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K66" s="2" t="inlineStr"/>
-      <c r="L66" s="2" t="inlineStr">
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K67" s="2" t="inlineStr"/>
+      <c r="L67" s="2" t="inlineStr">
         <is>
           <t>https://www.adzuna.de/land/ad/5848296401?se=lphMSjui8RGhLffPfv7Txw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CDA6039E4CB2826923EB7E2E7ECB163DB4CFE919</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr"/>
-      <c r="B67" t="n">
-        <v>54</v>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>Lidl Stiftung &amp; Co. KG</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr"/>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
-      </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K67" t="inlineStr"/>
-      <c r="L67" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
         </is>
       </c>
     </row>
@@ -3592,12 +3590,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Marc O'Polo</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3606,11 +3604,7 @@
         </is>
       </c>
       <c r="F68" t="inlineStr"/>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
+      <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3618,7 +3612,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -3629,7 +3623,7 @@
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
         </is>
       </c>
     </row>
@@ -3640,21 +3634,25 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>Marc O'Polo</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Praktikum Marketing (m/w/d)</t>
+          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F69" t="inlineStr"/>
-      <c r="G69" t="inlineStr"/>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
       <c r="H69" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3673,7 +3671,7 @@
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899691?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3684,7 +3682,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -3694,14 +3692,14 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -3717,7 +3715,7 @@
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
+          <t>https://www.adzuna.de/details/5802899691?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3733,7 +3731,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Sales (m/w/d)</t>
+          <t>Praktikum Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -3750,7 +3748,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
@@ -3761,55 +3759,51 @@
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr">
         <is>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr"/>
+      <c r="B72" t="n">
+        <v>54</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Nestle Deutschland</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Praktikum Marketing &amp; Sales (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main, DE, 60329</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>fmcg</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr">
+        <is>
           <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-&amp;-Sales-%28mwd%29-60329/1425985633/</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B72" s="2" t="n">
-        <v>54</v>
-      </c>
-      <c r="C72" s="2" t="inlineStr">
-        <is>
-          <t>Nestle Deutschland</t>
-        </is>
-      </c>
-      <c r="D72" s="2" t="inlineStr">
-        <is>
-          <t>Praktikum Produktmarketing (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E72" s="2" t="inlineStr">
-        <is>
-          <t>Frankfurt am Main, DE, 60329</t>
-        </is>
-      </c>
-      <c r="F72" s="2" t="inlineStr"/>
-      <c r="G72" s="2" t="inlineStr"/>
-      <c r="H72" s="2" t="inlineStr">
-        <is>
-          <t>fmcg</t>
-        </is>
-      </c>
-      <c r="I72" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-      <c r="J72" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K72" s="2" t="inlineStr"/>
-      <c r="L72" s="2" t="inlineStr">
-        <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Produktmarketing-%28mwd%29-60329/1431039933/</t>
         </is>
       </c>
     </row>
@@ -3820,33 +3814,33 @@
         </is>
       </c>
       <c r="B73" s="2" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d) - In 3 Minuten erfolgreich bewerben</t>
+          <t>Praktikum Produktmarketing (m/w/d)</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr"/>
       <c r="G73" s="2" t="inlineStr"/>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr">
@@ -3857,7 +3851,7 @@
       <c r="K73" s="2" t="inlineStr"/>
       <c r="L73" s="2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5856295760?se=VqemWBmh8RGCZtbxFymUqg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A0E45C661705BA9D9ECDDCCACDFEEB182D4173F7</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Produktmarketing-%28mwd%29-60329/1431039933/</t>
         </is>
       </c>
     </row>
@@ -3868,27 +3862,21 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>LIGANOVA GmbH</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Praktikum Buying (all genders) – September 2026</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d) - In 3 Minuten erfolgreich bewerben</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
-        </is>
-      </c>
-      <c r="F74" t="n">
-        <v>6</v>
-      </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3896,7 +3884,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -3907,57 +3895,55 @@
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5849630691?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5856295760?se=VqemWBmh8RGCZtbxFymUqg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A0E45C661705BA9D9ECDDCCACDFEEB182D4173F7</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr"/>
-      <c r="B75" t="n">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="n">
         <v>52</v>
       </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>LIGANOVA I Karriere</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>Praktikum Buying (all genders) – September 2026</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>Mitte, Stuttgart</t>
-        </is>
-      </c>
-      <c r="F75" t="n">
-        <v>6</v>
-      </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="H75" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I75" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
-      </c>
-      <c r="J75" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K75" t="inlineStr"/>
-      <c r="L75" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5852669596?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>Handwerk Karriere</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr"/>
+      <c r="G75" s="2" t="inlineStr"/>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K75" s="2" t="inlineStr"/>
+      <c r="L75" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/land/ad/5859734477?se=2BMB0Auj8RGxSf1iGXKoQA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8912F76B99550481E2615DFD8E07B2F6745D01A7</t>
         </is>
       </c>
     </row>
@@ -3968,29 +3954,35 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>LIGANOVA GmbH</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Marketing &amp; Merchandising Assistant Trainee</t>
+          <t>Praktikum Buying (all genders) – September 2026</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>MILAN</t>
-        </is>
-      </c>
-      <c r="F76" t="inlineStr"/>
-      <c r="G76" t="inlineStr"/>
+          <t>Mitte, Stuttgart</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>6</v>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -4001,7 +3993,7 @@
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
+          <t>https://www.adzuna.de/details/5849630691?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4012,29 +4004,35 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>LIGANOVA I Karriere</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Marketing and Merchandising Assistant Trainee</t>
+          <t>Praktikum Buying (all genders) – September 2026</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>MILAN</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr"/>
-      <c r="G77" t="inlineStr"/>
+          <t>Mitte, Stuttgart</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>6</v>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -4045,7 +4043,7 @@
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing-and-Merchandising-Assistant-Trainee_JR128690</t>
+          <t>https://www.adzuna.de/details/5852669596?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4056,29 +4054,29 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Wonder Natural GmbH</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
+          <t>Marketing &amp; Merchandising Assistant Trainee</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -4089,35 +4087,35 @@
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr"/>
       <c r="B79" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Digitalagenten</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
+          <t>Marketing and Merchandising Assistant Trainee</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Charlottenburg, Berlin</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -4133,28 +4131,28 @@
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804948828?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing-and-Merchandising-Assistant-Trainee_JR128690</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr"/>
       <c r="B80" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>HardyTec Industries UG haftungsbeschränkt</t>
+          <t>Wonder Natural GmbH</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Business Development</t>
+          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Büderich, Meerbusch</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F80" t="inlineStr"/>
@@ -4166,7 +4164,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -4177,7 +4175,7 @@
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5848139968?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4188,17 +4186,17 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>LIMITD by Wunderproducts GmbH</t>
+          <t>Digitalagenten</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Kreuzberg, Berlin</t>
+          <t>Charlottenburg, Berlin</t>
         </is>
       </c>
       <c r="F81" t="inlineStr"/>
@@ -4221,7 +4219,7 @@
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804948828?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4232,25 +4230,21 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers GmbH WPG</t>
+          <t>HardyTec Industries UG haftungsbeschränkt</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
+          <t>Praktikum Marketing &amp; Business Development</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Büderich, Meerbusch</t>
         </is>
       </c>
       <c r="F82" t="inlineStr"/>
-      <c r="G82" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
+      <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4258,7 +4252,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -4269,7 +4263,7 @@
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5848139968?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4280,25 +4274,21 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>SERVICEPLAN Gruppe</t>
+          <t>LIMITD by Wunderproducts GmbH</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Sales (Marketing / New Business) (all genders)</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Kreuzberg, Berlin</t>
         </is>
       </c>
       <c r="F83" t="inlineStr"/>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4306,7 +4296,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -4317,7 +4307,7 @@
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4328,21 +4318,25 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>WirWinzer</t>
+          <t>PricewaterhouseCoopers GmbH WPG</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Praktikum Business Development Weinhandel (all genders)</t>
+          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
-      <c r="G84" t="inlineStr"/>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
       <c r="H84" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4361,32 +4355,36 @@
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr"/>
       <c r="B85" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>SERVICEPLAN Gruppe</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Praktikum Inside Sales (x/f/m)</t>
+          <t>Praktikum Business Development &amp; Sales (Marketing / New Business) (all genders)</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
-      <c r="G85" t="inlineStr"/>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H85" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4394,7 +4392,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -4405,40 +4403,40 @@
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7799489003</t>
+          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr"/>
       <c r="B86" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>WirWinzer</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Internship - High Jewelry Business Development Assistant</t>
+          <t>Praktikum Business Development Weinhandel (all genders)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -4449,7 +4447,7 @@
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
+          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4460,27 +4458,21 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>RÖDL</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Inside Sales (x/f/m)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Stuttgart, Baden-Württemberg</t>
-        </is>
-      </c>
-      <c r="F87" t="n">
-        <v>6</v>
-      </c>
-      <c r="G87" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>Berlin, Berlin, Germany</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4499,40 +4491,40 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5854352066?se=9tCS70-g8RGkr9xW060fUg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DBAD57A9DC2B84BE2128168013A758C1F47DCD27</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7799489003</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr"/>
       <c r="B88" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Brand Trust</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
+          <t>Internship - High Jewelry Business Development Assistant</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Gleißbühl, Nürnberg</t>
+          <t>PARIS</t>
         </is>
       </c>
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -4543,28 +4535,38 @@
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5669847401?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr"/>
       <c r="B89" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>RÖDL</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr"/>
-      <c r="F89" t="inlineStr"/>
-      <c r="G89" t="inlineStr"/>
+          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Stuttgart, Baden-Württemberg</t>
+        </is>
+      </c>
+      <c r="F89" t="n">
+        <v>6</v>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H89" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4572,7 +4574,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -4583,7 +4585,7 @@
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
+          <t>https://www.adzuna.de/land/ad/5854352066?se=9tCS70-g8RGkr9xW060fUg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DBAD57A9DC2B84BE2128168013A758C1F47DCD27</t>
         </is>
       </c>
     </row>
@@ -4594,17 +4596,17 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Brand Trust</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Praktikum B2B Event Marketing (x/f/m)</t>
+          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
+          <t>Gleißbühl, Nürnberg</t>
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
@@ -4616,7 +4618,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -4627,7 +4629,7 @@
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7820455003</t>
+          <t>https://www.adzuna.de/details/5669847401?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4642,17 +4644,17 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Codeso Living</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>Go To Market Strategy Hospitals (x/f/m)</t>
+          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
+          <t>Unterbilk, Düsseldorf</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr"/>
@@ -4664,7 +4666,7 @@
       </c>
       <c r="I91" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J91" s="2" t="inlineStr">
@@ -4675,7 +4677,7 @@
       <c r="K91" s="2" t="inlineStr"/>
       <c r="L91" s="2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7971471003</t>
+          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4686,19 +4688,15 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Genuine Parts Company</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Praktikum Category Management (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>Münster, Nordrhein-Westfalen</t>
-        </is>
-      </c>
+          <t>Marketing Intern - Trade Marketing</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
@@ -4708,7 +4706,7 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
@@ -4719,7 +4717,7 @@
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853760166?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
         </is>
       </c>
     </row>
@@ -4730,17 +4728,17 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
+          <t>Praktikum B2B Event Marketing (x/f/m)</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Benrath, Düsseldorf</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F93" t="inlineStr"/>
@@ -4752,7 +4750,7 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
@@ -4763,7 +4761,7 @@
       <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7820455003</t>
         </is>
       </c>
     </row>
@@ -4774,17 +4772,17 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
+          <t>Go To Market Strategy Hospitals (x/f/m)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Schwabing-Freimann, München</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F94" t="inlineStr"/>
@@ -4796,7 +4794,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
@@ -4807,7 +4805,7 @@
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7971471003</t>
         </is>
       </c>
     </row>
@@ -4818,29 +4816,29 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Genuine Parts Company</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
+          <t>Praktikum Category Management (m/w/d)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>DEU-Bayern-Unterhaching</t>
+          <t>Münster, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -4851,7 +4849,7 @@
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
+          <t>https://www.adzuna.de/details/5853760166?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4862,17 +4860,17 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>Benrath, Düsseldorf</t>
         </is>
       </c>
       <c r="F96" t="inlineStr"/>
@@ -4884,7 +4882,7 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
@@ -4895,7 +4893,7 @@
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4906,17 +4904,17 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Schwabing-Freimann, München</t>
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -4939,7 +4937,7 @@
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
+          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4950,24 +4948,24 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>DEU-Bayern-Unterhaching</t>
         </is>
       </c>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -4983,7 +4981,7 @@
       <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
         </is>
       </c>
     </row>
@@ -4994,17 +4992,17 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F99" t="inlineStr"/>
@@ -5027,7 +5025,7 @@
       <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
+          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5038,17 +5036,17 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F100" t="inlineStr"/>
@@ -5071,7 +5069,7 @@
       <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
         </is>
       </c>
     </row>
@@ -5082,17 +5080,17 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>RAG</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Gornhofen, Ravensburg</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F101" t="inlineStr"/>
@@ -5104,7 +5102,7 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
@@ -5115,28 +5113,28 @@
       <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr"/>
       <c r="B102" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>REWE Group</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F102" t="inlineStr"/>
@@ -5159,28 +5157,28 @@
       <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5712965755?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr"/>
       <c r="B103" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
         </is>
       </c>
       <c r="F103" t="inlineStr"/>
@@ -5203,28 +5201,28 @@
       <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr"/>
       <c r="B104" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>RAG</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Altstadt-Nord, Köln</t>
+          <t>Gornhofen, Ravensburg</t>
         </is>
       </c>
       <c r="F104" t="inlineStr"/>
@@ -5236,7 +5234,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -5247,28 +5245,28 @@
       <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr"/>
       <c r="B105" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Devoteam G Cloud Germany</t>
+          <t>REWE Group</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F105" t="inlineStr"/>
@@ -5291,28 +5289,28 @@
       <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811135653?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5712965755?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr"/>
       <c r="B106" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>freudio</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Wien, Österreich</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F106" t="inlineStr"/>
@@ -5324,7 +5322,7 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J106" t="inlineStr">
@@ -5335,28 +5333,28 @@
       <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/details/5836667156?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr"/>
       <c r="B107" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt-Nord, Köln</t>
         </is>
       </c>
       <c r="F107" t="inlineStr"/>
@@ -5379,7 +5377,7 @@
       <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5390,12 +5388,12 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>Devoteam G Cloud Germany</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -5423,7 +5421,7 @@
       <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5811135653?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5434,17 +5432,17 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>freudio</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Wien, Österreich</t>
         </is>
       </c>
       <c r="F109" t="inlineStr"/>
@@ -5456,7 +5454,7 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
@@ -5467,7 +5465,7 @@
       <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/details/5836667156?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5483,12 +5481,12 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F110" t="inlineStr"/>
@@ -5511,55 +5509,51 @@
       <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B111" s="2" t="n">
+      <c r="A111" t="inlineStr"/>
+      <c r="B111" t="n">
         <v>45</v>
       </c>
-      <c r="C111" s="2" t="inlineStr">
+      <c r="C111" t="inlineStr">
         <is>
           <t>prepmymeal GmbH</t>
         </is>
       </c>
-      <c r="D111" s="2" t="inlineStr">
-        <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d) - In 3 Minuten erfolgreich bewerben</t>
-        </is>
-      </c>
-      <c r="E111" s="2" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F111" s="2" t="inlineStr"/>
-      <c r="G111" s="2" t="inlineStr"/>
-      <c r="H111" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I111" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="J111" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K111" s="2" t="inlineStr"/>
-      <c r="L111" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5856292292?se=PMRjVxmh8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DF242745B4142F9871F0353F9B390FD5166A63B5</t>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr"/>
+      <c r="G111" t="inlineStr"/>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr"/>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5570,17 +5564,17 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>sailwithus</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F112" t="inlineStr"/>
@@ -5603,7 +5597,7 @@
       <c r="K112" t="inlineStr"/>
       <c r="L112" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5614,12 +5608,12 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>sailwithus</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -5647,12 +5641,144 @@
       <c r="K113" t="inlineStr"/>
       <c r="L113" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr"/>
+      <c r="B114" t="n">
+        <v>45</v>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>prepmymeal GmbH</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Praktikum Business Development (Französisch) (m/w/d) - In 3 Minuten erfolgreich bewerben</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr"/>
+      <c r="G114" t="inlineStr"/>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr"/>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/land/ad/5856292292?se=PMRjVxmh8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DF242745B4142F9871F0353F9B390FD5166A63B5</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr"/>
+      <c r="B115" t="n">
+        <v>45</v>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>sailwithus</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr"/>
+      <c r="G115" t="inlineStr"/>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr"/>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr"/>
+      <c r="B116" t="n">
+        <v>45</v>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>sailwithus</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr"/>
+      <c r="G116" t="inlineStr"/>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr"/>
+      <c r="L116" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5804544237?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L113"/>
+  <autoFilter ref="A1:L116"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5663,7 +5789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G97"/>
+  <dimension ref="A1:G99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -5794,7 +5920,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="C5" t="n">
         <v>84</v>
@@ -5819,7 +5945,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C6" t="n">
         <v>84</v>
@@ -5844,7 +5970,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C7" t="n">
         <v>84</v>
@@ -5877,7 +6003,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C8" t="n">
         <v>84</v>
@@ -5902,7 +6028,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C9" t="n">
         <v>84</v>
@@ -5927,7 +6053,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
@@ -5952,7 +6078,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C11" t="n">
         <v>84</v>
@@ -5977,7 +6103,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C12" t="n">
         <v>84</v>
@@ -6002,7 +6128,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C13" t="n">
         <v>84</v>
@@ -6027,7 +6153,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C14" t="n">
         <v>84</v>
@@ -6060,7 +6186,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C15" t="n">
         <v>84</v>
@@ -6110,7 +6236,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C17" t="n">
         <v>80</v>
@@ -6135,7 +6261,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C18" t="n">
         <v>79</v>
@@ -6210,7 +6336,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C21" t="n">
         <v>78</v>
@@ -6243,7 +6369,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C22" t="n">
         <v>78</v>
@@ -6268,7 +6394,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C23" t="n">
         <v>78</v>
@@ -6293,7 +6419,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C24" t="n">
         <v>74</v>
@@ -6326,7 +6452,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C25" t="n">
         <v>74</v>
@@ -6351,7 +6477,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C26" t="n">
         <v>74</v>
@@ -6376,7 +6502,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C27" t="n">
         <v>74</v>
@@ -6401,7 +6527,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C28" t="n">
         <v>73</v>
@@ -6459,7 +6585,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C30" t="n">
         <v>73</v>
@@ -6484,7 +6610,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="C31" t="n">
         <v>72</v>
@@ -6509,7 +6635,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C32" t="n">
         <v>72</v>
@@ -6559,7 +6685,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C34" t="n">
         <v>69</v>
@@ -6584,7 +6710,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C35" t="n">
         <v>68</v>
@@ -6659,7 +6785,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C38" t="n">
         <v>66</v>
@@ -6684,7 +6810,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C39" t="n">
         <v>65</v>
@@ -6709,7 +6835,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C40" t="n">
         <v>64</v>
@@ -6734,7 +6860,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C41" t="n">
         <v>62</v>
@@ -6759,7 +6885,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C42" t="n">
         <v>62</v>
@@ -6792,7 +6918,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C43" t="n">
         <v>62</v>
@@ -6817,7 +6943,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C44" t="n">
         <v>59</v>
@@ -6842,7 +6968,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C45" t="n">
         <v>59</v>
@@ -6867,7 +6993,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C46" t="n">
         <v>57</v>
@@ -6900,7 +7026,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C47" t="n">
         <v>56</v>
@@ -6925,7 +7051,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C48" t="n">
         <v>55</v>
@@ -7000,7 +7126,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C51" t="n">
         <v>53</v>
@@ -7025,7 +7151,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C52" t="n">
         <v>53</v>
@@ -7075,7 +7201,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C54" t="n">
         <v>52</v>
@@ -7100,7 +7226,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C55" t="n">
         <v>52</v>
@@ -7121,100 +7247,100 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Digitalagenten</t>
+          <t>Handwerk Karriere</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="C56" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>HardyTec Industries UG haftungsbeschränkt</t>
+          <t>Digitalagenten</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="C57" t="n">
         <v>51</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Business Development</t>
+          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
         </is>
       </c>
       <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>RÖDL</t>
+          <t>HardyTec Industries UG haftungsbeschränkt</t>
         </is>
       </c>
       <c r="B58" t="n">
         <v>1</v>
       </c>
       <c r="C58" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Marketing &amp; Business Development</t>
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Brand Trust</t>
+          <t>RÖDL</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="C59" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
+          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-25</t>
         </is>
       </c>
     </row>
@@ -7225,7 +7351,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C60" t="n">
         <v>49</v>
@@ -7250,7 +7376,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C61" t="n">
         <v>49</v>
@@ -7275,7 +7401,7 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C62" t="n">
         <v>49</v>
@@ -7296,43 +7422,43 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Genuine Parts Company</t>
+          <t>Brand Trust</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="C63" t="n">
         <v>49</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Praktikum Category Management (m/w/d)</t>
+          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>RAG</t>
+          <t>Genuine Parts Company</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C64" t="n">
         <v>49</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
+          <t>Praktikum Category Management (m/w/d)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
@@ -7346,68 +7472,68 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>REWE Group</t>
+          <t>RAG</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="C65" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Pflegia</t>
+          <t>Codeso Living</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C66" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Werkia</t>
+          <t>REWE Group</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="C67" t="n">
         <v>48</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d) - Datenanalyse &amp; Automatisierung</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
@@ -7421,18 +7547,18 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>paero</t>
+          <t>Pflegia</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C68" t="n">
         <v>48</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr"/>
@@ -7446,7 +7572,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Vivanta Gmbh</t>
+          <t>Werkia</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -7457,7 +7583,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/d) - Datenanalyse &amp; Automatisierung</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
@@ -7471,7 +7597,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Vitolus</t>
+          <t>paero</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -7482,7 +7608,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
@@ -7496,7 +7622,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>GrantLift GmbH</t>
+          <t>Vivanta Gmbh</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -7507,7 +7633,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr"/>
@@ -7521,7 +7647,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Otto Group one.O GmbH</t>
+          <t>Vitolus</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -7532,7 +7658,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Praktikum im Knowledge Management - Corporate Strategy (w/m/d)</t>
+          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr"/>
@@ -7546,18 +7672,18 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>AUTO1 Global Services SE &amp; Co. KG</t>
+          <t>GrantLift GmbH</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C73" t="n">
         <v>48</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (d/m/w)</t>
+          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr"/>
@@ -7571,18 +7697,18 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>SHAVENT - ARA Sustainable Products</t>
+          <t>Otto Group one.O GmbH</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C74" t="n">
         <v>48</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Praktikum Business Development in nachhaltigem Start-Up (w/m/d) Remote in DE</t>
+          <t>Praktikum im Knowledge Management - Corporate Strategy (w/m/d)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr"/>
@@ -7596,7 +7722,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CTG Consulting</t>
+          <t>AUTO1 Global Services SE &amp; Co. KG</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -7607,7 +7733,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Praktikum Sales/Business Development // Hamburg oder Berlin</t>
+          <t>Praktikum Business Development (d/m/w)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr"/>
@@ -7621,7 +7747,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Dronesperhour</t>
+          <t>SHAVENT - ARA Sustainable Products</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -7632,7 +7758,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development eines Startups (m/w/d)</t>
+          <t>Praktikum Business Development in nachhaltigem Start-Up (w/m/d) Remote in DE</t>
         </is>
       </c>
       <c r="E76" t="inlineStr"/>
@@ -7646,7 +7772,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>SINN Power</t>
+          <t>CTG Consulting</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -7657,7 +7783,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Praktikum im AI Business Development (m/w/d)</t>
+          <t>Praktikum Sales/Business Development // Hamburg oder Berlin</t>
         </is>
       </c>
       <c r="E77" t="inlineStr"/>
@@ -7671,7 +7797,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>innpuls</t>
+          <t>Dronesperhour</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -7682,7 +7808,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Praktikum im Business Development eines Startups (m/w/d)</t>
         </is>
       </c>
       <c r="E78" t="inlineStr"/>
@@ -7696,7 +7822,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Amolina</t>
+          <t>SINN Power</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -7707,7 +7833,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
+          <t>Praktikum im AI Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E79" t="inlineStr"/>
@@ -7721,18 +7847,18 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>innpuls</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>52</v>
+        <v>1</v>
       </c>
       <c r="C80" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E80" t="inlineStr"/>
@@ -7746,43 +7872,43 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>freudio</t>
+          <t>Amolina</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="C81" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
+          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
         </is>
       </c>
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>STARTPLATZ Gruppe</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>1</v>
+        <v>54</v>
       </c>
       <c r="C82" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Sales (m/w/d) – STARTPLATZ</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E82" t="inlineStr"/>
@@ -7796,32 +7922,32 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>spring.gate business consulting UG</t>
+          <t>freudio</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="C83" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development &amp; B2B Akquise (m/w/d)</t>
+          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
         </is>
       </c>
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>specter automation</t>
+          <t>STARTPLATZ Gruppe</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -7832,7 +7958,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Praktikum (M/W/D) im Business Development</t>
+          <t>Praktikum Business Development &amp; Sales (m/w/d) – STARTPLATZ</t>
         </is>
       </c>
       <c r="E84" t="inlineStr"/>
@@ -7846,18 +7972,18 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Closd Kunststoffprodukte GmbH</t>
+          <t>spring.gate business consulting UG</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C85" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Praktikum beim E-Commerce Startup Closd als Founders Associate (m/w/d)</t>
+          <t>Praktikum im Business Development &amp; B2B Akquise (m/w/d)</t>
         </is>
       </c>
       <c r="E85" t="inlineStr"/>
@@ -7871,18 +7997,18 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Bosch Rexroth AG</t>
+          <t>specter automation</t>
         </is>
       </c>
       <c r="B86" t="n">
         <v>1</v>
       </c>
       <c r="C86" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Praktikum Business Development – Software Defined Business</t>
+          <t>Praktikum (M/W/D) im Business Development</t>
         </is>
       </c>
       <c r="E86" t="inlineStr"/>
@@ -7896,18 +8022,18 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Weenect</t>
+          <t>Closd Kunststoffprodukte GmbH</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C87" t="n">
         <v>38</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d) – Markt DACH – Standort Brüssel</t>
+          <t>Praktikum beim E-Commerce Startup Closd als Founders Associate (m/w/d)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr"/>
@@ -7921,18 +8047,18 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Lidl Dienstleistung GmbH &amp; Co. KG</t>
+          <t>Bosch Rexroth AG</t>
         </is>
       </c>
       <c r="B88" t="n">
         <v>1</v>
       </c>
       <c r="C88" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Praktikum Business Development – Software Defined Business</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
@@ -7946,18 +8072,18 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Drägerwerk AG &amp; Co. KGaA</t>
+          <t>Weenect</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C89" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Praktikum New Business Development</t>
+          <t>Praktikum Business Development (m/w/d) – Markt DACH – Standort Brüssel</t>
         </is>
       </c>
       <c r="E89" t="inlineStr"/>
@@ -7971,18 +8097,18 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Arteus Energy</t>
+          <t>Lidl Dienstleistung GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="B90" t="n">
         <v>1</v>
       </c>
       <c r="C90" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Praktikum Business Development und Marketing Photovoltaik</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E90" t="inlineStr"/>
@@ -7996,18 +8122,18 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>aramido</t>
+          <t>Drägerwerk AG &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C91" t="n">
         <v>28</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/x)</t>
+          <t>Praktikum New Business Development</t>
         </is>
       </c>
       <c r="E91" t="inlineStr"/>
@@ -8021,7 +8147,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>pacemaker.ai by thyssenkrupp</t>
+          <t>Arteus Energy</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -8032,7 +8158,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Praktikum Business Development und Marketing Photovoltaik</t>
         </is>
       </c>
       <c r="E92" t="inlineStr"/>
@@ -8046,7 +8172,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Molly Suh GmbH</t>
+          <t>aramido</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -8057,7 +8183,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; B2B Sales (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/x)</t>
         </is>
       </c>
       <c r="E93" t="inlineStr"/>
@@ -8071,7 +8197,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>homewise</t>
+          <t>pacemaker.ai by thyssenkrupp</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -8082,7 +8208,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development &amp; Strategie (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr"/>
@@ -8096,7 +8222,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>ClipMyHorse.TV</t>
+          <t>Molly Suh GmbH</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -8107,7 +8233,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Praktikum HR &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Business Development &amp; B2B Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr"/>
@@ -8121,7 +8247,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>AUMOVIO</t>
+          <t>homewise</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -8132,7 +8258,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Praktikum - Administration/Assistenz &amp; Business Development</t>
+          <t>Praktikum im Business Development &amp; Strategie (m/w/d)</t>
         </is>
       </c>
       <c r="E96" t="inlineStr"/>
@@ -8146,7 +8272,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>TRUMPF Group</t>
+          <t>ClipMyHorse.TV</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -8157,7 +8283,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich Business Development für Smart Factory Solutions (WS26/27)</t>
+          <t>Praktikum HR &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr"/>
@@ -8168,8 +8294,58 @@
         </is>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>AUMOVIO</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>1</v>
+      </c>
+      <c r="C98" t="n">
+        <v>28</v>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Praktikum - Administration/Assistenz &amp; Business Development</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr"/>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>TRUMPF Group</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>1</v>
+      </c>
+      <c r="C99" t="n">
+        <v>28</v>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Praktikum im Bereich Business Development für Smart Factory Solutions (WS26/27)</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr"/>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G97"/>
+  <autoFilter ref="A1:G99"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Lauf 2026-08-31 12:51 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firmen entdeckt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$119</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$118</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$99</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L119"/>
+  <dimension ref="A1:L118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -856,12 +856,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Picnic</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Category Management Praktikum (m/w/d)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -891,7 +891,7 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5859954968?se=avT3yguj8RGEeLI7Dotn4Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FEC8C1664463BB6D76B4F51C80D7BE9A67B3E95</t>
+          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -912,7 +912,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -937,34 +937,36 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759088383?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="n">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Picnic</t>
+          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Category Management Praktikum (m/w/d)</t>
+          <t>Praktikum Brand Management National</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F11" t="n">
-        <v>6</v>
-      </c>
-      <c r="G11" t="inlineStr"/>
+          <t>Au-Haidhausen, München</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -983,34 +985,36 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759088383?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805399065?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management National</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Au-Haidhausen, München</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>6</v>
+      </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1031,7 +1035,7 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805399065?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1047,7 +1051,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1060,7 +1064,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1081,7 +1085,7 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5799961458?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1097,7 +1101,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1108,11 +1112,7 @@
       <c r="F14" t="n">
         <v>6</v>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1131,7 +1131,7 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5799961458?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1142,17 +1142,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Ferrero</t>
+          <t>L'Occitane</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikum (m/w/d) Trade Marketing</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Friedrichstadt, Düsseldorf</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1177,7 +1177,7 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5842049264?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1188,23 +1188,27 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>L'Occitane</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Praktikum (m/w/d) Trade Marketing</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Friedrichstadt, Düsseldorf</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F16" t="n">
         <v>6</v>
       </c>
-      <c r="G16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1212,7 +1216,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1223,7 +1227,7 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5842049264?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1239,12 +1243,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Praktikum Brand Management (m/w/d)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F17" t="n">
@@ -1252,7 +1256,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1273,38 +1277,32 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802899675?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d)</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F18" t="n">
-        <v>6</v>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1312,7 +1310,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1323,7 +1321,7 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899675?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5843630960?se=znNqlDyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=875B574D03DFD36B16B3A3ABE0AA46F858215182</t>
         </is>
       </c>
     </row>
@@ -1339,7 +1337,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1367,7 +1365,7 @@
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5843630960?se=znNqlDyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=875B574D03DFD36B16B3A3ABE0AA46F858215182</t>
+          <t>https://www.adzuna.de/land/ad/5843628966?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=3DAF9A0A7032477BEFBE4DD229577F81F1D32CF0</t>
         </is>
       </c>
     </row>
@@ -1383,7 +1381,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1411,7 +1409,7 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5843628966?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=3DAF9A0A7032477BEFBE4DD229577F81F1D32CF0</t>
+          <t>https://www.adzuna.de/land/ad/5843628932?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=65C46D18FCDB11FD2E933BD305E494E07D043D72</t>
         </is>
       </c>
     </row>
@@ -1422,21 +1420,27 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>HUGO BOSS</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Internship Buying &amp; Planning - Global Merchandising (m/f/d)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
+          <t>Metzingen, Reutlingen (Kreis)</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>6</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H21" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1444,7 +1448,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -1455,7 +1459,7 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5843628932?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=65C46D18FCDB11FD2E933BD305E494E07D043D72</t>
+          <t>https://www.adzuna.de/details/5856159470?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1466,27 +1470,21 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>HUGO BOSS</t>
+          <t>Miles &amp; More GmbH</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Internship Buying &amp; Planning - Global Merchandising (m/f/d)</t>
+          <t>Internship Marketing Strategy &amp; Delivery</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Metzingen, Reutlingen (Kreis)</t>
-        </is>
-      </c>
-      <c r="F22" t="n">
-        <v>6</v>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>Flughafen, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1494,7 +1492,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1505,7 +1503,7 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5856159470?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5828674997?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1516,20 +1514,22 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Miles &amp; More GmbH</t>
+          <t>coty</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Internship Marketing Strategy &amp; Delivery</t>
+          <t>Marketing Intern - Trade Marketing</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Flughafen, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr"/>
+          <t>Darmstadt, Hessen</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>6</v>
+      </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
@@ -1549,7 +1549,7 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5828674997?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1560,17 +1560,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Tchibo GmbH</t>
+          <t>P&amp;G</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing Eduscho (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F24" t="n">
@@ -1595,7 +1595,7 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5773205889?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2006,26 +2006,24 @@
     <row r="34">
       <c r="A34" t="inlineStr"/>
       <c r="B34" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F34" t="n">
-        <v>6</v>
-      </c>
+          <t>Hamburg, Deutschland</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
@@ -2034,7 +2032,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -2045,7 +2043,7 @@
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5859954968?se=avT3yguj8RGEeLI7Dotn4Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FEC8C1664463BB6D76B4F51C80D7BE9A67B3E95</t>
         </is>
       </c>
     </row>
@@ -2061,7 +2059,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
+          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2091,7 +2089,7 @@
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2107,7 +2105,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
+          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2118,11 +2116,7 @@
       <c r="F36" t="n">
         <v>6</v>
       </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2141,7 +2135,7 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2152,17 +2146,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Bosch Thermotechnik GmbH</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Praktikum im internationalen Brand Management</t>
+          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Wernau (Neckar), Esslingen (Kreis)</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -2170,7 +2164,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2191,7 +2185,7 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5799981240?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2202,17 +2196,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>Bosch Thermotechnik GmbH</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>Praktikum im internationalen Brand Management</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Wernau (Neckar), Esslingen (Kreis)</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -2220,7 +2214,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2241,34 +2235,38 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5799981240?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr"/>
       <c r="B39" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F39" t="n">
         <v>6</v>
       </c>
-      <c r="G39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
       <c r="H39" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2287,7 +2285,7 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2308,7 +2306,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Altstadt, Düsseldorf</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F40" t="n">
@@ -2333,40 +2331,42 @@
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr"/>
       <c r="B41" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Internship in Trade Marketing</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>DEU-Nordrhein-Westfalen-Köln</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr"/>
+          <t>Altstadt, Düsseldorf</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>6</v>
+      </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -2377,40 +2377,40 @@
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
+          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr"/>
       <c r="B42" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Calypso Ventures GmbH</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
+          <t>Internship in Trade Marketing</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>DEU-Nordrhein-Westfalen-Köln</t>
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -2421,7 +2421,7 @@
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
         </is>
       </c>
     </row>
@@ -2432,17 +2432,17 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>Calypso Ventures GmbH</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
@@ -2465,7 +2465,7 @@
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2481,7 +2481,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2498,7 +2498,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -2509,7 +2509,7 @@
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2520,22 +2520,20 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>FC Viktoria 1889 Berlin Frauen-Fußball GmbH</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>PRAKTIKUM // Business Development - In 3 Minuten erfolgreich bewerben</t>
+          <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F45" t="n">
-        <v>3</v>
-      </c>
+          <t>Düsseltal, Düsseldorf</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
@@ -2544,7 +2542,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -2555,7 +2553,7 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5856283303?se=PMRjVxmh8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0E222C24DC5860DC4AEB24D8BB5E4CB04740A32C</t>
+          <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2566,20 +2564,22 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>montamo GmbH</t>
+          <t>FC Viktoria 1889 Berlin Frauen-Fußball GmbH</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>PRAKTIKUM // Business Development - In 3 Minuten erfolgreich bewerben</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr"/>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>3</v>
+      </c>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -2599,7 +2599,7 @@
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5856889494?se=1M-3UDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=471483726C1FC3DB660B48A5B3DEDE0DC1A4DC20</t>
+          <t>https://www.adzuna.de/land/ad/5856283303?se=PMRjVxmh8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0E222C24DC5860DC4AEB24D8BB5E4CB04740A32C</t>
         </is>
       </c>
     </row>
@@ -2620,7 +2620,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F47" t="inlineStr"/>
@@ -2643,28 +2643,28 @@
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5857559039?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5856889494?se=1M-3UDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=471483726C1FC3DB660B48A5B3DEDE0DC1A4DC20</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr"/>
       <c r="B48" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>montamo GmbH</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Praktikum Retail Marketing | Fashion und Sport-Marken (w/m/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Wedding, Berlin</t>
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
@@ -2687,124 +2687,116 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/details/5857559039?utm_medium=api&amp;utm_source=e1fd92a2</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr"/>
+      <c r="B49" t="n">
+        <v>60</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Otto GmbH &amp; Co. KGaA</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Praktikum Retail Marketing | Fashion und Sport-Marken (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Hamburg, Deutschland</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/land/ad/5858188456?se=HMKESTui8RGfx5bEd-nhPg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=86B24D9EAAAA2322A41661C360015255B004809E</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="n">
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+      <c r="B50" t="n">
         <v>60</v>
       </c>
-      <c r="C49" s="2" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
-      <c r="D49" s="2" t="inlineStr">
+      <c r="D50" t="inlineStr">
         <is>
           <t>Praktikum Retail Marketing | Fashion und Sport-Marken (w/m/d)</t>
         </is>
       </c>
-      <c r="E49" s="2" t="inlineStr">
+      <c r="E50" t="inlineStr">
         <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="F49" s="2" t="inlineStr"/>
-      <c r="G49" s="2" t="inlineStr"/>
-      <c r="H49" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I49" s="2" t="inlineStr">
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="J49" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K49" s="2" t="inlineStr"/>
-      <c r="L49" s="2" t="inlineStr">
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr">
         <is>
           <t>https://www.adzuna.de/land/ad/5860650076?se=EGcET6Oj8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=E6646A9A107DD9C83D248D81843D6570367335AD</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>Praktikum Retail Marketing | Fashion und Sport-Marken (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>Hamburg-Altstadt, Hamburg</t>
-        </is>
-      </c>
-      <c r="F50" s="2" t="inlineStr"/>
-      <c r="G50" s="2" t="inlineStr"/>
-      <c r="H50" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I50" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
-      </c>
-      <c r="J50" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K50" s="2" t="inlineStr"/>
-      <c r="L50" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5860355819?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr"/>
       <c r="B51" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikum Retail Marketing | Fashion und Sport-Marken (w/m/d)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Hamburg-Altstadt, Hamburg</t>
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
@@ -2816,7 +2808,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -2827,7 +2819,7 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848400955?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=4E59A334AC360616EAEAAC474F72A07451A7C624</t>
+          <t>https://www.adzuna.de/details/5860355819?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2843,7 +2835,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2871,99 +2863,99 @@
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/land/ad/5848400955?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=4E59A334AC360616EAEAAC474F72A07451A7C624</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+      <c r="B53" t="n">
+        <v>59</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/land/ad/5848409009?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5C62DDCDA5E03F77D6089CD03CFA1D966DF15C96</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>NEU</t>
         </is>
       </c>
-      <c r="B53" s="2" t="n">
+      <c r="B54" s="2" t="n">
         <v>59</v>
       </c>
-      <c r="C53" s="2" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr">
         <is>
           <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
-      <c r="D53" s="2" t="inlineStr">
+      <c r="D54" s="2" t="inlineStr">
         <is>
           <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
-      <c r="E53" s="2" t="inlineStr">
+      <c r="E54" s="2" t="inlineStr">
         <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="F53" s="2" t="inlineStr"/>
-      <c r="G53" s="2" t="inlineStr"/>
-      <c r="H53" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I53" s="2" t="inlineStr">
+      <c r="F54" s="2" t="inlineStr"/>
+      <c r="G54" s="2" t="inlineStr"/>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="J53" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K53" s="2" t="inlineStr"/>
-      <c r="L53" s="2" t="inlineStr">
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr"/>
+      <c r="L54" s="2" t="inlineStr">
         <is>
           <t>https://www.adzuna.de/land/ad/5861203670?se=hvkm4GOk8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD0ED2E271738C13EE6613442755CC0DE68C0F5A</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr"/>
-      <c r="B54" t="n">
-        <v>59</v>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>Nahrungs- &amp; Genussmittel Karriere</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5848308031?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=C04FAD6E90B5FCF47A6B81E4A697BA781ADC04AF</t>
         </is>
       </c>
     </row>
@@ -2979,7 +2971,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -3007,7 +2999,7 @@
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5851105442?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8F6135545B7E9C415844F10F4AF49C0BFA63A4B2</t>
+          <t>https://www.adzuna.de/land/ad/5848308031?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=C04FAD6E90B5FCF47A6B81E4A697BA781ADC04AF</t>
         </is>
       </c>
     </row>
@@ -3023,7 +3015,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -3051,7 +3043,7 @@
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848347180?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8A3F28529B6340B7DCCD5131E2C4472FBD8CA361</t>
+          <t>https://www.adzuna.de/land/ad/5851105442?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8F6135545B7E9C415844F10F4AF49C0BFA63A4B2</t>
         </is>
       </c>
     </row>
@@ -3067,7 +3059,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -3095,7 +3087,7 @@
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848315177?se=nioaTDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B01A57BB52C4BDBB1DF6554A4A21C913096E1D0</t>
+          <t>https://www.adzuna.de/land/ad/5848347180?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8A3F28529B6340B7DCCD5131E2C4472FBD8CA361</t>
         </is>
       </c>
     </row>
@@ -3111,7 +3103,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -3139,7 +3131,7 @@
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848325009?se=nioaTDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8D26762D834367B41A848A3D14A62E41FD573B9B</t>
+          <t>https://www.adzuna.de/land/ad/5848315177?se=nioaTDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B01A57BB52C4BDBB1DF6554A4A21C913096E1D0</t>
         </is>
       </c>
     </row>
@@ -3150,12 +3142,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>P&amp;G</t>
+          <t>Nahrungs- &amp; Genussmittel Karriere</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -3172,7 +3164,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -3183,7 +3175,7 @@
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5848325009?se=nioaTDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8D26762D834367B41A848A3D14A62E41FD573B9B</t>
         </is>
       </c>
     </row>
@@ -3322,30 +3314,28 @@
     <row r="63">
       <c r="A63" t="inlineStr"/>
       <c r="B63" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>coty</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
+          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Darmstadt, Hessen</t>
-        </is>
-      </c>
-      <c r="F63" t="n">
-        <v>6</v>
-      </c>
+          <t>MILAN</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -3361,7 +3351,7 @@
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
         </is>
       </c>
     </row>
@@ -3372,29 +3362,29 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Wonder Natural GmbH</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
+          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
@@ -3405,28 +3395,28 @@
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
+          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr"/>
       <c r="B65" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Wonder Natural GmbH</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F65" t="inlineStr"/>
@@ -3438,7 +3428,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -3449,7 +3439,7 @@
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3470,7 +3460,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F66" t="inlineStr"/>
@@ -3493,31 +3483,33 @@
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr"/>
       <c r="B67" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>THE VERSE Ventures</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr"/>
+          <t>Berlin, Deutschland</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>6</v>
+      </c>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
         <is>
@@ -3537,33 +3529,31 @@
       <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr"/>
       <c r="B68" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>THE VERSE Ventures</t>
+          <t>Abrio</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
-        </is>
-      </c>
-      <c r="F68" t="n">
-        <v>6</v>
-      </c>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr">
         <is>
@@ -3583,7 +3573,7 @@
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3594,17 +3584,17 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Abrio</t>
+          <t>Groß- &amp; Einzelhandel Karriere</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F69" t="inlineStr"/>
@@ -3616,7 +3606,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -3627,7 +3617,7 @@
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5848296401?se=lphMSjui8RGhLffPfv7Txw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CDA6039E4CB2826923EB7E2E7ECB163DB4CFE919</t>
         </is>
       </c>
     </row>
@@ -3638,7 +3628,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Groß- &amp; Einzelhandel Karriere</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -3660,7 +3650,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -3671,7 +3661,7 @@
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848296401?se=lphMSjui8RGhLffPfv7Txw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CDA6039E4CB2826923EB7E2E7ECB163DB4CFE919</t>
+          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
         </is>
       </c>
     </row>
@@ -3682,12 +3672,12 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Lidl Stiftung &amp; Co. KG</t>
+          <t>Marc O'Polo</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
+          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -3696,7 +3686,11 @@
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
-      <c r="G71" t="inlineStr"/>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
       <c r="H71" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3704,7 +3698,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
@@ -3715,7 +3709,7 @@
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
+          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3726,25 +3720,21 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Marc O'Polo</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
+          <t>Praktikum Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F72" t="inlineStr"/>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
+      <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3763,7 +3753,7 @@
       <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802899691?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3774,7 +3764,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -3784,14 +3774,14 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -3807,7 +3797,7 @@
       <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899691?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
         </is>
       </c>
     </row>
@@ -3823,7 +3813,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Praktikum Marketing (m/w/d)</t>
+          <t>Praktikum Marketing &amp; Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3840,7 +3830,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -3851,7 +3841,7 @@
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-&amp;-Sales-%28mwd%29-60329/1425985633/</t>
         </is>
       </c>
     </row>
@@ -3867,7 +3857,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Sales (m/w/d)</t>
+          <t>Praktikum Produktmarketing (m/w/d)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3884,7 +3874,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
@@ -3895,40 +3885,40 @@
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-&amp;-Sales-%28mwd%29-60329/1425985633/</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Produktmarketing-%28mwd%29-60329/1431039933/</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr"/>
       <c r="B76" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Praktikum Produktmarketing (m/w/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d) - In 3 Minuten erfolgreich bewerben</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -3939,7 +3929,7 @@
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Produktmarketing-%28mwd%29-60329/1431039933/</t>
+          <t>https://www.adzuna.de/land/ad/5856295760?se=VqemWBmh8RGCZtbxFymUqg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A0E45C661705BA9D9ECDDCCACDFEEB182D4173F7</t>
         </is>
       </c>
     </row>
@@ -3950,12 +3940,12 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>Handwerk Karriere</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d) - In 3 Minuten erfolgreich bewerben</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3972,7 +3962,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -3983,7 +3973,7 @@
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5856295760?se=VqemWBmh8RGCZtbxFymUqg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A0E45C661705BA9D9ECDDCCACDFEEB182D4173F7</t>
+          <t>https://www.adzuna.de/land/ad/5859734477?se=2BMB0Auj8RGxSf1iGXKoQA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8912F76B99550481E2615DFD8E07B2F6745D01A7</t>
         </is>
       </c>
     </row>
@@ -3994,21 +3984,27 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Handwerk Karriere</t>
+          <t>LIGANOVA GmbH</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Buying (all genders) – September 2026</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr"/>
-      <c r="G78" t="inlineStr"/>
+          <t>Mitte, Stuttgart</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>6</v>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="H78" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4016,7 +4012,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -4027,7 +4023,7 @@
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5859734477?se=2BMB0Auj8RGxSf1iGXKoQA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8912F76B99550481E2615DFD8E07B2F6745D01A7</t>
+          <t>https://www.adzuna.de/details/5849630691?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4038,7 +4034,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>LIGANOVA GmbH</t>
+          <t>LIGANOVA I Karriere</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -4066,7 +4062,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -4077,7 +4073,7 @@
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5849630691?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5852669596?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4088,35 +4084,29 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>LIGANOVA I Karriere</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Praktikum Buying (all genders) – September 2026</t>
+          <t>Marketing &amp; Merchandising Assistant Trainee</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
-        </is>
-      </c>
-      <c r="F80" t="n">
-        <v>6</v>
-      </c>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+          <t>MILAN</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -4127,7 +4117,7 @@
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5852669596?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
         </is>
       </c>
     </row>
@@ -4143,7 +4133,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Marketing &amp; Merchandising Assistant Trainee</t>
+          <t>Marketing and Merchandising Assistant Trainee</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -4171,7 +4161,7 @@
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing-and-Merchandising-Assistant-Trainee_JR128690</t>
         </is>
       </c>
     </row>
@@ -4182,29 +4172,29 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Wonder Natural GmbH</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Marketing and Merchandising Assistant Trainee</t>
+          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>MILAN</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -4215,28 +4205,28 @@
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing-and-Merchandising-Assistant-Trainee_JR128690</t>
+          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr"/>
       <c r="B83" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Wonder Natural GmbH</t>
+          <t>Digitalagenten</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
+          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Charlottenburg, Berlin</t>
         </is>
       </c>
       <c r="F83" t="inlineStr"/>
@@ -4248,7 +4238,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -4259,7 +4249,7 @@
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804948828?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4270,17 +4260,17 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Digitalagenten</t>
+          <t>HardyTec Industries UG haftungsbeschränkt</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
+          <t>Praktikum Marketing &amp; Business Development</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Charlottenburg, Berlin</t>
+          <t>Büderich, Meerbusch</t>
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
@@ -4292,7 +4282,7 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
@@ -4303,7 +4293,7 @@
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804948828?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5848139968?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4314,17 +4304,17 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>HardyTec Industries UG haftungsbeschränkt</t>
+          <t>LIMITD by Wunderproducts GmbH</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Business Development</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Büderich, Meerbusch</t>
+          <t>Kreuzberg, Berlin</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
@@ -4336,7 +4326,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -4347,7 +4337,7 @@
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5848139968?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4358,21 +4348,25 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>LIMITD by Wunderproducts GmbH</t>
+          <t>PricewaterhouseCoopers GmbH WPG</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Kreuzberg, Berlin</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F86" t="inlineStr"/>
-      <c r="G86" t="inlineStr"/>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
       <c r="H86" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4391,7 +4385,7 @@
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4402,12 +4396,12 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers GmbH WPG</t>
+          <t>SERVICEPLAN Gruppe</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
+          <t>Praktikum Business Development &amp; Sales (Marketing / New Business) (all genders)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4418,7 +4412,7 @@
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -4428,7 +4422,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -4439,7 +4433,7 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4450,25 +4444,21 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>SERVICEPLAN Gruppe</t>
+          <t>WirWinzer</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Sales (Marketing / New Business) (all genders)</t>
+          <t>Praktikum Business Development Weinhandel (all genders)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F88" t="inlineStr"/>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4476,7 +4466,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -4487,28 +4477,28 @@
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr"/>
       <c r="B89" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>WirWinzer</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Praktikum Business Development Weinhandel (all genders)</t>
+          <t>Praktikum Inside Sales (x/f/m)</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F89" t="inlineStr"/>
@@ -4520,7 +4510,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -4531,7 +4521,7 @@
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7799489003</t>
         </is>
       </c>
     </row>
@@ -4542,29 +4532,29 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Praktikum Inside Sales (x/f/m)</t>
+          <t>Internship - High Jewelry Business Development Assistant</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
+          <t>PARIS</t>
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -4575,7 +4565,7 @@
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7799489003</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
         </is>
       </c>
     </row>
@@ -4586,29 +4576,35 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>RÖDL</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Internship - High Jewelry Business Development Assistant</t>
+          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>PARIS</t>
-        </is>
-      </c>
-      <c r="F91" t="inlineStr"/>
-      <c r="G91" t="inlineStr"/>
+          <t>Stuttgart, Baden-Württemberg</t>
+        </is>
+      </c>
+      <c r="F91" t="n">
+        <v>6</v>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -4619,38 +4615,32 @@
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
+          <t>https://www.adzuna.de/land/ad/5854352066?se=9tCS70-g8RGkr9xW060fUg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DBAD57A9DC2B84BE2128168013A758C1F47DCD27</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr"/>
       <c r="B92" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>RÖDL</t>
+          <t>Brand Trust</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Stuttgart, Baden-Württemberg</t>
-        </is>
-      </c>
-      <c r="F92" t="n">
-        <v>6</v>
-      </c>
-      <c r="G92" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>Gleißbühl, Nürnberg</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4658,7 +4648,7 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
@@ -4669,7 +4659,7 @@
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5854352066?se=9tCS70-g8RGkr9xW060fUg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DBAD57A9DC2B84BE2128168013A758C1F47DCD27</t>
+          <t>https://www.adzuna.de/details/5669847401?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4680,17 +4670,17 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Brand Trust</t>
+          <t>Codeso Living</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
+          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Gleißbühl, Nürnberg</t>
+          <t>Unterbilk, Düsseldorf</t>
         </is>
       </c>
       <c r="F93" t="inlineStr"/>
@@ -4702,7 +4692,7 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
@@ -4713,7 +4703,7 @@
       <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5669847401?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4724,19 +4714,15 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Codeso Living</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>Unterbilk, Düsseldorf</t>
-        </is>
-      </c>
+          <t>Marketing Intern - Trade Marketing</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
@@ -4746,7 +4732,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
@@ -4757,7 +4743,7 @@
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
         </is>
       </c>
     </row>
@@ -4768,15 +4754,19 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
-        </is>
-      </c>
-      <c r="E95" t="inlineStr"/>
+          <t>Praktikum B2B Event Marketing (x/f/m)</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Berlin, Berlin, Germany</t>
+        </is>
+      </c>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
@@ -4786,7 +4776,7 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -4797,7 +4787,7 @@
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7820455003</t>
         </is>
       </c>
     </row>
@@ -4813,7 +4803,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Praktikum B2B Event Marketing (x/f/m)</t>
+          <t>Go To Market Strategy Hospitals (x/f/m)</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -4830,7 +4820,7 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
@@ -4841,7 +4831,7 @@
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7820455003</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7971471003</t>
         </is>
       </c>
     </row>
@@ -4852,17 +4842,17 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Genuine Parts Company</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Go To Market Strategy Hospitals (x/f/m)</t>
+          <t>Praktikum Category Management (m/w/d)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
+          <t>Münster, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -4874,7 +4864,7 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
@@ -4885,7 +4875,7 @@
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7971471003</t>
+          <t>https://www.adzuna.de/details/5853760166?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4896,17 +4886,17 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Genuine Parts Company</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Praktikum Category Management (m/w/d)</t>
+          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Münster, Nordrhein-Westfalen</t>
+          <t>Benrath, Düsseldorf</t>
         </is>
       </c>
       <c r="F98" t="inlineStr"/>
@@ -4918,7 +4908,7 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
@@ -4929,7 +4919,7 @@
       <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853760166?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4940,17 +4930,17 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Benrath, Düsseldorf</t>
+          <t>Schwabing-Freimann, München</t>
         </is>
       </c>
       <c r="F99" t="inlineStr"/>
@@ -4962,7 +4952,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
@@ -4973,7 +4963,7 @@
       <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4984,24 +4974,24 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
+          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Schwabing-Freimann, München</t>
+          <t>DEU-Bayern-Unterhaching</t>
         </is>
       </c>
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -5017,7 +5007,7 @@
       <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
         </is>
       </c>
     </row>
@@ -5028,24 +5018,24 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>DEU-Bayern-Unterhaching</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr"/>
       <c r="H101" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -5061,7 +5051,7 @@
       <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
+          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5072,17 +5062,17 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F102" t="inlineStr"/>
@@ -5105,7 +5095,7 @@
       <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
         </is>
       </c>
     </row>
@@ -5121,7 +5111,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -5149,7 +5139,7 @@
       <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
+          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
         </is>
       </c>
     </row>
@@ -5165,7 +5155,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -5193,7 +5183,7 @@
       <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
+          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
         </is>
       </c>
     </row>
@@ -5204,17 +5194,17 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
         </is>
       </c>
       <c r="F105" t="inlineStr"/>
@@ -5237,7 +5227,7 @@
       <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
+          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5248,17 +5238,17 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>RAG</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+          <t>Gornhofen, Ravensburg</t>
         </is>
       </c>
       <c r="F106" t="inlineStr"/>
@@ -5270,7 +5260,7 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J106" t="inlineStr">
@@ -5281,28 +5271,28 @@
       <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr"/>
       <c r="B107" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>RAG</t>
+          <t>REWE Group</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Gornhofen, Ravensburg</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F107" t="inlineStr"/>
@@ -5314,7 +5304,7 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
@@ -5325,28 +5315,28 @@
       <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5712965755?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr"/>
       <c r="B108" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>REWE Group</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F108" t="inlineStr"/>
@@ -5369,7 +5359,7 @@
       <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5712965755?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5390,7 +5380,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Altstadt-Nord, Köln</t>
         </is>
       </c>
       <c r="F109" t="inlineStr"/>
@@ -5413,28 +5403,28 @@
       <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr"/>
       <c r="B110" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>Devoteam G Cloud Germany</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Altstadt-Nord, Köln</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F110" t="inlineStr"/>
@@ -5457,7 +5447,7 @@
       <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5811135653?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5468,17 +5458,17 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Devoteam G Cloud Germany</t>
+          <t>freudio</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Wien, Österreich</t>
         </is>
       </c>
       <c r="F111" t="inlineStr"/>
@@ -5490,7 +5480,7 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
@@ -5501,7 +5491,7 @@
       <c r="K111" t="inlineStr"/>
       <c r="L111" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811135653?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/details/5836667156?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5512,17 +5502,17 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>freudio</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Wien, Österreich</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F112" t="inlineStr"/>
@@ -5534,7 +5524,7 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
@@ -5545,7 +5535,7 @@
       <c r="K112" t="inlineStr"/>
       <c r="L112" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/details/5836667156?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5561,7 +5551,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -5589,7 +5579,7 @@
       <c r="K113" t="inlineStr"/>
       <c r="L113" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5605,12 +5595,12 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F114" t="inlineStr"/>
@@ -5633,7 +5623,7 @@
       <c r="K114" t="inlineStr"/>
       <c r="L114" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5649,7 +5639,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -5677,7 +5667,7 @@
       <c r="K115" t="inlineStr"/>
       <c r="L115" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5693,12 +5683,12 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d) - In 3 Minuten erfolgreich bewerben</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F116" t="inlineStr"/>
@@ -5710,7 +5700,7 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
@@ -5721,7 +5711,7 @@
       <c r="K116" t="inlineStr"/>
       <c r="L116" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5856292292?se=PMRjVxmh8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DF242745B4142F9871F0353F9B390FD5166A63B5</t>
         </is>
       </c>
     </row>
@@ -5732,17 +5722,17 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>sailwithus</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d) - In 3 Minuten erfolgreich bewerben</t>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F117" t="inlineStr"/>
@@ -5754,7 +5744,7 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
@@ -5765,7 +5755,7 @@
       <c r="K117" t="inlineStr"/>
       <c r="L117" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5856292292?se=PMRjVxmh8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DF242745B4142F9871F0353F9B390FD5166A63B5</t>
+          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5786,7 +5776,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F118" t="inlineStr"/>
@@ -5809,56 +5799,12 @@
       <c r="K118" t="inlineStr"/>
       <c r="L118" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr"/>
-      <c r="B119" t="n">
-        <v>45</v>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>sailwithus</t>
-        </is>
-      </c>
-      <c r="D119" t="inlineStr">
-        <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
-        </is>
-      </c>
-      <c r="E119" t="inlineStr">
-        <is>
-          <t>Altstadt, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F119" t="inlineStr"/>
-      <c r="G119" t="inlineStr"/>
-      <c r="H119" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I119" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J119" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K119" t="inlineStr"/>
-      <c r="L119" t="inlineStr">
-        <is>
           <t>https://www.adzuna.de/details/5804544237?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L119"/>
+  <autoFilter ref="A1:L118"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5975,7 +5921,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C4" t="n">
         <v>89</v>
@@ -6025,7 +5971,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="C6" t="n">
         <v>84</v>
@@ -6050,7 +5996,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C7" t="n">
         <v>84</v>
@@ -6075,7 +6021,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C8" t="n">
         <v>84</v>
@@ -6100,7 +6046,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C9" t="n">
         <v>84</v>
@@ -6133,7 +6079,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
@@ -6158,7 +6104,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C11" t="n">
         <v>84</v>
@@ -6183,7 +6129,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C12" t="n">
         <v>84</v>
@@ -6204,43 +6150,51 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers GmbH WPG</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C13" t="n">
         <v>84</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
+          <t>Praktikum Product Marketing (x/f/m)</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>greenhouse</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-23</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Carwow</t>
+          <t>PricewaterhouseCoopers GmbH WPG</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C14" t="n">
         <v>84</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Media (m/w/d) - OEM Partnerships @ Carwow</t>
+          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
@@ -6254,33 +6208,25 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Carwow</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C15" t="n">
         <v>84</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Praktikum Product Marketing (x/f/m)</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>greenhouse</t>
-        </is>
-      </c>
+          <t>Praktikum Business Development &amp; Media (m/w/d) - OEM Partnerships @ Carwow</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
@@ -6291,7 +6237,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C16" t="n">
         <v>84</v>
@@ -6341,7 +6287,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C18" t="n">
         <v>80</v>
@@ -6366,7 +6312,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C19" t="n">
         <v>79</v>
@@ -6441,7 +6387,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C22" t="n">
         <v>78</v>
@@ -6474,7 +6420,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C23" t="n">
         <v>78</v>
@@ -6499,7 +6445,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C24" t="n">
         <v>78</v>
@@ -6524,7 +6470,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C25" t="n">
         <v>74</v>
@@ -6557,7 +6503,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C26" t="n">
         <v>74</v>
@@ -6582,7 +6528,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C27" t="n">
         <v>74</v>
@@ -6607,7 +6553,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C28" t="n">
         <v>73</v>
@@ -6665,7 +6611,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C30" t="n">
         <v>73</v>
@@ -6690,7 +6636,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C31" t="n">
         <v>72</v>
@@ -6715,7 +6661,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C32" t="n">
         <v>72</v>
@@ -6790,7 +6736,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C35" t="n">
         <v>68</v>
@@ -6865,7 +6811,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C38" t="n">
         <v>66</v>
@@ -6890,7 +6836,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C39" t="n">
         <v>65</v>
@@ -6915,7 +6861,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C40" t="n">
         <v>64</v>
@@ -6940,7 +6886,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C41" t="n">
         <v>62</v>
@@ -6965,7 +6911,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C42" t="n">
         <v>62</v>
@@ -6998,7 +6944,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C43" t="n">
         <v>62</v>
@@ -7023,7 +6969,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C44" t="n">
         <v>59</v>
@@ -7073,7 +7019,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C46" t="n">
         <v>57</v>
@@ -7106,7 +7052,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C47" t="n">
         <v>56</v>
@@ -7131,7 +7077,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C48" t="n">
         <v>55</v>
@@ -7206,7 +7152,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C51" t="n">
         <v>53</v>
@@ -7231,7 +7177,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C52" t="n">
         <v>53</v>
@@ -7281,7 +7227,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C54" t="n">
         <v>52</v>
@@ -7306,7 +7252,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C55" t="n">
         <v>52</v>
@@ -7356,7 +7302,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C57" t="n">
         <v>51</v>
@@ -7431,7 +7377,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C60" t="n">
         <v>49</v>
@@ -7456,7 +7402,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C61" t="n">
         <v>49</v>
@@ -7481,7 +7427,7 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C62" t="n">
         <v>49</v>
@@ -7531,7 +7477,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C64" t="n">
         <v>49</v>
@@ -7556,7 +7502,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C65" t="n">
         <v>49</v>
@@ -7581,7 +7527,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C66" t="n">
         <v>49</v>
@@ -7981,7 +7927,7 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C82" t="n">
         <v>46</v>
@@ -8006,7 +7952,7 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C83" t="n">
         <v>45</v>

</xml_diff>

<commit_message>
Lauf 2026-09-02 10:48 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -664,12 +664,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Nestle</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -703,7 +703,7 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Category-Management%2C-Brand-Activation-und-Sales-%28mwd%29-60329/1427883433/</t>
         </is>
       </c>
     </row>
@@ -714,35 +714,31 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Hamburg-Altstadt, Hamburg</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>5</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -753,53 +749,57 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Category-Management%2C-Brand-Activation-und-Sales-%28mwd%29-60329/1427883433/</t>
+          <t>https://www.adzuna.de/details/5829732882?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="n">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
         <v>84</v>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Hamburg-Altstadt, Hamburg</t>
         </is>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5829732882?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5865920988?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -852,27 +852,29 @@
     <row r="9">
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="n">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Picnic</t>
+          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Category Management Praktikum (m/w/d)</t>
+          <t>Praktikum Brand Management National</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G9" t="inlineStr"/>
+          <t>Au-Haidhausen, München</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -891,34 +893,36 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759088383?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805399065?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management National</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Au-Haidhausen, München</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>6</v>
+      </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -939,7 +943,7 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805399065?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -955,7 +959,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -968,7 +972,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -989,7 +993,7 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5799961458?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1005,7 +1009,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1016,11 +1020,7 @@
       <c r="F12" t="n">
         <v>6</v>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1039,7 +1039,7 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5799961458?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1050,17 +1050,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Ferrero</t>
+          <t>L'Occitane</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikum (m/w/d) Trade Marketing</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Friedrichstadt, Düsseldorf</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1085,7 +1085,7 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5842049264?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1096,23 +1096,27 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>L'Occitane</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Praktikum (m/w/d) Trade Marketing</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Friedrichstadt, Düsseldorf</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F14" t="n">
         <v>6</v>
       </c>
-      <c r="G14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1120,7 +1124,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1131,7 +1135,7 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5842049264?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1147,12 +1151,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Praktikum Brand Management (m/w/d)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -1160,7 +1164,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1181,7 +1185,7 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802899675?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1192,27 +1196,23 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>Nestle</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d)</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F16" t="n">
         <v>6</v>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1231,7 +1231,7 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899675?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1464,25 +1464,25 @@
     <row r="22">
       <c r="A22" t="inlineStr"/>
       <c r="B22" t="n">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>coty</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
+          <t>Praktikum Business Development &amp; Talent Partnerships (m/w/d)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Darmstadt, Hessen</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1503,32 +1503,32 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5851100606?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>P&amp;G</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum im B2B-Vertrieb &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
@@ -1538,7 +1538,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1549,7 +1549,7 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5851898375?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1560,21 +1560,21 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>markenbaumarkt24</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Talent Partnerships (m/w/d)</t>
+          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Feuersbach, Siegen</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
@@ -1584,7 +1584,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -1595,33 +1595,31 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5851100606?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>PARSA Haar- und Modeartikel GmbH</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Praktikum im B2B-Vertrieb &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
-        </is>
-      </c>
-      <c r="F25" t="n">
-        <v>5</v>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
@@ -1630,7 +1628,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -1641,33 +1639,31 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5851898375?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
       <c r="B26" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>markenbaumarkt24</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
+          <t>Praktikum Product Marketing (x/f/m)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Feuersbach, Siegen</t>
-        </is>
-      </c>
-      <c r="F26" t="n">
-        <v>2</v>
-      </c>
+          <t>Berlin, Berlin, Germany</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
@@ -1676,7 +1672,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -1687,23 +1683,23 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5842051017?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>PARSA Haar- und Modeartikel GmbH</t>
+          <t>Groß- &amp; Einzelhandel Karriere</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1720,7 +1716,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -1731,7 +1727,7 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
+          <t>https://www.adzuna.de/land/ad/5848300231?se=1ucgSzui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=BF61BDCA3F28DD382163849647345A68CC617C45</t>
         </is>
       </c>
     </row>
@@ -1742,17 +1738,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Praktikum Product Marketing (x/f/m)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F28" t="inlineStr"/>
@@ -1764,7 +1760,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -1775,7 +1771,7 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5842051017?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
         </is>
       </c>
     </row>
@@ -1786,7 +1782,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Groß- &amp; Einzelhandel Karriere</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1808,7 +1804,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -1819,7 +1815,7 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848300231?se=1ucgSzui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=BF61BDCA3F28DD382163849647345A68CC617C45</t>
+          <t>https://www.adzuna.de/land/ad/5849209692?se=qJaID2Kc8RGlrvMe-VN8Yg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B8E6A551D4E75B7916A5994DC13A8DA3451895D</t>
         </is>
       </c>
     </row>
@@ -1830,22 +1826,20 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Lidl Stiftung</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food in Neckarsulm</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F30" t="n">
-        <v>6</v>
-      </c>
+          <t>Hamburg, Deutschland</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
@@ -1854,7 +1848,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -1865,75 +1859,81 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813494719?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5859954968?se=avT3yguj8RGEeLI7Dotn4Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FEC8C1664463BB6D76B4F51C80D7BE9A67B3E95</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr"/>
-      <c r="B31" t="n">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="n">
         <v>69</v>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Hamburg, Deutschland</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr"/>
+      <c r="G31" s="2" t="inlineStr"/>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr"/>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/land/ad/5864785114?se=tDVxHrqm8RG47MvhImrnRA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=ABFCC49076160E6370E149C31FFE29D13C38563D</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr"/>
       <c r="B32" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr"/>
+          <t>Köln, Nordrhein-Westfalen</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>6</v>
+      </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
@@ -1942,7 +1942,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -1953,31 +1953,33 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5849209692?se=qJaID2Kc8RGlrvMe-VN8Yg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B8E6A551D4E75B7916A5994DC13A8DA3451895D</t>
+          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr"/>
       <c r="B33" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr"/>
+          <t>Köln, Nordrhein-Westfalen</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>6</v>
+      </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
@@ -1986,7 +1988,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -1997,7 +1999,7 @@
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5859954968?se=avT3yguj8RGEeLI7Dotn4Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FEC8C1664463BB6D76B4F51C80D7BE9A67B3E95</t>
+          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2013,7 +2015,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
+          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2024,7 +2026,11 @@
       <c r="F34" t="n">
         <v>6</v>
       </c>
-      <c r="G34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H34" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2043,7 +2049,7 @@
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2054,23 +2060,27 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F35" t="n">
         <v>6</v>
       </c>
-      <c r="G35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
       <c r="H35" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2089,46 +2099,40 @@
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="n">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
+          <t>Internship in Trade Marketing</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F36" t="n">
-        <v>6</v>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>DEU-Nordrhein-Westfalen-Köln</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -2139,38 +2143,32 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="n">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Bosch Thermotechnik GmbH</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Praktikum im internationalen Brand Management</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Wernau (Neckar), Esslingen (Kreis)</t>
-        </is>
-      </c>
-      <c r="F37" t="n">
-        <v>6</v>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2189,38 +2187,32 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5799981240?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="n">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
-        </is>
-      </c>
-      <c r="F38" t="n">
-        <v>6</v>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>2026-11-01</t>
-        </is>
-      </c>
+          <t>Altstadt, Düsseldorf</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2239,40 +2231,40 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr"/>
       <c r="B39" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Calypso Ventures GmbH</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Internship in Trade Marketing</t>
+          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>DEU-Nordrhein-Westfalen-Köln</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -2283,7 +2275,7 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
+          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2294,17 +2286,17 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
@@ -2327,7 +2319,7 @@
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2338,17 +2330,17 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Altstadt, Düsseldorf</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
@@ -2360,7 +2352,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -2371,51 +2363,55 @@
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr"/>
-      <c r="B42" t="n">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="n">
         <v>62</v>
       </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Calypso Ventures GmbH</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Berlin, Deutschland</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Exclusive Associates</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum im Sales &amp; Business Development – B2B (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Düsseltal, Düsseldorf</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr"/>
+      <c r="G42" s="2" t="inlineStr"/>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr"/>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5866225907?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2426,20 +2422,22 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>FC Viktoria 1889 Berlin Frauen-Fußball GmbH</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>PRAKTIKUM // Business Development - In 3 Minuten erfolgreich bewerben</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr"/>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>3</v>
+      </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
@@ -2448,7 +2446,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -2459,7 +2457,7 @@
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5856283303?se=PMRjVxmh8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0E222C24DC5860DC4AEB24D8BB5E4CB04740A32C</t>
         </is>
       </c>
     </row>
@@ -2470,17 +2468,17 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>montamo GmbH</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
@@ -2492,7 +2490,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -2503,7 +2501,7 @@
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5856889494?se=1M-3UDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=471483726C1FC3DB660B48A5B3DEDE0DC1A4DC20</t>
         </is>
       </c>
     </row>
@@ -2514,22 +2512,20 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>FC Viktoria 1889 Berlin Frauen-Fußball GmbH</t>
+          <t>montamo GmbH</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>PRAKTIKUM // Business Development - In 3 Minuten erfolgreich bewerben</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F45" t="n">
-        <v>3</v>
-      </c>
+          <t>Wedding, Berlin</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
@@ -2538,7 +2534,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -2549,28 +2545,28 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5856283303?se=PMRjVxmh8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0E222C24DC5860DC4AEB24D8BB5E4CB04740A32C</t>
+          <t>https://www.adzuna.de/details/5857559039?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr"/>
       <c r="B46" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>montamo GmbH</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Retail Marketing | Fashion und Sport-Marken (w/m/d)</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F46" t="inlineStr"/>
@@ -2593,28 +2589,28 @@
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5856889494?se=1M-3UDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=471483726C1FC3DB660B48A5B3DEDE0DC1A4DC20</t>
+          <t>https://www.adzuna.de/land/ad/5858188456?se=HMKESTui8RGfx5bEd-nhPg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=86B24D9EAAAA2322A41661C360015255B004809E</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr"/>
       <c r="B47" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>montamo GmbH</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Retail Marketing | Fashion und Sport-Marken (w/m/d)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F47" t="inlineStr"/>
@@ -2626,7 +2622,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -2637,7 +2633,7 @@
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5857559039?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5860650076?se=EGcET6Oj8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=E6646A9A107DD9C83D248D81843D6570367335AD</t>
         </is>
       </c>
     </row>
@@ -2658,7 +2654,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Hamburg-Altstadt, Hamburg</t>
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
@@ -2670,7 +2666,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -2681,23 +2677,23 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5858188456?se=HMKESTui8RGfx5bEd-nhPg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=86B24D9EAAAA2322A41661C360015255B004809E</t>
+          <t>https://www.adzuna.de/details/5860355819?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr"/>
       <c r="B49" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Praktikum Retail Marketing | Fashion und Sport-Marken (w/m/d)</t>
+          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2714,7 +2710,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -2725,28 +2721,28 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5860650076?se=EGcET6Oj8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=E6646A9A107DD9C83D248D81843D6570367335AD</t>
+          <t>https://www.adzuna.de/land/ad/5848400955?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=4E59A334AC360616EAEAAC474F72A07451A7C624</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr"/>
       <c r="B50" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Praktikum Retail Marketing | Fashion und Sport-Marken (w/m/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Hamburg-Altstadt, Hamburg</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F50" t="inlineStr"/>
@@ -2758,7 +2754,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -2769,7 +2765,7 @@
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5860355819?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5848409009?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5C62DDCDA5E03F77D6089CD03CFA1D966DF15C96</t>
         </is>
       </c>
     </row>
@@ -2785,7 +2781,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2802,7 +2798,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -2813,7 +2809,7 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848400955?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=4E59A334AC360616EAEAAC474F72A07451A7C624</t>
+          <t>https://www.adzuna.de/land/ad/5861203670?se=hvkm4GOk8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD0ED2E271738C13EE6613442755CC0DE68C0F5A</t>
         </is>
       </c>
     </row>
@@ -2824,12 +2820,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>Nahrungs- &amp; Genussmittel Karriere</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2846,7 +2842,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -2857,7 +2853,7 @@
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848409009?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5C62DDCDA5E03F77D6089CD03CFA1D966DF15C96</t>
+          <t>https://www.adzuna.de/land/ad/5848308031?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=C04FAD6E90B5FCF47A6B81E4A697BA781ADC04AF</t>
         </is>
       </c>
     </row>
@@ -2868,12 +2864,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>Nahrungs- &amp; Genussmittel Karriere</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2890,7 +2886,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -2901,7 +2897,7 @@
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5861203670?se=hvkm4GOk8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD0ED2E271738C13EE6613442755CC0DE68C0F5A</t>
+          <t>https://www.adzuna.de/land/ad/5851105442?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8F6135545B7E9C415844F10F4AF49C0BFA63A4B2</t>
         </is>
       </c>
     </row>
@@ -2917,7 +2913,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2945,7 +2941,7 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848308031?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=C04FAD6E90B5FCF47A6B81E4A697BA781ADC04AF</t>
+          <t>https://www.adzuna.de/land/ad/5848347180?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8A3F28529B6340B7DCCD5131E2C4472FBD8CA361</t>
         </is>
       </c>
     </row>
@@ -2961,7 +2957,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2989,7 +2985,7 @@
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5851105442?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8F6135545B7E9C415844F10F4AF49C0BFA63A4B2</t>
+          <t>https://www.adzuna.de/land/ad/5848315177?se=nioaTDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B01A57BB52C4BDBB1DF6554A4A21C913096E1D0</t>
         </is>
       </c>
     </row>
@@ -3005,7 +3001,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -3033,7 +3029,7 @@
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848347180?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8A3F28529B6340B7DCCD5131E2C4472FBD8CA361</t>
+          <t>https://www.adzuna.de/land/ad/5848325009?se=nioaTDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8D26762D834367B41A848A3D14A62E41FD573B9B</t>
         </is>
       </c>
     </row>
@@ -3044,12 +3040,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Nahrungs- &amp; Genussmittel Karriere</t>
+          <t>P&amp;G</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -3066,7 +3062,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -3077,7 +3073,7 @@
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848315177?se=nioaTDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B01A57BB52C4BDBB1DF6554A4A21C913096E1D0</t>
+          <t>https://www.adzuna.de/details/5681669004?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3088,12 +3084,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Nahrungs- &amp; Genussmittel Karriere</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -3110,7 +3106,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
@@ -3121,7 +3117,7 @@
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848325009?se=nioaTDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8D26762D834367B41A848A3D14A62E41FD573B9B</t>
+          <t>https://www.adzuna.de/land/ad/5848363308?se=OLEhDWKc8RGNPOjEPgN71g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=60107C204BD9BC811A91BB2CBB46D624738C18B4</t>
         </is>
       </c>
     </row>
@@ -3137,7 +3133,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -3154,7 +3150,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -3165,7 +3161,7 @@
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848363308?se=OLEhDWKc8RGNPOjEPgN71g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=60107C204BD9BC811A91BB2CBB46D624738C18B4</t>
+          <t>https://www.adzuna.de/land/ad/5851125720?se=InV_50-g8RGMGcGGm7sUnA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=7C64FF6DD3C490D2F3D0F3435DB5EA282FEC5BCD</t>
         </is>
       </c>
     </row>
@@ -3181,7 +3177,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -3198,7 +3194,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
@@ -3209,7 +3205,7 @@
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5851125720?se=InV_50-g8RGMGcGGm7sUnA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=7C64FF6DD3C490D2F3D0F3435DB5EA282FEC5BCD</t>
+          <t>https://www.adzuna.de/land/ad/5858349551?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1A4BC151031E238D2948A5C0796DC467B8176359</t>
         </is>
       </c>
     </row>
@@ -3220,12 +3216,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Picnic</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Category Management Praktikum (m/w/d)</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -3242,7 +3238,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -3253,35 +3249,37 @@
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5858349551?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=1A4BC151031E238D2948A5C0796DC467B8176359</t>
+          <t>https://www.adzuna.de/details/5759088383?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr"/>
       <c r="B62" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>coty</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
+          <t>Marketing Intern - Trade Marketing</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>MILAN</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr"/>
+          <t>Darmstadt, Hessen</t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v>6</v>
+      </c>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3297,7 +3295,7 @@
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
+          <t>https://www.adzuna.de/details/5790418556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3308,29 +3306,29 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Wonder Natural GmbH</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
+          <t>VM &amp; Wholesale Trade Marketing Trainee</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
@@ -3341,28 +3339,28 @@
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/VM---Wholesale-Trade-Marketing-Trainee_JR132215</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr"/>
       <c r="B64" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Upsters Energy GmbH</t>
+          <t>Wonder Natural GmbH</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (w/m/d) | Startup</t>
+          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F64" t="inlineStr"/>
@@ -3374,7 +3372,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
@@ -3385,7 +3383,7 @@
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3406,7 +3404,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F65" t="inlineStr"/>
@@ -3429,33 +3427,31 @@
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957389?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr"/>
       <c r="B66" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>THE VERSE Ventures</t>
+          <t>Upsters Energy GmbH</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Praktikum im Business Development (w/m/d) | Startup</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
-        </is>
-      </c>
-      <c r="F66" t="n">
-        <v>6</v>
-      </c>
+          <t>Altstadt, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
         <is>
@@ -3475,31 +3471,33 @@
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804542553?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr"/>
       <c r="B67" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Abrio</t>
+          <t>THE VERSE Ventures</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr"/>
+          <t>Berlin, Deutschland</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>6</v>
+      </c>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
         <is>
@@ -3519,7 +3517,7 @@
       <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5780534752?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3530,17 +3528,17 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Groß- &amp; Einzelhandel Karriere</t>
+          <t>Abrio</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
+          <t>Praktikum im UX/UI Design für E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F68" t="inlineStr"/>
@@ -3552,7 +3550,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -3563,7 +3561,7 @@
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848296401?se=lphMSjui8RGhLffPfv7Txw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CDA6039E4CB2826923EB7E2E7ECB163DB4CFE919</t>
+          <t>https://www.adzuna.de/details/5675505079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3574,7 +3572,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Lidl Stiftung &amp; Co. KG</t>
+          <t>Groß- &amp; Einzelhandel Karriere</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -3596,7 +3594,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -3607,7 +3605,7 @@
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
+          <t>https://www.adzuna.de/land/ad/5848296401?se=lphMSjui8RGhLffPfv7Txw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CDA6039E4CB2826923EB7E2E7ECB163DB4CFE919</t>
         </is>
       </c>
     </row>
@@ -3618,12 +3616,12 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Marc O'Polo</t>
+          <t>Lidl Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
+          <t>Praktikum Marketing International - Product Content &amp; Packaging Non Food</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3632,11 +3630,7 @@
         </is>
       </c>
       <c r="F70" t="inlineStr"/>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
+      <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3644,7 +3638,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -3655,7 +3649,7 @@
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5851953335?se=FiG3lvOd8RG1ZOZIEyO4Fw&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=F4371871A1D89A69EB1819E9C78C7A66AE16AE6B</t>
         </is>
       </c>
     </row>
@@ -3666,21 +3660,25 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>Marc O'Polo</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Praktikum Marketing (m/w/d)</t>
+          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
-      <c r="G71" t="inlineStr"/>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
       <c r="H71" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3699,7 +3697,7 @@
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899691?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5801857079?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3710,7 +3708,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -3720,14 +3718,14 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -3743,7 +3741,7 @@
       <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
+          <t>https://www.adzuna.de/details/5802899691?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -3759,7 +3757,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Sales (m/w/d)</t>
+          <t>Praktikum Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3776,7 +3774,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -3787,7 +3785,7 @@
       <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-&amp;-Sales-%28mwd%29-60329/1425985633/</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-%28mwd%29-60329/1404395733/</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3801,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Praktikum Produktmarketing (m/w/d)</t>
+          <t>Praktikum Marketing &amp; Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3820,7 +3818,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -3831,40 +3829,40 @@
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Produktmarketing-%28mwd%29-60329/1431039933/</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Marketing-&amp;-Sales-%28mwd%29-60329/1425985633/</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr"/>
       <c r="B75" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d) - In 3 Minuten erfolgreich bewerben</t>
+          <t>Praktikum Produktmarketing (m/w/d)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
@@ -3875,7 +3873,7 @@
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5856295760?se=VqemWBmh8RGCZtbxFymUqg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A0E45C661705BA9D9ECDDCCACDFEEB182D4173F7</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Produktmarketing-%28mwd%29-60329/1431039933/</t>
         </is>
       </c>
     </row>
@@ -3886,12 +3884,12 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Handwerk Karriere</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d) - In 3 Minuten erfolgreich bewerben</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -3908,7 +3906,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -3919,7 +3917,7 @@
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5859734477?se=2BMB0Auj8RGxSf1iGXKoQA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8912F76B99550481E2615DFD8E07B2F6745D01A7</t>
+          <t>https://www.adzuna.de/land/ad/5856295760?se=VqemWBmh8RGCZtbxFymUqg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A0E45C661705BA9D9ECDDCCACDFEEB182D4173F7</t>
         </is>
       </c>
     </row>
@@ -3930,27 +3928,21 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>LIGANOVA GmbH</t>
+          <t>Handwerk Karriere</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Praktikum Buying (all genders) – September 2026</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Mitte, Stuttgart</t>
-        </is>
-      </c>
-      <c r="F77" t="n">
-        <v>6</v>
-      </c>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -3958,7 +3950,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -3969,7 +3961,7 @@
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5849630691?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5859734477?se=2BMB0Auj8RGxSf1iGXKoQA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8912F76B99550481E2615DFD8E07B2F6745D01A7</t>
         </is>
       </c>
     </row>
@@ -3980,7 +3972,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>LIGANOVA I Karriere</t>
+          <t>LIGANOVA GmbH</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -4008,7 +4000,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -4019,7 +4011,7 @@
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5852669596?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5849630691?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4030,29 +4022,35 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>LIGANOVA I Karriere</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Marketing &amp; Merchandising Assistant Trainee</t>
+          <t>Praktikum Buying (all genders) – September 2026</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>MILAN</t>
-        </is>
-      </c>
-      <c r="F79" t="inlineStr"/>
-      <c r="G79" t="inlineStr"/>
+          <t>Mitte, Stuttgart</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>6</v>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -4063,7 +4061,7 @@
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
+          <t>https://www.adzuna.de/details/5852669596?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4079,7 +4077,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Marketing and Merchandising Assistant Trainee</t>
+          <t>Marketing &amp; Merchandising Assistant Trainee</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -4107,7 +4105,7 @@
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing-and-Merchandising-Assistant-Trainee_JR128690</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing---Merchandising-Assistant-Trainee_JR131638-1</t>
         </is>
       </c>
     </row>
@@ -4118,29 +4116,29 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Wonder Natural GmbH</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
+          <t>Marketing and Merchandising Assistant Trainee</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>MILAN</t>
         </is>
       </c>
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -4151,28 +4149,28 @@
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing-and-Merchandising-Assistant-Trainee_JR128690</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr"/>
       <c r="B82" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Digitalagenten</t>
+          <t>Wonder Natural GmbH</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Charlottenburg, Berlin</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F82" t="inlineStr"/>
@@ -4184,7 +4182,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -4195,7 +4193,7 @@
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804948828?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4206,17 +4204,17 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>HardyTec Industries UG haftungsbeschränkt</t>
+          <t>Digitalagenten</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Business Development</t>
+          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Büderich, Meerbusch</t>
+          <t>Charlottenburg, Berlin</t>
         </is>
       </c>
       <c r="F83" t="inlineStr"/>
@@ -4228,7 +4226,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -4239,7 +4237,7 @@
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5848139968?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804948828?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4250,17 +4248,17 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>LIMITD by Wunderproducts GmbH</t>
+          <t>HardyTec Industries UG haftungsbeschränkt</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Praktikum Marketing &amp; Business Development</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Kreuzberg, Berlin</t>
+          <t>Büderich, Meerbusch</t>
         </is>
       </c>
       <c r="F84" t="inlineStr"/>
@@ -4272,7 +4270,7 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
@@ -4283,7 +4281,7 @@
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5848139968?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4294,25 +4292,21 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers GmbH WPG</t>
+          <t>LIMITD by Wunderproducts GmbH</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
+          <t>Praktikum - Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Kreuzberg, Berlin</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
+      <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4331,7 +4325,7 @@
       <c r="K85" t="inlineStr"/>
       <c r="L85" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4342,12 +4336,12 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>SERVICEPLAN Gruppe</t>
+          <t>PricewaterhouseCoopers GmbH WPG</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Sales (Marketing / New Business) (all genders)</t>
+          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -4358,7 +4352,7 @@
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -4368,7 +4362,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -4379,7 +4373,7 @@
       <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4390,21 +4384,25 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>WirWinzer</t>
+          <t>SERVICEPLAN Gruppe</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Praktikum Business Development Weinhandel (all genders)</t>
+          <t>Praktikum Business Development &amp; Sales (Marketing / New Business) (all genders)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F87" t="inlineStr"/>
-      <c r="G87" t="inlineStr"/>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H87" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4412,7 +4410,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -4423,28 +4421,28 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr"/>
       <c r="B88" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>WirWinzer</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Praktikum Inside Sales (x/f/m)</t>
+          <t>Praktikum Business Development Weinhandel (all genders)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F88" t="inlineStr"/>
@@ -4456,7 +4454,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -4467,7 +4465,7 @@
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7799489003</t>
+          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4478,29 +4476,29 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Internship - High Jewelry Business Development Assistant</t>
+          <t>Praktikum Inside Sales (x/f/m)</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -4511,7 +4509,7 @@
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7799489003</t>
         </is>
       </c>
     </row>
@@ -4522,35 +4520,29 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>RÖDL</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
+          <t>Internship - High Jewelry Business Development Assistant</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Stuttgart, Baden-Württemberg</t>
-        </is>
-      </c>
-      <c r="F90" t="n">
-        <v>6</v>
-      </c>
-      <c r="G90" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -4561,32 +4553,38 @@
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5854352066?se=9tCS70-g8RGkr9xW060fUg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DBAD57A9DC2B84BE2128168013A758C1F47DCD27</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr"/>
       <c r="B91" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Brand Trust</t>
+          <t>RÖDL</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
+          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Gleißbühl, Nürnberg</t>
-        </is>
-      </c>
-      <c r="F91" t="inlineStr"/>
-      <c r="G91" t="inlineStr"/>
+          <t>Stuttgart, Baden-Württemberg</t>
+        </is>
+      </c>
+      <c r="F91" t="n">
+        <v>6</v>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H91" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4594,7 +4592,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -4605,99 +4603,99 @@
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
+          <t>https://www.adzuna.de/land/ad/5854352066?se=9tCS70-g8RGkr9xW060fUg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DBAD57A9DC2B84BE2128168013A758C1F47DCD27</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr"/>
+      <c r="B92" t="n">
+        <v>49</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Brand Trust</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Gleißbühl, Nürnberg</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr"/>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr"/>
+      <c r="L92" t="inlineStr">
+        <is>
           <t>https://www.adzuna.de/details/5669847401?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" s="2" t="inlineStr">
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
         <is>
           <t>NEU</t>
         </is>
       </c>
-      <c r="B92" s="2" t="n">
+      <c r="B93" s="2" t="n">
         <v>49</v>
       </c>
-      <c r="C92" s="2" t="inlineStr">
+      <c r="C93" s="2" t="inlineStr">
         <is>
           <t>Clarios Germany GmbH &amp; Co. KG</t>
         </is>
       </c>
-      <c r="D92" s="2" t="inlineStr">
+      <c r="D93" s="2" t="inlineStr">
         <is>
           <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
         </is>
       </c>
-      <c r="E92" s="2" t="inlineStr">
+      <c r="E93" s="2" t="inlineStr">
         <is>
           <t>Hannover, Region Hannover (Kreis)</t>
         </is>
       </c>
-      <c r="F92" s="2" t="inlineStr"/>
-      <c r="G92" s="2" t="inlineStr"/>
-      <c r="H92" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I92" s="2" t="inlineStr">
+      <c r="F93" s="2" t="inlineStr"/>
+      <c r="G93" s="2" t="inlineStr"/>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I93" s="2" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="J92" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K92" s="2" t="inlineStr"/>
-      <c r="L92" s="2" t="inlineStr">
+      <c r="J93" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K93" s="2" t="inlineStr"/>
+      <c r="L93" s="2" t="inlineStr">
         <is>
           <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr"/>
-      <c r="B93" t="n">
-        <v>49</v>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>Codeso Living</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>Unterbilk, Düsseldorf</t>
-        </is>
-      </c>
-      <c r="F93" t="inlineStr"/>
-      <c r="G93" t="inlineStr"/>
-      <c r="H93" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I93" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
-      </c>
-      <c r="J93" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K93" t="inlineStr"/>
-      <c r="L93" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4708,15 +4706,19 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Codeso Living</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr"/>
+          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Unterbilk, Düsseldorf</t>
+        </is>
+      </c>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
@@ -4726,7 +4728,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
@@ -4737,7 +4739,7 @@
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
+          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4748,19 +4750,15 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Praktikum B2B Event Marketing (x/f/m)</t>
-        </is>
-      </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>Berlin, Berlin, Germany</t>
-        </is>
-      </c>
+          <t>Marketing Intern - Trade Marketing</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
@@ -4770,7 +4768,7 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -4781,7 +4779,7 @@
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7820455003</t>
+          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4795,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Go To Market Strategy Hospitals (x/f/m)</t>
+          <t>Praktikum B2B Event Marketing (x/f/m)</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -4814,7 +4812,7 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
@@ -4825,7 +4823,7 @@
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7971471003</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7820455003</t>
         </is>
       </c>
     </row>
@@ -4836,17 +4834,17 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Genuine Parts Company</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Praktikum Category Management (m/w/d)</t>
+          <t>Go To Market Strategy Hospitals (x/f/m)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Münster, Nordrhein-Westfalen</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -4858,7 +4856,7 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
@@ -4869,7 +4867,7 @@
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853760166?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7971471003</t>
         </is>
       </c>
     </row>
@@ -4880,17 +4878,17 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>Genuine Parts Company</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
+          <t>Praktikum Category Management (m/w/d)</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Benrath, Düsseldorf</t>
+          <t>Münster, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F98" t="inlineStr"/>
@@ -4902,7 +4900,7 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
@@ -4913,7 +4911,7 @@
       <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5853760166?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4924,17 +4922,17 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Henkel</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
+          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Schwabing-Freimann, München</t>
+          <t>Benrath, Düsseldorf</t>
         </is>
       </c>
       <c r="F99" t="inlineStr"/>
@@ -4946,7 +4944,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
@@ -4957,7 +4955,7 @@
       <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4968,24 +4966,24 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>DEU-Bayern-Unterhaching</t>
+          <t>Schwabing-Freimann, München</t>
         </is>
       </c>
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -5001,7 +4999,7 @@
       <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
+          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5012,24 +5010,24 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>DEU-Bayern-Unterhaching</t>
         </is>
       </c>
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr"/>
       <c r="H101" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -5045,51 +5043,55 @@
       <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" t="inlineStr"/>
-      <c r="B102" t="n">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="n">
         <v>49</v>
       </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
-        </is>
-      </c>
-      <c r="D102" t="inlineStr">
-        <is>
-          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
-        </is>
-      </c>
-      <c r="F102" t="inlineStr"/>
-      <c r="G102" t="inlineStr"/>
-      <c r="H102" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I102" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J102" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K102" t="inlineStr"/>
-      <c r="L102" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>Mars</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>2 Standorte</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr"/>
+      <c r="G102" s="2" t="inlineStr"/>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
+          <t>fmcg</t>
+        </is>
+      </c>
+      <c r="I102" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="J102" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K102" s="2" t="inlineStr"/>
+      <c r="L102" s="2" t="inlineStr">
+        <is>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
         </is>
       </c>
     </row>
@@ -5100,17 +5102,17 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F103" t="inlineStr"/>
@@ -5133,7 +5135,7 @@
       <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
+          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5149,7 +5151,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -5177,7 +5179,7 @@
       <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
+          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
         </is>
       </c>
     </row>
@@ -5188,17 +5190,17 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F105" t="inlineStr"/>
@@ -5221,7 +5223,7 @@
       <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
         </is>
       </c>
     </row>
@@ -5232,17 +5234,17 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>RAG</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Gornhofen, Ravensburg</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F106" t="inlineStr"/>
@@ -5254,7 +5256,7 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J106" t="inlineStr">
@@ -5265,76 +5267,72 @@
       <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
         </is>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B107" s="2" t="n">
-        <v>48</v>
-      </c>
-      <c r="C107" s="2" t="inlineStr">
-        <is>
-          <t>Konzernzentrale</t>
-        </is>
-      </c>
-      <c r="D107" s="2" t="inlineStr">
-        <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E107" s="2" t="inlineStr">
-        <is>
-          <t>Braunsfeld, Köln</t>
-        </is>
-      </c>
-      <c r="F107" s="2" t="inlineStr"/>
-      <c r="G107" s="2" t="inlineStr"/>
-      <c r="H107" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I107" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="J107" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K107" s="2" t="inlineStr"/>
-      <c r="L107" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5864351176?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="A107" t="inlineStr"/>
+      <c r="B107" t="n">
+        <v>49</v>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Procter &amp; Gamble</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr"/>
+      <c r="G107" t="inlineStr"/>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr"/>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr"/>
       <c r="B108" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>REWE Group</t>
+          <t>RAG</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Gornhofen, Ravensburg</t>
         </is>
       </c>
       <c r="F108" t="inlineStr"/>
@@ -5346,7 +5344,7 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
@@ -5357,51 +5355,55 @@
       <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5712965755?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="109">
-      <c r="A109" t="inlineStr"/>
-      <c r="B109" t="n">
-        <v>46</v>
-      </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>SUPA - Sport Und Party App</t>
-        </is>
-      </c>
-      <c r="D109" t="inlineStr">
-        <is>
-          <t>Business Development Praktikum</t>
-        </is>
-      </c>
-      <c r="E109" t="inlineStr">
-        <is>
-          <t>Köln, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F109" t="inlineStr"/>
-      <c r="G109" t="inlineStr"/>
-      <c r="H109" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I109" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J109" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K109" t="inlineStr"/>
-      <c r="L109" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>Konzernzentrale</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>Braunsfeld, Köln</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr"/>
+      <c r="G109" s="2" t="inlineStr"/>
+      <c r="H109" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I109" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="J109" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K109" s="2" t="inlineStr"/>
+      <c r="L109" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5864351176?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5422,7 +5424,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Altstadt-Nord, Köln</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F110" t="inlineStr"/>
@@ -5445,28 +5447,28 @@
       <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr"/>
       <c r="B111" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Devoteam G Cloud Germany</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt-Nord, Köln</t>
         </is>
       </c>
       <c r="F111" t="inlineStr"/>
@@ -5489,7 +5491,7 @@
       <c r="K111" t="inlineStr"/>
       <c r="L111" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811135653?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5963,7 +5965,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C4" t="n">
         <v>89</v>
@@ -6013,7 +6015,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="C6" t="n">
         <v>84</v>
@@ -6038,7 +6040,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C7" t="n">
         <v>84</v>
@@ -6063,7 +6065,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="C8" t="n">
         <v>84</v>
@@ -6088,7 +6090,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C9" t="n">
         <v>84</v>
@@ -6121,7 +6123,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
@@ -6146,7 +6148,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C11" t="n">
         <v>84</v>
@@ -6179,7 +6181,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C12" t="n">
         <v>84</v>
@@ -6204,7 +6206,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C13" t="n">
         <v>84</v>
@@ -6229,7 +6231,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C14" t="n">
         <v>84</v>
@@ -6254,7 +6256,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C15" t="n">
         <v>84</v>
@@ -6304,7 +6306,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C17" t="n">
         <v>84</v>
@@ -6329,7 +6331,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C18" t="n">
         <v>80</v>
@@ -6354,7 +6356,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C19" t="n">
         <v>79</v>
@@ -6429,7 +6431,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C22" t="n">
         <v>78</v>
@@ -6462,7 +6464,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C23" t="n">
         <v>78</v>
@@ -6487,7 +6489,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C24" t="n">
         <v>78</v>
@@ -6512,7 +6514,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C25" t="n">
         <v>74</v>
@@ -6545,7 +6547,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C26" t="n">
         <v>74</v>
@@ -6570,7 +6572,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C27" t="n">
         <v>74</v>
@@ -6595,7 +6597,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C28" t="n">
         <v>73</v>
@@ -6653,7 +6655,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C30" t="n">
         <v>73</v>
@@ -6678,7 +6680,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C31" t="n">
         <v>72</v>
@@ -6703,7 +6705,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C32" t="n">
         <v>72</v>
@@ -6778,7 +6780,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C35" t="n">
         <v>68</v>
@@ -6853,7 +6855,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C38" t="n">
         <v>66</v>
@@ -6878,7 +6880,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C39" t="n">
         <v>65</v>
@@ -6903,7 +6905,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C40" t="n">
         <v>64</v>
@@ -6928,7 +6930,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C41" t="n">
         <v>62</v>
@@ -6953,7 +6955,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C42" t="n">
         <v>62</v>
@@ -6986,7 +6988,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C43" t="n">
         <v>62</v>
@@ -7011,7 +7013,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C44" t="n">
         <v>59</v>
@@ -7061,7 +7063,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C46" t="n">
         <v>57</v>
@@ -7094,7 +7096,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C47" t="n">
         <v>56</v>
@@ -7119,7 +7121,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C48" t="n">
         <v>55</v>
@@ -7194,7 +7196,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="C51" t="n">
         <v>53</v>
@@ -7219,7 +7221,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C52" t="n">
         <v>53</v>
@@ -7269,7 +7271,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C54" t="n">
         <v>52</v>
@@ -7294,7 +7296,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C55" t="n">
         <v>52</v>
@@ -7344,7 +7346,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C57" t="n">
         <v>51</v>
@@ -7394,7 +7396,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C59" t="n">
         <v>50</v>
@@ -7419,7 +7421,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C60" t="n">
         <v>49</v>
@@ -7444,7 +7446,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C61" t="n">
         <v>49</v>
@@ -7469,7 +7471,7 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C62" t="n">
         <v>49</v>
@@ -7519,7 +7521,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C64" t="n">
         <v>49</v>
@@ -7544,7 +7546,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C65" t="n">
         <v>49</v>
@@ -7569,7 +7571,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C66" t="n">
         <v>49</v>
@@ -7594,7 +7596,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C67" t="n">
         <v>49</v>
@@ -7815,32 +7817,32 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>AUTO1 Global Services SE &amp; Co. KG</t>
+          <t>Konzernzentrale</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C76" t="n">
         <v>48</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (d/m/w)</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-01</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>SHAVENT - ARA Sustainable Products</t>
+          <t>AUTO1 Global Services SE &amp; Co. KG</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -7851,7 +7853,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Praktikum Business Development in nachhaltigem Start-Up (w/m/d) Remote in DE</t>
+          <t>Praktikum Business Development (d/m/w)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr"/>
@@ -7865,7 +7867,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CTG Consulting</t>
+          <t>SHAVENT - ARA Sustainable Products</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -7876,7 +7878,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Praktikum Sales/Business Development // Hamburg oder Berlin</t>
+          <t>Praktikum Business Development in nachhaltigem Start-Up (w/m/d) Remote in DE</t>
         </is>
       </c>
       <c r="E78" t="inlineStr"/>
@@ -7890,7 +7892,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Dronesperhour</t>
+          <t>CTG Consulting</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -7901,7 +7903,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development eines Startups (m/w/d)</t>
+          <t>Praktikum Sales/Business Development // Hamburg oder Berlin</t>
         </is>
       </c>
       <c r="E79" t="inlineStr"/>
@@ -7915,7 +7917,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>SINN Power</t>
+          <t>Dronesperhour</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -7926,7 +7928,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Praktikum im AI Business Development (m/w/d)</t>
+          <t>Praktikum im Business Development eines Startups (m/w/d)</t>
         </is>
       </c>
       <c r="E80" t="inlineStr"/>
@@ -7940,7 +7942,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>innpuls</t>
+          <t>SINN Power</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -7951,7 +7953,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Praktikum im AI Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E81" t="inlineStr"/>
@@ -7965,7 +7967,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Amolina</t>
+          <t>innpuls</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -7976,7 +7978,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E82" t="inlineStr"/>
@@ -7990,7 +7992,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Konzernzentrale</t>
+          <t>Amolina</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -8001,14 +8003,14 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
         </is>
       </c>
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
@@ -8019,7 +8021,7 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C84" t="n">
         <v>46</v>
@@ -8044,7 +8046,7 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C85" t="n">
         <v>45</v>

</xml_diff>

<commit_message>
Lauf 2026-09-04 10:46 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$124</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$102</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -754,50 +754,46 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="n">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="n">
         <v>84</v>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Hamburg-Altstadt, Hamburg</t>
         </is>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="F7" t="n">
         <v>6</v>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
         <is>
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
         <is>
           <t>https://www.adzuna.de/details/5865920988?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
@@ -902,29 +898,27 @@
     <row r="10">
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="n">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management National</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Au-Haidhausen, München</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>6</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -943,36 +937,34 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805399065?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Ferrero</t>
+          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikum Brand Management National</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F11" t="n">
-        <v>6</v>
-      </c>
+          <t>Au-Haidhausen, München</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -993,7 +985,7 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805399065?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1001,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1022,7 +1014,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1043,7 +1035,7 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5799961458?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1059,7 +1051,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1070,7 +1062,11 @@
       <c r="F13" t="n">
         <v>6</v>
       </c>
-      <c r="G13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1089,7 +1085,7 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5799961458?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1914,48 +1910,44 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="n">
+      <c r="A32" t="inlineStr"/>
+      <c r="B32" t="n">
         <v>69</v>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr"/>
-      <c r="G32" s="2" t="inlineStr"/>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I32" s="2" t="inlineStr">
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
         <is>
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="J32" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K32" s="2" t="inlineStr"/>
-      <c r="L32" s="2" t="inlineStr">
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr">
         <is>
           <t>https://www.adzuna.de/land/ad/5864785114?se=tDVxHrqm8RG47MvhImrnRA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=ABFCC49076160E6370E149C31FFE29D13C38563D</t>
         </is>
@@ -2514,48 +2506,44 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="n">
+      <c r="A45" t="inlineStr"/>
+      <c r="B45" t="n">
         <v>62</v>
       </c>
-      <c r="C45" s="2" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>Exclusive Associates</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>Praktikum im Sales &amp; Business Development – B2B (m/w/d)</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr"/>
-      <c r="G45" s="2" t="inlineStr"/>
-      <c r="H45" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I45" s="2" t="inlineStr">
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
         <is>
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="J45" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K45" s="2" t="inlineStr"/>
-      <c r="L45" s="2" t="inlineStr">
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr">
         <is>
           <t>https://www.adzuna.de/details/5866225907?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
@@ -5290,48 +5278,44 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B107" s="2" t="n">
+      <c r="A107" t="inlineStr"/>
+      <c r="B107" t="n">
         <v>49</v>
       </c>
-      <c r="C107" s="2" t="inlineStr">
+      <c r="C107" t="inlineStr">
         <is>
           <t>Mars</t>
         </is>
       </c>
-      <c r="D107" s="2" t="inlineStr">
+      <c r="D107" t="inlineStr">
         <is>
           <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
         </is>
       </c>
-      <c r="E107" s="2" t="inlineStr">
+      <c r="E107" t="inlineStr">
         <is>
           <t>2 Standorte</t>
         </is>
       </c>
-      <c r="F107" s="2" t="inlineStr"/>
-      <c r="G107" s="2" t="inlineStr"/>
-      <c r="H107" s="2" t="inlineStr">
+      <c r="F107" t="inlineStr"/>
+      <c r="G107" t="inlineStr"/>
+      <c r="H107" t="inlineStr">
         <is>
           <t>fmcg</t>
         </is>
       </c>
-      <c r="I107" s="2" t="inlineStr">
+      <c r="I107" t="inlineStr">
         <is>
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="J107" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K107" s="2" t="inlineStr"/>
-      <c r="L107" s="2" t="inlineStr">
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr"/>
+      <c r="L107" t="inlineStr">
         <is>
           <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
         </is>
@@ -6097,7 +6081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G101"/>
+  <dimension ref="A1:G102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -6203,7 +6187,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C4" t="n">
         <v>89</v>
@@ -6253,7 +6237,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="C6" t="n">
         <v>84</v>
@@ -6278,7 +6262,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C7" t="n">
         <v>84</v>
@@ -6303,7 +6287,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="C8" t="n">
         <v>84</v>
@@ -6328,7 +6312,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C9" t="n">
         <v>84</v>
@@ -6361,7 +6345,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
@@ -6386,7 +6370,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C11" t="n">
         <v>84</v>
@@ -6419,7 +6403,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C12" t="n">
         <v>84</v>
@@ -6444,7 +6428,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C13" t="n">
         <v>84</v>
@@ -6469,7 +6453,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C14" t="n">
         <v>84</v>
@@ -6494,7 +6478,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C15" t="n">
         <v>84</v>
@@ -6565,22 +6549,30 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>32</v>
+        <v>93</v>
       </c>
       <c r="C18" t="n">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management National</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>successfactors</t>
+        </is>
+      </c>
       <c r="G18" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -6590,18 +6582,18 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Marc O'Polo</t>
+          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C19" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
+          <t>Praktikum Brand Management National</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
@@ -6615,18 +6607,18 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>EAT HAPPY GROUP</t>
+          <t>Marc O'Polo</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="C20" t="n">
         <v>79</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Praktikum Brand Marketing (m/w/d) Marketing · Köln</t>
+          <t>Praktikum Buying Retail &amp; eCom m/w/d</t>
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
@@ -6640,18 +6632,18 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Yogi Tea</t>
+          <t>EAT HAPPY GROUP</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C21" t="n">
         <v>79</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Praktikum im Marketing - Brand &amp; Product / mindestens 5 Monate</t>
+          <t>Praktikum Brand Marketing (m/w/d) Marketing · Köln</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
@@ -6665,30 +6657,22 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Ferrero</t>
+          <t>Yogi Tea</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>91</v>
+        <v>4</v>
       </c>
       <c r="C22" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>successfactors</t>
-        </is>
-      </c>
+          <t>Praktikum im Marketing - Brand &amp; Product / mindestens 5 Monate</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -6702,7 +6686,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C23" t="n">
         <v>78</v>
@@ -6727,7 +6711,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C24" t="n">
         <v>78</v>
@@ -6752,7 +6736,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C25" t="n">
         <v>74</v>
@@ -6785,7 +6769,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C26" t="n">
         <v>74</v>
@@ -6810,7 +6794,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C27" t="n">
         <v>74</v>
@@ -6835,7 +6819,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C28" t="n">
         <v>73</v>
@@ -6893,7 +6877,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C30" t="n">
         <v>73</v>
@@ -6918,7 +6902,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C31" t="n">
         <v>72</v>
@@ -6943,7 +6927,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C32" t="n">
         <v>72</v>
@@ -7018,7 +7002,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C35" t="n">
         <v>68</v>
@@ -7093,7 +7077,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C38" t="n">
         <v>66</v>
@@ -7118,7 +7102,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C39" t="n">
         <v>65</v>
@@ -7143,7 +7127,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C40" t="n">
         <v>64</v>
@@ -7168,7 +7152,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C41" t="n">
         <v>62</v>
@@ -7193,7 +7177,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C42" t="n">
         <v>62</v>
@@ -7226,7 +7210,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C43" t="n">
         <v>62</v>
@@ -7251,7 +7235,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C44" t="n">
         <v>59</v>
@@ -7301,7 +7285,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="C46" t="n">
         <v>57</v>
@@ -7334,7 +7318,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C47" t="n">
         <v>56</v>
@@ -7359,7 +7343,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C48" t="n">
         <v>55</v>
@@ -7434,7 +7418,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C51" t="n">
         <v>53</v>
@@ -7459,7 +7443,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C52" t="n">
         <v>53</v>
@@ -7509,7 +7493,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C54" t="n">
         <v>52</v>
@@ -7534,7 +7518,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C55" t="n">
         <v>52</v>
@@ -7634,7 +7618,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C59" t="n">
         <v>50</v>
@@ -7659,7 +7643,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C60" t="n">
         <v>49</v>
@@ -7684,7 +7668,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C61" t="n">
         <v>49</v>
@@ -7709,7 +7693,7 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C62" t="n">
         <v>49</v>
@@ -7759,7 +7743,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C64" t="n">
         <v>49</v>
@@ -7784,7 +7768,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C65" t="n">
         <v>49</v>
@@ -7809,7 +7793,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C66" t="n">
         <v>49</v>
@@ -7855,43 +7839,43 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>REWE Group</t>
+          <t>Clarios</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="C68" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
         </is>
       </c>
       <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-04</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Pflegia</t>
+          <t>REWE Group</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="C69" t="n">
         <v>48</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
@@ -7905,57 +7889,57 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Konzernzentrale</t>
+          <t>Pflegia</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C70" t="n">
         <v>48</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Werkia</t>
+          <t>Konzernzentrale</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C71" t="n">
         <v>48</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d) - Datenanalyse &amp; Automatisierung</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-01</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>paero</t>
+          <t>Werkia</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -7966,7 +7950,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/d) - Datenanalyse &amp; Automatisierung</t>
         </is>
       </c>
       <c r="E72" t="inlineStr"/>
@@ -7980,7 +7964,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Vivanta Gmbh</t>
+          <t>paero</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -7991,7 +7975,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr"/>
@@ -8005,7 +7989,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Vitolus</t>
+          <t>Vivanta Gmbh</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -8016,7 +8000,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr"/>
@@ -8030,7 +8014,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>GrantLift GmbH</t>
+          <t>Vitolus</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -8041,7 +8025,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
+          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr"/>
@@ -8055,7 +8039,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Otto Group one.O GmbH</t>
+          <t>GrantLift GmbH</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -8066,7 +8050,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Praktikum im Knowledge Management - Corporate Strategy (w/m/d)</t>
+          <t>Praktikant Business Development &amp; Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr"/>
@@ -8080,18 +8064,18 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>AUTO1 Global Services SE &amp; Co. KG</t>
+          <t>Otto Group one.O GmbH</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C77" t="n">
         <v>48</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (d/m/w)</t>
+          <t>Praktikum im Knowledge Management - Corporate Strategy (w/m/d)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr"/>
@@ -8105,7 +8089,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>SHAVENT - ARA Sustainable Products</t>
+          <t>AUTO1 Global Services SE &amp; Co. KG</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -8116,7 +8100,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Praktikum Business Development in nachhaltigem Start-Up (w/m/d) Remote in DE</t>
+          <t>Praktikum Business Development (d/m/w)</t>
         </is>
       </c>
       <c r="E78" t="inlineStr"/>
@@ -8130,7 +8114,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CTG Consulting</t>
+          <t>SHAVENT - ARA Sustainable Products</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -8141,7 +8125,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Praktikum Sales/Business Development // Hamburg oder Berlin</t>
+          <t>Praktikum Business Development in nachhaltigem Start-Up (w/m/d) Remote in DE</t>
         </is>
       </c>
       <c r="E79" t="inlineStr"/>
@@ -8155,7 +8139,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Dronesperhour</t>
+          <t>CTG Consulting</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -8166,7 +8150,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development eines Startups (m/w/d)</t>
+          <t>Praktikum Sales/Business Development // Hamburg oder Berlin</t>
         </is>
       </c>
       <c r="E80" t="inlineStr"/>
@@ -8180,7 +8164,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>SINN Power</t>
+          <t>Dronesperhour</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -8191,7 +8175,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Praktikum im AI Business Development (m/w/d)</t>
+          <t>Praktikum im Business Development eines Startups (m/w/d)</t>
         </is>
       </c>
       <c r="E81" t="inlineStr"/>
@@ -8205,7 +8189,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>innpuls</t>
+          <t>SINN Power</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -8216,7 +8200,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Praktikum im Sales / Business Development (m/w/d)</t>
+          <t>Praktikum im AI Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E82" t="inlineStr"/>
@@ -8230,7 +8214,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Amolina</t>
+          <t>innpuls</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -8241,7 +8225,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
+          <t>Praktikum im Sales / Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E83" t="inlineStr"/>
@@ -8255,18 +8239,18 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>Amolina</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>64</v>
+        <v>1</v>
       </c>
       <c r="C84" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Business Development &amp; Operations Praktikum im Startup (m/w/d)</t>
         </is>
       </c>
       <c r="E84" t="inlineStr"/>
@@ -8280,57 +8264,57 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>freudio</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>23</v>
+        <v>66</v>
       </c>
       <c r="C85" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>STARTPLATZ Gruppe</t>
+          <t>freudio</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="C86" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Sales (m/w/d) – STARTPLATZ</t>
+          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>spring.gate business consulting UG</t>
+          <t>STARTPLATZ Gruppe</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -8341,7 +8325,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development &amp; B2B Akquise (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Sales (m/w/d) – STARTPLATZ</t>
         </is>
       </c>
       <c r="E87" t="inlineStr"/>
@@ -8355,7 +8339,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>specter automation</t>
+          <t>spring.gate business consulting UG</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -8366,7 +8350,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Praktikum (M/W/D) im Business Development</t>
+          <t>Praktikum im Business Development &amp; B2B Akquise (m/w/d)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
@@ -8380,18 +8364,18 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Closd Kunststoffprodukte GmbH</t>
+          <t>specter automation</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C89" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Praktikum beim E-Commerce Startup Closd als Founders Associate (m/w/d)</t>
+          <t>Praktikum (M/W/D) im Business Development</t>
         </is>
       </c>
       <c r="E89" t="inlineStr"/>
@@ -8405,18 +8389,18 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Bosch Rexroth AG</t>
+          <t>Closd Kunststoffprodukte GmbH</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C90" t="n">
         <v>38</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Praktikum Business Development – Software Defined Business</t>
+          <t>Praktikum beim E-Commerce Startup Closd als Founders Associate (m/w/d)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr"/>
@@ -8430,7 +8414,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Weenect</t>
+          <t>Bosch Rexroth AG</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -8441,7 +8425,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d) – Markt DACH – Standort Brüssel</t>
+          <t>Praktikum Business Development – Software Defined Business</t>
         </is>
       </c>
       <c r="E91" t="inlineStr"/>
@@ -8455,18 +8439,18 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Lidl Dienstleistung GmbH &amp; Co. KG</t>
+          <t>Weenect</t>
         </is>
       </c>
       <c r="B92" t="n">
         <v>1</v>
       </c>
       <c r="C92" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
+          <t>Praktikum Business Development (m/w/d) – Markt DACH – Standort Brüssel</t>
         </is>
       </c>
       <c r="E92" t="inlineStr"/>
@@ -8480,18 +8464,18 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Drägerwerk AG &amp; Co. KGaA</t>
+          <t>Lidl Dienstleistung GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C93" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Praktikum New Business Development</t>
+          <t>Praktikum Omnichannel &amp; E-Commerce Strategie</t>
         </is>
       </c>
       <c r="E93" t="inlineStr"/>
@@ -8505,18 +8489,18 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Arteus Energy</t>
+          <t>Drägerwerk AG &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C94" t="n">
         <v>28</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Praktikum Business Development und Marketing Photovoltaik</t>
+          <t>Praktikum New Business Development</t>
         </is>
       </c>
       <c r="E94" t="inlineStr"/>
@@ -8530,7 +8514,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>aramido</t>
+          <t>Arteus Energy</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -8541,7 +8525,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/x)</t>
+          <t>Praktikum Business Development und Marketing Photovoltaik</t>
         </is>
       </c>
       <c r="E95" t="inlineStr"/>
@@ -8555,7 +8539,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>pacemaker.ai by thyssenkrupp</t>
+          <t>aramido</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -8566,7 +8550,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/x)</t>
         </is>
       </c>
       <c r="E96" t="inlineStr"/>
@@ -8580,7 +8564,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Molly Suh GmbH</t>
+          <t>pacemaker.ai by thyssenkrupp</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -8591,7 +8575,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; B2B Sales (m/w/d)</t>
+          <t>Praktikum Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr"/>
@@ -8605,7 +8589,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>homewise</t>
+          <t>Molly Suh GmbH</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -8616,7 +8600,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development &amp; Strategie (m/w/d)</t>
+          <t>Praktikum Business Development &amp; B2B Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E98" t="inlineStr"/>
@@ -8630,7 +8614,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>ClipMyHorse.TV</t>
+          <t>homewise</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -8641,7 +8625,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Praktikum HR &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im Business Development &amp; Strategie (m/w/d)</t>
         </is>
       </c>
       <c r="E99" t="inlineStr"/>
@@ -8655,7 +8639,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>AUMOVIO</t>
+          <t>ClipMyHorse.TV</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -8666,7 +8650,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Praktikum - Administration/Assistenz &amp; Business Development</t>
+          <t>Praktikum HR &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E100" t="inlineStr"/>
@@ -8680,7 +8664,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>TRUMPF Group</t>
+          <t>AUMOVIO</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -8691,7 +8675,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich Business Development für Smart Factory Solutions (WS26/27)</t>
+          <t>Praktikum - Administration/Assistenz &amp; Business Development</t>
         </is>
       </c>
       <c r="E101" t="inlineStr"/>
@@ -8702,8 +8686,33 @@
         </is>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>TRUMPF Group</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>1</v>
+      </c>
+      <c r="C102" t="n">
+        <v>28</v>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Praktikum im Bereich Business Development für Smart Factory Solutions (WS26/27)</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr"/>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G101"/>
+  <autoFilter ref="A1:G102"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Lauf 2026-09-05 10:09 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -6331,7 +6331,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="C2" t="n">
         <v>109</v>
@@ -6406,7 +6406,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="C5" t="n">
         <v>89</v>
@@ -6456,7 +6456,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7" t="n">
         <v>87</v>
@@ -6477,18 +6477,18 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="C8" t="n">
         <v>84</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
@@ -6502,18 +6502,18 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="C9" t="n">
         <v>84</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
@@ -6531,7 +6531,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
@@ -6564,7 +6564,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="C11" t="n">
         <v>84</v>
@@ -6597,7 +6597,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C12" t="n">
         <v>84</v>
@@ -6622,7 +6622,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C13" t="n">
         <v>84</v>
@@ -6647,7 +6647,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C14" t="n">
         <v>84</v>
@@ -6672,7 +6672,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C15" t="n">
         <v>84</v>
@@ -6697,7 +6697,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C16" t="n">
         <v>84</v>
@@ -6772,7 +6772,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C19" t="n">
         <v>83</v>
@@ -6805,7 +6805,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C20" t="n">
         <v>80</v>
@@ -6830,7 +6830,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C21" t="n">
         <v>79</v>
@@ -6905,7 +6905,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C24" t="n">
         <v>78</v>
@@ -6930,7 +6930,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C25" t="n">
         <v>78</v>
@@ -6955,7 +6955,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C26" t="n">
         <v>74</v>
@@ -6988,7 +6988,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C27" t="n">
         <v>74</v>
@@ -7013,7 +7013,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C28" t="n">
         <v>74</v>
@@ -7038,7 +7038,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C29" t="n">
         <v>73</v>
@@ -7096,7 +7096,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C31" t="n">
         <v>73</v>
@@ -7121,7 +7121,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="C32" t="n">
         <v>72</v>
@@ -7146,7 +7146,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C33" t="n">
         <v>72</v>
@@ -7221,7 +7221,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C36" t="n">
         <v>68</v>
@@ -7296,7 +7296,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C39" t="n">
         <v>66</v>
@@ -7321,7 +7321,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C40" t="n">
         <v>65</v>
@@ -7346,7 +7346,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C41" t="n">
         <v>64</v>
@@ -7371,7 +7371,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C42" t="n">
         <v>62</v>
@@ -7396,7 +7396,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C43" t="n">
         <v>62</v>
@@ -7429,7 +7429,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C44" t="n">
         <v>62</v>
@@ -7454,7 +7454,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="C45" t="n">
         <v>59</v>
@@ -7504,7 +7504,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="C47" t="n">
         <v>57</v>
@@ -7537,7 +7537,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C48" t="n">
         <v>56</v>
@@ -7562,7 +7562,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C49" t="n">
         <v>55</v>
@@ -7637,7 +7637,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="C52" t="n">
         <v>53</v>
@@ -7662,7 +7662,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C53" t="n">
         <v>53</v>
@@ -7712,7 +7712,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C55" t="n">
         <v>52</v>
@@ -7737,7 +7737,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C56" t="n">
         <v>52</v>
@@ -7837,7 +7837,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C60" t="n">
         <v>50</v>
@@ -7862,7 +7862,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C61" t="n">
         <v>49</v>
@@ -7887,7 +7887,7 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C62" t="n">
         <v>49</v>
@@ -7912,7 +7912,7 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C63" t="n">
         <v>49</v>
@@ -7962,7 +7962,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C65" t="n">
         <v>49</v>
@@ -7987,7 +7987,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C66" t="n">
         <v>49</v>
@@ -8012,7 +8012,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C67" t="n">
         <v>49</v>
@@ -8037,7 +8037,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C68" t="n">
         <v>49</v>
@@ -8058,32 +8058,32 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Clarios</t>
+          <t>ABOUT YOU</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C69" t="n">
         <v>49</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
+          <t>Intern Marketing &amp; GTM Strategy (all genders)Hamburg, Germany</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ABOUT YOU</t>
+          <t>Clarios</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -8094,14 +8094,14 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Intern Marketing &amp; GTM Strategy (all genders)Hamburg, Germany</t>
+          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-04</t>
         </is>
       </c>
     </row>
@@ -8133,32 +8133,32 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Pflegia</t>
+          <t>Konzernzentrale</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C72" t="n">
         <v>48</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Praktikum im Business Development (m/w/d)</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-01</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Konzernzentrale</t>
+          <t>Pflegia</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -8169,14 +8169,14 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Praktikum im Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>
@@ -8512,7 +8512,7 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C87" t="n">
         <v>46</v>

</xml_diff>

<commit_message>
Lauf 2026-09-06 10:26 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firmen entdeckt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$128</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$127</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$104</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L128"/>
+  <dimension ref="A1:L127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -764,12 +764,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Nestle</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -787,12 +787,12 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -803,7 +803,7 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Category-Management%2C-Brand-Activation-und-Sales-%28mwd%29-60329/1427883433/</t>
         </is>
       </c>
     </row>
@@ -814,35 +814,31 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Hamburg-Altstadt, Hamburg</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -853,7 +849,7 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Category-Management%2C-Brand-Activation-und-Sales-%28mwd%29-60329/1427883433/</t>
+          <t>https://www.adzuna.de/details/5829732882?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -869,12 +865,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Hamburg-Altstadt, Hamburg</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -888,7 +884,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -899,7 +895,7 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
+          <t>https://www.adzuna.de/details/5865920988?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -920,7 +916,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Hamburg-Altstadt, Hamburg</t>
+          <t>Barmbek-Süd, Hamburg</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -934,7 +930,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -945,7 +941,7 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5829732882?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5867772905?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -956,12 +952,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Picnic</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Category Management Praktikum (m/w/d)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -980,7 +976,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -991,34 +987,36 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5859954968?se=avT3yguj8RGEeLI7Dotn4Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FEC8C1664463BB6D76B4F51C80D7BE9A67B3E95</t>
+          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="n">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Praktikum Brand Management National</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Hamburg-Altstadt, Hamburg</t>
-        </is>
-      </c>
-      <c r="F12" t="n">
-        <v>6</v>
-      </c>
-      <c r="G12" t="inlineStr"/>
+          <t>Au-Haidhausen, München</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1026,7 +1024,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1037,34 +1035,38 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5865920988?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805399065?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="n">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Barmbek-Süd, Hamburg</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F13" t="n">
         <v>6</v>
       </c>
-      <c r="G13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1072,7 +1074,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1083,34 +1085,38 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5867772905?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5843628932?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=65C46D18FCDB11FD2E933BD305E494E07D043D72</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="n">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Picnic</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Category Management Praktikum (m/w/d)</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F14" t="n">
         <v>6</v>
       </c>
-      <c r="G14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1129,23 +1135,23 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="n">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1158,7 +1164,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1168,7 +1174,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1179,14 +1185,14 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5843628932?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=65C46D18FCDB11FD2E933BD305E494E07D043D72</t>
+          <t>https://www.adzuna.de/details/5799961458?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="n">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1232,29 +1238,27 @@
     <row r="17">
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
+          <t>L'Occitane</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management National</t>
+          <t>Praktikum (m/w/d) Trade Marketing</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Au-Haidhausen, München</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
+          <t>Friedrichstadt, Düsseldorf</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>6</v>
+      </c>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1262,7 +1266,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1273,7 +1277,7 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805399065?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5842049264?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1284,17 +1288,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Ferrero</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F18" t="n">
@@ -1302,7 +1306,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1323,7 +1327,7 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1334,17 +1338,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Ferrero</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikum Brand Management (m/w/d)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F19" t="n">
@@ -1352,7 +1356,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1373,7 +1377,7 @@
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5799961458?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802899675?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1384,17 +1388,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>L'Occitane</t>
+          <t>Nestle</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Praktikum (m/w/d) Trade Marketing</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Friedrichstadt, Düsseldorf</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F20" t="n">
@@ -1408,7 +1412,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1419,38 +1423,32 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5842049264?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
       <c r="B21" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F21" t="n">
-        <v>6</v>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1458,7 +1456,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -1469,28 +1467,28 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5843628966?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=3DAF9A0A7032477BEFBE4DD229577F81F1D32CF0</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr"/>
       <c r="B22" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>HUGO BOSS</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d)</t>
+          <t>Internship Buying &amp; Planning - Global Merchandising (m/f/d)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
+          <t>Metzingen, Reutlingen (Kreis)</t>
         </is>
       </c>
       <c r="F22" t="n">
@@ -1498,7 +1496,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1508,7 +1506,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1519,7 +1517,7 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899675?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5856159470?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1530,17 +1528,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>Miles &amp; More GmbH</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
+          <t>Internship Marketing Strategy &amp; Delivery</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Flughafen, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F23" t="inlineStr"/>
@@ -1552,7 +1550,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1563,38 +1561,34 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5843628966?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=3DAF9A0A7032477BEFBE4DD229577F81F1D32CF0</t>
+          <t>https://www.adzuna.de/details/5828674997?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="n">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>HUGO BOSS</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Internship Buying &amp; Planning - Global Merchandising (m/f/d)</t>
+          <t>Praktikum Business Development &amp; Talent Partnerships (m/w/d)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Metzingen, Reutlingen (Kreis)</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>6</v>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1602,7 +1596,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -1613,31 +1607,33 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5856159470?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5851100606?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="n">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Miles &amp; More GmbH</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Internship Marketing Strategy &amp; Delivery</t>
+          <t>Praktikum im B2B-Vertrieb &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Flughafen, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr"/>
+          <t>Düsseltal, Düsseldorf</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>5</v>
+      </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
@@ -1646,7 +1642,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -1657,7 +1653,7 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5828674997?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5851898375?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1668,21 +1664,21 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>markenbaumarkt24</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Talent Partnerships (m/w/d)</t>
+          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Feuersbach, Siegen</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
@@ -1692,7 +1688,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -1703,33 +1699,31 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5851100606?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>PARSA Haar- und Modeartikel GmbH</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Praktikum im B2B-Vertrieb &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
-        </is>
-      </c>
-      <c r="F27" t="n">
-        <v>5</v>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
@@ -1738,7 +1732,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -1749,33 +1743,31 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5851898375?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>markenbaumarkt24</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
+          <t>Praktikum Product Marketing (x/f/m)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Feuersbach, Siegen</t>
-        </is>
-      </c>
-      <c r="F28" t="n">
-        <v>2</v>
-      </c>
+          <t>Berlin, Berlin, Germany</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
@@ -1784,7 +1776,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -1795,23 +1787,23 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5842051017?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>PARSA Haar- und Modeartikel GmbH</t>
+          <t>Groß- &amp; Einzelhandel Karriere</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1828,7 +1820,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -1839,7 +1831,7 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
+          <t>https://www.adzuna.de/land/ad/5848300231?se=1ucgSzui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=BF61BDCA3F28DD382163849647345A68CC617C45</t>
         </is>
       </c>
     </row>
@@ -1850,17 +1842,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Praktikum Product Marketing (x/f/m)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
@@ -1872,7 +1864,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -1883,7 +1875,7 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5842051017?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
         </is>
       </c>
     </row>
@@ -1894,7 +1886,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Groß- &amp; Einzelhandel Karriere</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1916,7 +1908,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -1927,7 +1919,7 @@
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848300231?se=1ucgSzui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=BF61BDCA3F28DD382163849647345A68CC617C45</t>
+          <t>https://www.adzuna.de/land/ad/5849209692?se=qJaID2Kc8RGlrvMe-VN8Yg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B8E6A551D4E75B7916A5994DC13A8DA3451895D</t>
         </is>
       </c>
     </row>
@@ -1943,12 +1935,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
@@ -1960,7 +1952,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -1971,7 +1963,7 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5849209692?se=qJaID2Kc8RGlrvMe-VN8Yg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B8E6A551D4E75B7916A5994DC13A8DA3451895D</t>
+          <t>https://www.adzuna.de/land/ad/5859954968?se=avT3yguj8RGEeLI7Dotn4Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FEC8C1664463BB6D76B4F51C80D7BE9A67B3E95</t>
         </is>
       </c>
     </row>
@@ -5346,17 +5338,17 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Henkel</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Praktikum Key Account Management Henkel Consumer Brands</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Benrath, Düsseldorf</t>
+          <t>Schwabing-Freimann, München</t>
         </is>
       </c>
       <c r="F108" t="inlineStr"/>
@@ -5368,7 +5360,7 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
@@ -5379,7 +5371,7 @@
       <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5816484283?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5390,24 +5382,24 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
+          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Schwabing-Freimann, München</t>
+          <t>DEU-Bayern-Unterhaching</t>
         </is>
       </c>
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr"/>
       <c r="H109" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -5423,7 +5415,7 @@
       <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
         </is>
       </c>
     </row>
@@ -5439,12 +5431,12 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
+          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>DEU-Bayern-Unterhaching</t>
+          <t>2 Standorte</t>
         </is>
       </c>
       <c r="F110" t="inlineStr"/>
@@ -5456,7 +5448,7 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
@@ -5467,7 +5459,7 @@
       <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
         </is>
       </c>
     </row>
@@ -5478,29 +5470,29 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>2 Standorte</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
@@ -5511,7 +5503,7 @@
       <c r="K111" t="inlineStr"/>
       <c r="L111" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
+          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5522,17 +5514,17 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F112" t="inlineStr"/>
@@ -5555,7 +5547,7 @@
       <c r="K112" t="inlineStr"/>
       <c r="L112" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
         </is>
       </c>
     </row>
@@ -5571,7 +5563,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -5599,7 +5591,7 @@
       <c r="K113" t="inlineStr"/>
       <c r="L113" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
+          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
         </is>
       </c>
     </row>
@@ -5615,7 +5607,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -5643,7 +5635,7 @@
       <c r="K114" t="inlineStr"/>
       <c r="L114" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
+          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
         </is>
       </c>
     </row>
@@ -5654,17 +5646,17 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
         </is>
       </c>
       <c r="F115" t="inlineStr"/>
@@ -5687,7 +5679,7 @@
       <c r="K115" t="inlineStr"/>
       <c r="L115" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
+          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5698,17 +5690,17 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>RAG</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+          <t>Gornhofen, Ravensburg</t>
         </is>
       </c>
       <c r="F116" t="inlineStr"/>
@@ -5720,7 +5712,7 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
@@ -5731,28 +5723,28 @@
       <c r="K116" t="inlineStr"/>
       <c r="L116" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr"/>
       <c r="B117" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>RAG</t>
+          <t>Konzernzentrale</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Gornhofen, Ravensburg</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F117" t="inlineStr"/>
@@ -5764,7 +5756,7 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
@@ -5775,28 +5767,28 @@
       <c r="K117" t="inlineStr"/>
       <c r="L117" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5864351176?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr"/>
       <c r="B118" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Konzernzentrale</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F118" t="inlineStr"/>
@@ -5808,7 +5800,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
@@ -5819,7 +5811,7 @@
       <c r="K118" t="inlineStr"/>
       <c r="L118" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5864351176?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5840,7 +5832,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Altstadt-Nord, Köln</t>
         </is>
       </c>
       <c r="F119" t="inlineStr"/>
@@ -5863,28 +5855,28 @@
       <c r="K119" t="inlineStr"/>
       <c r="L119" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr"/>
       <c r="B120" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>freudio</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Altstadt-Nord, Köln</t>
+          <t>Wien, Österreich</t>
         </is>
       </c>
       <c r="F120" t="inlineStr"/>
@@ -5896,7 +5888,7 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
@@ -5907,7 +5899,7 @@
       <c r="K120" t="inlineStr"/>
       <c r="L120" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/details/5836667156?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5918,17 +5910,17 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>freudio</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Wien, Österreich</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F121" t="inlineStr"/>
@@ -5940,7 +5932,7 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
@@ -5951,7 +5943,7 @@
       <c r="K121" t="inlineStr"/>
       <c r="L121" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/details/5836667156?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5967,7 +5959,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -5995,7 +5987,7 @@
       <c r="K122" t="inlineStr"/>
       <c r="L122" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -6011,12 +6003,12 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F123" t="inlineStr"/>
@@ -6039,7 +6031,7 @@
       <c r="K123" t="inlineStr"/>
       <c r="L123" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -6055,7 +6047,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -6083,7 +6075,7 @@
       <c r="K124" t="inlineStr"/>
       <c r="L124" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -6099,12 +6091,12 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d) - In 3 Minuten erfolgreich bewerben</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F125" t="inlineStr"/>
@@ -6116,7 +6108,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
@@ -6127,7 +6119,7 @@
       <c r="K125" t="inlineStr"/>
       <c r="L125" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5856292292?se=PMRjVxmh8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DF242745B4142F9871F0353F9B390FD5166A63B5</t>
         </is>
       </c>
     </row>
@@ -6138,17 +6130,17 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>sailwithus</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d) - In 3 Minuten erfolgreich bewerben</t>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F126" t="inlineStr"/>
@@ -6160,7 +6152,7 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
@@ -6171,7 +6163,7 @@
       <c r="K126" t="inlineStr"/>
       <c r="L126" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5856292292?se=PMRjVxmh8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DF242745B4142F9871F0353F9B390FD5166A63B5</t>
+          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -6192,7 +6184,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F127" t="inlineStr"/>
@@ -6215,56 +6207,12 @@
       <c r="K127" t="inlineStr"/>
       <c r="L127" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="inlineStr"/>
-      <c r="B128" t="n">
-        <v>45</v>
-      </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>sailwithus</t>
-        </is>
-      </c>
-      <c r="D128" t="inlineStr">
-        <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
-        </is>
-      </c>
-      <c r="E128" t="inlineStr">
-        <is>
-          <t>Altstadt, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F128" t="inlineStr"/>
-      <c r="G128" t="inlineStr"/>
-      <c r="H128" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I128" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J128" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K128" t="inlineStr"/>
-      <c r="L128" t="inlineStr">
-        <is>
           <t>https://www.adzuna.de/details/5804544237?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L128"/>
+  <autoFilter ref="A1:L127"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6331,7 +6279,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="C2" t="n">
         <v>109</v>
@@ -6406,7 +6354,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C5" t="n">
         <v>89</v>
@@ -6456,7 +6404,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C7" t="n">
         <v>87</v>
@@ -6481,7 +6429,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="C8" t="n">
         <v>84</v>
@@ -6506,7 +6454,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C9" t="n">
         <v>84</v>
@@ -6531,7 +6479,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
@@ -6564,7 +6512,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="C11" t="n">
         <v>84</v>
@@ -6597,7 +6545,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C12" t="n">
         <v>84</v>
@@ -6622,7 +6570,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C13" t="n">
         <v>84</v>
@@ -6647,7 +6595,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C14" t="n">
         <v>84</v>
@@ -6672,7 +6620,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C15" t="n">
         <v>84</v>
@@ -6697,7 +6645,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C16" t="n">
         <v>84</v>
@@ -6772,7 +6720,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C19" t="n">
         <v>83</v>
@@ -6805,7 +6753,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C20" t="n">
         <v>80</v>
@@ -6830,7 +6778,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C21" t="n">
         <v>79</v>
@@ -6905,7 +6853,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C24" t="n">
         <v>78</v>
@@ -6930,7 +6878,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C25" t="n">
         <v>78</v>
@@ -6955,7 +6903,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C26" t="n">
         <v>74</v>
@@ -6988,7 +6936,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C27" t="n">
         <v>74</v>
@@ -7038,7 +6986,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C29" t="n">
         <v>73</v>
@@ -7096,7 +7044,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C31" t="n">
         <v>73</v>
@@ -7121,7 +7069,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="C32" t="n">
         <v>72</v>
@@ -7146,7 +7094,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C33" t="n">
         <v>72</v>
@@ -7221,7 +7169,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C36" t="n">
         <v>68</v>
@@ -7296,7 +7244,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C39" t="n">
         <v>66</v>
@@ -7321,7 +7269,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C40" t="n">
         <v>65</v>
@@ -7346,7 +7294,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C41" t="n">
         <v>64</v>
@@ -7371,7 +7319,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C42" t="n">
         <v>62</v>
@@ -7396,7 +7344,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C43" t="n">
         <v>62</v>
@@ -7429,7 +7377,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C44" t="n">
         <v>62</v>
@@ -7454,7 +7402,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C45" t="n">
         <v>59</v>
@@ -7504,7 +7452,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C47" t="n">
         <v>57</v>
@@ -7537,7 +7485,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C48" t="n">
         <v>56</v>
@@ -7562,7 +7510,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C49" t="n">
         <v>55</v>
@@ -7637,7 +7585,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="C52" t="n">
         <v>53</v>
@@ -7662,7 +7610,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C53" t="n">
         <v>53</v>
@@ -7712,7 +7660,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C55" t="n">
         <v>52</v>
@@ -7737,7 +7685,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C56" t="n">
         <v>52</v>
@@ -7837,7 +7785,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C60" t="n">
         <v>50</v>
@@ -7862,7 +7810,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C61" t="n">
         <v>49</v>
@@ -7887,7 +7835,7 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C62" t="n">
         <v>49</v>
@@ -7912,7 +7860,7 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C63" t="n">
         <v>49</v>
@@ -7962,7 +7910,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C65" t="n">
         <v>49</v>
@@ -7987,7 +7935,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C66" t="n">
         <v>49</v>
@@ -8012,7 +7960,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C67" t="n">
         <v>49</v>
@@ -8037,7 +7985,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C68" t="n">
         <v>49</v>
@@ -8062,7 +8010,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C69" t="n">
         <v>49</v>
@@ -8137,7 +8085,7 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C72" t="n">
         <v>48</v>
@@ -8512,7 +8460,7 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C87" t="n">
         <v>46</v>

</xml_diff>

<commit_message>
Lauf 2026-09-07 11:44 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -518,31 +518,27 @@
     <row r="2">
       <c r="A2" t="inlineStr"/>
       <c r="B2" t="n">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>ABRIO GmbH</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikum - Digital Marketing &amp; E-Commerce (m/w/d)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Bockenheim, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>6</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -550,7 +546,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -561,57 +557,53 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5843630960?se=znNqlDyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=875B574D03DFD36B16B3A3ABE0AA46F858215182</t>
+          <t>https://www.adzuna.de/details/5871278891?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>87</v>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>ABRIO GmbH</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Praktikum - Digital Marketing &amp; E-Commerce (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Bockenheim, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="n">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="n">
+        <v>84</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Carwow</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Praktikum Business Development &amp; Media (m/w/d) - OEM Partnerships @ Carwow</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>München, München (Kreis)</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
         <v>3</v>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-05</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr"/>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5871278891?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5822522402?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -622,17 +614,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Carwow</t>
+          <t>FC Viktoria 1889 Berlin Frauen-Fußball GmbH</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Media (m/w/d) - OEM Partnerships @ Carwow</t>
+          <t>PRAKTIKUM // Business Development</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Mitte, Berlin</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -657,7 +649,7 @@
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5822522402?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802962068?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -668,23 +660,27 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>FC Viktoria 1889 Berlin Frauen-Fußball GmbH</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>PRAKTIKUM // Business Development</t>
+          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Mitte, Berlin</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G5" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -692,7 +688,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -703,7 +699,7 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802962068?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5858231617?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -714,17 +710,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>Nestle</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -732,7 +728,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -742,7 +738,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -753,7 +749,7 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5858231617?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1046,12 +1042,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1064,7 +1060,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1074,7 +1070,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1085,7 +1081,7 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5843628932?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=65C46D18FCDB11FD2E933BD305E494E07D043D72</t>
+          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1097,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1114,7 +1110,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1135,7 +1131,7 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5799961458?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1147,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1162,11 +1158,7 @@
       <c r="F15" t="n">
         <v>6</v>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1185,7 +1177,7 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5799961458?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1196,17 +1188,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Ferrero</t>
+          <t>L'Occitane</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikum (m/w/d) Trade Marketing</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Friedrichstadt, Düsseldorf</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -1220,7 +1212,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1231,7 +1223,7 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5842049264?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1242,23 +1234,27 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>L'Occitane</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Praktikum (m/w/d) Trade Marketing</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Friedrichstadt, Düsseldorf</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F17" t="n">
         <v>6</v>
       </c>
-      <c r="G17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
       <c r="H17" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1266,7 +1262,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1277,7 +1273,7 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5842049264?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1293,12 +1289,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Praktikum Brand Management (m/w/d)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F18" t="n">
@@ -1306,7 +1302,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1327,38 +1323,32 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802899675?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
       <c r="B19" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d)</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F19" t="n">
-        <v>6</v>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1366,7 +1356,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1377,33 +1367,31 @@
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899675?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5843630960?se=znNqlDyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=875B574D03DFD36B16B3A3ABE0AA46F858215182</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Nestle</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
-        </is>
-      </c>
-      <c r="F20" t="n">
-        <v>6</v>
-      </c>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
@@ -1412,7 +1400,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1423,7 +1411,7 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5843628966?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=3DAF9A0A7032477BEFBE4DD229577F81F1D32CF0</t>
         </is>
       </c>
     </row>
@@ -1439,7 +1427,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1467,7 +1455,7 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5843628966?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=3DAF9A0A7032477BEFBE4DD229577F81F1D32CF0</t>
+          <t>https://www.adzuna.de/land/ad/5843628932?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=65C46D18FCDB11FD2E933BD305E494E07D043D72</t>
         </is>
       </c>
     </row>
@@ -1979,7 +1967,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Stepstone geprüft - Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1996,7 +1984,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -2007,7 +1995,7 @@
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5864785114?se=tDVxHrqm8RG47MvhImrnRA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=ABFCC49076160E6370E149C31FFE29D13C38563D</t>
+          <t>https://www.adzuna.de/land/ad/5868159571?se=Ur2Ws4On8RGeD7WukCg86Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD828F897C614DE600F1B21C5501265E349B7241</t>
         </is>
       </c>
     </row>
@@ -2023,7 +2011,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Stepstone geprüft - Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Stepstone geprüft - Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2051,31 +2039,33 @@
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5868159571?se=Ur2Ws4On8RGeD7WukCg86Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD828F897C614DE600F1B21C5501265E349B7241</t>
+          <t>https://www.adzuna.de/land/ad/5868159685?se=Ur2Ws4On8RGeD7WukCg86Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DA869B4EFE837366B3946FD4F30C27AACFC1FE6D</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr"/>
       <c r="B35" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Stepstone geprüft - Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr"/>
+          <t>Köln, Nordrhein-Westfalen</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>6</v>
+      </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
@@ -2084,7 +2074,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -2095,7 +2085,7 @@
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5868159685?se=Ur2Ws4On8RGeD7WukCg86Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DA869B4EFE837366B3946FD4F30C27AACFC1FE6D</t>
+          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2111,7 +2101,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
+          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2141,7 +2131,7 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2157,7 +2147,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
+          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2168,7 +2158,11 @@
       <c r="F37" t="n">
         <v>6</v>
       </c>
-      <c r="G37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H37" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2187,7 +2181,7 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2198,17 +2192,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -2216,7 +2210,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2237,46 +2231,40 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr"/>
       <c r="B39" t="n">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>Internship in Trade Marketing</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
-        </is>
-      </c>
-      <c r="F39" t="n">
-        <v>6</v>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>2026-11-01</t>
-        </is>
-      </c>
+          <t>DEU-Nordrhein-Westfalen-Köln</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -2287,40 +2275,40 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr"/>
       <c r="B40" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Internship in Trade Marketing</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>DEU-Nordrhein-Westfalen-Köln</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -2331,7 +2319,7 @@
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
+          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2352,7 +2340,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
+          <t>Altstadt, Düsseldorf</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
@@ -2375,7 +2363,7 @@
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2386,17 +2374,17 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>Calypso Ventures GmbH</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Altstadt, Düsseldorf</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
@@ -2419,7 +2407,7 @@
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2430,17 +2418,17 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Calypso Ventures GmbH</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
+          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
@@ -2463,7 +2451,7 @@
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2479,7 +2467,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2496,7 +2484,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -2507,7 +2495,7 @@
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2523,7 +2511,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im Sales &amp; Business Development – B2B (m/w/d)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2540,7 +2528,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -2551,7 +2539,7 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5866225907?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2567,7 +2555,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Praktikum im Sales &amp; Business Development – B2B (m/w/d)</t>
+          <t>Sales &amp; Business Development Praktikum B2B (m/w/d)</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2584,7 +2572,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -2595,55 +2583,53 @@
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5866225907?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5871334687?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="n">
+      <c r="A47" t="inlineStr"/>
+      <c r="B47" t="n">
         <v>62</v>
       </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>Exclusive Associates</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>Sales &amp; Business Development Praktikum B2B (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>Düsseltal, Düsseldorf</t>
-        </is>
-      </c>
-      <c r="F47" s="2" t="inlineStr"/>
-      <c r="G47" s="2" t="inlineStr"/>
-      <c r="H47" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I47" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-05</t>
-        </is>
-      </c>
-      <c r="J47" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K47" s="2" t="inlineStr"/>
-      <c r="L47" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5871334687?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>FC Viktoria 1889 Berlin Frauen-Fußball GmbH</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>PRAKTIKUM // Business Development - In 3 Minuten erfolgreich bewerben</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>3</v>
+      </c>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/land/ad/5856283303?se=PMRjVxmh8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0E222C24DC5860DC4AEB24D8BB5E4CB04740A32C</t>
         </is>
       </c>
     </row>
@@ -2654,22 +2640,20 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>FC Viktoria 1889 Berlin Frauen-Fußball GmbH</t>
+          <t>montamo GmbH</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>PRAKTIKUM // Business Development - In 3 Minuten erfolgreich bewerben</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F48" t="n">
-        <v>3</v>
-      </c>
+          <t>Berlin, Deutschland</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
@@ -2678,7 +2662,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -2689,7 +2673,7 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5856283303?se=PMRjVxmh8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0E222C24DC5860DC4AEB24D8BB5E4CB04740A32C</t>
+          <t>https://www.adzuna.de/land/ad/5856889494?se=1M-3UDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=471483726C1FC3DB660B48A5B3DEDE0DC1A4DC20</t>
         </is>
       </c>
     </row>
@@ -2710,7 +2694,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Wedding, Berlin</t>
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
@@ -2733,28 +2717,28 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5856889494?se=1M-3UDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=471483726C1FC3DB660B48A5B3DEDE0DC1A4DC20</t>
+          <t>https://www.adzuna.de/details/5857559039?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr"/>
       <c r="B50" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>montamo GmbH</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Retail Marketing | Fashion und Sport-Marken (w/m/d)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F50" t="inlineStr"/>
@@ -2777,7 +2761,7 @@
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5857559039?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5858188456?se=HMKESTui8RGfx5bEd-nhPg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=86B24D9EAAAA2322A41661C360015255B004809E</t>
         </is>
       </c>
     </row>
@@ -2798,7 +2782,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
@@ -2810,7 +2794,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -2821,7 +2805,7 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5858188456?se=HMKESTui8RGfx5bEd-nhPg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=86B24D9EAAAA2322A41661C360015255B004809E</t>
+          <t>https://www.adzuna.de/land/ad/5860650076?se=EGcET6Oj8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=E6646A9A107DD9C83D248D81843D6570367335AD</t>
         </is>
       </c>
     </row>
@@ -2842,7 +2826,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Hamburg-Altstadt, Hamburg</t>
         </is>
       </c>
       <c r="F52" t="inlineStr"/>
@@ -2865,28 +2849,28 @@
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5860650076?se=EGcET6Oj8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=E6646A9A107DD9C83D248D81843D6570367335AD</t>
+          <t>https://www.adzuna.de/details/5860355819?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr"/>
       <c r="B53" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Praktikum Retail Marketing | Fashion und Sport-Marken (w/m/d)</t>
+          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Hamburg-Altstadt, Hamburg</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F53" t="inlineStr"/>
@@ -2898,7 +2882,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -2909,7 +2893,7 @@
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5860355819?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5848400955?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=4E59A334AC360616EAEAAC474F72A07451A7C624</t>
         </is>
       </c>
     </row>
@@ -2925,7 +2909,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2953,7 +2937,7 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848400955?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=4E59A334AC360616EAEAAC474F72A07451A7C624</t>
+          <t>https://www.adzuna.de/land/ad/5848409009?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5C62DDCDA5E03F77D6089CD03CFA1D966DF15C96</t>
         </is>
       </c>
     </row>
@@ -2969,7 +2953,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2986,7 +2970,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -2997,7 +2981,7 @@
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848409009?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5C62DDCDA5E03F77D6089CD03CFA1D966DF15C96</t>
+          <t>https://www.adzuna.de/land/ad/5861203670?se=hvkm4GOk8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD0ED2E271738C13EE6613442755CC0DE68C0F5A</t>
         </is>
       </c>
     </row>
@@ -3008,12 +2992,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>Nahrungs- &amp; Genussmittel Karriere</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -3030,7 +3014,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -3041,7 +3025,7 @@
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5861203670?se=hvkm4GOk8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD0ED2E271738C13EE6613442755CC0DE68C0F5A</t>
+          <t>https://www.adzuna.de/land/ad/5848308031?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=C04FAD6E90B5FCF47A6B81E4A697BA781ADC04AF</t>
         </is>
       </c>
     </row>
@@ -3057,7 +3041,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -3085,7 +3069,7 @@
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848308031?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=C04FAD6E90B5FCF47A6B81E4A697BA781ADC04AF</t>
+          <t>https://www.adzuna.de/land/ad/5851105442?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8F6135545B7E9C415844F10F4AF49C0BFA63A4B2</t>
         </is>
       </c>
     </row>
@@ -3101,7 +3085,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -3129,7 +3113,7 @@
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5851105442?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8F6135545B7E9C415844F10F4AF49C0BFA63A4B2</t>
+          <t>https://www.adzuna.de/land/ad/5848347180?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8A3F28529B6340B7DCCD5131E2C4472FBD8CA361</t>
         </is>
       </c>
     </row>
@@ -3145,7 +3129,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
+          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -3173,7 +3157,7 @@
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848347180?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8A3F28529B6340B7DCCD5131E2C4472FBD8CA361</t>
+          <t>https://www.adzuna.de/land/ad/5848315177?se=nioaTDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B01A57BB52C4BDBB1DF6554A4A21C913096E1D0</t>
         </is>
       </c>
     </row>
@@ -3189,7 +3173,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -3217,7 +3201,7 @@
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848315177?se=nioaTDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B01A57BB52C4BDBB1DF6554A4A21C913096E1D0</t>
+          <t>https://www.adzuna.de/land/ad/5848325009?se=nioaTDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8D26762D834367B41A848A3D14A62E41FD573B9B</t>
         </is>
       </c>
     </row>
@@ -3228,12 +3212,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Nahrungs- &amp; Genussmittel Karriere</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -3250,7 +3234,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -3261,7 +3245,7 @@
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848325009?se=nioaTDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8D26762D834367B41A848A3D14A62E41FD573B9B</t>
+          <t>https://www.adzuna.de/land/ad/5864785114?se=tDVxHrqm8RG47MvhImrnRA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=ABFCC49076160E6370E149C31FFE29D13C38563D</t>
         </is>
       </c>
     </row>
@@ -4430,46 +4414,50 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" t="inlineStr"/>
-      <c r="B88" t="n">
-        <v>51</v>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>Digitalagenten</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr">
-        <is>
-          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>Charlottenburg, Berlin</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr"/>
-      <c r="G88" t="inlineStr"/>
-      <c r="H88" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I88" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J88" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K88" t="inlineStr"/>
-      <c r="L88" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5804948828?utm_medium=api&amp;utm_source=e1fd92a2</t>
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>montamo GmbH</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr"/>
+      <c r="G88" s="2" t="inlineStr"/>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K88" s="2" t="inlineStr"/>
+      <c r="L88" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/land/ad/5871424623?se=gmRR3q-q8RGogquEo3zAlQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=453E406F424C8AB021346B1F246ACB2280C9B284</t>
         </is>
       </c>
     </row>
@@ -4480,17 +4468,17 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>HardyTec Industries UG haftungsbeschränkt</t>
+          <t>Digitalagenten</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Business Development</t>
+          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Büderich, Meerbusch</t>
+          <t>Charlottenburg, Berlin</t>
         </is>
       </c>
       <c r="F89" t="inlineStr"/>
@@ -4502,7 +4490,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -4513,7 +4501,7 @@
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5848139968?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804948828?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4658,52 +4646,48 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B93" s="2" t="n">
+      <c r="A93" t="inlineStr"/>
+      <c r="B93" t="n">
         <v>51</v>
       </c>
-      <c r="C93" s="2" t="inlineStr">
+      <c r="C93" t="inlineStr">
         <is>
           <t>SERVICEPLAN Gruppe</t>
         </is>
       </c>
-      <c r="D93" s="2" t="inlineStr">
+      <c r="D93" t="inlineStr">
         <is>
           <t>Praktikum Business Development, Marketing &amp; Sales (all genders)</t>
         </is>
       </c>
-      <c r="E93" s="2" t="inlineStr">
+      <c r="E93" t="inlineStr">
         <is>
           <t>München, München (Kreis)</t>
         </is>
       </c>
-      <c r="F93" s="2" t="inlineStr"/>
-      <c r="G93" s="2" t="inlineStr">
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr">
         <is>
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="H93" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I93" s="2" t="inlineStr">
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
         <is>
           <t>2026-09-05</t>
         </is>
       </c>
-      <c r="J93" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K93" s="2" t="inlineStr"/>
-      <c r="L93" s="2" t="inlineStr">
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr"/>
+      <c r="L93" t="inlineStr">
         <is>
           <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
@@ -4940,44 +4924,40 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B99" s="2" t="n">
+      <c r="A99" t="inlineStr"/>
+      <c r="B99" t="n">
         <v>49</v>
       </c>
-      <c r="C99" s="2" t="inlineStr">
+      <c r="C99" t="inlineStr">
         <is>
           <t>ABOUT YOU</t>
         </is>
       </c>
-      <c r="D99" s="2" t="inlineStr">
+      <c r="D99" t="inlineStr">
         <is>
           <t>Intern Marketing &amp; GTM Strategy (all genders)Hamburg, Germany</t>
         </is>
       </c>
-      <c r="E99" s="2" t="inlineStr"/>
-      <c r="F99" s="2" t="inlineStr"/>
-      <c r="G99" s="2" t="inlineStr"/>
-      <c r="H99" s="2" t="inlineStr">
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr"/>
+      <c r="G99" t="inlineStr"/>
+      <c r="H99" t="inlineStr">
         <is>
           <t>fashion</t>
         </is>
       </c>
-      <c r="I99" s="2" t="inlineStr">
+      <c r="I99" t="inlineStr">
         <is>
           <t>2026-09-05</t>
         </is>
       </c>
-      <c r="J99" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K99" s="2" t="inlineStr"/>
-      <c r="L99" s="2" t="inlineStr">
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr"/>
+      <c r="L99" t="inlineStr">
         <is>
           <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-gtm-strategy-all-genders-hamburg-germany</t>
         </is>
@@ -6279,7 +6259,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="C2" t="n">
         <v>109</v>
@@ -6354,7 +6334,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C5" t="n">
         <v>89</v>
@@ -6404,7 +6384,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C7" t="n">
         <v>87</v>
@@ -6429,7 +6409,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="C8" t="n">
         <v>84</v>
@@ -6454,7 +6434,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C9" t="n">
         <v>84</v>
@@ -6479,7 +6459,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
@@ -6512,7 +6492,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="C11" t="n">
         <v>84</v>
@@ -6545,7 +6525,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C12" t="n">
         <v>84</v>
@@ -6570,7 +6550,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C13" t="n">
         <v>84</v>
@@ -6595,7 +6575,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C14" t="n">
         <v>84</v>
@@ -6620,7 +6600,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C15" t="n">
         <v>84</v>
@@ -6645,7 +6625,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C16" t="n">
         <v>84</v>
@@ -6720,7 +6700,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C19" t="n">
         <v>83</v>
@@ -6753,7 +6733,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C20" t="n">
         <v>80</v>
@@ -6778,7 +6758,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C21" t="n">
         <v>79</v>
@@ -6853,7 +6833,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C24" t="n">
         <v>78</v>
@@ -6878,7 +6858,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C25" t="n">
         <v>78</v>
@@ -6903,7 +6883,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C26" t="n">
         <v>74</v>
@@ -6936,7 +6916,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C27" t="n">
         <v>74</v>
@@ -6986,7 +6966,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C29" t="n">
         <v>73</v>
@@ -7044,7 +7024,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C31" t="n">
         <v>73</v>
@@ -7069,7 +7049,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="C32" t="n">
         <v>72</v>
@@ -7094,7 +7074,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C33" t="n">
         <v>72</v>
@@ -7169,7 +7149,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C36" t="n">
         <v>68</v>
@@ -7244,7 +7224,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C39" t="n">
         <v>66</v>
@@ -7269,7 +7249,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C40" t="n">
         <v>65</v>
@@ -7294,7 +7274,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C41" t="n">
         <v>64</v>
@@ -7319,7 +7299,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C42" t="n">
         <v>62</v>
@@ -7344,7 +7324,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C43" t="n">
         <v>62</v>
@@ -7377,7 +7357,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C44" t="n">
         <v>62</v>
@@ -7402,7 +7382,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="C45" t="n">
         <v>59</v>
@@ -7452,7 +7432,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C47" t="n">
         <v>57</v>
@@ -7485,7 +7465,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C48" t="n">
         <v>56</v>
@@ -7510,7 +7490,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C49" t="n">
         <v>55</v>
@@ -7585,7 +7565,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="C52" t="n">
         <v>53</v>
@@ -7610,7 +7590,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C53" t="n">
         <v>53</v>
@@ -7660,7 +7640,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C55" t="n">
         <v>52</v>
@@ -7685,7 +7665,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C56" t="n">
         <v>52</v>
@@ -7785,7 +7765,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C60" t="n">
         <v>50</v>
@@ -7810,7 +7790,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C61" t="n">
         <v>49</v>
@@ -7835,7 +7815,7 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C62" t="n">
         <v>49</v>
@@ -7860,7 +7840,7 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C63" t="n">
         <v>49</v>
@@ -7910,7 +7890,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C65" t="n">
         <v>49</v>
@@ -7935,7 +7915,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C66" t="n">
         <v>49</v>
@@ -7960,7 +7940,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C67" t="n">
         <v>49</v>
@@ -7985,7 +7965,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C68" t="n">
         <v>49</v>
@@ -8010,7 +7990,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C69" t="n">
         <v>49</v>
@@ -8085,7 +8065,7 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C72" t="n">
         <v>48</v>
@@ -8460,7 +8440,7 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C87" t="n">
         <v>46</v>

</xml_diff>

<commit_message>
Lauf 2026-09-08 10:45 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firmen entdeckt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$127</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$125</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$104</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L127"/>
+  <dimension ref="A1:L125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -710,12 +710,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Nestle</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -728,17 +728,17 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -749,7 +749,7 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Category-Management%2C-Brand-Activation-und-Sales-%28mwd%29-60329/1427883433/</t>
         </is>
       </c>
     </row>
@@ -760,35 +760,31 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Hamburg-Altstadt, Hamburg</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>5</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -799,7 +795,7 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Category-Management%2C-Brand-Activation-und-Sales-%28mwd%29-60329/1427883433/</t>
+          <t>https://www.adzuna.de/details/5829732882?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -815,7 +811,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -834,7 +830,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -845,7 +841,7 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5829732882?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5865920988?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -861,12 +857,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Hamburg-Altstadt, Hamburg</t>
+          <t>Barmbek-Süd, Hamburg</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -880,7 +876,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -891,7 +887,7 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5865920988?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5867772905?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -902,17 +898,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Picnic</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Category Management Praktikum (m/w/d)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Barmbek-Süd, Hamburg</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -926,7 +922,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -937,34 +933,36 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5867772905?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="n">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Picnic</t>
+          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Category Management Praktikum (m/w/d)</t>
+          <t>Praktikum Brand Management National</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
-        </is>
-      </c>
-      <c r="F11" t="n">
-        <v>6</v>
-      </c>
-      <c r="G11" t="inlineStr"/>
+          <t>Au-Haidhausen, München</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -983,34 +981,36 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805399065?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management National</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Au-Haidhausen, München</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>6</v>
+      </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1031,7 +1031,7 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805399065?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1047,7 +1047,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1060,7 +1060,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1081,7 +1081,7 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5799961458?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1097,7 +1097,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1108,11 +1108,7 @@
       <c r="F14" t="n">
         <v>6</v>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1131,7 +1127,7 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5799961458?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1142,17 +1138,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Ferrero</t>
+          <t>L'Occitane</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikum (m/w/d) Trade Marketing</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Friedrichstadt, Düsseldorf</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -1166,7 +1162,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1177,7 +1173,7 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5842049264?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1188,23 +1184,27 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>L'Occitane</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Praktikum (m/w/d) Trade Marketing</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Friedrichstadt, Düsseldorf</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F16" t="n">
         <v>6</v>
       </c>
-      <c r="G16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1212,7 +1212,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1223,7 +1223,7 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5842049264?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1239,12 +1239,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Praktikum Brand Management (m/w/d)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F17" t="n">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1273,7 +1273,7 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802899675?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1284,27 +1284,23 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>Nestle</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d)</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F18" t="n">
         <v>6</v>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1323,7 +1319,7 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899675?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1879,12 +1875,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
@@ -1896,7 +1892,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -1907,7 +1903,7 @@
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5849209692?se=qJaID2Kc8RGlrvMe-VN8Yg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B8E6A551D4E75B7916A5994DC13A8DA3451895D</t>
+          <t>https://www.adzuna.de/land/ad/5859954968?se=avT3yguj8RGEeLI7Dotn4Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FEC8C1664463BB6D76B4F51C80D7BE9A67B3E95</t>
         </is>
       </c>
     </row>
@@ -1923,12 +1919,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Stepstone geprüft - Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
@@ -1940,7 +1936,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -1951,7 +1947,7 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5859954968?se=avT3yguj8RGEeLI7Dotn4Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FEC8C1664463BB6D76B4F51C80D7BE9A67B3E95</t>
+          <t>https://www.adzuna.de/land/ad/5868159571?se=Ur2Ws4On8RGeD7WukCg86Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD828F897C614DE600F1B21C5501265E349B7241</t>
         </is>
       </c>
     </row>
@@ -1967,7 +1963,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Stepstone geprüft - Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Stepstone geprüft - Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1995,31 +1991,33 @@
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5868159571?se=Ur2Ws4On8RGeD7WukCg86Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD828F897C614DE600F1B21C5501265E349B7241</t>
+          <t>https://www.adzuna.de/land/ad/5868159685?se=Ur2Ws4On8RGeD7WukCg86Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DA869B4EFE837366B3946FD4F30C27AACFC1FE6D</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr"/>
       <c r="B34" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Stepstone geprüft - Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr"/>
+          <t>Köln, Nordrhein-Westfalen</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>6</v>
+      </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
@@ -2028,7 +2026,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -2039,7 +2037,7 @@
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5868159685?se=Ur2Ws4On8RGeD7WukCg86Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DA869B4EFE837366B3946FD4F30C27AACFC1FE6D</t>
+          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2055,7 +2053,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
+          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2085,7 +2083,7 @@
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2099,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
+          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2112,7 +2110,11 @@
       <c r="F36" t="n">
         <v>6</v>
       </c>
-      <c r="G36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H36" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2131,7 +2133,7 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2142,17 +2144,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -2160,7 +2162,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2181,46 +2183,40 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="n">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>Internship in Trade Marketing</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
-        </is>
-      </c>
-      <c r="F38" t="n">
-        <v>6</v>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>2026-11-01</t>
-        </is>
-      </c>
+          <t>DEU-Nordrhein-Westfalen-Köln</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -2231,40 +2227,40 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr"/>
       <c r="B39" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Internship in Trade Marketing</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>DEU-Nordrhein-Westfalen-Köln</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -2275,7 +2271,7 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
+          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2296,7 +2292,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
+          <t>Altstadt, Düsseldorf</t>
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
@@ -2319,7 +2315,7 @@
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2330,17 +2326,17 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>Calypso Ventures GmbH</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Altstadt, Düsseldorf</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
@@ -2363,7 +2359,7 @@
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2374,17 +2370,17 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Calypso Ventures GmbH</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
+          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
@@ -2407,7 +2403,7 @@
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2423,7 +2419,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2440,7 +2436,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -2451,7 +2447,7 @@
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2463,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum im Sales &amp; Business Development – B2B (m/w/d)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2484,7 +2480,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -2495,7 +2491,7 @@
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5866225907?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2511,7 +2507,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Praktikum im Sales &amp; Business Development – B2B (m/w/d)</t>
+          <t>Sales &amp; Business Development Praktikum B2B (m/w/d)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2528,7 +2524,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -2539,7 +2535,7 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5866225907?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5871334687?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2550,20 +2546,22 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>FC Viktoria 1889 Berlin Frauen-Fußball GmbH</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Sales &amp; Business Development Praktikum B2B (m/w/d)</t>
+          <t>PRAKTIKUM // Business Development - In 3 Minuten erfolgreich bewerben</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr"/>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>3</v>
+      </c>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
@@ -2572,7 +2570,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -2583,7 +2581,7 @@
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5871334687?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5856283303?se=PMRjVxmh8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0E222C24DC5860DC4AEB24D8BB5E4CB04740A32C</t>
         </is>
       </c>
     </row>
@@ -2594,22 +2592,20 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>FC Viktoria 1889 Berlin Frauen-Fußball GmbH</t>
+          <t>montamo GmbH</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>PRAKTIKUM // Business Development - In 3 Minuten erfolgreich bewerben</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F47" t="n">
-        <v>3</v>
-      </c>
+          <t>Berlin, Deutschland</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
@@ -2618,7 +2614,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -2629,7 +2625,7 @@
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5856283303?se=PMRjVxmh8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0E222C24DC5860DC4AEB24D8BB5E4CB04740A32C</t>
+          <t>https://www.adzuna.de/land/ad/5856889494?se=1M-3UDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=471483726C1FC3DB660B48A5B3DEDE0DC1A4DC20</t>
         </is>
       </c>
     </row>
@@ -2650,7 +2646,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Wedding, Berlin</t>
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
@@ -2673,28 +2669,28 @@
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5856889494?se=1M-3UDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=471483726C1FC3DB660B48A5B3DEDE0DC1A4DC20</t>
+          <t>https://www.adzuna.de/details/5857559039?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr"/>
       <c r="B49" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>montamo GmbH</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Retail Marketing | Fashion und Sport-Marken (w/m/d)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
@@ -2717,7 +2713,7 @@
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5857559039?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5858188456?se=HMKESTui8RGfx5bEd-nhPg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=86B24D9EAAAA2322A41661C360015255B004809E</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2734,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F50" t="inlineStr"/>
@@ -2750,7 +2746,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -2761,7 +2757,7 @@
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5858188456?se=HMKESTui8RGfx5bEd-nhPg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=86B24D9EAAAA2322A41661C360015255B004809E</t>
+          <t>https://www.adzuna.de/land/ad/5860650076?se=EGcET6Oj8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=E6646A9A107DD9C83D248D81843D6570367335AD</t>
         </is>
       </c>
     </row>
@@ -2782,7 +2778,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Hamburg-Altstadt, Hamburg</t>
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
@@ -2805,28 +2801,28 @@
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5860650076?se=EGcET6Oj8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=E6646A9A107DD9C83D248D81843D6570367335AD</t>
+          <t>https://www.adzuna.de/details/5860355819?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr"/>
       <c r="B52" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Praktikum Retail Marketing | Fashion und Sport-Marken (w/m/d)</t>
+          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Hamburg-Altstadt, Hamburg</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F52" t="inlineStr"/>
@@ -2838,7 +2834,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -2849,7 +2845,7 @@
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5860355819?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5848400955?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=4E59A334AC360616EAEAAC474F72A07451A7C624</t>
         </is>
       </c>
     </row>
@@ -2865,7 +2861,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2893,7 +2889,7 @@
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848400955?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=4E59A334AC360616EAEAAC474F72A07451A7C624</t>
+          <t>https://www.adzuna.de/land/ad/5848409009?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5C62DDCDA5E03F77D6089CD03CFA1D966DF15C96</t>
         </is>
       </c>
     </row>
@@ -2909,7 +2905,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2926,7 +2922,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -2937,7 +2933,7 @@
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848409009?se=QG1VEGKc8RGPGoOo2YYCJg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=5C62DDCDA5E03F77D6089CD03CFA1D966DF15C96</t>
+          <t>https://www.adzuna.de/land/ad/5861203670?se=hvkm4GOk8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD0ED2E271738C13EE6613442755CC0DE68C0F5A</t>
         </is>
       </c>
     </row>
@@ -2948,12 +2944,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>Nahrungs- &amp; Genussmittel Karriere</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2970,7 +2966,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -2981,7 +2977,7 @@
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5861203670?se=hvkm4GOk8RGcfKYe_cIpvA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD0ED2E271738C13EE6613442755CC0DE68C0F5A</t>
+          <t>https://www.adzuna.de/land/ad/5848308031?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=C04FAD6E90B5FCF47A6B81E4A697BA781ADC04AF</t>
         </is>
       </c>
     </row>
@@ -2997,7 +2993,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -3025,7 +3021,7 @@
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848308031?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=C04FAD6E90B5FCF47A6B81E4A697BA781ADC04AF</t>
+          <t>https://www.adzuna.de/land/ad/5851105442?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8F6135545B7E9C415844F10F4AF49C0BFA63A4B2</t>
         </is>
       </c>
     </row>
@@ -3041,7 +3037,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -3069,7 +3065,7 @@
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5851105442?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8F6135545B7E9C415844F10F4AF49C0BFA63A4B2</t>
+          <t>https://www.adzuna.de/land/ad/5848347180?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8A3F28529B6340B7DCCD5131E2C4472FBD8CA361</t>
         </is>
       </c>
     </row>
@@ -3085,7 +3081,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
+          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -3113,7 +3109,7 @@
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848347180?se=rlOKSDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8A3F28529B6340B7DCCD5131E2C4472FBD8CA361</t>
+          <t>https://www.adzuna.de/land/ad/5848315177?se=nioaTDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B01A57BB52C4BDBB1DF6554A4A21C913096E1D0</t>
         </is>
       </c>
     </row>
@@ -3129,7 +3125,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -3157,7 +3153,7 @@
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848315177?se=nioaTDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B01A57BB52C4BDBB1DF6554A4A21C913096E1D0</t>
+          <t>https://www.adzuna.de/land/ad/5848325009?se=nioaTDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8D26762D834367B41A848A3D14A62E41FD573B9B</t>
         </is>
       </c>
     </row>
@@ -3168,12 +3164,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Nahrungs- &amp; Genussmittel Karriere</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -3190,7 +3186,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
@@ -3201,7 +3197,7 @@
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848325009?se=nioaTDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8D26762D834367B41A848A3D14A62E41FD573B9B</t>
+          <t>https://www.adzuna.de/land/ad/5849209692?se=qJaID2Kc8RGlrvMe-VN8Yg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=6B8E6A551D4E75B7916A5994DC13A8DA3451895D</t>
         </is>
       </c>
     </row>
@@ -4326,67 +4322,71 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" t="inlineStr"/>
-      <c r="B86" t="n">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>NEU</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="n">
         <v>52</v>
       </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>Richemont</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t>Marketing and Merchandising Assistant Trainee</t>
-        </is>
-      </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>MILAN</t>
-        </is>
-      </c>
-      <c r="F86" t="inlineStr"/>
-      <c r="G86" t="inlineStr"/>
-      <c r="H86" t="inlineStr">
-        <is>
-          <t>fashion</t>
-        </is>
-      </c>
-      <c r="I86" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J86" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K86" t="inlineStr"/>
-      <c r="L86" t="inlineStr">
-        <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/MILAN/Marketing-and-Merchandising-Assistant-Trainee_JR128690</t>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>montamo GmbH</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr"/>
+      <c r="G86" s="2" t="inlineStr"/>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K86" s="2" t="inlineStr"/>
+      <c r="L86" s="2" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/land/ad/5871424623?se=gmRR3q-q8RGogquEo3zAlQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=453E406F424C8AB021346B1F246ACB2280C9B284</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr"/>
       <c r="B87" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Wonder Natural GmbH</t>
+          <t>Digitalagenten</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Operations (m/w/d)</t>
+          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Charlottenburg, Berlin</t>
         </is>
       </c>
       <c r="F87" t="inlineStr"/>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -4409,55 +4409,51 @@
       <c r="K87" t="inlineStr"/>
       <c r="L87" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5350026741?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804948828?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="2" t="inlineStr">
-        <is>
-          <t>NEU</t>
-        </is>
-      </c>
-      <c r="B88" s="2" t="n">
-        <v>52</v>
-      </c>
-      <c r="C88" s="2" t="inlineStr">
-        <is>
-          <t>montamo GmbH</t>
-        </is>
-      </c>
-      <c r="D88" s="2" t="inlineStr">
-        <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
-        </is>
-      </c>
-      <c r="E88" s="2" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F88" s="2" t="inlineStr"/>
-      <c r="G88" s="2" t="inlineStr"/>
-      <c r="H88" s="2" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I88" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
-      <c r="J88" s="2" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K88" s="2" t="inlineStr"/>
-      <c r="L88" s="2" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/land/ad/5871424623?se=gmRR3q-q8RGogquEo3zAlQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=453E406F424C8AB021346B1F246ACB2280C9B284</t>
+      <c r="A88" t="inlineStr"/>
+      <c r="B88" t="n">
+        <v>51</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>LIMITD by Wunderproducts GmbH</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Praktikum - Business Development (m/w/d)</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Kreuzberg, Berlin</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr"/>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>entdeckt</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr"/>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4468,21 +4464,25 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Digitalagenten</t>
+          <t>PricewaterhouseCoopers GmbH WPG</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Pflichtpraktikant Business Development, HR &amp; Office Management (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Charlottenburg, Berlin</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F89" t="inlineStr"/>
-      <c r="G89" t="inlineStr"/>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
       <c r="H89" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4501,7 +4501,7 @@
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804948828?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4512,21 +4512,25 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>LIMITD by Wunderproducts GmbH</t>
+          <t>SERVICEPLAN Gruppe</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Praktikum - Business Development (m/w/d)</t>
+          <t>Praktikum Business Development &amp; Sales (Marketing / New Business) (all genders)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Kreuzberg, Berlin</t>
+          <t>München, München (Kreis)</t>
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
-      <c r="G90" t="inlineStr"/>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H90" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4534,7 +4538,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -4545,7 +4549,7 @@
       <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5818261480?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4556,12 +4560,12 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>PricewaterhouseCoopers GmbH WPG</t>
+          <t>SERVICEPLAN Gruppe</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Marketing (w/m/d)</t>
+          <t>Praktikum Business Development, Marketing &amp; Sales (all genders)</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4572,7 +4576,7 @@
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -4582,7 +4586,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -4593,7 +4597,7 @@
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5630602276?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4604,25 +4608,21 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>SERVICEPLAN Gruppe</t>
+          <t>WirWinzer</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Sales (Marketing / New Business) (all genders)</t>
+          <t>Praktikum Business Development Weinhandel (all genders)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Altstadt-Lehel, München</t>
         </is>
       </c>
       <c r="F92" t="inlineStr"/>
-      <c r="G92" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4630,7 +4630,7 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
@@ -4641,36 +4641,32 @@
       <c r="K92" t="inlineStr"/>
       <c r="L92" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr"/>
       <c r="B93" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>SERVICEPLAN Gruppe</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Praktikum Business Development, Marketing &amp; Sales (all genders)</t>
+          <t>Praktikum Inside Sales (x/f/m)</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>München, München (Kreis)</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F93" t="inlineStr"/>
-      <c r="G93" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4678,7 +4674,7 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
@@ -4689,32 +4685,36 @@
       <c r="K93" t="inlineStr"/>
       <c r="L93" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5838464092?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7799489003</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr"/>
       <c r="B94" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>WirWinzer</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Praktikum Business Development Weinhandel (all genders)</t>
+          <t>Praktikum Human Resources  (x/f/m)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Altstadt-Lehel, München</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F94" t="inlineStr"/>
-      <c r="G94" t="inlineStr"/>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H94" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4722,7 +4722,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
@@ -4733,7 +4733,7 @@
       <c r="K94" t="inlineStr"/>
       <c r="L94" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5198895349?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7984297003</t>
         </is>
       </c>
     </row>
@@ -4744,29 +4744,29 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Praktikum Inside Sales (x/f/m)</t>
+          <t>Internship - High Jewelry Business Development Assistant</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
+          <t>PARIS</t>
         </is>
       </c>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fashion</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -4777,7 +4777,7 @@
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7799489003</t>
+          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
         </is>
       </c>
     </row>
@@ -4788,20 +4788,22 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>RÖDL</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Praktikum Human Resources  (x/f/m)</t>
+          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
-        </is>
-      </c>
-      <c r="F96" t="inlineStr"/>
+          <t>Stuttgart, Baden-Württemberg</t>
+        </is>
+      </c>
+      <c r="F96" t="n">
+        <v>6</v>
+      </c>
       <c r="G96" t="inlineStr">
         <is>
           <t>2026-10-01</t>
@@ -4814,7 +4816,7 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
@@ -4825,30 +4827,26 @@
       <c r="K96" t="inlineStr"/>
       <c r="L96" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7984297003</t>
+          <t>https://www.adzuna.de/land/ad/5854352066?se=9tCS70-g8RGkr9xW060fUg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DBAD57A9DC2B84BE2128168013A758C1F47DCD27</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr"/>
       <c r="B97" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>ABOUT YOU</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Internship - High Jewelry Business Development Assistant</t>
-        </is>
-      </c>
-      <c r="E97" t="inlineStr">
-        <is>
-          <t>PARIS</t>
-        </is>
-      </c>
+          <t>Intern Marketing &amp; GTM Strategy (all genders)Hamburg, Germany</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr"/>
       <c r="H97" t="inlineStr">
@@ -4858,7 +4856,7 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
@@ -4869,38 +4867,32 @@
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
-          <t>https://richemont.wd3.myworkdayjobs.com/broadbean_external/job/PARIS/Internship---High-Jewelry-Business-Development-Assistant_JR132227</t>
+          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-gtm-strategy-all-genders-hamburg-germany</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr"/>
       <c r="B98" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>RÖDL</t>
+          <t>Brand Trust</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Praktikum Marketing &amp; Business Development (m/w/d)</t>
+          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Stuttgart, Baden-Württemberg</t>
-        </is>
-      </c>
-      <c r="F98" t="n">
-        <v>6</v>
-      </c>
-      <c r="G98" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>Gleißbühl, Nürnberg</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr"/>
+      <c r="G98" t="inlineStr"/>
       <c r="H98" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -4908,7 +4900,7 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
@@ -4919,7 +4911,7 @@
       <c r="K98" t="inlineStr"/>
       <c r="L98" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5854352066?se=9tCS70-g8RGkr9xW060fUg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DBAD57A9DC2B84BE2128168013A758C1F47DCD27</t>
+          <t>https://www.adzuna.de/details/5669847401?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -4930,25 +4922,29 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>ABOUT YOU</t>
+          <t>Clarios Germany GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Intern Marketing &amp; GTM Strategy (all genders)Hamburg, Germany</t>
-        </is>
-      </c>
-      <c r="E99" t="inlineStr"/>
+          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Hannover, Region Hannover (Kreis)</t>
+        </is>
+      </c>
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr"/>
       <c r="H99" t="inlineStr">
         <is>
-          <t>fashion</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
@@ -4959,7 +4955,7 @@
       <c r="K99" t="inlineStr"/>
       <c r="L99" t="inlineStr">
         <is>
-          <t>https://corporate.aboutyou.de/en/career/jobs/intern-marketing-gtm-strategy-all-genders-hamburg-germany</t>
+          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
         </is>
       </c>
     </row>
@@ -4970,17 +4966,17 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Brand Trust</t>
+          <t>Clarios Germany GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management - Consulting Managementberatung (m/w/d)</t>
+          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Gleißbühl, Nürnberg</t>
+          <t>Bult, Hannover</t>
         </is>
       </c>
       <c r="F100" t="inlineStr"/>
@@ -4992,7 +4988,7 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
@@ -5003,7 +4999,7 @@
       <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5669847401?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5867940737?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5014,17 +5010,17 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Clarios Germany GmbH &amp; Co. KG</t>
+          <t>Codeso Living</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
+          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Hannover, Region Hannover (Kreis)</t>
+          <t>Unterbilk, Düsseldorf</t>
         </is>
       </c>
       <c r="F101" t="inlineStr"/>
@@ -5036,7 +5032,7 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
@@ -5047,7 +5043,7 @@
       <c r="K101" t="inlineStr"/>
       <c r="L101" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5863103277?se=cHct3_Sl8RGGYI73n1NTOA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=8215B1B43E9B962681510343497F2E51686F98B2</t>
+          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5058,19 +5054,15 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Clarios Germany GmbH &amp; Co. KG</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Praktikant (m/w/d) im Bereich Trade Marketing DACH</t>
-        </is>
-      </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>Bult, Hannover</t>
-        </is>
-      </c>
+          <t>Marketing Intern - Trade Marketing</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr"/>
       <c r="H102" t="inlineStr">
@@ -5080,7 +5072,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -5091,7 +5083,7 @@
       <c r="K102" t="inlineStr"/>
       <c r="L102" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5867940737?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
         </is>
       </c>
     </row>
@@ -5102,17 +5094,17 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Codeso Living</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Praktikum Online Marketing &amp; E-Commerce (w/m/d)</t>
+          <t>Praktikum B2B Event Marketing (x/f/m)</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Unterbilk, Düsseldorf</t>
+          <t>Berlin, Berlin, Germany</t>
         </is>
       </c>
       <c r="F103" t="inlineStr"/>
@@ -5124,7 +5116,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -5135,7 +5127,7 @@
       <c r="K103" t="inlineStr"/>
       <c r="L103" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5859740097?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7820455003</t>
         </is>
       </c>
     </row>
@@ -5146,15 +5138,19 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Marketing Intern - Trade Marketing</t>
-        </is>
-      </c>
-      <c r="E104" t="inlineStr"/>
+          <t>Go To Market Strategy Hospitals (x/f/m)</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Berlin, Berlin, Germany</t>
+        </is>
+      </c>
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr"/>
       <c r="H104" t="inlineStr">
@@ -5164,7 +5160,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -5175,7 +5171,7 @@
       <c r="K104" t="inlineStr"/>
       <c r="L104" t="inlineStr">
         <is>
-          <t>https://careers.coty.com/job/Darmstadt-Marketing-Intern-Trade-Marketing-HE-64295/1400261133/</t>
+          <t>https://job-boards.greenhouse.io/doctolib/jobs/7971471003</t>
         </is>
       </c>
     </row>
@@ -5186,17 +5182,17 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Genuine Parts Company</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Praktikum B2B Event Marketing (x/f/m)</t>
+          <t>Praktikum Category Management (m/w/d)</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
+          <t>Münster, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F105" t="inlineStr"/>
@@ -5208,7 +5204,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
@@ -5219,7 +5215,7 @@
       <c r="K105" t="inlineStr"/>
       <c r="L105" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7820455003</t>
+          <t>https://www.adzuna.de/details/5853760166?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5230,17 +5226,17 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Honest Catch</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Go To Market Strategy Hospitals (x/f/m)</t>
+          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
+          <t>Schwabing-Freimann, München</t>
         </is>
       </c>
       <c r="F106" t="inlineStr"/>
@@ -5252,7 +5248,7 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J106" t="inlineStr">
@@ -5263,7 +5259,7 @@
       <c r="K106" t="inlineStr"/>
       <c r="L106" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/doctolib/jobs/7971471003</t>
+          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5274,29 +5270,29 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Genuine Parts Company</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Praktikum Category Management (m/w/d)</t>
+          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Münster, Nordrhein-Westfalen</t>
+          <t>DEU-Bayern-Unterhaching</t>
         </is>
       </c>
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr"/>
       <c r="H107" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
@@ -5307,7 +5303,7 @@
       <c r="K107" t="inlineStr"/>
       <c r="L107" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853760166?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
         </is>
       </c>
     </row>
@@ -5318,29 +5314,29 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Honest Catch</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Praktikum E-Commerce &amp; Marketing (m/w/d)</t>
+          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Schwabing-Freimann, München</t>
+          <t>2 Standorte</t>
         </is>
       </c>
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr"/>
       <c r="H108" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
@@ -5351,7 +5347,7 @@
       <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5727345086?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
         </is>
       </c>
     </row>
@@ -5362,24 +5358,24 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Molkerei A.Müller GmbH&amp;Co</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Intern Brand Marketing Gum&amp;Mints Portfolio</t>
+          <t>Praktikum Trade Marketing &amp; Category Management</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>DEU-Bayern-Unterhaching</t>
+          <t>Fischach, Augsburg (Kreis)</t>
         </is>
       </c>
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr"/>
       <c r="H109" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -5395,7 +5391,7 @@
       <c r="K109" t="inlineStr"/>
       <c r="L109" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Bayern-Unterhaching/Intern-Brand-Marketing-Gum-Mints-Portfolio_R160981-1</t>
+          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5406,29 +5402,29 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Summer 2027 Mars Snacking MBA Marketing and Brand Management Internship</t>
+          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>2 Standorte</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
@@ -5439,7 +5435,7 @@
       <c r="K110" t="inlineStr"/>
       <c r="L110" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/USA-Illinois-Chicago/Summer-2027-Mars-Snacking-MBA-Marketing-and-Brand-Management-Internship_R152836-1</t>
+          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
         </is>
       </c>
     </row>
@@ -5450,17 +5446,17 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Molkerei A.Müller GmbH&amp;Co</t>
+          <t>PEPSICO DEUTSCHLAND GMBH</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Praktikum Trade Marketing &amp; Category Management</t>
+          <t>Praktikum Brand Management Snacks (m/w/d)</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Fischach, Augsburg (Kreis)</t>
+          <t>Neu-Isenburg, Offenbach (Kreis)</t>
         </is>
       </c>
       <c r="F111" t="inlineStr"/>
@@ -5483,7 +5479,7 @@
       <c r="K111" t="inlineStr"/>
       <c r="L111" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5811751898?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
         </is>
       </c>
     </row>
@@ -5499,7 +5495,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Carbonated Soft Drinks (m/w/d)</t>
+          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -5527,7 +5523,7 @@
       <c r="K112" t="inlineStr"/>
       <c r="L112" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5826399222?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FB3613C8F86AA7B6ED71C39D94BF8376129100A</t>
+          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
         </is>
       </c>
     </row>
@@ -5538,17 +5534,17 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>Procter &amp; Gamble</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Snacks (m/w/d)</t>
+          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
         </is>
       </c>
       <c r="F113" t="inlineStr"/>
@@ -5571,7 +5567,7 @@
       <c r="K113" t="inlineStr"/>
       <c r="L113" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5818522668?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=104C2D280C31290047D8390DB2FF091D02938FF9</t>
+          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5582,17 +5578,17 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>PEPSICO DEUTSCHLAND GMBH</t>
+          <t>RAG</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management Rockstar Energy (m/w/d)</t>
+          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Neu-Isenburg, Offenbach (Kreis)</t>
+          <t>Gornhofen, Ravensburg</t>
         </is>
       </c>
       <c r="F114" t="inlineStr"/>
@@ -5604,7 +5600,7 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
@@ -5615,28 +5611,28 @@
       <c r="K114" t="inlineStr"/>
       <c r="L114" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5828401052?se=DkDUl2eQ8RGLwZkdgahNug&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=59C0F55727CD16CD2B3635C4136676B5D7BB1A17</t>
+          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr"/>
       <c r="B115" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Procter &amp; Gamble</t>
+          <t>Konzernzentrale</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Double Internship - Sales &amp; Brand Management (m/f/d)</t>
+          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Schwalbach am Taunus, Main-Taunus-Kreis</t>
+          <t>Braunsfeld, Köln</t>
         </is>
       </c>
       <c r="F115" t="inlineStr"/>
@@ -5648,7 +5644,7 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
@@ -5659,28 +5655,28 @@
       <c r="K115" t="inlineStr"/>
       <c r="L115" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5680986556?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5864351176?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr"/>
       <c r="B116" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>RAG</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Praktikum Internationales Trade Marketing (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Gornhofen, Ravensburg</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F116" t="inlineStr"/>
@@ -5692,7 +5688,7 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
@@ -5703,28 +5699,28 @@
       <c r="K116" t="inlineStr"/>
       <c r="L116" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5853715081?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr"/>
       <c r="B117" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Konzernzentrale</t>
+          <t>SUPA - Sport Und Party App</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Initiativbewerbung Trainee Einkauf (m/w/d)</t>
+          <t>Business Development Praktikum</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Altstadt-Nord, Köln</t>
         </is>
       </c>
       <c r="F117" t="inlineStr"/>
@@ -5736,7 +5732,7 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
@@ -5747,28 +5743,28 @@
       <c r="K117" t="inlineStr"/>
       <c r="L117" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5864351176?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr"/>
       <c r="B118" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>freudio</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
+          <t>Wien, Österreich</t>
         </is>
       </c>
       <c r="F118" t="inlineStr"/>
@@ -5780,7 +5776,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
@@ -5791,28 +5787,28 @@
       <c r="K118" t="inlineStr"/>
       <c r="L118" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802971085?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.at/details/5836667156?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr"/>
       <c r="B119" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>SUPA - Sport Und Party App</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Business Development Praktikum</t>
+          <t>Praktikum Business Development/ Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Altstadt-Nord, Köln</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F119" t="inlineStr"/>
@@ -5835,7 +5831,7 @@
       <c r="K119" t="inlineStr"/>
       <c r="L119" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804561224?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5846,17 +5842,17 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>freudio</t>
+          <t>prepmymeal GmbH</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Founder's Associate - Business Development (Vollzeit/Praktikum/Studienbegleitend)</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Wien, Österreich</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F120" t="inlineStr"/>
@@ -5868,7 +5864,7 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
@@ -5879,7 +5875,7 @@
       <c r="K120" t="inlineStr"/>
       <c r="L120" t="inlineStr">
         <is>
-          <t>https://www.adzuna.at/details/5836667156?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5900,7 +5896,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F121" t="inlineStr"/>
@@ -5923,7 +5919,7 @@
       <c r="K121" t="inlineStr"/>
       <c r="L121" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802957658?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5944,7 +5940,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F122" t="inlineStr"/>
@@ -5967,7 +5963,7 @@
       <c r="K122" t="inlineStr"/>
       <c r="L122" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802966683?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -5983,12 +5979,12 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Praktikum Business Development/ Sales (m/w/d)</t>
+          <t>Praktikum Business Development (Französisch) (m/w/d) - In 3 Minuten erfolgreich bewerben</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F123" t="inlineStr"/>
@@ -6000,7 +5996,7 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
@@ -6011,7 +6007,7 @@
       <c r="K123" t="inlineStr"/>
       <c r="L123" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804543221?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5856292292?se=PMRjVxmh8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DF242745B4142F9871F0353F9B390FD5166A63B5</t>
         </is>
       </c>
     </row>
@@ -6022,17 +6018,17 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>sailwithus</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d)</t>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Altstadt, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F124" t="inlineStr"/>
@@ -6055,7 +6051,7 @@
       <c r="K124" t="inlineStr"/>
       <c r="L124" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804557902?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -6066,17 +6062,17 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>prepmymeal GmbH</t>
+          <t>sailwithus</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Praktikum Business Development (Französisch) (m/w/d) - In 3 Minuten erfolgreich bewerben</t>
+          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Altstadt, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F125" t="inlineStr"/>
@@ -6088,7 +6084,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
@@ -6099,100 +6095,12 @@
       <c r="K125" t="inlineStr"/>
       <c r="L125" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5856292292?se=PMRjVxmh8RG7j7TsS0oVjg&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DF242745B4142F9871F0353F9B390FD5166A63B5</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr"/>
-      <c r="B126" t="n">
-        <v>45</v>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>sailwithus</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
-        </is>
-      </c>
-      <c r="E126" t="inlineStr">
-        <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F126" t="inlineStr"/>
-      <c r="G126" t="inlineStr"/>
-      <c r="H126" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I126" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J126" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K126" t="inlineStr"/>
-      <c r="L126" t="inlineStr">
-        <is>
-          <t>https://www.adzuna.de/details/5802958025?utm_medium=api&amp;utm_source=e1fd92a2</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr"/>
-      <c r="B127" t="n">
-        <v>45</v>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>sailwithus</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr">
-        <is>
-          <t>Praktikum Pflichtpraktikum Business Development (m/w/d) in Frankfurt nach Absprache</t>
-        </is>
-      </c>
-      <c r="E127" t="inlineStr">
-        <is>
-          <t>Altstadt, Frankfurt am Main</t>
-        </is>
-      </c>
-      <c r="F127" t="inlineStr"/>
-      <c r="G127" t="inlineStr"/>
-      <c r="H127" t="inlineStr">
-        <is>
-          <t>entdeckt</t>
-        </is>
-      </c>
-      <c r="I127" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J127" t="inlineStr">
-        <is>
-          <t>neu</t>
-        </is>
-      </c>
-      <c r="K127" t="inlineStr"/>
-      <c r="L127" t="inlineStr">
-        <is>
           <t>https://www.adzuna.de/details/5804544237?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L127"/>
+  <autoFilter ref="A1:L125"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6259,7 +6167,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="C2" t="n">
         <v>109</v>
@@ -6334,7 +6242,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C5" t="n">
         <v>89</v>
@@ -6384,7 +6292,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C7" t="n">
         <v>87</v>
@@ -6409,7 +6317,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="C8" t="n">
         <v>84</v>
@@ -6434,7 +6342,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C9" t="n">
         <v>84</v>
@@ -6459,7 +6367,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C10" t="n">
         <v>84</v>
@@ -6492,7 +6400,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="C11" t="n">
         <v>84</v>
@@ -6525,7 +6433,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C12" t="n">
         <v>84</v>
@@ -6550,7 +6458,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C13" t="n">
         <v>84</v>
@@ -6575,7 +6483,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C14" t="n">
         <v>84</v>
@@ -6600,7 +6508,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C15" t="n">
         <v>84</v>
@@ -6625,7 +6533,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C16" t="n">
         <v>84</v>
@@ -6700,7 +6608,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C19" t="n">
         <v>83</v>
@@ -6733,7 +6641,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C20" t="n">
         <v>80</v>
@@ -6758,7 +6666,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C21" t="n">
         <v>79</v>
@@ -6833,7 +6741,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C24" t="n">
         <v>78</v>
@@ -6858,7 +6766,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C25" t="n">
         <v>78</v>
@@ -6883,7 +6791,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C26" t="n">
         <v>74</v>
@@ -6916,7 +6824,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C27" t="n">
         <v>74</v>
@@ -6966,7 +6874,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C29" t="n">
         <v>73</v>
@@ -7024,7 +6932,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C31" t="n">
         <v>73</v>
@@ -7049,7 +6957,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="C32" t="n">
         <v>72</v>
@@ -7074,7 +6982,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C33" t="n">
         <v>72</v>
@@ -7149,7 +7057,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C36" t="n">
         <v>68</v>
@@ -7224,7 +7132,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C39" t="n">
         <v>66</v>
@@ -7249,7 +7157,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C40" t="n">
         <v>65</v>
@@ -7274,7 +7182,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C41" t="n">
         <v>64</v>
@@ -7299,7 +7207,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C42" t="n">
         <v>62</v>
@@ -7324,7 +7232,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C43" t="n">
         <v>62</v>
@@ -7357,7 +7265,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C44" t="n">
         <v>62</v>
@@ -7382,7 +7290,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="C45" t="n">
         <v>59</v>
@@ -7432,7 +7340,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C47" t="n">
         <v>57</v>
@@ -7465,7 +7373,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C48" t="n">
         <v>56</v>
@@ -7490,7 +7398,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C49" t="n">
         <v>55</v>
@@ -7565,7 +7473,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="C52" t="n">
         <v>53</v>
@@ -7590,7 +7498,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C53" t="n">
         <v>53</v>
@@ -7640,7 +7548,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C55" t="n">
         <v>52</v>
@@ -7665,7 +7573,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C56" t="n">
         <v>52</v>
@@ -7765,7 +7673,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C60" t="n">
         <v>50</v>
@@ -7790,7 +7698,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C61" t="n">
         <v>49</v>
@@ -7815,7 +7723,7 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C62" t="n">
         <v>49</v>
@@ -7840,7 +7748,7 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C63" t="n">
         <v>49</v>
@@ -7890,7 +7798,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C65" t="n">
         <v>49</v>
@@ -7915,7 +7823,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C66" t="n">
         <v>49</v>
@@ -7940,7 +7848,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C67" t="n">
         <v>49</v>
@@ -7965,7 +7873,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C68" t="n">
         <v>49</v>
@@ -7990,7 +7898,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C69" t="n">
         <v>49</v>
@@ -8065,7 +7973,7 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C72" t="n">
         <v>48</v>
@@ -8440,7 +8348,7 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C87" t="n">
         <v>46</v>

</xml_diff>

<commit_message>
Lauf 2026-09-10 10:47 UTC
</commit_message>
<xml_diff>
--- a/docs/praktika.xlsx
+++ b/docs/praktika.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Firmen entdeckt" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$118</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$105</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Treffer'!$A$1:$L$119</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Firmen entdeckt'!$A$1:$G$106</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L118"/>
+  <dimension ref="A1:L119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -614,21 +614,21 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>FC Viktoria 1889 Berlin Frauen-Fußball GmbH</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>PRAKTIKUM // Business Development</t>
+          <t>Praktikum Product Marketing (x/f/m)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Mitte, Berlin</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
@@ -638,7 +638,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -649,7 +649,7 @@
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802962068?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5842051017?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -660,27 +660,23 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>FC Viktoria 1889 Berlin Frauen-Fußball GmbH</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
+          <t>PRAKTIKUM // Business Development</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Mitte, Berlin</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>5</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -688,7 +684,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -699,7 +695,7 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5858231617?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802962068?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -710,7 +706,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Nestle Deutschland</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -720,7 +716,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -733,12 +729,12 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -749,7 +745,7 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Category-Management%2C-Brand-Activation-und-Sales-%28mwd%29-60329/1427883433/</t>
+          <t>https://www.adzuna.de/details/5858231617?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -760,31 +756,35 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Nestle Deutschland</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Category Management, Brand Activation und Sales (m/w/d)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Hamburg-Altstadt, Hamburg</t>
+          <t>Frankfurt am Main, DE, 60329</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>6</v>
-      </c>
-      <c r="G7" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -795,7 +795,7 @@
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5829732882?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://jobdetails.nestle.com/job/Frankfurt-am-Main-Praktikum-Category-Management%2C-Brand-Activation-und-Sales-%28mwd%29-60329/1427883433/</t>
         </is>
       </c>
     </row>
@@ -811,7 +811,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -830,7 +830,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -841,7 +841,7 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5865920988?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5829732882?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -857,12 +857,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Barmbek-Süd, Hamburg</t>
+          <t>Hamburg-Altstadt, Hamburg</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -876,7 +876,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -887,7 +887,7 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5867772905?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5865920988?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -898,17 +898,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Picnic</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Category Management Praktikum (m/w/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Barmbek-Süd, Hamburg</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -922,7 +922,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -933,36 +933,34 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5867772905?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="n">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
+          <t>Picnic</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management National</t>
+          <t>Category Management Praktikum (m/w/d)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Au-Haidhausen, München</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
+          <t>Hamburg, Deutschland</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>6</v>
+      </c>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -981,38 +979,34 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805399065?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5797390477?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="n">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Ferrero</t>
+          <t>Picnic</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Category Management Praktikum (m/w/d)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F12" t="n">
         <v>6</v>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1031,34 +1025,36 @@
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759088383?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Ferrero</t>
+          <t>Paulaner Brauerei Gruppe Sales &amp; Marketing</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikum Brand Management National</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F13" t="n">
-        <v>6</v>
-      </c>
-      <c r="G13" t="inlineStr"/>
+          <t>Au-Haidhausen, München</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1077,7 +1073,7 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805399065?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1088,23 +1084,27 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>L'Occitane</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Praktikum (m/w/d) Trade Marketing</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Friedrichstadt, Düsseldorf</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F14" t="n">
         <v>6</v>
       </c>
-      <c r="G14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1112,7 +1112,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1123,7 +1123,7 @@
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5842049264?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907198?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1134,27 +1134,23 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Nespresso Deutschland GmbH</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Bahnhofsviertel, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F15" t="n">
         <v>6</v>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1173,7 +1169,7 @@
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5759907162?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1180,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Nestle</t>
+          <t>L'Occitane</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Praktikum Brand Management (m/w/d(</t>
+          <t>Praktikum (m/w/d) Trade Marketing</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, DE, 60329</t>
+          <t>Friedrichstadt, Düsseldorf</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -1208,7 +1204,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1219,32 +1215,38 @@
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5842049264?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>Nespresso Deutschland GmbH</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
+          <t>Bahnhofsviertel, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>6</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
       <c r="H17" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1252,7 +1254,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1263,31 +1265,33 @@
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5843630960?se=znNqlDyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=875B574D03DFD36B16B3A3ABE0AA46F858215182</t>
+          <t>https://www.adzuna.de/details/5802899677?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>FERRERO MSC GmbH &amp; Co. KG</t>
+          <t>Nestle</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
+          <t>Praktikum Brand Management (m/w/d(</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Frankfurt am Main, Hessen</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr"/>
+          <t>Frankfurt am Main, DE, 60329</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>6</v>
+      </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
@@ -1296,7 +1300,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1307,7 +1311,7 @@
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5843628966?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=3DAF9A0A7032477BEFBE4DD229577F81F1D32CF0</t>
+          <t>https://www.adzuna.de/details/5798579537?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1323,7 +1327,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Praktikant Trade Marketing (w/m/d)</t>
+          <t>Praktikant Category Management &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1351,7 +1355,7 @@
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5843628932?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=65C46D18FCDB11FD2E933BD305E494E07D043D72</t>
+          <t>https://www.adzuna.de/land/ad/5843630960?se=znNqlDyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=875B574D03DFD36B16B3A3ABE0AA46F858215182</t>
         </is>
       </c>
     </row>
@@ -1362,27 +1366,21 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>HUGO BOSS</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Internship Buying &amp; Planning - Global Merchandising (m/f/d)</t>
+          <t>Praktikant Trade Marketing - Innovation &amp; Shopper Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Metzingen, Reutlingen (Kreis)</t>
-        </is>
-      </c>
-      <c r="F20" t="n">
-        <v>6</v>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+          <t>Frankfurt am Main, Hessen</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1390,7 +1388,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1401,7 +1399,7 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5856159470?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5843628966?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=3DAF9A0A7032477BEFBE4DD229577F81F1D32CF0</t>
         </is>
       </c>
     </row>
@@ -1412,17 +1410,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Miles &amp; More GmbH</t>
+          <t>FERRERO MSC GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Internship Marketing Strategy &amp; Delivery</t>
+          <t>Praktikant Trade Marketing (w/m/d)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Flughafen, Frankfurt am Main</t>
+          <t>Frankfurt am Main, Hessen</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
@@ -1434,7 +1432,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -1445,34 +1443,38 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5828674997?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5843628932?se=qGM2lTyZ8RGH5-2hxadZjA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=65C46D18FCDB11FD2E933BD305E494E07D043D72</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr"/>
       <c r="B22" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>HUGO BOSS</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Praktikum Business Development &amp; Talent Partnerships (m/w/d)</t>
+          <t>Internship Buying &amp; Planning - Global Merchandising (m/f/d)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Metzingen, Reutlingen (Kreis)</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>5</v>
-      </c>
-      <c r="G22" t="inlineStr"/>
+        <v>6</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -1480,7 +1482,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1491,33 +1493,31 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5851100606?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5856159470?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>Miles &amp; More GmbH</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Praktikum im B2B-Vertrieb &amp; Business Development (m/w/d)</t>
+          <t>Internship Marketing Strategy &amp; Delivery</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
-        </is>
-      </c>
-      <c r="F23" t="n">
-        <v>5</v>
-      </c>
+          <t>Flughafen, Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
@@ -1526,7 +1526,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1537,7 +1537,7 @@
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5851898375?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5828674997?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -1548,21 +1548,21 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>markenbaumarkt24</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
+          <t>Praktikum Business Development &amp; Talent Partnerships (m/w/d)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Feuersbach, Siegen</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
@@ -1572,7 +1572,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -1583,31 +1583,33 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5851100606?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>PARSA Haar- und Modeartikel GmbH</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
+          <t>Praktikum im B2B-Vertrieb &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr"/>
+          <t>Düsseltal, Düsseldorf</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>5</v>
+      </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
@@ -1616,7 +1618,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -1627,31 +1629,33 @@
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
+          <t>https://www.adzuna.de/details/5851898375?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
       <c r="B26" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>markenbaumarkt24</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Praktikum Product Marketing (x/f/m)</t>
+          <t>Praktikum im E-Commerce: Vertrieb &amp; Online Marketing</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Berlin, Berlin, Germany</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr"/>
+          <t>Feuersbach, Siegen</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>2</v>
+      </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
@@ -1660,7 +1664,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -1671,23 +1675,23 @@
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5842051017?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5357624909?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Groß- &amp; Einzelhandel Karriere</t>
+          <t>PARSA Haar- und Modeartikel GmbH</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Praktikum Marketing | Brand Management &amp; Unternehmenskommunikation (m/w/d)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1704,7 +1708,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -1715,7 +1719,7 @@
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5848300231?se=1ucgSzui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=BF61BDCA3F28DD382163849647345A68CC617C45</t>
+          <t>https://www.adzuna.de/land/ad/5803505649?se=pJ2M1PSS8RGmkIYMEaL09g&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=CA862AD7625CBBB2DC0F4C6FE9C15D94665B9158</t>
         </is>
       </c>
     </row>
@@ -1726,7 +1730,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Otto GmbH &amp; Co. KGaA</t>
+          <t>Groß- &amp; Einzelhandel Karriere</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1736,7 +1740,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Hamburg, Deutschland</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="F28" t="inlineStr"/>
@@ -1748,7 +1752,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -1759,7 +1763,7 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
+          <t>https://www.adzuna.de/land/ad/5848300231?se=1ucgSzui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=BF61BDCA3F28DD382163849647345A68CC617C45</t>
         </is>
       </c>
     </row>
@@ -1775,7 +1779,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1792,7 +1796,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -1803,7 +1807,7 @@
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5859954968?se=avT3yguj8RGEeLI7Dotn4Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FEC8C1664463BB6D76B4F51C80D7BE9A67B3E95</t>
+          <t>https://www.adzuna.de/land/ad/5824205429?se=FKokm2eQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=A5DADCE1B254FED787BA48C9712705406358AC57</t>
         </is>
       </c>
     </row>
@@ -1824,7 +1828,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
@@ -1836,7 +1840,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -1847,7 +1851,7 @@
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5864785114?se=tDVxHrqm8RG47MvhImrnRA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=ABFCC49076160E6370E149C31FFE29D13C38563D</t>
+          <t>https://www.adzuna.de/land/ad/5859954968?se=avT3yguj8RGEeLI7Dotn4Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=0FEC8C1664463BB6D76B4F51C80D7BE9A67B3E95</t>
         </is>
       </c>
     </row>
@@ -1863,7 +1867,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Stepstone geprüft - Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
+          <t>Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1880,7 +1884,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -1891,7 +1895,7 @@
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5868159571?se=Ur2Ws4On8RGeD7WukCg86Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD828F897C614DE600F1B21C5501265E349B7241</t>
+          <t>https://www.adzuna.de/land/ad/5864785114?se=tDVxHrqm8RG47MvhImrnRA&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=ABFCC49076160E6370E149C31FFE29D13C38563D</t>
         </is>
       </c>
     </row>
@@ -1907,7 +1911,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Stepstone geprüft - Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
+          <t>Stepstone geprüft - Praktikum Category Management | Sortimente Notebook, PC, Drucker, Monitore, SmartHome und IT-Zubehör (w/m/d)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1935,33 +1939,31 @@
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5868159685?se=Ur2Ws4On8RGeD7WukCg86Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DA869B4EFE837366B3946FD4F30C27AACFC1FE6D</t>
+          <t>https://www.adzuna.de/land/ad/5868159571?se=Ur2Ws4On8RGeD7WukCg86Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DD828F897C614DE600F1B21C5501265E349B7241</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr"/>
       <c r="B33" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Barilla</t>
+          <t>Otto GmbH &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
+          <t>Stepstone geprüft - Praktikum Einkauf | Category Management Bedding (w/m/d)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Köln, Nordrhein-Westfalen</t>
-        </is>
-      </c>
-      <c r="F33" t="n">
-        <v>6</v>
-      </c>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
@@ -1970,7 +1972,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -1981,7 +1983,7 @@
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5868159685?se=Ur2Ws4On8RGeD7WukCg86Q&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=DA869B4EFE837366B3946FD4F30C27AACFC1FE6D</t>
         </is>
       </c>
     </row>
@@ -1997,7 +1999,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
+          <t>Praktikum im Trade Marketing - Barilla Pasta</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2027,7 +2029,7 @@
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5795117090?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2043,7 +2045,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
+          <t>Praktikum im Trade Marketing - Barilla Pesto</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2054,11 +2056,7 @@
       <c r="F35" t="n">
         <v>6</v>
       </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
+      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
           <t>entdeckt</t>
@@ -2077,7 +2075,7 @@
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5805819284?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2088,17 +2086,17 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>PENNY International</t>
+          <t>Barilla</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
+          <t>Praktikum im Trade Marketing - Brand Barilla Food Services</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Braunsfeld, Köln</t>
+          <t>Köln, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -2106,7 +2104,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -2127,40 +2125,46 @@
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5790607767?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>PENNY International</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Internship in Trade Marketing</t>
+          <t>Praktikum Category Management / Einkauf International Trockensortiment (m/w/d)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>DEU-Nordrhein-Westfalen-Köln</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
+          <t>Braunsfeld, Köln</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>6</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2026-11-01</t>
+        </is>
+      </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>fmcg</t>
+          <t>entdeckt</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -2171,40 +2175,40 @@
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
-          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
+          <t>https://www.adzuna.de/details/5796260359?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>CRAVIES GmbH</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Internship in Trade Marketing</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Düsseldorf, Nordrhein-Westfalen</t>
+          <t>DEU-Nordrhein-Westfalen-Köln</t>
         </is>
       </c>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
-          <t>entdeckt</t>
+          <t>fmcg</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -2215,7 +2219,7 @@
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://mars.wd3.myworkdayjobs.com/External/job/DEU-Nordrhein-Westfalen-Kln/Internship-in-Trade-Marketing_R163385-1</t>
         </is>
       </c>
     </row>
@@ -2236,7 +2240,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Altstadt, Düsseldorf</t>
+          <t>Düsseldorf, Nordrhein-Westfalen</t>
         </is>
       </c>
       <c r="F39" t="inlineStr"/>
@@ -2259,7 +2263,7 @@
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5802953160?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2270,17 +2274,17 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Calypso Ventures GmbH</t>
+          <t>CRAVIES GmbH</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
+          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Altstadt, Düsseldorf</t>
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
@@ -2303,7 +2307,7 @@
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5804552463?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2314,17 +2318,17 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Exclusive Associates</t>
+          <t>Calypso Ventures GmbH</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Business Development Manager Praktikum - Künstliche Intelligenz</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Düsseltal, Düsseldorf</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
@@ -2347,7 +2351,7 @@
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5752979910?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2363,7 +2367,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
+          <t>Praktikum B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2380,7 +2384,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -2391,7 +2395,7 @@
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5813913108?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2407,7 +2411,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Praktikum im Sales &amp; Business Development – B2B (m/w/d)</t>
+          <t>Praktikum im Bereich B2B Sales &amp; Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2424,7 +2428,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -2435,7 +2439,7 @@
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5866225907?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5846892540?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2451,7 +2455,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Sales &amp; Business Development Praktikum B2B (m/w/d)</t>
+          <t>Praktikum im Sales &amp; Business Development – B2B (m/w/d)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2468,7 +2472,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -2479,7 +2483,7 @@
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5871334687?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/details/5866225907?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2490,17 +2494,17 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>montamo GmbH</t>
+          <t>Exclusive Associates</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Praktikum Sales &amp; Business Development (m/w/d)</t>
+          <t>Sales &amp; Business Development Praktikum B2B (m/w/d)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Berlin, Deutschland</t>
+          <t>Düsseltal, Düsseldorf</t>
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
@@ -2512,7 +2516,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -2523,7 +2527,7 @@
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/land/ad/5856889494?se=1M-3UDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=471483726C1FC3DB660B48A5B3DEDE0DC1A4DC20</t>
+          <t>https://www.adzuna.de/details/5871334687?utm_medium=api&amp;utm_source=e1fd92a2</t>
         </is>
       </c>
     </row>
@@ -2544,7 +2548,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Wedding, Berlin</t>
+          <t>Berlin, Deutschland</t>
         </is>
       </c>
       <c r="F46" t="inlineStr"/>
@@ -2567,28 +2571,28 @@
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr">
         <is>
-          <t>https://www.adzuna.de/details/5857559039?utm_medium=api&amp;utm_source=e1fd92a2</t>
+          <t>https://www.adzuna.de/land/ad/5856889494?se=1M-3UDui8RGJ35lZBgd8oQ&amp;utm_medium=api&amp;utm_source=e1fd92a2&amp;v=471483726C1FC3DB660B48A5B3DEDE0DC1A4DC20</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr"/>
       <c r="B47" t="n">
-  